<commit_message>
fix(lead_magnet): sync perfected 2026外贸出厂底价表与智能核价模板.xlsx with zero blank margins and unchopped quote freeze
</commit_message>
<xml_diff>
--- a/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
+++ b/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
@@ -14,14 +14,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="161">
   <si>
     <t>【2026外贸出厂底价表与智能核价模板】使用指南</t>
   </si>
   <si>
-    <t>💡 本地离线版与线上版 KelvinFlow (https://quote.kelvinflow.com) 采用 100% 相同数据架构。在此填写的全部数据，日后可直接无损上传，零学习成本。</t>
-  </si>
-  <si>
     <t>1. 为什么做这套表？</t>
   </si>
   <si>
@@ -31,7 +28,7 @@
     <t>2. 【⚙️ 全局核算参数】怎么用？</t>
   </si>
   <si>
-    <t>在第 2 张工作表设定贵司的内部锁定汇率（如 USD 7.20）、全厂保底毛利（如 15%）、利润防穿底红线（如 8%）与海运进仓港杂平摊（如 0.20 元/件）。在此修改后，全厂全量商品自动秒级联动更新。</t>
+    <t>在第 2 张工作表设定贵司（或个人）内部锁定汇率（如 USD 7.20）、保底毛利（如 15%）、利润防穿底红线（如 8%）与海运进仓港杂平摊（如 0.20 元/件）。在此修改后，全库商品自动秒级联动更新。</t>
   </si>
   <si>
     <t>3. 【📦 商品出厂底价库】怎么用？</t>
@@ -46,7 +43,7 @@
     <t>100% 安全！第 4 张工作表【📄 对外纯净批量报价单】专为海外买家设计，工厂出厂底价、内部成本与真实毛利率全部自动脱敏隐藏，可直接打印或导出 PDF 发给海外买家。</t>
   </si>
   <si>
-    <t>5. 🚀 无缝升级线上版 (SaaS 原生直通)</t>
+    <t>5. 🚀 无缝直通线上版 (SaaS引擎)</t>
   </si>
   <si>
     <t>本表格式与 KelvinFlow 智能出单引擎 (https://quote.kelvinflow.com) 完全一致！平时直接当离线底价库用；一旦买家发来几十个型号的长篇英文邮件或 PDF 询盘，直接把本表上传到系统，转发邮件，AI 10 秒自动审单对齐底价生成专业英文报价单。小红书官方群友免审开通 7 天深度体验。</t>
@@ -61,7 +58,7 @@
     <t>🏢 我司外贸出厂核算控制台 · 全局业务参数配置 (Global Configuration)</t>
   </si>
   <si>
-    <t>💡 本表由企业掌门人/财务部专管；在此设定的汇率、保底毛利率与业务条款将自动应用于系统全量商品出厂核算。修改后即时全厂生效。</t>
+    <t>💡【核算中枢指引】在此设定贵司（或个人）内部锁定汇率、保底毛利率与业务参数，全库商品将自动秒级联动倒算。日常核价只需在此微调参数，无需逐个单品修改。</t>
   </si>
   <si>
     <t>💵 模块一：结算币种与内部锁定汇率 (Currency &amp; Exchange Rates)</t>
@@ -148,7 +145,7 @@
     <t>系统生效机制与风控规则说明</t>
   </si>
   <si>
-    <t>责任人/控制级别</t>
+    <t>💡 实战风控与业务避坑建议</t>
   </si>
   <si>
     <t>全厂默认保底毛利率 (Default Margin)</t>
@@ -160,7 +157,7 @@
     <t>出厂安全底价基础上浮动加价；单品未设时自动继承此参数</t>
   </si>
   <si>
-    <t>企业掌门人 / 老板</t>
+    <t>建议常规大货订单基准，给买家还价预留 3%~5% 安全博弈空间</t>
   </si>
   <si>
     <t>最低保护红线毛利率 (Floor Margin)</t>
@@ -172,7 +169,7 @@
     <t>业务员最低授权底线，低于此红线系统强制拦截并报警打回</t>
   </si>
   <si>
-    <t>老板 / 财务总监</t>
+    <t>底线防御警戒线！低于此值系统自动标红警报，防止业务员算亏</t>
   </si>
   <si>
     <t>样品打样费上浮倍率 (Sample Multiplier)</t>
@@ -184,7 +181,7 @@
     <t>覆盖小批量散单模具调机成本，后续批量达标全额抵扣货款</t>
   </si>
   <si>
-    <t>厂长 / 工程部</t>
+    <t>覆盖小批量散单机台调机损耗，可在合同中约定大货满额全额返还</t>
   </si>
   <si>
     <t>报价单默认有效期 (Price Validity)</t>
@@ -199,7 +196,7 @@
     <t>超出 30 天需重新核实原材料成本与外币汇率波动情况</t>
   </si>
   <si>
-    <t>外贸部主管</t>
+    <t>严防海运费与汇率剧烈波动风险，超期需重新核算，避免履约亏损</t>
   </si>
   <si>
     <t>🚢 模块三：默认贸易术语与杂费基准 (Incoterms &amp; Port Charges)</t>
@@ -472,7 +469,7 @@
     <t>Trade Term: FOB Shenzhen (Incoterms 2020)  |  Currency: USD ($)</t>
   </si>
   <si>
-    <t>Payment: 30% Deposit, 70% Before Shipment  |  Price Validity: 30 Days</t>
+    <t>Payment: 30% T/T Deposit, 70% Balance Before Shipment  |  Price Validity: 30 Days</t>
   </si>
   <si>
     <t>Item</t>
@@ -516,7 +513,7 @@
     <numFmt numFmtId="170" formatCode="0.000"/>
     <numFmt numFmtId="171" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -528,12 +525,6 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="13"/>
-      <name val="Microsoft YaHei"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF475569"/>
-      <sz val="9.5"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
@@ -648,17 +639,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFDBEAFE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
     <fill>
@@ -704,201 +695,198 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="17" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="18" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="14" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="19" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="19" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1240,78 +1228,70 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:C10"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="92" customWidth="1"/>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="96" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="38" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="1" ht="38" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-    </row>
-    <row r="3" ht="30" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+      <c r="B1" s="1"/>
+    </row>
+    <row r="2" ht="52" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="5" ht="52" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="3" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="4" t="s">
+    </row>
+    <row r="3" ht="52" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" ht="52" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" ht="52" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" ht="88" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="B6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" ht="75" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="4" t="s">
+    </row>
+    <row r="7" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>13</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1320,479 +1300,479 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
-    <col min="5" max="5" width="54" customWidth="1"/>
+    <col min="5" max="5" width="66" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+    <row r="2" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+    </row>
+    <row r="3" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-    </row>
-    <row r="4" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-    </row>
-    <row r="5" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="8" t="s">
         <v>21</v>
       </c>
+      <c r="B5" s="9">
+        <v>7.2</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="10">
-        <v>7.2</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="12" t="s">
+      <c r="A6" s="12" t="s">
         <v>25</v>
       </c>
+      <c r="B6" s="13">
+        <v>7.85</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="14">
-        <v>7.85</v>
-      </c>
-      <c r="C7" s="15" t="s">
+      <c r="A7" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="9">
+        <v>9.1</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>29</v>
+      <c r="E7" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="10">
-        <v>9.1</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="12" t="s">
+      <c r="A8" s="12" t="s">
         <v>32</v>
       </c>
+      <c r="B8" s="13">
+        <v>4.8</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" s="14">
-        <v>4.8</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="16" t="s">
+      <c r="A9" s="8" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+      <c r="B9" s="9">
+        <v>5.3</v>
+      </c>
+      <c r="C9" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="10">
-        <v>5.3</v>
-      </c>
-      <c r="C10" s="11" t="s">
+      <c r="D9" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="12" t="s">
+    </row>
+    <row r="11" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="12" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+    </row>
+    <row r="12" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
+      <c r="B12" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="8" t="s">
+      <c r="A13" s="16" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+      <c r="B13" s="17">
+        <v>0.15</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="18">
-        <v>0.15</v>
-      </c>
-      <c r="C14" s="11" t="s">
+      <c r="D13" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="E13" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="12" t="s">
+    </row>
+    <row r="14" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="B14" s="19">
+        <v>0.08</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="20">
-        <v>0.08</v>
-      </c>
-      <c r="C15" s="21" t="s">
+      <c r="D14" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="22" t="s">
+      <c r="E14" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="22" t="s">
+    </row>
+    <row r="15" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="16" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
+      <c r="B15" s="22">
+        <v>2.5</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="23">
-        <v>2.5</v>
-      </c>
-      <c r="C16" s="11" t="s">
+      <c r="D15" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="E15" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E16" s="12" t="s">
+    </row>
+    <row r="16" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="23" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="24" t="s">
+      <c r="B16" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="C16" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="D16" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="D17" s="16" t="s">
+      <c r="E16" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="16" t="s">
+    </row>
+    <row r="18" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="19" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+    </row>
+    <row r="19" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-    </row>
-    <row r="20" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="E20" s="8" t="s">
         <v>67</v>
       </c>
+      <c r="B20" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="24">
+        <v>0</v>
+      </c>
+      <c r="D20" s="24">
+        <v>0</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>69</v>
+      <c r="A21" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>71</v>
       </c>
       <c r="C21" s="25">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D21" s="25">
-        <v>0</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>70</v>
+        <v>1500</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="C22" s="26">
-        <v>0.2</v>
-      </c>
-      <c r="D22" s="26">
-        <v>1500</v>
-      </c>
-      <c r="E22" s="16" t="s">
+      <c r="A22" s="8" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="23" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
+      <c r="B22" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="C22" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="D22" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="E22" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="E23" s="12" t="s">
+    </row>
+    <row r="24" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="25" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+    </row>
+    <row r="25" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-    </row>
-    <row r="26" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="D25" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="E25" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E26" s="8" t="s">
+    </row>
+    <row r="26" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="16" t="s">
         <v>84</v>
       </c>
+      <c r="B26" s="26">
+        <v>-0.02</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" s="27">
+        <v>0</v>
+      </c>
+      <c r="C27" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="27">
-        <v>-0.02</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="E27" s="12" t="s">
-        <v>88</v>
+      <c r="D27" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="E27" s="15" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="B28" s="28">
-        <v>0</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="E28" s="16" t="s">
+      <c r="A28" s="16" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="29" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
+      <c r="B28" s="26">
+        <v>0.015</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="B29" s="27">
-        <v>0.015</v>
-      </c>
-      <c r="C29" s="11" t="s">
+      <c r="D28" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="E28" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E29" s="12" t="s">
+    </row>
+    <row r="30" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="31" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-    </row>
-    <row r="32" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="8" t="s">
+      <c r="B31" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="C31" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="D31" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="D32" s="8" t="s">
+      <c r="E31" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="E32" s="8" t="s">
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="16" t="s">
         <v>101</v>
       </c>
+      <c r="B32" s="28">
+        <v>28</v>
+      </c>
+      <c r="C32" s="28">
+        <v>33.2</v>
+      </c>
+      <c r="D32" s="29">
+        <v>21800</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="33" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="17" t="s">
-        <v>102</v>
-      </c>
-      <c r="B33" s="29">
-        <v>28</v>
-      </c>
-      <c r="C33" s="29">
-        <v>33.2</v>
-      </c>
-      <c r="D33" s="30">
-        <v>21800</v>
-      </c>
-      <c r="E33" s="12" t="s">
+      <c r="A33" s="23" t="s">
         <v>103</v>
       </c>
+      <c r="B33" s="30">
+        <v>58</v>
+      </c>
+      <c r="C33" s="30">
+        <v>67.7</v>
+      </c>
+      <c r="D33" s="31">
+        <v>26000</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="34" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="24" t="s">
-        <v>104</v>
-      </c>
-      <c r="B34" s="31">
-        <v>58</v>
-      </c>
-      <c r="C34" s="31">
-        <v>67.7</v>
-      </c>
-      <c r="D34" s="32">
+      <c r="A34" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B34" s="28">
+        <v>68</v>
+      </c>
+      <c r="C34" s="28">
+        <v>76.3</v>
+      </c>
+      <c r="D34" s="29">
         <v>26000</v>
       </c>
-      <c r="E34" s="16" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="17" t="s">
+      <c r="E34" s="11" t="s">
         <v>106</v>
-      </c>
-      <c r="B35" s="29">
-        <v>68</v>
-      </c>
-      <c r="C35" s="29">
-        <v>76.3</v>
-      </c>
-      <c r="D35" s="30">
-        <v>26000</v>
-      </c>
-      <c r="E35" s="12" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A30:E30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1821,366 +1801,366 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="32" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="32" t="s">
         <v>108</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="C1" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="C1" s="33" t="s">
+      <c r="D1" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="E1" s="32" t="s">
         <v>111</v>
       </c>
-      <c r="E1" s="33" t="s">
+      <c r="F1" s="32" t="s">
         <v>112</v>
       </c>
-      <c r="F1" s="33" t="s">
+      <c r="G1" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="G1" s="33" t="s">
+      <c r="H1" s="32" t="s">
         <v>114</v>
       </c>
-      <c r="H1" s="33" t="s">
+      <c r="I1" s="32" t="s">
         <v>115</v>
       </c>
-      <c r="I1" s="33" t="s">
+      <c r="J1" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="J1" s="33" t="s">
+      <c r="K1" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="K1" s="33" t="s">
+      <c r="L1" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="L1" s="34" t="s">
+      <c r="M1" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="M1" s="34" t="s">
+      <c r="N1" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="N1" s="34" t="s">
+      <c r="O1" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="O1" s="34" t="s">
+      <c r="P1" s="33" t="s">
         <v>122</v>
       </c>
-      <c r="P1" s="34" t="s">
+      <c r="Q1" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="Q1" s="34" t="s">
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="34" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="2" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="B2" s="35" t="s">
         <v>125</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="C2" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="36" t="s">
+      <c r="D2" s="36">
+        <v>15.5</v>
+      </c>
+      <c r="E2" s="37">
+        <v>500</v>
+      </c>
+      <c r="F2" s="37">
+        <v>50</v>
+      </c>
+      <c r="G2" s="38">
+        <v>0.045</v>
+      </c>
+      <c r="H2" s="39">
+        <v>14.5</v>
+      </c>
+      <c r="I2" s="40"/>
+      <c r="J2" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="37">
-        <v>15.5</v>
-      </c>
-      <c r="E2" s="38">
-        <v>500</v>
-      </c>
-      <c r="F2" s="38">
+      <c r="K2" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="L2" s="41">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
+      </c>
+      <c r="M2" s="42">
+        <f>IF(ISBLANK(I2), '⚙️ 全局核算参数 (Config)'!$B$13, I2)</f>
+      </c>
+      <c r="N2" s="43">
+        <f>ROUND(((D2 * (1 + M2) + L2) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
+      </c>
+      <c r="O2" s="44">
+        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G2)) * F2, "-")</f>
+      </c>
+      <c r="P2" s="44">
+        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G2)) * F2, "-")</f>
+      </c>
+      <c r="Q2" s="45">
+        <f>IF(M2&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M2&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="46" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="47" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3" s="47" t="s">
+        <v>131</v>
+      </c>
+      <c r="D3" s="48">
+        <v>0.85</v>
+      </c>
+      <c r="E3" s="49">
+        <v>5000</v>
+      </c>
+      <c r="F3" s="49">
+        <v>1000</v>
+      </c>
+      <c r="G3" s="50">
+        <v>0.02</v>
+      </c>
+      <c r="H3" s="51">
+        <v>18</v>
+      </c>
+      <c r="I3" s="52">
+        <v>0.18</v>
+      </c>
+      <c r="J3" s="46" t="s">
+        <v>132</v>
+      </c>
+      <c r="K3" s="46" t="s">
+        <v>133</v>
+      </c>
+      <c r="L3" s="41">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
+      </c>
+      <c r="M3" s="42">
+        <f>IF(ISBLANK(I3), '⚙️ 全局核算参数 (Config)'!$B$13, I3)</f>
+      </c>
+      <c r="N3" s="43">
+        <f>ROUND(((D3 * (1 + M3) + L3) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
+      </c>
+      <c r="O3" s="44">
+        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G3)) * F3, "-")</f>
+      </c>
+      <c r="P3" s="44">
+        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G3)) * F3, "-")</f>
+      </c>
+      <c r="Q3" s="45">
+        <f>IF(M3&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M3&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="B4" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="D4" s="36">
+        <v>185</v>
+      </c>
+      <c r="E4" s="37">
         <v>50</v>
       </c>
-      <c r="G2" s="39">
-        <v>0.045</v>
-      </c>
-      <c r="H2" s="40">
-        <v>14.5</v>
-      </c>
-      <c r="I2" s="41"/>
-      <c r="J2" s="35" t="s">
-        <v>128</v>
-      </c>
-      <c r="K2" s="35" t="s">
-        <v>129</v>
-      </c>
-      <c r="L2" s="42">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M2" s="43">
-        <f>IF(ISBLANK(I2), '⚙️ 全局核算参数 (Config)'!$B$14, I2)</f>
-      </c>
-      <c r="N2" s="44">
-        <f>ROUND(((D2 * (1 + M2) + L2) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O2" s="45">
-        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G2)) * F2, "-")</f>
-      </c>
-      <c r="P2" s="45">
-        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G2)) * F2, "-")</f>
-      </c>
-      <c r="Q2" s="46">
-        <f>IF(M2&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M2&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="47" t="s">
-        <v>130</v>
-      </c>
-      <c r="B3" s="48" t="s">
-        <v>131</v>
-      </c>
-      <c r="C3" s="48" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" s="49">
-        <v>0.85</v>
-      </c>
-      <c r="E3" s="50">
-        <v>5000</v>
-      </c>
-      <c r="F3" s="50">
-        <v>1000</v>
-      </c>
-      <c r="G3" s="51">
-        <v>0.02</v>
-      </c>
-      <c r="H3" s="52">
-        <v>18</v>
-      </c>
-      <c r="I3" s="53">
-        <v>0.18</v>
-      </c>
-      <c r="J3" s="47" t="s">
-        <v>133</v>
-      </c>
-      <c r="K3" s="47" t="s">
-        <v>134</v>
-      </c>
-      <c r="L3" s="42">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M3" s="43">
-        <f>IF(ISBLANK(I3), '⚙️ 全局核算参数 (Config)'!$B$14, I3)</f>
-      </c>
-      <c r="N3" s="44">
-        <f>ROUND(((D3 * (1 + M3) + L3) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O3" s="45">
-        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G3)) * F3, "-")</f>
-      </c>
-      <c r="P3" s="45">
-        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G3)) * F3, "-")</f>
-      </c>
-      <c r="Q3" s="46">
-        <f>IF(M3&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M3&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>136</v>
-      </c>
-      <c r="C4" s="36" t="s">
+      <c r="F4" s="37">
+        <v>1</v>
+      </c>
+      <c r="G4" s="38">
+        <v>0.16</v>
+      </c>
+      <c r="H4" s="39">
+        <v>16.2</v>
+      </c>
+      <c r="I4" s="40">
+        <v>0.25</v>
+      </c>
+      <c r="J4" s="34" t="s">
         <v>137</v>
       </c>
-      <c r="D4" s="37">
-        <v>185</v>
-      </c>
-      <c r="E4" s="38">
-        <v>50</v>
-      </c>
-      <c r="F4" s="38">
-        <v>1</v>
-      </c>
-      <c r="G4" s="39">
-        <v>0.16</v>
-      </c>
-      <c r="H4" s="40">
-        <v>16.2</v>
-      </c>
-      <c r="I4" s="41">
-        <v>0.25</v>
-      </c>
-      <c r="J4" s="35" t="s">
+      <c r="K4" s="34" t="s">
         <v>138</v>
       </c>
-      <c r="K4" s="35" t="s">
+      <c r="L4" s="41">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
+      </c>
+      <c r="M4" s="42">
+        <f>IF(ISBLANK(I4), '⚙️ 全局核算参数 (Config)'!$B$13, I4)</f>
+      </c>
+      <c r="N4" s="43">
+        <f>ROUND(((D4 * (1 + M4) + L4) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
+      </c>
+      <c r="O4" s="44">
+        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G4)) * F4, "-")</f>
+      </c>
+      <c r="P4" s="44">
+        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G4)) * F4, "-")</f>
+      </c>
+      <c r="Q4" s="45">
+        <f>IF(M4&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M4&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="46" t="s">
         <v>139</v>
       </c>
-      <c r="L4" s="42">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M4" s="43">
-        <f>IF(ISBLANK(I4), '⚙️ 全局核算参数 (Config)'!$B$14, I4)</f>
-      </c>
-      <c r="N4" s="44">
-        <f>ROUND(((D4 * (1 + M4) + L4) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O4" s="45">
-        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G4)) * F4, "-")</f>
-      </c>
-      <c r="P4" s="45">
-        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G4)) * F4, "-")</f>
-      </c>
-      <c r="Q4" s="46">
-        <f>IF(M4&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M4&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="47" t="s">
+      <c r="B5" s="47" t="s">
         <v>140</v>
       </c>
-      <c r="B5" s="48" t="s">
+      <c r="C5" s="47" t="s">
         <v>141</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="D5" s="48">
+        <v>38</v>
+      </c>
+      <c r="E5" s="49">
+        <v>200</v>
+      </c>
+      <c r="F5" s="49">
+        <v>5</v>
+      </c>
+      <c r="G5" s="50">
+        <v>0.08</v>
+      </c>
+      <c r="H5" s="51">
+        <v>11</v>
+      </c>
+      <c r="I5" s="52"/>
+      <c r="J5" s="46" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="49">
-        <v>38</v>
-      </c>
-      <c r="E5" s="50">
-        <v>200</v>
-      </c>
-      <c r="F5" s="50">
-        <v>5</v>
-      </c>
-      <c r="G5" s="51">
-        <v>0.08</v>
-      </c>
-      <c r="H5" s="52">
-        <v>11</v>
-      </c>
-      <c r="I5" s="53"/>
-      <c r="J5" s="47" t="s">
+      <c r="K5" s="46" t="s">
         <v>143</v>
       </c>
-      <c r="K5" s="47" t="s">
+      <c r="L5" s="41">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
+      </c>
+      <c r="M5" s="42">
+        <f>IF(ISBLANK(I5), '⚙️ 全局核算参数 (Config)'!$B$13, I5)</f>
+      </c>
+      <c r="N5" s="43">
+        <f>ROUND(((D5 * (1 + M5) + L5) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
+      </c>
+      <c r="O5" s="44">
+        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G5)) * F5, "-")</f>
+      </c>
+      <c r="P5" s="44">
+        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G5)) * F5, "-")</f>
+      </c>
+      <c r="Q5" s="45">
+        <f>IF(M5&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M5&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" s="34" t="s">
         <v>144</v>
       </c>
-      <c r="L5" s="42">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M5" s="43">
-        <f>IF(ISBLANK(I5), '⚙️ 全局核算参数 (Config)'!$B$14, I5)</f>
-      </c>
-      <c r="N5" s="44">
-        <f>ROUND(((D5 * (1 + M5) + L5) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O5" s="45">
-        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G5)) * F5, "-")</f>
-      </c>
-      <c r="P5" s="45">
-        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G5)) * F5, "-")</f>
-      </c>
-      <c r="Q5" s="46">
-        <f>IF(M5&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M5&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="35" t="s">
+      <c r="B6" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="C6" s="35" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="36" t="s">
+      <c r="D6" s="36">
+        <v>24</v>
+      </c>
+      <c r="E6" s="37">
+        <v>300</v>
+      </c>
+      <c r="F6" s="37">
+        <v>20</v>
+      </c>
+      <c r="G6" s="38">
+        <v>0.055</v>
+      </c>
+      <c r="H6" s="39">
+        <v>9.5</v>
+      </c>
+      <c r="I6" s="40"/>
+      <c r="J6" s="34" t="s">
+        <v>127</v>
+      </c>
+      <c r="K6" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="L6" s="41">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
+      </c>
+      <c r="M6" s="42">
+        <f>IF(ISBLANK(I6), '⚙️ 全局核算参数 (Config)'!$B$13, I6)</f>
+      </c>
+      <c r="N6" s="43">
+        <f>ROUND(((D6 * (1 + M6) + L6) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
+      </c>
+      <c r="O6" s="44">
+        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G6)) * F6, "-")</f>
+      </c>
+      <c r="P6" s="44">
+        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G6)) * F6, "-")</f>
+      </c>
+      <c r="Q6" s="45">
+        <f>IF(M6&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M6&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="46" t="s">
         <v>147</v>
       </c>
-      <c r="D6" s="37">
-        <v>24</v>
-      </c>
-      <c r="E6" s="38">
+      <c r="B7" s="47" t="s">
+        <v>148</v>
+      </c>
+      <c r="C7" s="47" t="s">
+        <v>146</v>
+      </c>
+      <c r="D7" s="48">
+        <v>25</v>
+      </c>
+      <c r="E7" s="49">
         <v>300</v>
       </c>
-      <c r="F6" s="38">
+      <c r="F7" s="49">
         <v>20</v>
       </c>
-      <c r="G6" s="39">
+      <c r="G7" s="50">
         <v>0.055</v>
       </c>
-      <c r="H6" s="40">
+      <c r="H7" s="51">
         <v>9.5</v>
       </c>
-      <c r="I6" s="41"/>
-      <c r="J6" s="35" t="s">
-        <v>128</v>
-      </c>
-      <c r="K6" s="35" t="s">
-        <v>144</v>
-      </c>
-      <c r="L6" s="42">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M6" s="43">
-        <f>IF(ISBLANK(I6), '⚙️ 全局核算参数 (Config)'!$B$14, I6)</f>
-      </c>
-      <c r="N6" s="44">
-        <f>ROUND(((D6 * (1 + M6) + L6) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O6" s="45">
-        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G6)) * F6, "-")</f>
-      </c>
-      <c r="P6" s="45">
-        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G6)) * F6, "-")</f>
-      </c>
-      <c r="Q6" s="46">
-        <f>IF(M6&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M6&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="47" t="s">
-        <v>148</v>
-      </c>
-      <c r="B7" s="48" t="s">
-        <v>149</v>
-      </c>
-      <c r="C7" s="48" t="s">
-        <v>147</v>
-      </c>
-      <c r="D7" s="49">
-        <v>25</v>
-      </c>
-      <c r="E7" s="50">
-        <v>300</v>
-      </c>
-      <c r="F7" s="50">
-        <v>20</v>
-      </c>
-      <c r="G7" s="51">
-        <v>0.055</v>
-      </c>
-      <c r="H7" s="52">
-        <v>9.5</v>
-      </c>
-      <c r="I7" s="53"/>
-      <c r="J7" s="47" t="s">
-        <v>128</v>
-      </c>
-      <c r="K7" s="47" t="s">
-        <v>144</v>
-      </c>
-      <c r="L7" s="42">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$22</f>
-      </c>
-      <c r="M7" s="43">
-        <f>IF(ISBLANK(I7), '⚙️ 全局核算参数 (Config)'!$B$14, I7)</f>
-      </c>
-      <c r="N7" s="44">
-        <f>ROUND(((D7 * (1 + M7) + L7) / '⚙️ 全局核算参数 (Config)'!$B$6), 2)</f>
-      </c>
-      <c r="O7" s="45">
-        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$33 / G7)) * F7, "-")</f>
-      </c>
-      <c r="P7" s="45">
-        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$35 / G7)) * F7, "-")</f>
-      </c>
-      <c r="Q7" s="46">
-        <f>IF(M7&lt;'⚙️ 全局核算参数 (Config)'!$B$15, "🚨 穿透红线", IF(M7&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      <c r="I7" s="52"/>
+      <c r="J7" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="K7" s="46" t="s">
+        <v>143</v>
+      </c>
+      <c r="L7" s="41">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
+      </c>
+      <c r="M7" s="42">
+        <f>IF(ISBLANK(I7), '⚙️ 全局核算参数 (Config)'!$B$13, I7)</f>
+      </c>
+      <c r="N7" s="43">
+        <f>ROUND(((D7 * (1 + M7) + L7) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
+      </c>
+      <c r="O7" s="44">
+        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G7)) * F7, "-")</f>
+      </c>
+      <c r="P7" s="44">
+        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G7)) * F7, "-")</f>
+      </c>
+      <c r="Q7" s="45">
+        <f>IF(M7&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M7&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
       </c>
     </row>
   </sheetData>
@@ -2204,233 +2184,233 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="53" t="s">
+        <v>149</v>
+      </c>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="54" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-    </row>
-    <row r="2" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="55" t="s">
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="55" t="s">
         <v>151</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="56" t="s">
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+    </row>
+    <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="56" t="s">
         <v>152</v>
       </c>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
-    </row>
-    <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="B3" s="56" t="s">
         <v>153</v>
       </c>
-      <c r="B3" s="57" t="s">
+      <c r="C3" s="56" t="s">
         <v>154</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="D3" s="56" t="s">
         <v>155</v>
       </c>
-      <c r="D3" s="57" t="s">
+      <c r="E3" s="56" t="s">
         <v>156</v>
       </c>
-      <c r="E3" s="57" t="s">
+      <c r="F3" s="56" t="s">
         <v>157</v>
       </c>
-      <c r="F3" s="57" t="s">
+      <c r="G3" s="56" t="s">
         <v>158</v>
       </c>
-      <c r="G3" s="57" t="s">
+      <c r="H3" s="56" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="57" t="s">
+      <c r="I3" s="56" t="s">
         <v>160</v>
       </c>
-      <c r="I3" s="57" t="s">
-        <v>161</v>
-      </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="58">
+      <c r="A4" s="57">
         <v>1</v>
       </c>
-      <c r="B4" s="58">
+      <c r="B4" s="57">
         <f>'📦 商品出厂底价库 (Products)'!A2</f>
       </c>
-      <c r="C4" s="59">
+      <c r="C4" s="58">
         <f>'📦 商品出厂底价库 (Products)'!C2</f>
       </c>
-      <c r="D4" s="60">
+      <c r="D4" s="59">
         <f>'📦 商品出厂底价库 (Products)'!E2</f>
       </c>
-      <c r="E4" s="61">
+      <c r="E4" s="60">
         <f>'📦 商品出厂底价库 (Products)'!N2</f>
       </c>
-      <c r="F4" s="60">
+      <c r="F4" s="59">
         <f>'📦 商品出厂底价库 (Products)'!F2</f>
       </c>
-      <c r="G4" s="60">
+      <c r="G4" s="59">
         <f>'📦 商品出厂底价库 (Products)'!O2</f>
       </c>
-      <c r="H4" s="60">
+      <c r="H4" s="59">
         <f>'📦 商品出厂底价库 (Products)'!P2</f>
       </c>
-      <c r="I4" s="58">
+      <c r="I4" s="57">
         <f>'📦 商品出厂底价库 (Products)'!J2</f>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="62">
+      <c r="A5" s="61">
         <v>2</v>
       </c>
-      <c r="B5" s="62">
+      <c r="B5" s="61">
         <f>'📦 商品出厂底价库 (Products)'!A3</f>
       </c>
-      <c r="C5" s="63">
+      <c r="C5" s="62">
         <f>'📦 商品出厂底价库 (Products)'!C3</f>
       </c>
-      <c r="D5" s="64">
+      <c r="D5" s="63">
         <f>'📦 商品出厂底价库 (Products)'!E3</f>
       </c>
-      <c r="E5" s="65">
+      <c r="E5" s="64">
         <f>'📦 商品出厂底价库 (Products)'!N3</f>
       </c>
-      <c r="F5" s="64">
+      <c r="F5" s="63">
         <f>'📦 商品出厂底价库 (Products)'!F3</f>
       </c>
-      <c r="G5" s="64">
+      <c r="G5" s="63">
         <f>'📦 商品出厂底价库 (Products)'!O3</f>
       </c>
-      <c r="H5" s="64">
+      <c r="H5" s="63">
         <f>'📦 商品出厂底价库 (Products)'!P3</f>
       </c>
-      <c r="I5" s="62">
+      <c r="I5" s="61">
         <f>'📦 商品出厂底价库 (Products)'!J3</f>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="58">
+      <c r="A6" s="57">
         <v>3</v>
       </c>
-      <c r="B6" s="58">
+      <c r="B6" s="57">
         <f>'📦 商品出厂底价库 (Products)'!A4</f>
       </c>
-      <c r="C6" s="59">
+      <c r="C6" s="58">
         <f>'📦 商品出厂底价库 (Products)'!C4</f>
       </c>
-      <c r="D6" s="60">
+      <c r="D6" s="59">
         <f>'📦 商品出厂底价库 (Products)'!E4</f>
       </c>
-      <c r="E6" s="61">
+      <c r="E6" s="60">
         <f>'📦 商品出厂底价库 (Products)'!N4</f>
       </c>
-      <c r="F6" s="60">
+      <c r="F6" s="59">
         <f>'📦 商品出厂底价库 (Products)'!F4</f>
       </c>
-      <c r="G6" s="60">
+      <c r="G6" s="59">
         <f>'📦 商品出厂底价库 (Products)'!O4</f>
       </c>
-      <c r="H6" s="60">
+      <c r="H6" s="59">
         <f>'📦 商品出厂底价库 (Products)'!P4</f>
       </c>
-      <c r="I6" s="58">
+      <c r="I6" s="57">
         <f>'📦 商品出厂底价库 (Products)'!J4</f>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="62">
+      <c r="A7" s="61">
         <v>4</v>
       </c>
-      <c r="B7" s="62">
+      <c r="B7" s="61">
         <f>'📦 商品出厂底价库 (Products)'!A5</f>
       </c>
-      <c r="C7" s="63">
+      <c r="C7" s="62">
         <f>'📦 商品出厂底价库 (Products)'!C5</f>
       </c>
-      <c r="D7" s="64">
+      <c r="D7" s="63">
         <f>'📦 商品出厂底价库 (Products)'!E5</f>
       </c>
-      <c r="E7" s="65">
+      <c r="E7" s="64">
         <f>'📦 商品出厂底价库 (Products)'!N5</f>
       </c>
-      <c r="F7" s="64">
+      <c r="F7" s="63">
         <f>'📦 商品出厂底价库 (Products)'!F5</f>
       </c>
-      <c r="G7" s="64">
+      <c r="G7" s="63">
         <f>'📦 商品出厂底价库 (Products)'!O5</f>
       </c>
-      <c r="H7" s="64">
+      <c r="H7" s="63">
         <f>'📦 商品出厂底价库 (Products)'!P5</f>
       </c>
-      <c r="I7" s="62">
+      <c r="I7" s="61">
         <f>'📦 商品出厂底价库 (Products)'!J5</f>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="58">
+      <c r="A8" s="57">
         <v>5</v>
       </c>
-      <c r="B8" s="58">
+      <c r="B8" s="57">
         <f>'📦 商品出厂底价库 (Products)'!A6</f>
       </c>
-      <c r="C8" s="59">
+      <c r="C8" s="58">
         <f>'📦 商品出厂底价库 (Products)'!C6</f>
       </c>
-      <c r="D8" s="60">
+      <c r="D8" s="59">
         <f>'📦 商品出厂底价库 (Products)'!E6</f>
       </c>
-      <c r="E8" s="61">
+      <c r="E8" s="60">
         <f>'📦 商品出厂底价库 (Products)'!N6</f>
       </c>
-      <c r="F8" s="60">
+      <c r="F8" s="59">
         <f>'📦 商品出厂底价库 (Products)'!F6</f>
       </c>
-      <c r="G8" s="60">
+      <c r="G8" s="59">
         <f>'📦 商品出厂底价库 (Products)'!O6</f>
       </c>
-      <c r="H8" s="60">
+      <c r="H8" s="59">
         <f>'📦 商品出厂底价库 (Products)'!P6</f>
       </c>
-      <c r="I8" s="58">
+      <c r="I8" s="57">
         <f>'📦 商品出厂底价库 (Products)'!J6</f>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="62">
+      <c r="A9" s="61">
         <v>6</v>
       </c>
-      <c r="B9" s="62">
+      <c r="B9" s="61">
         <f>'📦 商品出厂底价库 (Products)'!A7</f>
       </c>
-      <c r="C9" s="63">
+      <c r="C9" s="62">
         <f>'📦 商品出厂底价库 (Products)'!C7</f>
       </c>
-      <c r="D9" s="64">
+      <c r="D9" s="63">
         <f>'📦 商品出厂底价库 (Products)'!E7</f>
       </c>
-      <c r="E9" s="65">
+      <c r="E9" s="64">
         <f>'📦 商品出厂底价库 (Products)'!N7</f>
       </c>
-      <c r="F9" s="64">
+      <c r="F9" s="63">
         <f>'📦 商品出厂底价库 (Products)'!F7</f>
       </c>
-      <c r="G9" s="64">
+      <c r="G9" s="63">
         <f>'📦 商品出厂底价库 (Products)'!O7</f>
       </c>
-      <c r="H9" s="64">
+      <c r="H9" s="63">
         <f>'📦 商品出厂底价库 (Products)'!P7</f>
       </c>
-      <c r="I9" s="62">
+      <c r="I9" s="61">
         <f>'📦 商品出厂底价库 (Products)'!J7</f>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(lead_magnet): apply clean freeze panes and outer border styling to quotation sheet
</commit_message>
<xml_diff>
--- a/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
+++ b/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="162">
   <si>
     <t>【2026外贸出厂底价表与智能核价模板】使用指南</t>
   </si>
@@ -463,10 +463,13 @@
     <t>3D Armrest Pro, PU Armrest Plus, 加强升降扶手, ARM-09</t>
   </si>
   <si>
-    <t>GLOBAL EXPORT FORMAL QUOTATION (COMMERCIAL OFFER)</t>
-  </si>
-  <si>
-    <t>Trade Term: FOB Shenzhen (Incoterms 2020)  |  Currency: USD ($)</t>
+    <t>GLOBAL EXPORT</t>
+  </si>
+  <si>
+    <t>FORMAL COMMERCIAL OFFER (FOB SHENZHEN)</t>
+  </si>
+  <si>
+    <t>Incoterms® 2020 · USD ($)</t>
   </si>
   <si>
     <t>Payment: 30% T/T Deposit, 70% Balance Before Shipment  |  Price Validity: 30 Days</t>
@@ -513,7 +516,7 @@
     <numFmt numFmtId="170" formatCode="0.000"/>
     <numFmt numFmtId="171" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -598,7 +601,20 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12.5"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <color rgb="FF1E293B"/>
+      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -668,7 +684,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -691,11 +707,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -853,40 +882,43 @@
     <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="19" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="20" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="17" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="18" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="18" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="19" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="20" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2175,12 +2207,11 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="55" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="9" width="20" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2188,237 +2219,240 @@
         <v>149</v>
       </c>
       <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
-      <c r="I1" s="53"/>
+      <c r="C1" s="54" t="s">
+        <v>150</v>
+      </c>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="54"/>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="54" t="s">
-        <v>150</v>
-      </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="55" t="s">
+      <c r="A2" s="55" t="s">
         <v>151</v>
       </c>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="56" t="s">
+        <v>152</v>
+      </c>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="56" t="s">
-        <v>152</v>
-      </c>
-      <c r="B3" s="56" t="s">
+      <c r="A3" s="57" t="s">
         <v>153</v>
       </c>
-      <c r="C3" s="56" t="s">
+      <c r="B3" s="57" t="s">
         <v>154</v>
       </c>
-      <c r="D3" s="56" t="s">
+      <c r="C3" s="57" t="s">
         <v>155</v>
       </c>
-      <c r="E3" s="56" t="s">
+      <c r="D3" s="57" t="s">
         <v>156</v>
       </c>
-      <c r="F3" s="56" t="s">
+      <c r="E3" s="57" t="s">
         <v>157</v>
       </c>
-      <c r="G3" s="56" t="s">
+      <c r="F3" s="57" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="56" t="s">
+      <c r="G3" s="57" t="s">
         <v>159</v>
       </c>
-      <c r="I3" s="56" t="s">
+      <c r="H3" s="57" t="s">
         <v>160</v>
       </c>
+      <c r="I3" s="57" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="57">
+      <c r="A4" s="58">
         <v>1</v>
       </c>
-      <c r="B4" s="57">
+      <c r="B4" s="58">
         <f>'📦 商品出厂底价库 (Products)'!A2</f>
       </c>
-      <c r="C4" s="58">
+      <c r="C4" s="59">
         <f>'📦 商品出厂底价库 (Products)'!C2</f>
       </c>
-      <c r="D4" s="59">
+      <c r="D4" s="60">
         <f>'📦 商品出厂底价库 (Products)'!E2</f>
       </c>
-      <c r="E4" s="60">
+      <c r="E4" s="61">
         <f>'📦 商品出厂底价库 (Products)'!N2</f>
       </c>
-      <c r="F4" s="59">
+      <c r="F4" s="60">
         <f>'📦 商品出厂底价库 (Products)'!F2</f>
       </c>
-      <c r="G4" s="59">
+      <c r="G4" s="60">
         <f>'📦 商品出厂底价库 (Products)'!O2</f>
       </c>
-      <c r="H4" s="59">
+      <c r="H4" s="60">
         <f>'📦 商品出厂底价库 (Products)'!P2</f>
       </c>
-      <c r="I4" s="57">
+      <c r="I4" s="58">
         <f>'📦 商品出厂底价库 (Products)'!J2</f>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="61">
+      <c r="A5" s="62">
         <v>2</v>
       </c>
-      <c r="B5" s="61">
+      <c r="B5" s="62">
         <f>'📦 商品出厂底价库 (Products)'!A3</f>
       </c>
-      <c r="C5" s="62">
+      <c r="C5" s="63">
         <f>'📦 商品出厂底价库 (Products)'!C3</f>
       </c>
-      <c r="D5" s="63">
+      <c r="D5" s="64">
         <f>'📦 商品出厂底价库 (Products)'!E3</f>
       </c>
-      <c r="E5" s="64">
+      <c r="E5" s="65">
         <f>'📦 商品出厂底价库 (Products)'!N3</f>
       </c>
-      <c r="F5" s="63">
+      <c r="F5" s="64">
         <f>'📦 商品出厂底价库 (Products)'!F3</f>
       </c>
-      <c r="G5" s="63">
+      <c r="G5" s="64">
         <f>'📦 商品出厂底价库 (Products)'!O3</f>
       </c>
-      <c r="H5" s="63">
+      <c r="H5" s="64">
         <f>'📦 商品出厂底价库 (Products)'!P3</f>
       </c>
-      <c r="I5" s="61">
+      <c r="I5" s="62">
         <f>'📦 商品出厂底价库 (Products)'!J3</f>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="57">
+      <c r="A6" s="58">
         <v>3</v>
       </c>
-      <c r="B6" s="57">
+      <c r="B6" s="58">
         <f>'📦 商品出厂底价库 (Products)'!A4</f>
       </c>
-      <c r="C6" s="58">
+      <c r="C6" s="59">
         <f>'📦 商品出厂底价库 (Products)'!C4</f>
       </c>
-      <c r="D6" s="59">
+      <c r="D6" s="60">
         <f>'📦 商品出厂底价库 (Products)'!E4</f>
       </c>
-      <c r="E6" s="60">
+      <c r="E6" s="61">
         <f>'📦 商品出厂底价库 (Products)'!N4</f>
       </c>
-      <c r="F6" s="59">
+      <c r="F6" s="60">
         <f>'📦 商品出厂底价库 (Products)'!F4</f>
       </c>
-      <c r="G6" s="59">
+      <c r="G6" s="60">
         <f>'📦 商品出厂底价库 (Products)'!O4</f>
       </c>
-      <c r="H6" s="59">
+      <c r="H6" s="60">
         <f>'📦 商品出厂底价库 (Products)'!P4</f>
       </c>
-      <c r="I6" s="57">
+      <c r="I6" s="58">
         <f>'📦 商品出厂底价库 (Products)'!J4</f>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="61">
+      <c r="A7" s="62">
         <v>4</v>
       </c>
-      <c r="B7" s="61">
+      <c r="B7" s="62">
         <f>'📦 商品出厂底价库 (Products)'!A5</f>
       </c>
-      <c r="C7" s="62">
+      <c r="C7" s="63">
         <f>'📦 商品出厂底价库 (Products)'!C5</f>
       </c>
-      <c r="D7" s="63">
+      <c r="D7" s="64">
         <f>'📦 商品出厂底价库 (Products)'!E5</f>
       </c>
-      <c r="E7" s="64">
+      <c r="E7" s="65">
         <f>'📦 商品出厂底价库 (Products)'!N5</f>
       </c>
-      <c r="F7" s="63">
+      <c r="F7" s="64">
         <f>'📦 商品出厂底价库 (Products)'!F5</f>
       </c>
-      <c r="G7" s="63">
+      <c r="G7" s="64">
         <f>'📦 商品出厂底价库 (Products)'!O5</f>
       </c>
-      <c r="H7" s="63">
+      <c r="H7" s="64">
         <f>'📦 商品出厂底价库 (Products)'!P5</f>
       </c>
-      <c r="I7" s="61">
+      <c r="I7" s="62">
         <f>'📦 商品出厂底价库 (Products)'!J5</f>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="57">
+      <c r="A8" s="58">
         <v>5</v>
       </c>
-      <c r="B8" s="57">
+      <c r="B8" s="58">
         <f>'📦 商品出厂底价库 (Products)'!A6</f>
       </c>
-      <c r="C8" s="58">
+      <c r="C8" s="59">
         <f>'📦 商品出厂底价库 (Products)'!C6</f>
       </c>
-      <c r="D8" s="59">
+      <c r="D8" s="60">
         <f>'📦 商品出厂底价库 (Products)'!E6</f>
       </c>
-      <c r="E8" s="60">
+      <c r="E8" s="61">
         <f>'📦 商品出厂底价库 (Products)'!N6</f>
       </c>
-      <c r="F8" s="59">
+      <c r="F8" s="60">
         <f>'📦 商品出厂底价库 (Products)'!F6</f>
       </c>
-      <c r="G8" s="59">
+      <c r="G8" s="60">
         <f>'📦 商品出厂底价库 (Products)'!O6</f>
       </c>
-      <c r="H8" s="59">
+      <c r="H8" s="60">
         <f>'📦 商品出厂底价库 (Products)'!P6</f>
       </c>
-      <c r="I8" s="57">
+      <c r="I8" s="58">
         <f>'📦 商品出厂底价库 (Products)'!J6</f>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="61">
+      <c r="A9" s="62">
         <v>6</v>
       </c>
-      <c r="B9" s="61">
+      <c r="B9" s="62">
         <f>'📦 商品出厂底价库 (Products)'!A7</f>
       </c>
-      <c r="C9" s="62">
+      <c r="C9" s="63">
         <f>'📦 商品出厂底价库 (Products)'!C7</f>
       </c>
-      <c r="D9" s="63">
+      <c r="D9" s="64">
         <f>'📦 商品出厂底价库 (Products)'!E7</f>
       </c>
-      <c r="E9" s="64">
+      <c r="E9" s="65">
         <f>'📦 商品出厂底价库 (Products)'!N7</f>
       </c>
-      <c r="F9" s="63">
+      <c r="F9" s="64">
         <f>'📦 商品出厂底价库 (Products)'!F7</f>
       </c>
-      <c r="G9" s="63">
+      <c r="G9" s="64">
         <f>'📦 商品出厂底价库 (Products)'!O7</f>
       </c>
-      <c r="H9" s="63">
+      <c r="H9" s="64">
         <f>'📦 商品出厂底价库 (Products)'!P7</f>
       </c>
-      <c r="I9" s="61">
+      <c r="I9" s="62">
         <f>'📦 商品出厂底价库 (Products)'!J7</f>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:I2"/>
+  <mergeCells count="4">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:I1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat(templates): implement Scheme A dynamic master currency controller and fix quote headers
</commit_message>
<xml_diff>
--- a/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
+++ b/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="161">
   <si>
     <t>【2026外贸出厂底价表与智能核价模板】使用指南</t>
   </si>
@@ -28,13 +28,13 @@
     <t>2. 【⚙️ 全局核算参数】怎么用？</t>
   </si>
   <si>
-    <t>在第 2 张工作表设定贵司（或个人）内部锁定汇率（如 USD 7.20）、保底毛利（如 15%）、利润防穿底红线（如 8%）与海运进仓港杂平摊（如 0.20 元/件）。在此修改后，全库商品自动秒级联动更新。</t>
+    <t>在第 2 张工作表顶部可【一键下拉切换主结算币种】（支持 USD / EUR / GBP / AUD / CAD），全库商品底价与对外报价单秒级自动自适应切换！同时可设定内部锁定汇率、保底毛利（如 15%）、利润防穿底红线（如 8%）与海运进仓港杂平摊（如 0.20 元/件）。在此微调后，全库商品自动秒级联动更新。</t>
   </si>
   <si>
     <t>3. 【📦 商品出厂底价库】怎么用？</t>
   </si>
   <si>
-    <t>在第 3 张工作表批量录入产品 SKU、出厂底价与包装尺寸。黄色公式区会自动联动倒算出精准 FOB 美金报价、自动算出 20GP/40HQ 可装柜件数；若某品毛利低于红线会自动闪烁警报。</t>
+    <t>在第 3 张工作表批量录入产品 SKU、出厂底价与包装尺寸。黄色公式区会自动联动倒算出精准 FOB 外币报价、自动算出 20GP/40HQ 可装柜件数；若某品毛利低于红线会自动闪烁警报。</t>
   </si>
   <si>
     <t>4. 对外发给买家安全吗？</t>
@@ -61,7 +61,16 @@
     <t>💡【核算中枢指引】在此设定贵司（或个人）内部锁定汇率、保底毛利率与业务参数，全库商品将自动秒级联动倒算。日常核价只需在此微调参数，无需逐个单品修改。</t>
   </si>
   <si>
-    <t>💵 模块一：结算币种与内部锁定汇率 (Currency &amp; Exchange Rates)</t>
+    <t>💵 模块一：结算币种与全局主报价切换 (Currency &amp; Master Active Currency)</t>
+  </si>
+  <si>
+    <t>🎯 当前全局核算与报价主币种 (Active Currency)</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>👈 下拉切换币种：底价库与对外脱敏报价单秒级全表自适应！</t>
   </si>
   <si>
     <t>外币币种 (Target Currency)</t>
@@ -79,13 +88,10 @@
     <t>适用采购区域 (采购商来源)</t>
   </si>
   <si>
-    <t>USD</t>
-  </si>
-  <si>
     <t>$</t>
   </si>
   <si>
-    <t>★ 基准主币种 (波动±3%保护)</t>
+    <t>★ 默认主币种 (波动±3%保护)</t>
   </si>
   <si>
     <t>北美、东南亚、全球主流外贸结算 (默认主币种)</t>
@@ -376,9 +382,6 @@
     <t>⚡ 生效核算毛利率</t>
   </si>
   <si>
-    <t>🎯 FOB美金单价(USD)</t>
-  </si>
-  <si>
     <t>📦 20GP小柜装量(PCS)</t>
   </si>
   <si>
@@ -469,9 +472,6 @@
     <t>FORMAL COMMERCIAL OFFER (FOB SHENZHEN)</t>
   </si>
   <si>
-    <t>Incoterms® 2020 · USD ($)</t>
-  </si>
-  <si>
     <t>Payment: 30% T/T Deposit, 70% Balance Before Shipment  |  Price Validity: 30 Days</t>
   </si>
   <si>
@@ -485,9 +485,6 @@
   </si>
   <si>
     <t>MOQ (PCS)</t>
-  </si>
-  <si>
-    <t>FOB Price (USD)</t>
   </si>
   <si>
     <t>Packing (PCS/CTN)</t>
@@ -506,7 +503,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="8">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="¥#,##0.00"/>
@@ -514,9 +511,8 @@
     <numFmt numFmtId="168" formatCode="0.0&quot; CBM&quot;"/>
     <numFmt numFmtId="169" formatCode="#,##0&quot; KG&quot;"/>
     <numFmt numFmtId="170" formatCode="0.000"/>
-    <numFmt numFmtId="171" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -550,6 +546,18 @@
       <b/>
       <color rgb="FF1E3A8A"/>
       <sz val="11"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1E3A8A"/>
+      <sz val="10.5"/>
+      <name val="Microsoft YaHei"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF475569"/>
+      <sz val="9.5"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
@@ -670,17 +678,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF2563EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD97706"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -724,7 +732,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -745,84 +753,99 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -831,7 +854,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -846,19 +869,19 @@
     <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="13" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -867,7 +890,7 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -882,43 +905,43 @@
     <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="20" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="21" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="22" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="19" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="20" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="21" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="22" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1281,7 +1304,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" ht="52" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" ht="64" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -1369,111 +1392,130 @@
       <c r="D3" s="6"/>
       <c r="E3" s="6"/>
     </row>
-    <row r="4" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="9">
+        <f>VLOOKUP(B4, A6:C10, 2, FALSE)</f>
+        <v>7.2</v>
+      </c>
+      <c r="D4" s="10" t="str">
+        <f>VLOOKUP(B4, A6:C10, 3, FALSE)</f>
+        <v>$</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="7" t="s">
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="B5" s="12" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="C5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="9">
+      <c r="D5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="14">
         <v>7.2</v>
       </c>
-      <c r="C5" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="11" t="s">
+      <c r="C6" s="15" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="D6" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="13">
+      <c r="E6" s="16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="18">
         <v>7.85</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="15" t="s">
+      <c r="C7" s="19" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="D7" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="9">
+      <c r="E7" s="20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="14">
         <v>9.1</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="C8" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="13">
+      <c r="D8" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="18">
         <v>4.8</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="C9" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="9">
+      <c r="D9" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="14">
         <v>5.3</v>
       </c>
-      <c r="C9" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>37</v>
+      <c r="C10" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1481,93 +1523,93 @@
       <c r="E11" s="6"/>
     </row>
     <row r="12" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="7" t="s">
+      <c r="A12" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="B12" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="C12" s="12" t="s">
         <v>43</v>
       </c>
+      <c r="D12" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="13" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="17">
+      <c r="A13" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="22">
         <v>0.15</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" s="11" t="s">
+      <c r="C13" s="15" t="s">
         <v>47</v>
       </c>
+      <c r="D13" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" s="19">
+      <c r="A14" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="24">
         <v>0.08</v>
       </c>
-      <c r="C14" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" s="21" t="s">
+      <c r="C14" s="25" t="s">
         <v>51</v>
       </c>
+      <c r="D14" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="15" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" s="22">
+      <c r="A15" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="27">
         <v>2.5</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="E15" s="11" t="s">
+      <c r="C15" s="15" t="s">
         <v>55</v>
       </c>
+      <c r="D15" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="16" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C16" s="14" t="s">
+      <c r="A16" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="B16" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="C16" s="19" t="s">
         <v>60</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1575,76 +1617,76 @@
       <c r="E18" s="6"/>
     </row>
     <row r="19" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="C19" s="7" t="s">
+      <c r="A19" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="B19" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="C19" s="12" t="s">
         <v>66</v>
       </c>
+      <c r="D19" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C20" s="24">
+      <c r="A20" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="29">
         <v>0</v>
       </c>
-      <c r="D20" s="24">
+      <c r="D20" s="29">
         <v>0</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>69</v>
+      <c r="E20" s="16" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="C21" s="25">
+      <c r="A21" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" s="30">
         <v>0.2</v>
       </c>
-      <c r="D21" s="25">
+      <c r="D21" s="30">
         <v>1500</v>
       </c>
-      <c r="E21" s="15" t="s">
-        <v>72</v>
+      <c r="E21" s="20" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="C22" s="10" t="s">
+      <c r="A22" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="B22" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="C22" s="15" t="s">
         <v>77</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1652,76 +1694,76 @@
       <c r="E24" s="6"/>
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C25" s="7" t="s">
+      <c r="A25" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="B25" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="C25" s="12" t="s">
         <v>83</v>
       </c>
+      <c r="D25" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="B26" s="26">
+      <c r="A26" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="B26" s="31">
         <v>-0.02</v>
       </c>
-      <c r="C26" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E26" s="11" t="s">
+      <c r="C26" s="15" t="s">
         <v>87</v>
       </c>
+      <c r="D26" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="B27" s="27">
+      <c r="A27" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" s="32">
         <v>0</v>
       </c>
-      <c r="C27" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="E27" s="15" t="s">
-        <v>90</v>
+      <c r="C27" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="E27" s="20" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="B28" s="26">
+      <c r="A28" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B28" s="31">
         <v>0.015</v>
       </c>
-      <c r="C28" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="E28" s="11" t="s">
+      <c r="C28" s="15" t="s">
         <v>94</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="30" ht="26" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -1729,71 +1771,71 @@
       <c r="E30" s="6"/>
     </row>
     <row r="31" ht="24" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C31" s="7" t="s">
+      <c r="A31" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="B31" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="C31" s="12" t="s">
         <v>100</v>
       </c>
+      <c r="D31" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="32" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="B32" s="28">
+      <c r="A32" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="B32" s="33">
         <v>28</v>
       </c>
-      <c r="C32" s="28">
+      <c r="C32" s="33">
         <v>33.2</v>
       </c>
-      <c r="D32" s="29">
+      <c r="D32" s="34">
         <v>21800</v>
       </c>
-      <c r="E32" s="11" t="s">
-        <v>102</v>
+      <c r="E32" s="16" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="B33" s="30">
+      <c r="A33" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="B33" s="35">
         <v>58</v>
       </c>
-      <c r="C33" s="30">
+      <c r="C33" s="35">
         <v>67.7</v>
       </c>
-      <c r="D33" s="31">
+      <c r="D33" s="36">
         <v>26000</v>
       </c>
-      <c r="E33" s="15" t="s">
-        <v>104</v>
+      <c r="E33" s="20" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="B34" s="28">
+      <c r="A34" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="B34" s="33">
         <v>68</v>
       </c>
-      <c r="C34" s="28">
+      <c r="C34" s="33">
         <v>76.3</v>
       </c>
-      <c r="D34" s="29">
+      <c r="D34" s="34">
         <v>26000</v>
       </c>
-      <c r="E34" s="11" t="s">
-        <v>106</v>
+      <c r="E34" s="16" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1806,6 +1848,11 @@
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A30:E30"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" sqref="B4">
+      <formula1>"USD,EUR,GBP,AUD,CAD"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1833,365 +1880,366 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="B1" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="C1" s="32" t="s">
+      <c r="A1" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="B1" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="E1" s="32" t="s">
+      <c r="C1" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="F1" s="32" t="s">
+      <c r="D1" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="G1" s="32" t="s">
+      <c r="E1" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="F1" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="I1" s="32" t="s">
+      <c r="G1" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="J1" s="32" t="s">
+      <c r="H1" s="37" t="s">
         <v>116</v>
       </c>
-      <c r="K1" s="32" t="s">
+      <c r="I1" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="L1" s="33" t="s">
+      <c r="J1" s="37" t="s">
         <v>118</v>
       </c>
-      <c r="M1" s="33" t="s">
+      <c r="K1" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="N1" s="33" t="s">
+      <c r="L1" s="38" t="s">
         <v>120</v>
       </c>
-      <c r="O1" s="33" t="s">
+      <c r="M1" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="P1" s="33" t="s">
+      <c r="N1" s="38" t="str">
+        <f>"🎯 FOB核算单价 (" &amp; '⚙️ 全局核算参数 (Config)'!$B$4 &amp; ")"</f>
+        <v>🎯 FOB核算单价 (USD)</v>
+      </c>
+      <c r="O1" s="38" t="s">
         <v>122</v>
       </c>
-      <c r="Q1" s="33" t="s">
+      <c r="P1" s="38" t="s">
         <v>123</v>
       </c>
+      <c r="Q1" s="38" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="34" t="s">
-        <v>124</v>
-      </c>
-      <c r="B2" s="35" t="s">
+      <c r="A2" s="39" t="s">
         <v>125</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="B2" s="40" t="s">
         <v>126</v>
       </c>
-      <c r="D2" s="36">
+      <c r="C2" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="D2" s="41">
         <v>15.5</v>
       </c>
-      <c r="E2" s="37">
+      <c r="E2" s="42">
         <v>500</v>
       </c>
-      <c r="F2" s="37">
+      <c r="F2" s="42">
         <v>50</v>
       </c>
-      <c r="G2" s="38">
+      <c r="G2" s="43">
         <v>0.045</v>
       </c>
-      <c r="H2" s="39">
+      <c r="H2" s="44">
         <v>14.5</v>
       </c>
-      <c r="I2" s="40"/>
-      <c r="J2" s="34" t="s">
-        <v>127</v>
-      </c>
-      <c r="K2" s="34" t="s">
+      <c r="I2" s="45"/>
+      <c r="J2" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="L2" s="41">
+      <c r="K2" s="39" t="s">
+        <v>129</v>
+      </c>
+      <c r="L2" s="46">
         <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
       </c>
-      <c r="M2" s="42">
+      <c r="M2" s="47">
         <f>IF(ISBLANK(I2), '⚙️ 全局核算参数 (Config)'!$B$13, I2)</f>
       </c>
-      <c r="N2" s="43">
-        <f>ROUND(((D2 * (1 + M2) + L2) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
-      </c>
-      <c r="O2" s="44">
+      <c r="N2" s="48">
+        <f>ROUND(((D2 * (1 + M2) + L2) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
+      </c>
+      <c r="O2" s="49">
         <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G2)) * F2, "-")</f>
       </c>
-      <c r="P2" s="44">
+      <c r="P2" s="49">
         <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G2)) * F2, "-")</f>
       </c>
-      <c r="Q2" s="45">
+      <c r="Q2" s="50">
         <f>IF(M2&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M2&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="46" t="s">
-        <v>129</v>
-      </c>
-      <c r="B3" s="47" t="s">
+      <c r="A3" s="51" t="s">
         <v>130</v>
       </c>
-      <c r="C3" s="47" t="s">
+      <c r="B3" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="D3" s="48">
+      <c r="C3" s="52" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" s="53">
         <v>0.85</v>
       </c>
-      <c r="E3" s="49">
+      <c r="E3" s="54">
         <v>5000</v>
       </c>
-      <c r="F3" s="49">
+      <c r="F3" s="54">
         <v>1000</v>
       </c>
-      <c r="G3" s="50">
+      <c r="G3" s="55">
         <v>0.02</v>
       </c>
-      <c r="H3" s="51">
+      <c r="H3" s="56">
         <v>18</v>
       </c>
-      <c r="I3" s="52">
+      <c r="I3" s="57">
         <v>0.18</v>
       </c>
-      <c r="J3" s="46" t="s">
-        <v>132</v>
-      </c>
-      <c r="K3" s="46" t="s">
+      <c r="J3" s="51" t="s">
         <v>133</v>
       </c>
-      <c r="L3" s="41">
+      <c r="K3" s="51" t="s">
+        <v>134</v>
+      </c>
+      <c r="L3" s="46">
         <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
       </c>
-      <c r="M3" s="42">
+      <c r="M3" s="47">
         <f>IF(ISBLANK(I3), '⚙️ 全局核算参数 (Config)'!$B$13, I3)</f>
       </c>
-      <c r="N3" s="43">
-        <f>ROUND(((D3 * (1 + M3) + L3) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
-      </c>
-      <c r="O3" s="44">
+      <c r="N3" s="48">
+        <f>ROUND(((D3 * (1 + M3) + L3) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
+      </c>
+      <c r="O3" s="49">
         <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G3)) * F3, "-")</f>
       </c>
-      <c r="P3" s="44">
+      <c r="P3" s="49">
         <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G3)) * F3, "-")</f>
       </c>
-      <c r="Q3" s="45">
+      <c r="Q3" s="50">
         <f>IF(M3&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M3&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="34" t="s">
-        <v>134</v>
-      </c>
-      <c r="B4" s="35" t="s">
+      <c r="A4" s="39" t="s">
         <v>135</v>
       </c>
-      <c r="C4" s="35" t="s">
+      <c r="B4" s="40" t="s">
         <v>136</v>
       </c>
-      <c r="D4" s="36">
+      <c r="C4" s="40" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="41">
         <v>185</v>
       </c>
-      <c r="E4" s="37">
+      <c r="E4" s="42">
         <v>50</v>
       </c>
-      <c r="F4" s="37">
+      <c r="F4" s="42">
         <v>1</v>
       </c>
-      <c r="G4" s="38">
+      <c r="G4" s="43">
         <v>0.16</v>
       </c>
-      <c r="H4" s="39">
+      <c r="H4" s="44">
         <v>16.2</v>
       </c>
-      <c r="I4" s="40">
+      <c r="I4" s="45">
         <v>0.25</v>
       </c>
-      <c r="J4" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="K4" s="34" t="s">
+      <c r="J4" s="39" t="s">
         <v>138</v>
       </c>
-      <c r="L4" s="41">
+      <c r="K4" s="39" t="s">
+        <v>139</v>
+      </c>
+      <c r="L4" s="46">
         <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
       </c>
-      <c r="M4" s="42">
+      <c r="M4" s="47">
         <f>IF(ISBLANK(I4), '⚙️ 全局核算参数 (Config)'!$B$13, I4)</f>
       </c>
-      <c r="N4" s="43">
-        <f>ROUND(((D4 * (1 + M4) + L4) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
-      </c>
-      <c r="O4" s="44">
+      <c r="N4" s="48">
+        <f>ROUND(((D4 * (1 + M4) + L4) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
+      </c>
+      <c r="O4" s="49">
         <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G4)) * F4, "-")</f>
       </c>
-      <c r="P4" s="44">
+      <c r="P4" s="49">
         <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G4)) * F4, "-")</f>
       </c>
-      <c r="Q4" s="45">
+      <c r="Q4" s="50">
         <f>IF(M4&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M4&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="46" t="s">
-        <v>139</v>
-      </c>
-      <c r="B5" s="47" t="s">
+      <c r="A5" s="51" t="s">
         <v>140</v>
       </c>
-      <c r="C5" s="47" t="s">
+      <c r="B5" s="52" t="s">
         <v>141</v>
       </c>
-      <c r="D5" s="48">
+      <c r="C5" s="52" t="s">
+        <v>142</v>
+      </c>
+      <c r="D5" s="53">
         <v>38</v>
       </c>
-      <c r="E5" s="49">
+      <c r="E5" s="54">
         <v>200</v>
       </c>
-      <c r="F5" s="49">
+      <c r="F5" s="54">
         <v>5</v>
       </c>
-      <c r="G5" s="50">
+      <c r="G5" s="55">
         <v>0.08</v>
       </c>
-      <c r="H5" s="51">
+      <c r="H5" s="56">
         <v>11</v>
       </c>
-      <c r="I5" s="52"/>
-      <c r="J5" s="46" t="s">
-        <v>142</v>
-      </c>
-      <c r="K5" s="46" t="s">
+      <c r="I5" s="57"/>
+      <c r="J5" s="51" t="s">
         <v>143</v>
       </c>
-      <c r="L5" s="41">
+      <c r="K5" s="51" t="s">
+        <v>144</v>
+      </c>
+      <c r="L5" s="46">
         <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
       </c>
-      <c r="M5" s="42">
+      <c r="M5" s="47">
         <f>IF(ISBLANK(I5), '⚙️ 全局核算参数 (Config)'!$B$13, I5)</f>
       </c>
-      <c r="N5" s="43">
-        <f>ROUND(((D5 * (1 + M5) + L5) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
-      </c>
-      <c r="O5" s="44">
+      <c r="N5" s="48">
+        <f>ROUND(((D5 * (1 + M5) + L5) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
+      </c>
+      <c r="O5" s="49">
         <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G5)) * F5, "-")</f>
       </c>
-      <c r="P5" s="44">
+      <c r="P5" s="49">
         <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G5)) * F5, "-")</f>
       </c>
-      <c r="Q5" s="45">
+      <c r="Q5" s="50">
         <f>IF(M5&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M5&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="39" t="s">
+        <v>145</v>
+      </c>
+      <c r="B6" s="40" t="s">
+        <v>146</v>
+      </c>
+      <c r="C6" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="D6" s="41">
+        <v>24</v>
+      </c>
+      <c r="E6" s="42">
+        <v>300</v>
+      </c>
+      <c r="F6" s="42">
+        <v>20</v>
+      </c>
+      <c r="G6" s="43">
+        <v>0.055</v>
+      </c>
+      <c r="H6" s="44">
+        <v>9.5</v>
+      </c>
+      <c r="I6" s="45"/>
+      <c r="J6" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="K6" s="39" t="s">
         <v>144</v>
       </c>
-      <c r="B6" s="35" t="s">
-        <v>145</v>
-      </c>
-      <c r="C6" s="35" t="s">
-        <v>146</v>
-      </c>
-      <c r="D6" s="36">
-        <v>24</v>
-      </c>
-      <c r="E6" s="37">
+      <c r="L6" s="46">
+        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
+      </c>
+      <c r="M6" s="47">
+        <f>IF(ISBLANK(I6), '⚙️ 全局核算参数 (Config)'!$B$13, I6)</f>
+      </c>
+      <c r="N6" s="48">
+        <f>ROUND(((D6 * (1 + M6) + L6) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
+      </c>
+      <c r="O6" s="49">
+        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G6)) * F6, "-")</f>
+      </c>
+      <c r="P6" s="49">
+        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G6)) * F6, "-")</f>
+      </c>
+      <c r="Q6" s="50">
+        <f>IF(M6&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M6&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" s="51" t="s">
+        <v>148</v>
+      </c>
+      <c r="B7" s="52" t="s">
+        <v>149</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>147</v>
+      </c>
+      <c r="D7" s="53">
+        <v>25</v>
+      </c>
+      <c r="E7" s="54">
         <v>300</v>
       </c>
-      <c r="F6" s="37">
+      <c r="F7" s="54">
         <v>20</v>
       </c>
-      <c r="G6" s="38">
+      <c r="G7" s="55">
         <v>0.055</v>
       </c>
-      <c r="H6" s="39">
+      <c r="H7" s="56">
         <v>9.5</v>
       </c>
-      <c r="I6" s="40"/>
-      <c r="J6" s="34" t="s">
-        <v>127</v>
-      </c>
-      <c r="K6" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="L6" s="41">
+      <c r="I7" s="57"/>
+      <c r="J7" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="K7" s="51" t="s">
+        <v>144</v>
+      </c>
+      <c r="L7" s="46">
         <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
       </c>
-      <c r="M6" s="42">
-        <f>IF(ISBLANK(I6), '⚙️ 全局核算参数 (Config)'!$B$13, I6)</f>
-      </c>
-      <c r="N6" s="43">
-        <f>ROUND(((D6 * (1 + M6) + L6) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
-      </c>
-      <c r="O6" s="44">
-        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G6)) * F6, "-")</f>
-      </c>
-      <c r="P6" s="44">
-        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G6)) * F6, "-")</f>
-      </c>
-      <c r="Q6" s="45">
-        <f>IF(M6&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M6&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="46" t="s">
-        <v>147</v>
-      </c>
-      <c r="B7" s="47" t="s">
-        <v>148</v>
-      </c>
-      <c r="C7" s="47" t="s">
-        <v>146</v>
-      </c>
-      <c r="D7" s="48">
-        <v>25</v>
-      </c>
-      <c r="E7" s="49">
-        <v>300</v>
-      </c>
-      <c r="F7" s="49">
-        <v>20</v>
-      </c>
-      <c r="G7" s="50">
-        <v>0.055</v>
-      </c>
-      <c r="H7" s="51">
-        <v>9.5</v>
-      </c>
-      <c r="I7" s="52"/>
-      <c r="J7" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="K7" s="46" t="s">
-        <v>143</v>
-      </c>
-      <c r="L7" s="41">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
-      </c>
-      <c r="M7" s="42">
+      <c r="M7" s="47">
         <f>IF(ISBLANK(I7), '⚙️ 全局核算参数 (Config)'!$B$13, I7)</f>
       </c>
-      <c r="N7" s="43">
-        <f>ROUND(((D7 * (1 + M7) + L7) / '⚙️ 全局核算参数 (Config)'!$B$5), 2)</f>
-      </c>
-      <c r="O7" s="44">
+      <c r="N7" s="48">
+        <f>ROUND(((D7 * (1 + M7) + L7) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
+      </c>
+      <c r="O7" s="49">
         <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G7)) * F7, "-")</f>
       </c>
-      <c r="P7" s="44">
+      <c r="P7" s="49">
         <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G7)) * F7, "-")</f>
       </c>
-      <c r="Q7" s="45">
+      <c r="Q7" s="50">
         <f>IF(M7&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M7&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
       </c>
     </row>
@@ -2211,239 +2259,243 @@
     <col min="3" max="3" width="48" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="9" width="16" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="53" t="s">
-        <v>149</v>
-      </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="54" t="s">
+      <c r="A1" s="58" t="s">
         <v>150</v>
       </c>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="59" t="s">
+        <v>151</v>
+      </c>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="55" t="s">
-        <v>151</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="56" t="s">
+      <c r="A2" s="60" t="str">
+        <f>"Trade Term: FOB · " &amp; '⚙️ 全局核算参数 (Config)'!$B$4 &amp; " (" &amp; '⚙️ 全局核算参数 (Config)'!$D$4 &amp; ")"</f>
+        <v>Trade Term: FOB · USD ($)</v>
+      </c>
+      <c r="B2" s="60"/>
+      <c r="C2" s="61" t="s">
         <v>152</v>
       </c>
-      <c r="D2" s="56"/>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="56"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="62" t="s">
         <v>153</v>
       </c>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="62" t="s">
         <v>154</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="62" t="s">
         <v>155</v>
       </c>
-      <c r="D3" s="57" t="s">
+      <c r="D3" s="62" t="s">
         <v>156</v>
       </c>
-      <c r="E3" s="57" t="s">
+      <c r="E3" s="62" t="str">
+        <f>"FOB Price (" &amp; '⚙️ 全局核算参数 (Config)'!$B$4 &amp; ")"</f>
+        <v>FOB Price (USD)</v>
+      </c>
+      <c r="F3" s="62" t="s">
         <v>157</v>
       </c>
-      <c r="F3" s="57" t="s">
+      <c r="G3" s="62" t="s">
         <v>158</v>
       </c>
-      <c r="G3" s="57" t="s">
+      <c r="H3" s="62" t="s">
         <v>159</v>
       </c>
-      <c r="H3" s="57" t="s">
+      <c r="I3" s="62" t="s">
         <v>160</v>
       </c>
-      <c r="I3" s="57" t="s">
-        <v>161</v>
-      </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="58">
+      <c r="A4" s="63">
         <v>1</v>
       </c>
-      <c r="B4" s="58">
+      <c r="B4" s="63">
         <f>'📦 商品出厂底价库 (Products)'!A2</f>
       </c>
-      <c r="C4" s="59">
+      <c r="C4" s="64">
         <f>'📦 商品出厂底价库 (Products)'!C2</f>
       </c>
-      <c r="D4" s="60">
+      <c r="D4" s="65">
         <f>'📦 商品出厂底价库 (Products)'!E2</f>
       </c>
-      <c r="E4" s="61">
+      <c r="E4" s="66">
         <f>'📦 商品出厂底价库 (Products)'!N2</f>
       </c>
-      <c r="F4" s="60">
+      <c r="F4" s="65">
         <f>'📦 商品出厂底价库 (Products)'!F2</f>
       </c>
-      <c r="G4" s="60">
+      <c r="G4" s="65">
         <f>'📦 商品出厂底价库 (Products)'!O2</f>
       </c>
-      <c r="H4" s="60">
+      <c r="H4" s="65">
         <f>'📦 商品出厂底价库 (Products)'!P2</f>
       </c>
-      <c r="I4" s="58">
+      <c r="I4" s="63">
         <f>'📦 商品出厂底价库 (Products)'!J2</f>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="62">
+      <c r="A5" s="67">
         <v>2</v>
       </c>
-      <c r="B5" s="62">
+      <c r="B5" s="67">
         <f>'📦 商品出厂底价库 (Products)'!A3</f>
       </c>
-      <c r="C5" s="63">
+      <c r="C5" s="68">
         <f>'📦 商品出厂底价库 (Products)'!C3</f>
       </c>
-      <c r="D5" s="64">
+      <c r="D5" s="69">
         <f>'📦 商品出厂底价库 (Products)'!E3</f>
       </c>
-      <c r="E5" s="65">
+      <c r="E5" s="70">
         <f>'📦 商品出厂底价库 (Products)'!N3</f>
       </c>
-      <c r="F5" s="64">
+      <c r="F5" s="69">
         <f>'📦 商品出厂底价库 (Products)'!F3</f>
       </c>
-      <c r="G5" s="64">
+      <c r="G5" s="69">
         <f>'📦 商品出厂底价库 (Products)'!O3</f>
       </c>
-      <c r="H5" s="64">
+      <c r="H5" s="69">
         <f>'📦 商品出厂底价库 (Products)'!P3</f>
       </c>
-      <c r="I5" s="62">
+      <c r="I5" s="67">
         <f>'📦 商品出厂底价库 (Products)'!J3</f>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="58">
+      <c r="A6" s="63">
         <v>3</v>
       </c>
-      <c r="B6" s="58">
+      <c r="B6" s="63">
         <f>'📦 商品出厂底价库 (Products)'!A4</f>
       </c>
-      <c r="C6" s="59">
+      <c r="C6" s="64">
         <f>'📦 商品出厂底价库 (Products)'!C4</f>
       </c>
-      <c r="D6" s="60">
+      <c r="D6" s="65">
         <f>'📦 商品出厂底价库 (Products)'!E4</f>
       </c>
-      <c r="E6" s="61">
+      <c r="E6" s="66">
         <f>'📦 商品出厂底价库 (Products)'!N4</f>
       </c>
-      <c r="F6" s="60">
+      <c r="F6" s="65">
         <f>'📦 商品出厂底价库 (Products)'!F4</f>
       </c>
-      <c r="G6" s="60">
+      <c r="G6" s="65">
         <f>'📦 商品出厂底价库 (Products)'!O4</f>
       </c>
-      <c r="H6" s="60">
+      <c r="H6" s="65">
         <f>'📦 商品出厂底价库 (Products)'!P4</f>
       </c>
-      <c r="I6" s="58">
+      <c r="I6" s="63">
         <f>'📦 商品出厂底价库 (Products)'!J4</f>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="62">
+      <c r="A7" s="67">
         <v>4</v>
       </c>
-      <c r="B7" s="62">
+      <c r="B7" s="67">
         <f>'📦 商品出厂底价库 (Products)'!A5</f>
       </c>
-      <c r="C7" s="63">
+      <c r="C7" s="68">
         <f>'📦 商品出厂底价库 (Products)'!C5</f>
       </c>
-      <c r="D7" s="64">
+      <c r="D7" s="69">
         <f>'📦 商品出厂底价库 (Products)'!E5</f>
       </c>
-      <c r="E7" s="65">
+      <c r="E7" s="70">
         <f>'📦 商品出厂底价库 (Products)'!N5</f>
       </c>
-      <c r="F7" s="64">
+      <c r="F7" s="69">
         <f>'📦 商品出厂底价库 (Products)'!F5</f>
       </c>
-      <c r="G7" s="64">
+      <c r="G7" s="69">
         <f>'📦 商品出厂底价库 (Products)'!O5</f>
       </c>
-      <c r="H7" s="64">
+      <c r="H7" s="69">
         <f>'📦 商品出厂底价库 (Products)'!P5</f>
       </c>
-      <c r="I7" s="62">
+      <c r="I7" s="67">
         <f>'📦 商品出厂底价库 (Products)'!J5</f>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="58">
+      <c r="A8" s="63">
         <v>5</v>
       </c>
-      <c r="B8" s="58">
+      <c r="B8" s="63">
         <f>'📦 商品出厂底价库 (Products)'!A6</f>
       </c>
-      <c r="C8" s="59">
+      <c r="C8" s="64">
         <f>'📦 商品出厂底价库 (Products)'!C6</f>
       </c>
-      <c r="D8" s="60">
+      <c r="D8" s="65">
         <f>'📦 商品出厂底价库 (Products)'!E6</f>
       </c>
-      <c r="E8" s="61">
+      <c r="E8" s="66">
         <f>'📦 商品出厂底价库 (Products)'!N6</f>
       </c>
-      <c r="F8" s="60">
+      <c r="F8" s="65">
         <f>'📦 商品出厂底价库 (Products)'!F6</f>
       </c>
-      <c r="G8" s="60">
+      <c r="G8" s="65">
         <f>'📦 商品出厂底价库 (Products)'!O6</f>
       </c>
-      <c r="H8" s="60">
+      <c r="H8" s="65">
         <f>'📦 商品出厂底价库 (Products)'!P6</f>
       </c>
-      <c r="I8" s="58">
+      <c r="I8" s="63">
         <f>'📦 商品出厂底价库 (Products)'!J6</f>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="62">
+      <c r="A9" s="67">
         <v>6</v>
       </c>
-      <c r="B9" s="62">
+      <c r="B9" s="67">
         <f>'📦 商品出厂底价库 (Products)'!A7</f>
       </c>
-      <c r="C9" s="63">
+      <c r="C9" s="68">
         <f>'📦 商品出厂底价库 (Products)'!C7</f>
       </c>
-      <c r="D9" s="64">
+      <c r="D9" s="69">
         <f>'📦 商品出厂底价库 (Products)'!E7</f>
       </c>
-      <c r="E9" s="65">
+      <c r="E9" s="70">
         <f>'📦 商品出厂底价库 (Products)'!N7</f>
       </c>
-      <c r="F9" s="64">
+      <c r="F9" s="69">
         <f>'📦 商品出厂底价库 (Products)'!F7</f>
       </c>
-      <c r="G9" s="64">
+      <c r="G9" s="69">
         <f>'📦 商品出厂底价库 (Products)'!O7</f>
       </c>
-      <c r="H9" s="64">
+      <c r="H9" s="69">
         <f>'📦 商品出厂底价库 (Products)'!P7</f>
       </c>
-      <c r="I9" s="62">
+      <c r="I9" s="67">
         <f>'📦 商品出厂底价库 (Products)'!J7</f>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(lead_magnets): expand column widths, increase quote row height, and pre-populate 30 smart formula rows
</commit_message>
<xml_diff>
--- a/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
+++ b/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="160">
   <si>
     <t>【2026外贸出厂底价表与智能核价模板】使用指南</t>
   </si>
@@ -70,7 +70,7 @@
     <t>USD</t>
   </si>
   <si>
-    <t>👈 下拉切换币种：底价库与对外脱敏报价单秒级全表自适应！</t>
+    <t>👈 下拉切换主币种：全库底价与对外报价单秒级自适应！</t>
   </si>
   <si>
     <t>外币币种 (Target Currency)</t>
@@ -470,9 +470,6 @@
   </si>
   <si>
     <t>FORMAL COMMERCIAL OFFER (FOB SHENZHEN)</t>
-  </si>
-  <si>
-    <t>Payment: 30% T/T Deposit, 70% Balance Before Shipment  |  Price Validity: 30 Days</t>
   </si>
   <si>
     <t>Item</t>
@@ -732,7 +729,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -854,6 +851,9 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="166" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -890,6 +890,9 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="166" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -921,28 +924,28 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="3" fontId="21" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="22" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="3" fontId="21" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="22" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1358,11 +1361,11 @@
   <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="1" max="1" width="48" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
-    <col min="5" max="5" width="66" customWidth="1"/>
+    <col min="5" max="5" width="72" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1860,7 +1863,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1940,101 +1943,101 @@
       <c r="B2" s="40" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="40" t="s">
+      <c r="C2" s="41" t="s">
         <v>127</v>
       </c>
-      <c r="D2" s="41">
+      <c r="D2" s="42">
         <v>15.5</v>
       </c>
-      <c r="E2" s="42">
+      <c r="E2" s="43">
         <v>500</v>
       </c>
-      <c r="F2" s="42">
+      <c r="F2" s="43">
         <v>50</v>
       </c>
-      <c r="G2" s="43">
+      <c r="G2" s="44">
         <v>0.045</v>
       </c>
-      <c r="H2" s="44">
+      <c r="H2" s="45">
         <v>14.5</v>
       </c>
-      <c r="I2" s="45"/>
+      <c r="I2" s="46"/>
       <c r="J2" s="39" t="s">
         <v>128</v>
       </c>
       <c r="K2" s="39" t="s">
         <v>129</v>
       </c>
-      <c r="L2" s="46">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
-      </c>
-      <c r="M2" s="47">
-        <f>IF(ISBLANK(I2), '⚙️ 全局核算参数 (Config)'!$B$13, I2)</f>
-      </c>
-      <c r="N2" s="48">
-        <f>ROUND(((D2 * (1 + M2) + L2) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
-      </c>
-      <c r="O2" s="49">
-        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G2)) * F2, "-")</f>
-      </c>
-      <c r="P2" s="49">
-        <f>IF(AND(G2&gt;0, F2&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G2)) * F2, "-")</f>
-      </c>
-      <c r="Q2" s="50">
-        <f>IF(M2&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M2&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="51" t="s">
+      <c r="L2" s="47">
+        <f>IF(ISBLANK(D2), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M2" s="48">
+        <f>IF(ISBLANK(D2), "", IF(ISBLANK(I2), '⚙️ 全局核算参数 (Config)'!$B$13, I2))</f>
+      </c>
+      <c r="N2" s="49">
+        <f>IF(ISBLANK(D2), "", ROUND(((D2 * (1 + M2) + L2) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O2" s="50">
+        <f>IF(OR(ISBLANK(D2), NOT(AND(G2&gt;0, F2&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G2)) * F2)</f>
+      </c>
+      <c r="P2" s="50">
+        <f>IF(OR(ISBLANK(D2), NOT(AND(G2&gt;0, F2&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G2)) * F2)</f>
+      </c>
+      <c r="Q2" s="51">
+        <f>IF(ISBLANK(D2), "", IF(M2&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M2&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="52" t="s">
         <v>130</v>
       </c>
-      <c r="B3" s="52" t="s">
+      <c r="B3" s="53" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="52" t="s">
+      <c r="C3" s="54" t="s">
         <v>132</v>
       </c>
-      <c r="D3" s="53">
+      <c r="D3" s="55">
         <v>0.85</v>
       </c>
-      <c r="E3" s="54">
+      <c r="E3" s="56">
         <v>5000</v>
       </c>
-      <c r="F3" s="54">
+      <c r="F3" s="56">
         <v>1000</v>
       </c>
-      <c r="G3" s="55">
+      <c r="G3" s="57">
         <v>0.02</v>
       </c>
-      <c r="H3" s="56">
+      <c r="H3" s="58">
         <v>18</v>
       </c>
-      <c r="I3" s="57">
+      <c r="I3" s="59">
         <v>0.18</v>
       </c>
-      <c r="J3" s="51" t="s">
+      <c r="J3" s="52" t="s">
         <v>133</v>
       </c>
-      <c r="K3" s="51" t="s">
+      <c r="K3" s="52" t="s">
         <v>134</v>
       </c>
-      <c r="L3" s="46">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
-      </c>
-      <c r="M3" s="47">
-        <f>IF(ISBLANK(I3), '⚙️ 全局核算参数 (Config)'!$B$13, I3)</f>
-      </c>
-      <c r="N3" s="48">
-        <f>ROUND(((D3 * (1 + M3) + L3) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
-      </c>
-      <c r="O3" s="49">
-        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G3)) * F3, "-")</f>
-      </c>
-      <c r="P3" s="49">
-        <f>IF(AND(G3&gt;0, F3&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G3)) * F3, "-")</f>
-      </c>
-      <c r="Q3" s="50">
-        <f>IF(M3&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M3&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      <c r="L3" s="47">
+        <f>IF(ISBLANK(D3), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M3" s="48">
+        <f>IF(ISBLANK(D3), "", IF(ISBLANK(I3), '⚙️ 全局核算参数 (Config)'!$B$13, I3))</f>
+      </c>
+      <c r="N3" s="49">
+        <f>IF(ISBLANK(D3), "", ROUND(((D3 * (1 + M3) + L3) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O3" s="50">
+        <f>IF(OR(ISBLANK(D3), NOT(AND(G3&gt;0, F3&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G3)) * F3)</f>
+      </c>
+      <c r="P3" s="50">
+        <f>IF(OR(ISBLANK(D3), NOT(AND(G3&gt;0, F3&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G3)) * F3)</f>
+      </c>
+      <c r="Q3" s="51">
+        <f>IF(ISBLANK(D3), "", IF(M3&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M3&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -2044,25 +2047,25 @@
       <c r="B4" s="40" t="s">
         <v>136</v>
       </c>
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="41" t="s">
         <v>137</v>
       </c>
-      <c r="D4" s="41">
+      <c r="D4" s="42">
         <v>185</v>
       </c>
-      <c r="E4" s="42">
+      <c r="E4" s="43">
         <v>50</v>
       </c>
-      <c r="F4" s="42">
+      <c r="F4" s="43">
         <v>1</v>
       </c>
-      <c r="G4" s="43">
+      <c r="G4" s="44">
         <v>0.16</v>
       </c>
-      <c r="H4" s="44">
+      <c r="H4" s="45">
         <v>16.2</v>
       </c>
-      <c r="I4" s="45">
+      <c r="I4" s="46">
         <v>0.25</v>
       </c>
       <c r="J4" s="39" t="s">
@@ -2071,74 +2074,74 @@
       <c r="K4" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="L4" s="46">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
-      </c>
-      <c r="M4" s="47">
-        <f>IF(ISBLANK(I4), '⚙️ 全局核算参数 (Config)'!$B$13, I4)</f>
-      </c>
-      <c r="N4" s="48">
-        <f>ROUND(((D4 * (1 + M4) + L4) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
-      </c>
-      <c r="O4" s="49">
-        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G4)) * F4, "-")</f>
-      </c>
-      <c r="P4" s="49">
-        <f>IF(AND(G4&gt;0, F4&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G4)) * F4, "-")</f>
-      </c>
-      <c r="Q4" s="50">
-        <f>IF(M4&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M4&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      <c r="L4" s="47">
+        <f>IF(ISBLANK(D4), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M4" s="48">
+        <f>IF(ISBLANK(D4), "", IF(ISBLANK(I4), '⚙️ 全局核算参数 (Config)'!$B$13, I4))</f>
+      </c>
+      <c r="N4" s="49">
+        <f>IF(ISBLANK(D4), "", ROUND(((D4 * (1 + M4) + L4) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O4" s="50">
+        <f>IF(OR(ISBLANK(D4), NOT(AND(G4&gt;0, F4&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G4)) * F4)</f>
+      </c>
+      <c r="P4" s="50">
+        <f>IF(OR(ISBLANK(D4), NOT(AND(G4&gt;0, F4&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G4)) * F4)</f>
+      </c>
+      <c r="Q4" s="51">
+        <f>IF(ISBLANK(D4), "", IF(M4&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M4&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="52" t="s">
         <v>140</v>
       </c>
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="53" t="s">
         <v>141</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="54" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="53">
+      <c r="D5" s="55">
         <v>38</v>
       </c>
-      <c r="E5" s="54">
+      <c r="E5" s="56">
         <v>200</v>
       </c>
-      <c r="F5" s="54">
+      <c r="F5" s="56">
         <v>5</v>
       </c>
-      <c r="G5" s="55">
+      <c r="G5" s="57">
         <v>0.08</v>
       </c>
-      <c r="H5" s="56">
+      <c r="H5" s="58">
         <v>11</v>
       </c>
-      <c r="I5" s="57"/>
-      <c r="J5" s="51" t="s">
+      <c r="I5" s="59"/>
+      <c r="J5" s="52" t="s">
         <v>143</v>
       </c>
-      <c r="K5" s="51" t="s">
+      <c r="K5" s="52" t="s">
         <v>144</v>
       </c>
-      <c r="L5" s="46">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
-      </c>
-      <c r="M5" s="47">
-        <f>IF(ISBLANK(I5), '⚙️ 全局核算参数 (Config)'!$B$13, I5)</f>
-      </c>
-      <c r="N5" s="48">
-        <f>ROUND(((D5 * (1 + M5) + L5) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
-      </c>
-      <c r="O5" s="49">
-        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G5)) * F5, "-")</f>
-      </c>
-      <c r="P5" s="49">
-        <f>IF(AND(G5&gt;0, F5&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G5)) * F5, "-")</f>
-      </c>
-      <c r="Q5" s="50">
-        <f>IF(M5&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M5&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      <c r="L5" s="47">
+        <f>IF(ISBLANK(D5), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M5" s="48">
+        <f>IF(ISBLANK(D5), "", IF(ISBLANK(I5), '⚙️ 全局核算参数 (Config)'!$B$13, I5))</f>
+      </c>
+      <c r="N5" s="49">
+        <f>IF(ISBLANK(D5), "", ROUND(((D5 * (1 + M5) + L5) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O5" s="50">
+        <f>IF(OR(ISBLANK(D5), NOT(AND(G5&gt;0, F5&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G5)) * F5)</f>
+      </c>
+      <c r="P5" s="50">
+        <f>IF(OR(ISBLANK(D5), NOT(AND(G5&gt;0, F5&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G5)) * F5)</f>
+      </c>
+      <c r="Q5" s="51">
+        <f>IF(ISBLANK(D5), "", IF(M5&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M5&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -2148,99 +2151,843 @@
       <c r="B6" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="40" t="s">
+      <c r="C6" s="41" t="s">
         <v>147</v>
       </c>
-      <c r="D6" s="41">
+      <c r="D6" s="42">
         <v>24</v>
       </c>
-      <c r="E6" s="42">
+      <c r="E6" s="43">
         <v>300</v>
       </c>
-      <c r="F6" s="42">
+      <c r="F6" s="43">
         <v>20</v>
       </c>
-      <c r="G6" s="43">
+      <c r="G6" s="44">
         <v>0.055</v>
       </c>
-      <c r="H6" s="44">
+      <c r="H6" s="45">
         <v>9.5</v>
       </c>
-      <c r="I6" s="45"/>
+      <c r="I6" s="46"/>
       <c r="J6" s="39" t="s">
         <v>128</v>
       </c>
       <c r="K6" s="39" t="s">
         <v>144</v>
       </c>
-      <c r="L6" s="46">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
-      </c>
-      <c r="M6" s="47">
-        <f>IF(ISBLANK(I6), '⚙️ 全局核算参数 (Config)'!$B$13, I6)</f>
-      </c>
-      <c r="N6" s="48">
-        <f>ROUND(((D6 * (1 + M6) + L6) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
-      </c>
-      <c r="O6" s="49">
-        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G6)) * F6, "-")</f>
-      </c>
-      <c r="P6" s="49">
-        <f>IF(AND(G6&gt;0, F6&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G6)) * F6, "-")</f>
-      </c>
-      <c r="Q6" s="50">
-        <f>IF(M6&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M6&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      <c r="L6" s="47">
+        <f>IF(ISBLANK(D6), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M6" s="48">
+        <f>IF(ISBLANK(D6), "", IF(ISBLANK(I6), '⚙️ 全局核算参数 (Config)'!$B$13, I6))</f>
+      </c>
+      <c r="N6" s="49">
+        <f>IF(ISBLANK(D6), "", ROUND(((D6 * (1 + M6) + L6) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O6" s="50">
+        <f>IF(OR(ISBLANK(D6), NOT(AND(G6&gt;0, F6&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G6)) * F6)</f>
+      </c>
+      <c r="P6" s="50">
+        <f>IF(OR(ISBLANK(D6), NOT(AND(G6&gt;0, F6&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G6)) * F6)</f>
+      </c>
+      <c r="Q6" s="51">
+        <f>IF(ISBLANK(D6), "", IF(M6&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M6&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="51" t="s">
+      <c r="A7" s="52" t="s">
         <v>148</v>
       </c>
-      <c r="B7" s="52" t="s">
+      <c r="B7" s="53" t="s">
         <v>149</v>
       </c>
-      <c r="C7" s="52" t="s">
+      <c r="C7" s="54" t="s">
         <v>147</v>
       </c>
-      <c r="D7" s="53">
+      <c r="D7" s="55">
         <v>25</v>
       </c>
-      <c r="E7" s="54">
+      <c r="E7" s="56">
         <v>300</v>
       </c>
-      <c r="F7" s="54">
+      <c r="F7" s="56">
         <v>20</v>
       </c>
-      <c r="G7" s="55">
+      <c r="G7" s="57">
         <v>0.055</v>
       </c>
-      <c r="H7" s="56">
+      <c r="H7" s="58">
         <v>9.5</v>
       </c>
-      <c r="I7" s="57"/>
-      <c r="J7" s="51" t="s">
+      <c r="I7" s="59"/>
+      <c r="J7" s="52" t="s">
         <v>128</v>
       </c>
-      <c r="K7" s="51" t="s">
+      <c r="K7" s="52" t="s">
         <v>144</v>
       </c>
-      <c r="L7" s="46">
-        <f>'⚙️ 全局核算参数 (Config)'!$C$21</f>
-      </c>
-      <c r="M7" s="47">
-        <f>IF(ISBLANK(I7), '⚙️ 全局核算参数 (Config)'!$B$13, I7)</f>
-      </c>
-      <c r="N7" s="48">
-        <f>ROUND(((D7 * (1 + M7) + L7) / '⚙️ 全局核算参数 (Config)'!$C$4), 2)</f>
-      </c>
-      <c r="O7" s="49">
-        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G7)) * F7, "-")</f>
-      </c>
-      <c r="P7" s="49">
-        <f>IF(AND(G7&gt;0, F7&gt;0), INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G7)) * F7, "-")</f>
-      </c>
-      <c r="Q7" s="50">
-        <f>IF(M7&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M7&gt;=0.25, "💎 高毛利款", "✅ 利润健康"))</f>
+      <c r="L7" s="47">
+        <f>IF(ISBLANK(D7), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M7" s="48">
+        <f>IF(ISBLANK(D7), "", IF(ISBLANK(I7), '⚙️ 全局核算参数 (Config)'!$B$13, I7))</f>
+      </c>
+      <c r="N7" s="49">
+        <f>IF(ISBLANK(D7), "", ROUND(((D7 * (1 + M7) + L7) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O7" s="50">
+        <f>IF(OR(ISBLANK(D7), NOT(AND(G7&gt;0, F7&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G7)) * F7)</f>
+      </c>
+      <c r="P7" s="50">
+        <f>IF(OR(ISBLANK(D7), NOT(AND(G7&gt;0, F7&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G7)) * F7)</f>
+      </c>
+      <c r="Q7" s="51">
+        <f>IF(ISBLANK(D7), "", IF(M7&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M7&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" s="39"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="46"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="47">
+        <f>IF(ISBLANK(D8), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M8" s="48">
+        <f>IF(ISBLANK(D8), "", IF(ISBLANK(I8), '⚙️ 全局核算参数 (Config)'!$B$13, I8))</f>
+      </c>
+      <c r="N8" s="49">
+        <f>IF(ISBLANK(D8), "", ROUND(((D8 * (1 + M8) + L8) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O8" s="50">
+        <f>IF(OR(ISBLANK(D8), NOT(AND(G8&gt;0, F8&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G8)) * F8)</f>
+      </c>
+      <c r="P8" s="50">
+        <f>IF(OR(ISBLANK(D8), NOT(AND(G8&gt;0, F8&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G8)) * F8)</f>
+      </c>
+      <c r="Q8" s="51">
+        <f>IF(ISBLANK(D8), "", IF(M8&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M8&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="52"/>
+      <c r="B9" s="53"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="55"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="57"/>
+      <c r="H9" s="58"/>
+      <c r="I9" s="59"/>
+      <c r="J9" s="52"/>
+      <c r="K9" s="52"/>
+      <c r="L9" s="47">
+        <f>IF(ISBLANK(D9), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M9" s="48">
+        <f>IF(ISBLANK(D9), "", IF(ISBLANK(I9), '⚙️ 全局核算参数 (Config)'!$B$13, I9))</f>
+      </c>
+      <c r="N9" s="49">
+        <f>IF(ISBLANK(D9), "", ROUND(((D9 * (1 + M9) + L9) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O9" s="50">
+        <f>IF(OR(ISBLANK(D9), NOT(AND(G9&gt;0, F9&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G9)) * F9)</f>
+      </c>
+      <c r="P9" s="50">
+        <f>IF(OR(ISBLANK(D9), NOT(AND(G9&gt;0, F9&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G9)) * F9)</f>
+      </c>
+      <c r="Q9" s="51">
+        <f>IF(ISBLANK(D9), "", IF(M9&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M9&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" s="39"/>
+      <c r="B10" s="40"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="45"/>
+      <c r="I10" s="46"/>
+      <c r="J10" s="39"/>
+      <c r="K10" s="39"/>
+      <c r="L10" s="47">
+        <f>IF(ISBLANK(D10), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M10" s="48">
+        <f>IF(ISBLANK(D10), "", IF(ISBLANK(I10), '⚙️ 全局核算参数 (Config)'!$B$13, I10))</f>
+      </c>
+      <c r="N10" s="49">
+        <f>IF(ISBLANK(D10), "", ROUND(((D10 * (1 + M10) + L10) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O10" s="50">
+        <f>IF(OR(ISBLANK(D10), NOT(AND(G10&gt;0, F10&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G10)) * F10)</f>
+      </c>
+      <c r="P10" s="50">
+        <f>IF(OR(ISBLANK(D10), NOT(AND(G10&gt;0, F10&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G10)) * F10)</f>
+      </c>
+      <c r="Q10" s="51">
+        <f>IF(ISBLANK(D10), "", IF(M10&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M10&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" s="52"/>
+      <c r="B11" s="53"/>
+      <c r="C11" s="54"/>
+      <c r="D11" s="55"/>
+      <c r="E11" s="56"/>
+      <c r="F11" s="56"/>
+      <c r="G11" s="57"/>
+      <c r="H11" s="58"/>
+      <c r="I11" s="59"/>
+      <c r="J11" s="52"/>
+      <c r="K11" s="52"/>
+      <c r="L11" s="47">
+        <f>IF(ISBLANK(D11), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M11" s="48">
+        <f>IF(ISBLANK(D11), "", IF(ISBLANK(I11), '⚙️ 全局核算参数 (Config)'!$B$13, I11))</f>
+      </c>
+      <c r="N11" s="49">
+        <f>IF(ISBLANK(D11), "", ROUND(((D11 * (1 + M11) + L11) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O11" s="50">
+        <f>IF(OR(ISBLANK(D11), NOT(AND(G11&gt;0, F11&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G11)) * F11)</f>
+      </c>
+      <c r="P11" s="50">
+        <f>IF(OR(ISBLANK(D11), NOT(AND(G11&gt;0, F11&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G11)) * F11)</f>
+      </c>
+      <c r="Q11" s="51">
+        <f>IF(ISBLANK(D11), "", IF(M11&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M11&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" s="39"/>
+      <c r="B12" s="40"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="46"/>
+      <c r="J12" s="39"/>
+      <c r="K12" s="39"/>
+      <c r="L12" s="47">
+        <f>IF(ISBLANK(D12), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M12" s="48">
+        <f>IF(ISBLANK(D12), "", IF(ISBLANK(I12), '⚙️ 全局核算参数 (Config)'!$B$13, I12))</f>
+      </c>
+      <c r="N12" s="49">
+        <f>IF(ISBLANK(D12), "", ROUND(((D12 * (1 + M12) + L12) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O12" s="50">
+        <f>IF(OR(ISBLANK(D12), NOT(AND(G12&gt;0, F12&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G12)) * F12)</f>
+      </c>
+      <c r="P12" s="50">
+        <f>IF(OR(ISBLANK(D12), NOT(AND(G12&gt;0, F12&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G12)) * F12)</f>
+      </c>
+      <c r="Q12" s="51">
+        <f>IF(ISBLANK(D12), "", IF(M12&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M12&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" s="52"/>
+      <c r="B13" s="53"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="55"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="56"/>
+      <c r="G13" s="57"/>
+      <c r="H13" s="58"/>
+      <c r="I13" s="59"/>
+      <c r="J13" s="52"/>
+      <c r="K13" s="52"/>
+      <c r="L13" s="47">
+        <f>IF(ISBLANK(D13), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M13" s="48">
+        <f>IF(ISBLANK(D13), "", IF(ISBLANK(I13), '⚙️ 全局核算参数 (Config)'!$B$13, I13))</f>
+      </c>
+      <c r="N13" s="49">
+        <f>IF(ISBLANK(D13), "", ROUND(((D13 * (1 + M13) + L13) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O13" s="50">
+        <f>IF(OR(ISBLANK(D13), NOT(AND(G13&gt;0, F13&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G13)) * F13)</f>
+      </c>
+      <c r="P13" s="50">
+        <f>IF(OR(ISBLANK(D13), NOT(AND(G13&gt;0, F13&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G13)) * F13)</f>
+      </c>
+      <c r="Q13" s="51">
+        <f>IF(ISBLANK(D13), "", IF(M13&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M13&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" s="39"/>
+      <c r="B14" s="40"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="45"/>
+      <c r="I14" s="46"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
+      <c r="L14" s="47">
+        <f>IF(ISBLANK(D14), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M14" s="48">
+        <f>IF(ISBLANK(D14), "", IF(ISBLANK(I14), '⚙️ 全局核算参数 (Config)'!$B$13, I14))</f>
+      </c>
+      <c r="N14" s="49">
+        <f>IF(ISBLANK(D14), "", ROUND(((D14 * (1 + M14) + L14) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O14" s="50">
+        <f>IF(OR(ISBLANK(D14), NOT(AND(G14&gt;0, F14&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G14)) * F14)</f>
+      </c>
+      <c r="P14" s="50">
+        <f>IF(OR(ISBLANK(D14), NOT(AND(G14&gt;0, F14&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G14)) * F14)</f>
+      </c>
+      <c r="Q14" s="51">
+        <f>IF(ISBLANK(D14), "", IF(M14&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M14&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" s="52"/>
+      <c r="B15" s="53"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="55"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="56"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="58"/>
+      <c r="I15" s="59"/>
+      <c r="J15" s="52"/>
+      <c r="K15" s="52"/>
+      <c r="L15" s="47">
+        <f>IF(ISBLANK(D15), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M15" s="48">
+        <f>IF(ISBLANK(D15), "", IF(ISBLANK(I15), '⚙️ 全局核算参数 (Config)'!$B$13, I15))</f>
+      </c>
+      <c r="N15" s="49">
+        <f>IF(ISBLANK(D15), "", ROUND(((D15 * (1 + M15) + L15) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O15" s="50">
+        <f>IF(OR(ISBLANK(D15), NOT(AND(G15&gt;0, F15&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G15)) * F15)</f>
+      </c>
+      <c r="P15" s="50">
+        <f>IF(OR(ISBLANK(D15), NOT(AND(G15&gt;0, F15&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G15)) * F15)</f>
+      </c>
+      <c r="Q15" s="51">
+        <f>IF(ISBLANK(D15), "", IF(M15&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M15&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" s="39"/>
+      <c r="B16" s="40"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="44"/>
+      <c r="H16" s="45"/>
+      <c r="I16" s="46"/>
+      <c r="J16" s="39"/>
+      <c r="K16" s="39"/>
+      <c r="L16" s="47">
+        <f>IF(ISBLANK(D16), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M16" s="48">
+        <f>IF(ISBLANK(D16), "", IF(ISBLANK(I16), '⚙️ 全局核算参数 (Config)'!$B$13, I16))</f>
+      </c>
+      <c r="N16" s="49">
+        <f>IF(ISBLANK(D16), "", ROUND(((D16 * (1 + M16) + L16) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O16" s="50">
+        <f>IF(OR(ISBLANK(D16), NOT(AND(G16&gt;0, F16&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G16)) * F16)</f>
+      </c>
+      <c r="P16" s="50">
+        <f>IF(OR(ISBLANK(D16), NOT(AND(G16&gt;0, F16&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G16)) * F16)</f>
+      </c>
+      <c r="Q16" s="51">
+        <f>IF(ISBLANK(D16), "", IF(M16&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M16&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" s="52"/>
+      <c r="B17" s="53"/>
+      <c r="C17" s="54"/>
+      <c r="D17" s="55"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="56"/>
+      <c r="G17" s="57"/>
+      <c r="H17" s="58"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="52"/>
+      <c r="K17" s="52"/>
+      <c r="L17" s="47">
+        <f>IF(ISBLANK(D17), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M17" s="48">
+        <f>IF(ISBLANK(D17), "", IF(ISBLANK(I17), '⚙️ 全局核算参数 (Config)'!$B$13, I17))</f>
+      </c>
+      <c r="N17" s="49">
+        <f>IF(ISBLANK(D17), "", ROUND(((D17 * (1 + M17) + L17) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O17" s="50">
+        <f>IF(OR(ISBLANK(D17), NOT(AND(G17&gt;0, F17&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G17)) * F17)</f>
+      </c>
+      <c r="P17" s="50">
+        <f>IF(OR(ISBLANK(D17), NOT(AND(G17&gt;0, F17&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G17)) * F17)</f>
+      </c>
+      <c r="Q17" s="51">
+        <f>IF(ISBLANK(D17), "", IF(M17&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M17&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" s="39"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="44"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="39"/>
+      <c r="L18" s="47">
+        <f>IF(ISBLANK(D18), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M18" s="48">
+        <f>IF(ISBLANK(D18), "", IF(ISBLANK(I18), '⚙️ 全局核算参数 (Config)'!$B$13, I18))</f>
+      </c>
+      <c r="N18" s="49">
+        <f>IF(ISBLANK(D18), "", ROUND(((D18 * (1 + M18) + L18) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O18" s="50">
+        <f>IF(OR(ISBLANK(D18), NOT(AND(G18&gt;0, F18&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G18)) * F18)</f>
+      </c>
+      <c r="P18" s="50">
+        <f>IF(OR(ISBLANK(D18), NOT(AND(G18&gt;0, F18&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G18)) * F18)</f>
+      </c>
+      <c r="Q18" s="51">
+        <f>IF(ISBLANK(D18), "", IF(M18&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M18&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A19" s="52"/>
+      <c r="B19" s="53"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="55"/>
+      <c r="E19" s="56"/>
+      <c r="F19" s="56"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="58"/>
+      <c r="I19" s="59"/>
+      <c r="J19" s="52"/>
+      <c r="K19" s="52"/>
+      <c r="L19" s="47">
+        <f>IF(ISBLANK(D19), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M19" s="48">
+        <f>IF(ISBLANK(D19), "", IF(ISBLANK(I19), '⚙️ 全局核算参数 (Config)'!$B$13, I19))</f>
+      </c>
+      <c r="N19" s="49">
+        <f>IF(ISBLANK(D19), "", ROUND(((D19 * (1 + M19) + L19) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O19" s="50">
+        <f>IF(OR(ISBLANK(D19), NOT(AND(G19&gt;0, F19&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G19)) * F19)</f>
+      </c>
+      <c r="P19" s="50">
+        <f>IF(OR(ISBLANK(D19), NOT(AND(G19&gt;0, F19&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G19)) * F19)</f>
+      </c>
+      <c r="Q19" s="51">
+        <f>IF(ISBLANK(D19), "", IF(M19&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M19&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A20" s="39"/>
+      <c r="B20" s="40"/>
+      <c r="C20" s="41"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="44"/>
+      <c r="H20" s="45"/>
+      <c r="I20" s="46"/>
+      <c r="J20" s="39"/>
+      <c r="K20" s="39"/>
+      <c r="L20" s="47">
+        <f>IF(ISBLANK(D20), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M20" s="48">
+        <f>IF(ISBLANK(D20), "", IF(ISBLANK(I20), '⚙️ 全局核算参数 (Config)'!$B$13, I20))</f>
+      </c>
+      <c r="N20" s="49">
+        <f>IF(ISBLANK(D20), "", ROUND(((D20 * (1 + M20) + L20) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O20" s="50">
+        <f>IF(OR(ISBLANK(D20), NOT(AND(G20&gt;0, F20&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G20)) * F20)</f>
+      </c>
+      <c r="P20" s="50">
+        <f>IF(OR(ISBLANK(D20), NOT(AND(G20&gt;0, F20&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G20)) * F20)</f>
+      </c>
+      <c r="Q20" s="51">
+        <f>IF(ISBLANK(D20), "", IF(M20&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M20&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A21" s="52"/>
+      <c r="B21" s="53"/>
+      <c r="C21" s="54"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="56"/>
+      <c r="F21" s="56"/>
+      <c r="G21" s="57"/>
+      <c r="H21" s="58"/>
+      <c r="I21" s="59"/>
+      <c r="J21" s="52"/>
+      <c r="K21" s="52"/>
+      <c r="L21" s="47">
+        <f>IF(ISBLANK(D21), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M21" s="48">
+        <f>IF(ISBLANK(D21), "", IF(ISBLANK(I21), '⚙️ 全局核算参数 (Config)'!$B$13, I21))</f>
+      </c>
+      <c r="N21" s="49">
+        <f>IF(ISBLANK(D21), "", ROUND(((D21 * (1 + M21) + L21) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O21" s="50">
+        <f>IF(OR(ISBLANK(D21), NOT(AND(G21&gt;0, F21&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G21)) * F21)</f>
+      </c>
+      <c r="P21" s="50">
+        <f>IF(OR(ISBLANK(D21), NOT(AND(G21&gt;0, F21&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G21)) * F21)</f>
+      </c>
+      <c r="Q21" s="51">
+        <f>IF(ISBLANK(D21), "", IF(M21&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M21&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A22" s="39"/>
+      <c r="B22" s="40"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="44"/>
+      <c r="H22" s="45"/>
+      <c r="I22" s="46"/>
+      <c r="J22" s="39"/>
+      <c r="K22" s="39"/>
+      <c r="L22" s="47">
+        <f>IF(ISBLANK(D22), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M22" s="48">
+        <f>IF(ISBLANK(D22), "", IF(ISBLANK(I22), '⚙️ 全局核算参数 (Config)'!$B$13, I22))</f>
+      </c>
+      <c r="N22" s="49">
+        <f>IF(ISBLANK(D22), "", ROUND(((D22 * (1 + M22) + L22) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O22" s="50">
+        <f>IF(OR(ISBLANK(D22), NOT(AND(G22&gt;0, F22&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G22)) * F22)</f>
+      </c>
+      <c r="P22" s="50">
+        <f>IF(OR(ISBLANK(D22), NOT(AND(G22&gt;0, F22&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G22)) * F22)</f>
+      </c>
+      <c r="Q22" s="51">
+        <f>IF(ISBLANK(D22), "", IF(M22&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M22&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A23" s="52"/>
+      <c r="B23" s="53"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="55"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="59"/>
+      <c r="J23" s="52"/>
+      <c r="K23" s="52"/>
+      <c r="L23" s="47">
+        <f>IF(ISBLANK(D23), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M23" s="48">
+        <f>IF(ISBLANK(D23), "", IF(ISBLANK(I23), '⚙️ 全局核算参数 (Config)'!$B$13, I23))</f>
+      </c>
+      <c r="N23" s="49">
+        <f>IF(ISBLANK(D23), "", ROUND(((D23 * (1 + M23) + L23) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O23" s="50">
+        <f>IF(OR(ISBLANK(D23), NOT(AND(G23&gt;0, F23&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G23)) * F23)</f>
+      </c>
+      <c r="P23" s="50">
+        <f>IF(OR(ISBLANK(D23), NOT(AND(G23&gt;0, F23&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G23)) * F23)</f>
+      </c>
+      <c r="Q23" s="51">
+        <f>IF(ISBLANK(D23), "", IF(M23&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M23&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A24" s="39"/>
+      <c r="B24" s="40"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="45"/>
+      <c r="I24" s="46"/>
+      <c r="J24" s="39"/>
+      <c r="K24" s="39"/>
+      <c r="L24" s="47">
+        <f>IF(ISBLANK(D24), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M24" s="48">
+        <f>IF(ISBLANK(D24), "", IF(ISBLANK(I24), '⚙️ 全局核算参数 (Config)'!$B$13, I24))</f>
+      </c>
+      <c r="N24" s="49">
+        <f>IF(ISBLANK(D24), "", ROUND(((D24 * (1 + M24) + L24) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O24" s="50">
+        <f>IF(OR(ISBLANK(D24), NOT(AND(G24&gt;0, F24&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G24)) * F24)</f>
+      </c>
+      <c r="P24" s="50">
+        <f>IF(OR(ISBLANK(D24), NOT(AND(G24&gt;0, F24&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G24)) * F24)</f>
+      </c>
+      <c r="Q24" s="51">
+        <f>IF(ISBLANK(D24), "", IF(M24&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M24&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A25" s="52"/>
+      <c r="B25" s="53"/>
+      <c r="C25" s="54"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="56"/>
+      <c r="F25" s="56"/>
+      <c r="G25" s="57"/>
+      <c r="H25" s="58"/>
+      <c r="I25" s="59"/>
+      <c r="J25" s="52"/>
+      <c r="K25" s="52"/>
+      <c r="L25" s="47">
+        <f>IF(ISBLANK(D25), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M25" s="48">
+        <f>IF(ISBLANK(D25), "", IF(ISBLANK(I25), '⚙️ 全局核算参数 (Config)'!$B$13, I25))</f>
+      </c>
+      <c r="N25" s="49">
+        <f>IF(ISBLANK(D25), "", ROUND(((D25 * (1 + M25) + L25) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O25" s="50">
+        <f>IF(OR(ISBLANK(D25), NOT(AND(G25&gt;0, F25&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G25)) * F25)</f>
+      </c>
+      <c r="P25" s="50">
+        <f>IF(OR(ISBLANK(D25), NOT(AND(G25&gt;0, F25&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G25)) * F25)</f>
+      </c>
+      <c r="Q25" s="51">
+        <f>IF(ISBLANK(D25), "", IF(M25&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M25&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A26" s="39"/>
+      <c r="B26" s="40"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="45"/>
+      <c r="I26" s="46"/>
+      <c r="J26" s="39"/>
+      <c r="K26" s="39"/>
+      <c r="L26" s="47">
+        <f>IF(ISBLANK(D26), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M26" s="48">
+        <f>IF(ISBLANK(D26), "", IF(ISBLANK(I26), '⚙️ 全局核算参数 (Config)'!$B$13, I26))</f>
+      </c>
+      <c r="N26" s="49">
+        <f>IF(ISBLANK(D26), "", ROUND(((D26 * (1 + M26) + L26) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O26" s="50">
+        <f>IF(OR(ISBLANK(D26), NOT(AND(G26&gt;0, F26&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G26)) * F26)</f>
+      </c>
+      <c r="P26" s="50">
+        <f>IF(OR(ISBLANK(D26), NOT(AND(G26&gt;0, F26&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G26)) * F26)</f>
+      </c>
+      <c r="Q26" s="51">
+        <f>IF(ISBLANK(D26), "", IF(M26&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M26&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A27" s="52"/>
+      <c r="B27" s="53"/>
+      <c r="C27" s="54"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="56"/>
+      <c r="F27" s="56"/>
+      <c r="G27" s="57"/>
+      <c r="H27" s="58"/>
+      <c r="I27" s="59"/>
+      <c r="J27" s="52"/>
+      <c r="K27" s="52"/>
+      <c r="L27" s="47">
+        <f>IF(ISBLANK(D27), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M27" s="48">
+        <f>IF(ISBLANK(D27), "", IF(ISBLANK(I27), '⚙️ 全局核算参数 (Config)'!$B$13, I27))</f>
+      </c>
+      <c r="N27" s="49">
+        <f>IF(ISBLANK(D27), "", ROUND(((D27 * (1 + M27) + L27) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O27" s="50">
+        <f>IF(OR(ISBLANK(D27), NOT(AND(G27&gt;0, F27&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G27)) * F27)</f>
+      </c>
+      <c r="P27" s="50">
+        <f>IF(OR(ISBLANK(D27), NOT(AND(G27&gt;0, F27&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G27)) * F27)</f>
+      </c>
+      <c r="Q27" s="51">
+        <f>IF(ISBLANK(D27), "", IF(M27&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M27&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A28" s="39"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="43"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="45"/>
+      <c r="I28" s="46"/>
+      <c r="J28" s="39"/>
+      <c r="K28" s="39"/>
+      <c r="L28" s="47">
+        <f>IF(ISBLANK(D28), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M28" s="48">
+        <f>IF(ISBLANK(D28), "", IF(ISBLANK(I28), '⚙️ 全局核算参数 (Config)'!$B$13, I28))</f>
+      </c>
+      <c r="N28" s="49">
+        <f>IF(ISBLANK(D28), "", ROUND(((D28 * (1 + M28) + L28) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O28" s="50">
+        <f>IF(OR(ISBLANK(D28), NOT(AND(G28&gt;0, F28&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G28)) * F28)</f>
+      </c>
+      <c r="P28" s="50">
+        <f>IF(OR(ISBLANK(D28), NOT(AND(G28&gt;0, F28&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G28)) * F28)</f>
+      </c>
+      <c r="Q28" s="51">
+        <f>IF(ISBLANK(D28), "", IF(M28&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M28&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A29" s="52"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="54"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
+      <c r="G29" s="57"/>
+      <c r="H29" s="58"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="52"/>
+      <c r="K29" s="52"/>
+      <c r="L29" s="47">
+        <f>IF(ISBLANK(D29), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M29" s="48">
+        <f>IF(ISBLANK(D29), "", IF(ISBLANK(I29), '⚙️ 全局核算参数 (Config)'!$B$13, I29))</f>
+      </c>
+      <c r="N29" s="49">
+        <f>IF(ISBLANK(D29), "", ROUND(((D29 * (1 + M29) + L29) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O29" s="50">
+        <f>IF(OR(ISBLANK(D29), NOT(AND(G29&gt;0, F29&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G29)) * F29)</f>
+      </c>
+      <c r="P29" s="50">
+        <f>IF(OR(ISBLANK(D29), NOT(AND(G29&gt;0, F29&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G29)) * F29)</f>
+      </c>
+      <c r="Q29" s="51">
+        <f>IF(ISBLANK(D29), "", IF(M29&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M29&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A30" s="39"/>
+      <c r="B30" s="40"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="43"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="45"/>
+      <c r="I30" s="46"/>
+      <c r="J30" s="39"/>
+      <c r="K30" s="39"/>
+      <c r="L30" s="47">
+        <f>IF(ISBLANK(D30), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M30" s="48">
+        <f>IF(ISBLANK(D30), "", IF(ISBLANK(I30), '⚙️ 全局核算参数 (Config)'!$B$13, I30))</f>
+      </c>
+      <c r="N30" s="49">
+        <f>IF(ISBLANK(D30), "", ROUND(((D30 * (1 + M30) + L30) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O30" s="50">
+        <f>IF(OR(ISBLANK(D30), NOT(AND(G30&gt;0, F30&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G30)) * F30)</f>
+      </c>
+      <c r="P30" s="50">
+        <f>IF(OR(ISBLANK(D30), NOT(AND(G30&gt;0, F30&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G30)) * F30)</f>
+      </c>
+      <c r="Q30" s="51">
+        <f>IF(ISBLANK(D30), "", IF(M30&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M30&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A31" s="52"/>
+      <c r="B31" s="53"/>
+      <c r="C31" s="54"/>
+      <c r="D31" s="55"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="56"/>
+      <c r="G31" s="57"/>
+      <c r="H31" s="58"/>
+      <c r="I31" s="59"/>
+      <c r="J31" s="52"/>
+      <c r="K31" s="52"/>
+      <c r="L31" s="47">
+        <f>IF(ISBLANK(D31), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M31" s="48">
+        <f>IF(ISBLANK(D31), "", IF(ISBLANK(I31), '⚙️ 全局核算参数 (Config)'!$B$13, I31))</f>
+      </c>
+      <c r="N31" s="49">
+        <f>IF(ISBLANK(D31), "", ROUND(((D31 * (1 + M31) + L31) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O31" s="50">
+        <f>IF(OR(ISBLANK(D31), NOT(AND(G31&gt;0, F31&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G31)) * F31)</f>
+      </c>
+      <c r="P31" s="50">
+        <f>IF(OR(ISBLANK(D31), NOT(AND(G31&gt;0, F31&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G31)) * F31)</f>
+      </c>
+      <c r="Q31" s="51">
+        <f>IF(ISBLANK(D31), "", IF(M31&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M31&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
       </c>
     </row>
   </sheetData>
@@ -2251,12 +2998,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="3" max="3" width="62" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
@@ -2265,238 +3012,935 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="60" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="59" t="s">
+      <c r="B1" s="60"/>
+      <c r="C1" s="61" t="s">
         <v>151</v>
       </c>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
     </row>
     <row r="2" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="60" t="str">
+      <c r="A2" s="62" t="str">
         <f>"Trade Term: FOB · " &amp; '⚙️ 全局核算参数 (Config)'!$B$4 &amp; " (" &amp; '⚙️ 全局核算参数 (Config)'!$D$4 &amp; ")"</f>
         <v>Trade Term: FOB · USD ($)</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="61" t="s">
+      <c r="B2" s="62"/>
+      <c r="C2" s="63" t="str">
+        <f>"Payment: 30% T/T Deposit, 70% Balance Before Shipment  |  Price Validity: " &amp; '⚙️ 全局核算参数 (Config)'!$B$16</f>
+        <v>Payment: 30% T/T Deposit, 70% Balance Before Shipment  |  Price Validity: 30 Days</v>
+      </c>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+    </row>
+    <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="64" t="s">
         <v>152</v>
       </c>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-    </row>
-    <row r="3" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="62" t="s">
+      <c r="B3" s="64" t="s">
         <v>153</v>
       </c>
-      <c r="B3" s="62" t="s">
+      <c r="C3" s="64" t="s">
         <v>154</v>
       </c>
-      <c r="C3" s="62" t="s">
+      <c r="D3" s="64" t="s">
         <v>155</v>
       </c>
-      <c r="D3" s="62" t="s">
-        <v>156</v>
-      </c>
-      <c r="E3" s="62" t="str">
+      <c r="E3" s="64" t="str">
         <f>"FOB Price (" &amp; '⚙️ 全局核算参数 (Config)'!$B$4 &amp; ")"</f>
         <v>FOB Price (USD)</v>
       </c>
-      <c r="F3" s="62" t="s">
+      <c r="F3" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="G3" s="64" t="s">
         <v>157</v>
       </c>
-      <c r="G3" s="62" t="s">
+      <c r="H3" s="64" t="s">
         <v>158</v>
       </c>
-      <c r="H3" s="62" t="s">
+      <c r="I3" s="64" t="s">
         <v>159</v>
       </c>
-      <c r="I3" s="62" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="63">
-        <v>1</v>
-      </c>
-      <c r="B4" s="63">
-        <f>'📦 商品出厂底价库 (Products)'!A2</f>
-      </c>
-      <c r="C4" s="64">
-        <f>'📦 商品出厂底价库 (Products)'!C2</f>
-      </c>
-      <c r="D4" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!E2</f>
-      </c>
-      <c r="E4" s="66">
-        <f>'📦 商品出厂底价库 (Products)'!N2</f>
-      </c>
-      <c r="F4" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!F2</f>
-      </c>
-      <c r="G4" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!O2</f>
-      </c>
-      <c r="H4" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!P2</f>
-      </c>
-      <c r="I4" s="63">
-        <f>'📦 商品出厂底价库 (Products)'!J2</f>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="67">
-        <v>2</v>
-      </c>
-      <c r="B5" s="67">
-        <f>'📦 商品出厂底价库 (Products)'!A3</f>
-      </c>
-      <c r="C5" s="68">
-        <f>'📦 商品出厂底价库 (Products)'!C3</f>
-      </c>
-      <c r="D5" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!E3</f>
-      </c>
-      <c r="E5" s="70">
-        <f>'📦 商品出厂底价库 (Products)'!N3</f>
-      </c>
-      <c r="F5" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!F3</f>
-      </c>
-      <c r="G5" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!O3</f>
-      </c>
-      <c r="H5" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!P3</f>
-      </c>
-      <c r="I5" s="67">
-        <f>'📦 商品出厂底价库 (Products)'!J3</f>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="63">
-        <v>3</v>
-      </c>
-      <c r="B6" s="63">
-        <f>'📦 商品出厂底价库 (Products)'!A4</f>
-      </c>
-      <c r="C6" s="64">
-        <f>'📦 商品出厂底价库 (Products)'!C4</f>
-      </c>
-      <c r="D6" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!E4</f>
-      </c>
-      <c r="E6" s="66">
-        <f>'📦 商品出厂底价库 (Products)'!N4</f>
-      </c>
-      <c r="F6" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!F4</f>
-      </c>
-      <c r="G6" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!O4</f>
-      </c>
-      <c r="H6" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!P4</f>
-      </c>
-      <c r="I6" s="63">
-        <f>'📦 商品出厂底价库 (Products)'!J4</f>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="67">
-        <v>4</v>
-      </c>
-      <c r="B7" s="67">
-        <f>'📦 商品出厂底价库 (Products)'!A5</f>
-      </c>
-      <c r="C7" s="68">
-        <f>'📦 商品出厂底价库 (Products)'!C5</f>
-      </c>
-      <c r="D7" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!E5</f>
-      </c>
-      <c r="E7" s="70">
-        <f>'📦 商品出厂底价库 (Products)'!N5</f>
-      </c>
-      <c r="F7" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!F5</f>
-      </c>
-      <c r="G7" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!O5</f>
-      </c>
-      <c r="H7" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!P5</f>
-      </c>
-      <c r="I7" s="67">
-        <f>'📦 商品出厂底价库 (Products)'!J5</f>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="63">
-        <v>5</v>
-      </c>
-      <c r="B8" s="63">
-        <f>'📦 商品出厂底价库 (Products)'!A6</f>
-      </c>
-      <c r="C8" s="64">
-        <f>'📦 商品出厂底价库 (Products)'!C6</f>
-      </c>
-      <c r="D8" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!E6</f>
-      </c>
-      <c r="E8" s="66">
-        <f>'📦 商品出厂底价库 (Products)'!N6</f>
-      </c>
-      <c r="F8" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!F6</f>
-      </c>
-      <c r="G8" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!O6</f>
-      </c>
-      <c r="H8" s="65">
-        <f>'📦 商品出厂底价库 (Products)'!P6</f>
-      </c>
-      <c r="I8" s="63">
-        <f>'📦 商品出厂底价库 (Products)'!J6</f>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="67">
-        <v>6</v>
-      </c>
-      <c r="B9" s="67">
-        <f>'📦 商品出厂底价库 (Products)'!A7</f>
-      </c>
-      <c r="C9" s="68">
-        <f>'📦 商品出厂底价库 (Products)'!C7</f>
-      </c>
-      <c r="D9" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!E7</f>
-      </c>
-      <c r="E9" s="70">
-        <f>'📦 商品出厂底价库 (Products)'!N7</f>
-      </c>
-      <c r="F9" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!F7</f>
-      </c>
-      <c r="G9" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!O7</f>
-      </c>
-      <c r="H9" s="69">
-        <f>'📦 商品出厂底价库 (Products)'!P7</f>
-      </c>
-      <c r="I9" s="67">
-        <f>'📦 商品出厂底价库 (Products)'!J7</f>
+    </row>
+    <row r="4" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A2), "", 1)</f>
+      </c>
+      <c r="B4" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A2), "", '📦 商品出厂底价库 (Products)'!A2)</f>
+      </c>
+      <c r="C4" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A2), "", '📦 商品出厂底价库 (Products)'!C2)</f>
+      </c>
+      <c r="D4" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A2), "", '📦 商品出厂底价库 (Products)'!E2)</f>
+      </c>
+      <c r="E4" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A2), "", '📦 商品出厂底价库 (Products)'!N2)</f>
+      </c>
+      <c r="F4" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A2), "", '📦 商品出厂底价库 (Products)'!F2)</f>
+      </c>
+      <c r="G4" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A2), "", '📦 商品出厂底价库 (Products)'!O2)</f>
+      </c>
+      <c r="H4" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A2), "", '📦 商品出厂底价库 (Products)'!P2)</f>
+      </c>
+      <c r="I4" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A2), "", '📦 商品出厂底价库 (Products)'!J2)</f>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A3), "", 2)</f>
+      </c>
+      <c r="B5" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A3), "", '📦 商品出厂底价库 (Products)'!A3)</f>
+      </c>
+      <c r="C5" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A3), "", '📦 商品出厂底价库 (Products)'!C3)</f>
+      </c>
+      <c r="D5" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A3), "", '📦 商品出厂底价库 (Products)'!E3)</f>
+      </c>
+      <c r="E5" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A3), "", '📦 商品出厂底价库 (Products)'!N3)</f>
+      </c>
+      <c r="F5" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A3), "", '📦 商品出厂底价库 (Products)'!F3)</f>
+      </c>
+      <c r="G5" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A3), "", '📦 商品出厂底价库 (Products)'!O3)</f>
+      </c>
+      <c r="H5" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A3), "", '📦 商品出厂底价库 (Products)'!P3)</f>
+      </c>
+      <c r="I5" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A3), "", '📦 商品出厂底价库 (Products)'!J3)</f>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A4), "", 3)</f>
+      </c>
+      <c r="B6" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A4), "", '📦 商品出厂底价库 (Products)'!A4)</f>
+      </c>
+      <c r="C6" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A4), "", '📦 商品出厂底价库 (Products)'!C4)</f>
+      </c>
+      <c r="D6" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A4), "", '📦 商品出厂底价库 (Products)'!E4)</f>
+      </c>
+      <c r="E6" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A4), "", '📦 商品出厂底价库 (Products)'!N4)</f>
+      </c>
+      <c r="F6" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A4), "", '📦 商品出厂底价库 (Products)'!F4)</f>
+      </c>
+      <c r="G6" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A4), "", '📦 商品出厂底价库 (Products)'!O4)</f>
+      </c>
+      <c r="H6" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A4), "", '📦 商品出厂底价库 (Products)'!P4)</f>
+      </c>
+      <c r="I6" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A4), "", '📦 商品出厂底价库 (Products)'!J4)</f>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A5), "", 4)</f>
+      </c>
+      <c r="B7" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A5), "", '📦 商品出厂底价库 (Products)'!A5)</f>
+      </c>
+      <c r="C7" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A5), "", '📦 商品出厂底价库 (Products)'!C5)</f>
+      </c>
+      <c r="D7" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A5), "", '📦 商品出厂底价库 (Products)'!E5)</f>
+      </c>
+      <c r="E7" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A5), "", '📦 商品出厂底价库 (Products)'!N5)</f>
+      </c>
+      <c r="F7" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A5), "", '📦 商品出厂底价库 (Products)'!F5)</f>
+      </c>
+      <c r="G7" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A5), "", '📦 商品出厂底价库 (Products)'!O5)</f>
+      </c>
+      <c r="H7" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A5), "", '📦 商品出厂底价库 (Products)'!P5)</f>
+      </c>
+      <c r="I7" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A5), "", '📦 商品出厂底价库 (Products)'!J5)</f>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A6), "", 5)</f>
+      </c>
+      <c r="B8" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A6), "", '📦 商品出厂底价库 (Products)'!A6)</f>
+      </c>
+      <c r="C8" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A6), "", '📦 商品出厂底价库 (Products)'!C6)</f>
+      </c>
+      <c r="D8" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A6), "", '📦 商品出厂底价库 (Products)'!E6)</f>
+      </c>
+      <c r="E8" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A6), "", '📦 商品出厂底价库 (Products)'!N6)</f>
+      </c>
+      <c r="F8" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A6), "", '📦 商品出厂底价库 (Products)'!F6)</f>
+      </c>
+      <c r="G8" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A6), "", '📦 商品出厂底价库 (Products)'!O6)</f>
+      </c>
+      <c r="H8" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A6), "", '📦 商品出厂底价库 (Products)'!P6)</f>
+      </c>
+      <c r="I8" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A6), "", '📦 商品出厂底价库 (Products)'!J6)</f>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A7), "", 6)</f>
+      </c>
+      <c r="B9" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A7), "", '📦 商品出厂底价库 (Products)'!A7)</f>
+      </c>
+      <c r="C9" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A7), "", '📦 商品出厂底价库 (Products)'!C7)</f>
+      </c>
+      <c r="D9" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A7), "", '📦 商品出厂底价库 (Products)'!E7)</f>
+      </c>
+      <c r="E9" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A7), "", '📦 商品出厂底价库 (Products)'!N7)</f>
+      </c>
+      <c r="F9" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A7), "", '📦 商品出厂底价库 (Products)'!F7)</f>
+      </c>
+      <c r="G9" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A7), "", '📦 商品出厂底价库 (Products)'!O7)</f>
+      </c>
+      <c r="H9" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A7), "", '📦 商品出厂底价库 (Products)'!P7)</f>
+      </c>
+      <c r="I9" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A7), "", '📦 商品出厂底价库 (Products)'!J7)</f>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A8), "", 7)</f>
+      </c>
+      <c r="B10" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A8), "", '📦 商品出厂底价库 (Products)'!A8)</f>
+      </c>
+      <c r="C10" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A8), "", '📦 商品出厂底价库 (Products)'!C8)</f>
+      </c>
+      <c r="D10" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A8), "", '📦 商品出厂底价库 (Products)'!E8)</f>
+      </c>
+      <c r="E10" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A8), "", '📦 商品出厂底价库 (Products)'!N8)</f>
+      </c>
+      <c r="F10" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A8), "", '📦 商品出厂底价库 (Products)'!F8)</f>
+      </c>
+      <c r="G10" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A8), "", '📦 商品出厂底价库 (Products)'!O8)</f>
+      </c>
+      <c r="H10" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A8), "", '📦 商品出厂底价库 (Products)'!P8)</f>
+      </c>
+      <c r="I10" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A8), "", '📦 商品出厂底价库 (Products)'!J8)</f>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A9), "", 8)</f>
+      </c>
+      <c r="B11" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A9), "", '📦 商品出厂底价库 (Products)'!A9)</f>
+      </c>
+      <c r="C11" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A9), "", '📦 商品出厂底价库 (Products)'!C9)</f>
+      </c>
+      <c r="D11" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A9), "", '📦 商品出厂底价库 (Products)'!E9)</f>
+      </c>
+      <c r="E11" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A9), "", '📦 商品出厂底价库 (Products)'!N9)</f>
+      </c>
+      <c r="F11" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A9), "", '📦 商品出厂底价库 (Products)'!F9)</f>
+      </c>
+      <c r="G11" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A9), "", '📦 商品出厂底价库 (Products)'!O9)</f>
+      </c>
+      <c r="H11" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A9), "", '📦 商品出厂底价库 (Products)'!P9)</f>
+      </c>
+      <c r="I11" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A9), "", '📦 商品出厂底价库 (Products)'!J9)</f>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A10), "", 9)</f>
+      </c>
+      <c r="B12" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A10), "", '📦 商品出厂底价库 (Products)'!A10)</f>
+      </c>
+      <c r="C12" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A10), "", '📦 商品出厂底价库 (Products)'!C10)</f>
+      </c>
+      <c r="D12" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A10), "", '📦 商品出厂底价库 (Products)'!E10)</f>
+      </c>
+      <c r="E12" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A10), "", '📦 商品出厂底价库 (Products)'!N10)</f>
+      </c>
+      <c r="F12" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A10), "", '📦 商品出厂底价库 (Products)'!F10)</f>
+      </c>
+      <c r="G12" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A10), "", '📦 商品出厂底价库 (Products)'!O10)</f>
+      </c>
+      <c r="H12" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A10), "", '📦 商品出厂底价库 (Products)'!P10)</f>
+      </c>
+      <c r="I12" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A10), "", '📦 商品出厂底价库 (Products)'!J10)</f>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A11), "", 10)</f>
+      </c>
+      <c r="B13" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A11), "", '📦 商品出厂底价库 (Products)'!A11)</f>
+      </c>
+      <c r="C13" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A11), "", '📦 商品出厂底价库 (Products)'!C11)</f>
+      </c>
+      <c r="D13" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A11), "", '📦 商品出厂底价库 (Products)'!E11)</f>
+      </c>
+      <c r="E13" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A11), "", '📦 商品出厂底价库 (Products)'!N11)</f>
+      </c>
+      <c r="F13" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A11), "", '📦 商品出厂底价库 (Products)'!F11)</f>
+      </c>
+      <c r="G13" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A11), "", '📦 商品出厂底价库 (Products)'!O11)</f>
+      </c>
+      <c r="H13" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A11), "", '📦 商品出厂底价库 (Products)'!P11)</f>
+      </c>
+      <c r="I13" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A11), "", '📦 商品出厂底价库 (Products)'!J11)</f>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A12), "", 11)</f>
+      </c>
+      <c r="B14" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A12), "", '📦 商品出厂底价库 (Products)'!A12)</f>
+      </c>
+      <c r="C14" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A12), "", '📦 商品出厂底价库 (Products)'!C12)</f>
+      </c>
+      <c r="D14" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A12), "", '📦 商品出厂底价库 (Products)'!E12)</f>
+      </c>
+      <c r="E14" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A12), "", '📦 商品出厂底价库 (Products)'!N12)</f>
+      </c>
+      <c r="F14" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A12), "", '📦 商品出厂底价库 (Products)'!F12)</f>
+      </c>
+      <c r="G14" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A12), "", '📦 商品出厂底价库 (Products)'!O12)</f>
+      </c>
+      <c r="H14" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A12), "", '📦 商品出厂底价库 (Products)'!P12)</f>
+      </c>
+      <c r="I14" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A12), "", '📦 商品出厂底价库 (Products)'!J12)</f>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A13), "", 12)</f>
+      </c>
+      <c r="B15" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A13), "", '📦 商品出厂底价库 (Products)'!A13)</f>
+      </c>
+      <c r="C15" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A13), "", '📦 商品出厂底价库 (Products)'!C13)</f>
+      </c>
+      <c r="D15" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A13), "", '📦 商品出厂底价库 (Products)'!E13)</f>
+      </c>
+      <c r="E15" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A13), "", '📦 商品出厂底价库 (Products)'!N13)</f>
+      </c>
+      <c r="F15" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A13), "", '📦 商品出厂底价库 (Products)'!F13)</f>
+      </c>
+      <c r="G15" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A13), "", '📦 商品出厂底价库 (Products)'!O13)</f>
+      </c>
+      <c r="H15" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A13), "", '📦 商品出厂底价库 (Products)'!P13)</f>
+      </c>
+      <c r="I15" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A13), "", '📦 商品出厂底价库 (Products)'!J13)</f>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A14), "", 13)</f>
+      </c>
+      <c r="B16" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A14), "", '📦 商品出厂底价库 (Products)'!A14)</f>
+      </c>
+      <c r="C16" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A14), "", '📦 商品出厂底价库 (Products)'!C14)</f>
+      </c>
+      <c r="D16" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A14), "", '📦 商品出厂底价库 (Products)'!E14)</f>
+      </c>
+      <c r="E16" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A14), "", '📦 商品出厂底价库 (Products)'!N14)</f>
+      </c>
+      <c r="F16" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A14), "", '📦 商品出厂底价库 (Products)'!F14)</f>
+      </c>
+      <c r="G16" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A14), "", '📦 商品出厂底价库 (Products)'!O14)</f>
+      </c>
+      <c r="H16" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A14), "", '📦 商品出厂底价库 (Products)'!P14)</f>
+      </c>
+      <c r="I16" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A14), "", '📦 商品出厂底价库 (Products)'!J14)</f>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A15), "", 14)</f>
+      </c>
+      <c r="B17" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A15), "", '📦 商品出厂底价库 (Products)'!A15)</f>
+      </c>
+      <c r="C17" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A15), "", '📦 商品出厂底价库 (Products)'!C15)</f>
+      </c>
+      <c r="D17" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A15), "", '📦 商品出厂底价库 (Products)'!E15)</f>
+      </c>
+      <c r="E17" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A15), "", '📦 商品出厂底价库 (Products)'!N15)</f>
+      </c>
+      <c r="F17" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A15), "", '📦 商品出厂底价库 (Products)'!F15)</f>
+      </c>
+      <c r="G17" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A15), "", '📦 商品出厂底价库 (Products)'!O15)</f>
+      </c>
+      <c r="H17" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A15), "", '📦 商品出厂底价库 (Products)'!P15)</f>
+      </c>
+      <c r="I17" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A15), "", '📦 商品出厂底价库 (Products)'!J15)</f>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A16), "", 15)</f>
+      </c>
+      <c r="B18" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A16), "", '📦 商品出厂底价库 (Products)'!A16)</f>
+      </c>
+      <c r="C18" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A16), "", '📦 商品出厂底价库 (Products)'!C16)</f>
+      </c>
+      <c r="D18" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A16), "", '📦 商品出厂底价库 (Products)'!E16)</f>
+      </c>
+      <c r="E18" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A16), "", '📦 商品出厂底价库 (Products)'!N16)</f>
+      </c>
+      <c r="F18" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A16), "", '📦 商品出厂底价库 (Products)'!F16)</f>
+      </c>
+      <c r="G18" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A16), "", '📦 商品出厂底价库 (Products)'!O16)</f>
+      </c>
+      <c r="H18" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A16), "", '📦 商品出厂底价库 (Products)'!P16)</f>
+      </c>
+      <c r="I18" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A16), "", '📦 商品出厂底价库 (Products)'!J16)</f>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A17), "", 16)</f>
+      </c>
+      <c r="B19" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A17), "", '📦 商品出厂底价库 (Products)'!A17)</f>
+      </c>
+      <c r="C19" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A17), "", '📦 商品出厂底价库 (Products)'!C17)</f>
+      </c>
+      <c r="D19" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A17), "", '📦 商品出厂底价库 (Products)'!E17)</f>
+      </c>
+      <c r="E19" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A17), "", '📦 商品出厂底价库 (Products)'!N17)</f>
+      </c>
+      <c r="F19" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A17), "", '📦 商品出厂底价库 (Products)'!F17)</f>
+      </c>
+      <c r="G19" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A17), "", '📦 商品出厂底价库 (Products)'!O17)</f>
+      </c>
+      <c r="H19" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A17), "", '📦 商品出厂底价库 (Products)'!P17)</f>
+      </c>
+      <c r="I19" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A17), "", '📦 商品出厂底价库 (Products)'!J17)</f>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A18), "", 17)</f>
+      </c>
+      <c r="B20" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A18), "", '📦 商品出厂底价库 (Products)'!A18)</f>
+      </c>
+      <c r="C20" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A18), "", '📦 商品出厂底价库 (Products)'!C18)</f>
+      </c>
+      <c r="D20" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A18), "", '📦 商品出厂底价库 (Products)'!E18)</f>
+      </c>
+      <c r="E20" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A18), "", '📦 商品出厂底价库 (Products)'!N18)</f>
+      </c>
+      <c r="F20" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A18), "", '📦 商品出厂底价库 (Products)'!F18)</f>
+      </c>
+      <c r="G20" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A18), "", '📦 商品出厂底价库 (Products)'!O18)</f>
+      </c>
+      <c r="H20" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A18), "", '📦 商品出厂底价库 (Products)'!P18)</f>
+      </c>
+      <c r="I20" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A18), "", '📦 商品出厂底价库 (Products)'!J18)</f>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A19), "", 18)</f>
+      </c>
+      <c r="B21" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A19), "", '📦 商品出厂底价库 (Products)'!A19)</f>
+      </c>
+      <c r="C21" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A19), "", '📦 商品出厂底价库 (Products)'!C19)</f>
+      </c>
+      <c r="D21" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A19), "", '📦 商品出厂底价库 (Products)'!E19)</f>
+      </c>
+      <c r="E21" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A19), "", '📦 商品出厂底价库 (Products)'!N19)</f>
+      </c>
+      <c r="F21" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A19), "", '📦 商品出厂底价库 (Products)'!F19)</f>
+      </c>
+      <c r="G21" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A19), "", '📦 商品出厂底价库 (Products)'!O19)</f>
+      </c>
+      <c r="H21" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A19), "", '📦 商品出厂底价库 (Products)'!P19)</f>
+      </c>
+      <c r="I21" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A19), "", '📦 商品出厂底价库 (Products)'!J19)</f>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A20), "", 19)</f>
+      </c>
+      <c r="B22" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A20), "", '📦 商品出厂底价库 (Products)'!A20)</f>
+      </c>
+      <c r="C22" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A20), "", '📦 商品出厂底价库 (Products)'!C20)</f>
+      </c>
+      <c r="D22" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A20), "", '📦 商品出厂底价库 (Products)'!E20)</f>
+      </c>
+      <c r="E22" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A20), "", '📦 商品出厂底价库 (Products)'!N20)</f>
+      </c>
+      <c r="F22" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A20), "", '📦 商品出厂底价库 (Products)'!F20)</f>
+      </c>
+      <c r="G22" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A20), "", '📦 商品出厂底价库 (Products)'!O20)</f>
+      </c>
+      <c r="H22" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A20), "", '📦 商品出厂底价库 (Products)'!P20)</f>
+      </c>
+      <c r="I22" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A20), "", '📦 商品出厂底价库 (Products)'!J20)</f>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A21), "", 20)</f>
+      </c>
+      <c r="B23" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A21), "", '📦 商品出厂底价库 (Products)'!A21)</f>
+      </c>
+      <c r="C23" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A21), "", '📦 商品出厂底价库 (Products)'!C21)</f>
+      </c>
+      <c r="D23" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A21), "", '📦 商品出厂底价库 (Products)'!E21)</f>
+      </c>
+      <c r="E23" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A21), "", '📦 商品出厂底价库 (Products)'!N21)</f>
+      </c>
+      <c r="F23" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A21), "", '📦 商品出厂底价库 (Products)'!F21)</f>
+      </c>
+      <c r="G23" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A21), "", '📦 商品出厂底价库 (Products)'!O21)</f>
+      </c>
+      <c r="H23" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A21), "", '📦 商品出厂底价库 (Products)'!P21)</f>
+      </c>
+      <c r="I23" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A21), "", '📦 商品出厂底价库 (Products)'!J21)</f>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A22), "", 21)</f>
+      </c>
+      <c r="B24" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A22), "", '📦 商品出厂底价库 (Products)'!A22)</f>
+      </c>
+      <c r="C24" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A22), "", '📦 商品出厂底价库 (Products)'!C22)</f>
+      </c>
+      <c r="D24" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A22), "", '📦 商品出厂底价库 (Products)'!E22)</f>
+      </c>
+      <c r="E24" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A22), "", '📦 商品出厂底价库 (Products)'!N22)</f>
+      </c>
+      <c r="F24" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A22), "", '📦 商品出厂底价库 (Products)'!F22)</f>
+      </c>
+      <c r="G24" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A22), "", '📦 商品出厂底价库 (Products)'!O22)</f>
+      </c>
+      <c r="H24" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A22), "", '📦 商品出厂底价库 (Products)'!P22)</f>
+      </c>
+      <c r="I24" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A22), "", '📦 商品出厂底价库 (Products)'!J22)</f>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A23), "", 22)</f>
+      </c>
+      <c r="B25" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A23), "", '📦 商品出厂底价库 (Products)'!A23)</f>
+      </c>
+      <c r="C25" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A23), "", '📦 商品出厂底价库 (Products)'!C23)</f>
+      </c>
+      <c r="D25" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A23), "", '📦 商品出厂底价库 (Products)'!E23)</f>
+      </c>
+      <c r="E25" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A23), "", '📦 商品出厂底价库 (Products)'!N23)</f>
+      </c>
+      <c r="F25" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A23), "", '📦 商品出厂底价库 (Products)'!F23)</f>
+      </c>
+      <c r="G25" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A23), "", '📦 商品出厂底价库 (Products)'!O23)</f>
+      </c>
+      <c r="H25" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A23), "", '📦 商品出厂底价库 (Products)'!P23)</f>
+      </c>
+      <c r="I25" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A23), "", '📦 商品出厂底价库 (Products)'!J23)</f>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A24), "", 23)</f>
+      </c>
+      <c r="B26" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A24), "", '📦 商品出厂底价库 (Products)'!A24)</f>
+      </c>
+      <c r="C26" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A24), "", '📦 商品出厂底价库 (Products)'!C24)</f>
+      </c>
+      <c r="D26" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A24), "", '📦 商品出厂底价库 (Products)'!E24)</f>
+      </c>
+      <c r="E26" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A24), "", '📦 商品出厂底价库 (Products)'!N24)</f>
+      </c>
+      <c r="F26" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A24), "", '📦 商品出厂底价库 (Products)'!F24)</f>
+      </c>
+      <c r="G26" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A24), "", '📦 商品出厂底价库 (Products)'!O24)</f>
+      </c>
+      <c r="H26" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A24), "", '📦 商品出厂底价库 (Products)'!P24)</f>
+      </c>
+      <c r="I26" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A24), "", '📦 商品出厂底价库 (Products)'!J24)</f>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A25), "", 24)</f>
+      </c>
+      <c r="B27" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A25), "", '📦 商品出厂底价库 (Products)'!A25)</f>
+      </c>
+      <c r="C27" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A25), "", '📦 商品出厂底价库 (Products)'!C25)</f>
+      </c>
+      <c r="D27" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A25), "", '📦 商品出厂底价库 (Products)'!E25)</f>
+      </c>
+      <c r="E27" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A25), "", '📦 商品出厂底价库 (Products)'!N25)</f>
+      </c>
+      <c r="F27" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A25), "", '📦 商品出厂底价库 (Products)'!F25)</f>
+      </c>
+      <c r="G27" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A25), "", '📦 商品出厂底价库 (Products)'!O25)</f>
+      </c>
+      <c r="H27" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A25), "", '📦 商品出厂底价库 (Products)'!P25)</f>
+      </c>
+      <c r="I27" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A25), "", '📦 商品出厂底价库 (Products)'!J25)</f>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A26), "", 25)</f>
+      </c>
+      <c r="B28" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A26), "", '📦 商品出厂底价库 (Products)'!A26)</f>
+      </c>
+      <c r="C28" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A26), "", '📦 商品出厂底价库 (Products)'!C26)</f>
+      </c>
+      <c r="D28" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A26), "", '📦 商品出厂底价库 (Products)'!E26)</f>
+      </c>
+      <c r="E28" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A26), "", '📦 商品出厂底价库 (Products)'!N26)</f>
+      </c>
+      <c r="F28" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A26), "", '📦 商品出厂底价库 (Products)'!F26)</f>
+      </c>
+      <c r="G28" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A26), "", '📦 商品出厂底价库 (Products)'!O26)</f>
+      </c>
+      <c r="H28" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A26), "", '📦 商品出厂底价库 (Products)'!P26)</f>
+      </c>
+      <c r="I28" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A26), "", '📦 商品出厂底价库 (Products)'!J26)</f>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A27), "", 26)</f>
+      </c>
+      <c r="B29" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A27), "", '📦 商品出厂底价库 (Products)'!A27)</f>
+      </c>
+      <c r="C29" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A27), "", '📦 商品出厂底价库 (Products)'!C27)</f>
+      </c>
+      <c r="D29" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A27), "", '📦 商品出厂底价库 (Products)'!E27)</f>
+      </c>
+      <c r="E29" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A27), "", '📦 商品出厂底价库 (Products)'!N27)</f>
+      </c>
+      <c r="F29" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A27), "", '📦 商品出厂底价库 (Products)'!F27)</f>
+      </c>
+      <c r="G29" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A27), "", '📦 商品出厂底价库 (Products)'!O27)</f>
+      </c>
+      <c r="H29" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A27), "", '📦 商品出厂底价库 (Products)'!P27)</f>
+      </c>
+      <c r="I29" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A27), "", '📦 商品出厂底价库 (Products)'!J27)</f>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A28), "", 27)</f>
+      </c>
+      <c r="B30" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A28), "", '📦 商品出厂底价库 (Products)'!A28)</f>
+      </c>
+      <c r="C30" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A28), "", '📦 商品出厂底价库 (Products)'!C28)</f>
+      </c>
+      <c r="D30" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A28), "", '📦 商品出厂底价库 (Products)'!E28)</f>
+      </c>
+      <c r="E30" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A28), "", '📦 商品出厂底价库 (Products)'!N28)</f>
+      </c>
+      <c r="F30" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A28), "", '📦 商品出厂底价库 (Products)'!F28)</f>
+      </c>
+      <c r="G30" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A28), "", '📦 商品出厂底价库 (Products)'!O28)</f>
+      </c>
+      <c r="H30" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A28), "", '📦 商品出厂底价库 (Products)'!P28)</f>
+      </c>
+      <c r="I30" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A28), "", '📦 商品出厂底价库 (Products)'!J28)</f>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A29), "", 28)</f>
+      </c>
+      <c r="B31" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A29), "", '📦 商品出厂底价库 (Products)'!A29)</f>
+      </c>
+      <c r="C31" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A29), "", '📦 商品出厂底价库 (Products)'!C29)</f>
+      </c>
+      <c r="D31" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A29), "", '📦 商品出厂底价库 (Products)'!E29)</f>
+      </c>
+      <c r="E31" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A29), "", '📦 商品出厂底价库 (Products)'!N29)</f>
+      </c>
+      <c r="F31" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A29), "", '📦 商品出厂底价库 (Products)'!F29)</f>
+      </c>
+      <c r="G31" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A29), "", '📦 商品出厂底价库 (Products)'!O29)</f>
+      </c>
+      <c r="H31" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A29), "", '📦 商品出厂底价库 (Products)'!P29)</f>
+      </c>
+      <c r="I31" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A29), "", '📦 商品出厂底价库 (Products)'!J29)</f>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A30), "", 29)</f>
+      </c>
+      <c r="B32" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A30), "", '📦 商品出厂底价库 (Products)'!A30)</f>
+      </c>
+      <c r="C32" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A30), "", '📦 商品出厂底价库 (Products)'!C30)</f>
+      </c>
+      <c r="D32" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A30), "", '📦 商品出厂底价库 (Products)'!E30)</f>
+      </c>
+      <c r="E32" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A30), "", '📦 商品出厂底价库 (Products)'!N30)</f>
+      </c>
+      <c r="F32" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A30), "", '📦 商品出厂底价库 (Products)'!F30)</f>
+      </c>
+      <c r="G32" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A30), "", '📦 商品出厂底价库 (Products)'!O30)</f>
+      </c>
+      <c r="H32" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A30), "", '📦 商品出厂底价库 (Products)'!P30)</f>
+      </c>
+      <c r="I32" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A30), "", '📦 商品出厂底价库 (Products)'!J30)</f>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", 30)</f>
+      </c>
+      <c r="B33" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", '📦 商品出厂底价库 (Products)'!A31)</f>
+      </c>
+      <c r="C33" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", '📦 商品出厂底价库 (Products)'!C31)</f>
+      </c>
+      <c r="D33" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", '📦 商品出厂底价库 (Products)'!E31)</f>
+      </c>
+      <c r="E33" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", '📦 商品出厂底价库 (Products)'!N31)</f>
+      </c>
+      <c r="F33" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", '📦 商品出厂底价库 (Products)'!F31)</f>
+      </c>
+      <c r="G33" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", '📦 商品出厂底价库 (Products)'!O31)</f>
+      </c>
+      <c r="H33" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", '📦 商品出厂底价库 (Products)'!P31)</f>
+      </c>
+      <c r="I33" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", '📦 商品出厂底价库 (Products)'!J31)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(lead_magnets): expand smart formula capacity to 100 pre-populated rows
</commit_message>
<xml_diff>
--- a/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
+++ b/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
@@ -1863,7 +1863,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q31"/>
+  <dimension ref="A1:Q101"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2990,6 +2990,2176 @@
         <f>IF(ISBLANK(D31), "", IF(M31&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M31&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
       </c>
     </row>
+    <row r="32" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A32" s="39"/>
+      <c r="B32" s="40"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="42"/>
+      <c r="E32" s="43"/>
+      <c r="F32" s="43"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="45"/>
+      <c r="I32" s="46"/>
+      <c r="J32" s="39"/>
+      <c r="K32" s="39"/>
+      <c r="L32" s="47">
+        <f>IF(ISBLANK(D32), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M32" s="48">
+        <f>IF(ISBLANK(D32), "", IF(ISBLANK(I32), '⚙️ 全局核算参数 (Config)'!$B$13, I32))</f>
+      </c>
+      <c r="N32" s="49">
+        <f>IF(ISBLANK(D32), "", ROUND(((D32 * (1 + M32) + L32) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O32" s="50">
+        <f>IF(OR(ISBLANK(D32), NOT(AND(G32&gt;0, F32&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G32)) * F32)</f>
+      </c>
+      <c r="P32" s="50">
+        <f>IF(OR(ISBLANK(D32), NOT(AND(G32&gt;0, F32&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G32)) * F32)</f>
+      </c>
+      <c r="Q32" s="51">
+        <f>IF(ISBLANK(D32), "", IF(M32&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M32&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A33" s="52"/>
+      <c r="B33" s="53"/>
+      <c r="C33" s="54"/>
+      <c r="D33" s="55"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="56"/>
+      <c r="G33" s="57"/>
+      <c r="H33" s="58"/>
+      <c r="I33" s="59"/>
+      <c r="J33" s="52"/>
+      <c r="K33" s="52"/>
+      <c r="L33" s="47">
+        <f>IF(ISBLANK(D33), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M33" s="48">
+        <f>IF(ISBLANK(D33), "", IF(ISBLANK(I33), '⚙️ 全局核算参数 (Config)'!$B$13, I33))</f>
+      </c>
+      <c r="N33" s="49">
+        <f>IF(ISBLANK(D33), "", ROUND(((D33 * (1 + M33) + L33) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O33" s="50">
+        <f>IF(OR(ISBLANK(D33), NOT(AND(G33&gt;0, F33&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G33)) * F33)</f>
+      </c>
+      <c r="P33" s="50">
+        <f>IF(OR(ISBLANK(D33), NOT(AND(G33&gt;0, F33&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G33)) * F33)</f>
+      </c>
+      <c r="Q33" s="51">
+        <f>IF(ISBLANK(D33), "", IF(M33&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M33&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A34" s="39"/>
+      <c r="B34" s="40"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="42"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="44"/>
+      <c r="H34" s="45"/>
+      <c r="I34" s="46"/>
+      <c r="J34" s="39"/>
+      <c r="K34" s="39"/>
+      <c r="L34" s="47">
+        <f>IF(ISBLANK(D34), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M34" s="48">
+        <f>IF(ISBLANK(D34), "", IF(ISBLANK(I34), '⚙️ 全局核算参数 (Config)'!$B$13, I34))</f>
+      </c>
+      <c r="N34" s="49">
+        <f>IF(ISBLANK(D34), "", ROUND(((D34 * (1 + M34) + L34) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O34" s="50">
+        <f>IF(OR(ISBLANK(D34), NOT(AND(G34&gt;0, F34&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G34)) * F34)</f>
+      </c>
+      <c r="P34" s="50">
+        <f>IF(OR(ISBLANK(D34), NOT(AND(G34&gt;0, F34&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G34)) * F34)</f>
+      </c>
+      <c r="Q34" s="51">
+        <f>IF(ISBLANK(D34), "", IF(M34&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M34&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A35" s="52"/>
+      <c r="B35" s="53"/>
+      <c r="C35" s="54"/>
+      <c r="D35" s="55"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="56"/>
+      <c r="G35" s="57"/>
+      <c r="H35" s="58"/>
+      <c r="I35" s="59"/>
+      <c r="J35" s="52"/>
+      <c r="K35" s="52"/>
+      <c r="L35" s="47">
+        <f>IF(ISBLANK(D35), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M35" s="48">
+        <f>IF(ISBLANK(D35), "", IF(ISBLANK(I35), '⚙️ 全局核算参数 (Config)'!$B$13, I35))</f>
+      </c>
+      <c r="N35" s="49">
+        <f>IF(ISBLANK(D35), "", ROUND(((D35 * (1 + M35) + L35) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O35" s="50">
+        <f>IF(OR(ISBLANK(D35), NOT(AND(G35&gt;0, F35&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G35)) * F35)</f>
+      </c>
+      <c r="P35" s="50">
+        <f>IF(OR(ISBLANK(D35), NOT(AND(G35&gt;0, F35&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G35)) * F35)</f>
+      </c>
+      <c r="Q35" s="51">
+        <f>IF(ISBLANK(D35), "", IF(M35&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M35&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A36" s="39"/>
+      <c r="B36" s="40"/>
+      <c r="C36" s="41"/>
+      <c r="D36" s="42"/>
+      <c r="E36" s="43"/>
+      <c r="F36" s="43"/>
+      <c r="G36" s="44"/>
+      <c r="H36" s="45"/>
+      <c r="I36" s="46"/>
+      <c r="J36" s="39"/>
+      <c r="K36" s="39"/>
+      <c r="L36" s="47">
+        <f>IF(ISBLANK(D36), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M36" s="48">
+        <f>IF(ISBLANK(D36), "", IF(ISBLANK(I36), '⚙️ 全局核算参数 (Config)'!$B$13, I36))</f>
+      </c>
+      <c r="N36" s="49">
+        <f>IF(ISBLANK(D36), "", ROUND(((D36 * (1 + M36) + L36) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O36" s="50">
+        <f>IF(OR(ISBLANK(D36), NOT(AND(G36&gt;0, F36&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G36)) * F36)</f>
+      </c>
+      <c r="P36" s="50">
+        <f>IF(OR(ISBLANK(D36), NOT(AND(G36&gt;0, F36&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G36)) * F36)</f>
+      </c>
+      <c r="Q36" s="51">
+        <f>IF(ISBLANK(D36), "", IF(M36&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M36&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A37" s="52"/>
+      <c r="B37" s="53"/>
+      <c r="C37" s="54"/>
+      <c r="D37" s="55"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
+      <c r="G37" s="57"/>
+      <c r="H37" s="58"/>
+      <c r="I37" s="59"/>
+      <c r="J37" s="52"/>
+      <c r="K37" s="52"/>
+      <c r="L37" s="47">
+        <f>IF(ISBLANK(D37), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M37" s="48">
+        <f>IF(ISBLANK(D37), "", IF(ISBLANK(I37), '⚙️ 全局核算参数 (Config)'!$B$13, I37))</f>
+      </c>
+      <c r="N37" s="49">
+        <f>IF(ISBLANK(D37), "", ROUND(((D37 * (1 + M37) + L37) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O37" s="50">
+        <f>IF(OR(ISBLANK(D37), NOT(AND(G37&gt;0, F37&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G37)) * F37)</f>
+      </c>
+      <c r="P37" s="50">
+        <f>IF(OR(ISBLANK(D37), NOT(AND(G37&gt;0, F37&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G37)) * F37)</f>
+      </c>
+      <c r="Q37" s="51">
+        <f>IF(ISBLANK(D37), "", IF(M37&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M37&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A38" s="39"/>
+      <c r="B38" s="40"/>
+      <c r="C38" s="41"/>
+      <c r="D38" s="42"/>
+      <c r="E38" s="43"/>
+      <c r="F38" s="43"/>
+      <c r="G38" s="44"/>
+      <c r="H38" s="45"/>
+      <c r="I38" s="46"/>
+      <c r="J38" s="39"/>
+      <c r="K38" s="39"/>
+      <c r="L38" s="47">
+        <f>IF(ISBLANK(D38), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M38" s="48">
+        <f>IF(ISBLANK(D38), "", IF(ISBLANK(I38), '⚙️ 全局核算参数 (Config)'!$B$13, I38))</f>
+      </c>
+      <c r="N38" s="49">
+        <f>IF(ISBLANK(D38), "", ROUND(((D38 * (1 + M38) + L38) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O38" s="50">
+        <f>IF(OR(ISBLANK(D38), NOT(AND(G38&gt;0, F38&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G38)) * F38)</f>
+      </c>
+      <c r="P38" s="50">
+        <f>IF(OR(ISBLANK(D38), NOT(AND(G38&gt;0, F38&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G38)) * F38)</f>
+      </c>
+      <c r="Q38" s="51">
+        <f>IF(ISBLANK(D38), "", IF(M38&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M38&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A39" s="52"/>
+      <c r="B39" s="53"/>
+      <c r="C39" s="54"/>
+      <c r="D39" s="55"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="56"/>
+      <c r="G39" s="57"/>
+      <c r="H39" s="58"/>
+      <c r="I39" s="59"/>
+      <c r="J39" s="52"/>
+      <c r="K39" s="52"/>
+      <c r="L39" s="47">
+        <f>IF(ISBLANK(D39), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M39" s="48">
+        <f>IF(ISBLANK(D39), "", IF(ISBLANK(I39), '⚙️ 全局核算参数 (Config)'!$B$13, I39))</f>
+      </c>
+      <c r="N39" s="49">
+        <f>IF(ISBLANK(D39), "", ROUND(((D39 * (1 + M39) + L39) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O39" s="50">
+        <f>IF(OR(ISBLANK(D39), NOT(AND(G39&gt;0, F39&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G39)) * F39)</f>
+      </c>
+      <c r="P39" s="50">
+        <f>IF(OR(ISBLANK(D39), NOT(AND(G39&gt;0, F39&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G39)) * F39)</f>
+      </c>
+      <c r="Q39" s="51">
+        <f>IF(ISBLANK(D39), "", IF(M39&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M39&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A40" s="39"/>
+      <c r="B40" s="40"/>
+      <c r="C40" s="41"/>
+      <c r="D40" s="42"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="44"/>
+      <c r="H40" s="45"/>
+      <c r="I40" s="46"/>
+      <c r="J40" s="39"/>
+      <c r="K40" s="39"/>
+      <c r="L40" s="47">
+        <f>IF(ISBLANK(D40), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M40" s="48">
+        <f>IF(ISBLANK(D40), "", IF(ISBLANK(I40), '⚙️ 全局核算参数 (Config)'!$B$13, I40))</f>
+      </c>
+      <c r="N40" s="49">
+        <f>IF(ISBLANK(D40), "", ROUND(((D40 * (1 + M40) + L40) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O40" s="50">
+        <f>IF(OR(ISBLANK(D40), NOT(AND(G40&gt;0, F40&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G40)) * F40)</f>
+      </c>
+      <c r="P40" s="50">
+        <f>IF(OR(ISBLANK(D40), NOT(AND(G40&gt;0, F40&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G40)) * F40)</f>
+      </c>
+      <c r="Q40" s="51">
+        <f>IF(ISBLANK(D40), "", IF(M40&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M40&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A41" s="52"/>
+      <c r="B41" s="53"/>
+      <c r="C41" s="54"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="56"/>
+      <c r="F41" s="56"/>
+      <c r="G41" s="57"/>
+      <c r="H41" s="58"/>
+      <c r="I41" s="59"/>
+      <c r="J41" s="52"/>
+      <c r="K41" s="52"/>
+      <c r="L41" s="47">
+        <f>IF(ISBLANK(D41), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M41" s="48">
+        <f>IF(ISBLANK(D41), "", IF(ISBLANK(I41), '⚙️ 全局核算参数 (Config)'!$B$13, I41))</f>
+      </c>
+      <c r="N41" s="49">
+        <f>IF(ISBLANK(D41), "", ROUND(((D41 * (1 + M41) + L41) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O41" s="50">
+        <f>IF(OR(ISBLANK(D41), NOT(AND(G41&gt;0, F41&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G41)) * F41)</f>
+      </c>
+      <c r="P41" s="50">
+        <f>IF(OR(ISBLANK(D41), NOT(AND(G41&gt;0, F41&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G41)) * F41)</f>
+      </c>
+      <c r="Q41" s="51">
+        <f>IF(ISBLANK(D41), "", IF(M41&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M41&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="42" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A42" s="39"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="43"/>
+      <c r="G42" s="44"/>
+      <c r="H42" s="45"/>
+      <c r="I42" s="46"/>
+      <c r="J42" s="39"/>
+      <c r="K42" s="39"/>
+      <c r="L42" s="47">
+        <f>IF(ISBLANK(D42), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M42" s="48">
+        <f>IF(ISBLANK(D42), "", IF(ISBLANK(I42), '⚙️ 全局核算参数 (Config)'!$B$13, I42))</f>
+      </c>
+      <c r="N42" s="49">
+        <f>IF(ISBLANK(D42), "", ROUND(((D42 * (1 + M42) + L42) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O42" s="50">
+        <f>IF(OR(ISBLANK(D42), NOT(AND(G42&gt;0, F42&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G42)) * F42)</f>
+      </c>
+      <c r="P42" s="50">
+        <f>IF(OR(ISBLANK(D42), NOT(AND(G42&gt;0, F42&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G42)) * F42)</f>
+      </c>
+      <c r="Q42" s="51">
+        <f>IF(ISBLANK(D42), "", IF(M42&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M42&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="43" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A43" s="52"/>
+      <c r="B43" s="53"/>
+      <c r="C43" s="54"/>
+      <c r="D43" s="55"/>
+      <c r="E43" s="56"/>
+      <c r="F43" s="56"/>
+      <c r="G43" s="57"/>
+      <c r="H43" s="58"/>
+      <c r="I43" s="59"/>
+      <c r="J43" s="52"/>
+      <c r="K43" s="52"/>
+      <c r="L43" s="47">
+        <f>IF(ISBLANK(D43), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M43" s="48">
+        <f>IF(ISBLANK(D43), "", IF(ISBLANK(I43), '⚙️ 全局核算参数 (Config)'!$B$13, I43))</f>
+      </c>
+      <c r="N43" s="49">
+        <f>IF(ISBLANK(D43), "", ROUND(((D43 * (1 + M43) + L43) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O43" s="50">
+        <f>IF(OR(ISBLANK(D43), NOT(AND(G43&gt;0, F43&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G43)) * F43)</f>
+      </c>
+      <c r="P43" s="50">
+        <f>IF(OR(ISBLANK(D43), NOT(AND(G43&gt;0, F43&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G43)) * F43)</f>
+      </c>
+      <c r="Q43" s="51">
+        <f>IF(ISBLANK(D43), "", IF(M43&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M43&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="44" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A44" s="39"/>
+      <c r="B44" s="40"/>
+      <c r="C44" s="41"/>
+      <c r="D44" s="42"/>
+      <c r="E44" s="43"/>
+      <c r="F44" s="43"/>
+      <c r="G44" s="44"/>
+      <c r="H44" s="45"/>
+      <c r="I44" s="46"/>
+      <c r="J44" s="39"/>
+      <c r="K44" s="39"/>
+      <c r="L44" s="47">
+        <f>IF(ISBLANK(D44), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M44" s="48">
+        <f>IF(ISBLANK(D44), "", IF(ISBLANK(I44), '⚙️ 全局核算参数 (Config)'!$B$13, I44))</f>
+      </c>
+      <c r="N44" s="49">
+        <f>IF(ISBLANK(D44), "", ROUND(((D44 * (1 + M44) + L44) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O44" s="50">
+        <f>IF(OR(ISBLANK(D44), NOT(AND(G44&gt;0, F44&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G44)) * F44)</f>
+      </c>
+      <c r="P44" s="50">
+        <f>IF(OR(ISBLANK(D44), NOT(AND(G44&gt;0, F44&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G44)) * F44)</f>
+      </c>
+      <c r="Q44" s="51">
+        <f>IF(ISBLANK(D44), "", IF(M44&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M44&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="45" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A45" s="52"/>
+      <c r="B45" s="53"/>
+      <c r="C45" s="54"/>
+      <c r="D45" s="55"/>
+      <c r="E45" s="56"/>
+      <c r="F45" s="56"/>
+      <c r="G45" s="57"/>
+      <c r="H45" s="58"/>
+      <c r="I45" s="59"/>
+      <c r="J45" s="52"/>
+      <c r="K45" s="52"/>
+      <c r="L45" s="47">
+        <f>IF(ISBLANK(D45), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M45" s="48">
+        <f>IF(ISBLANK(D45), "", IF(ISBLANK(I45), '⚙️ 全局核算参数 (Config)'!$B$13, I45))</f>
+      </c>
+      <c r="N45" s="49">
+        <f>IF(ISBLANK(D45), "", ROUND(((D45 * (1 + M45) + L45) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O45" s="50">
+        <f>IF(OR(ISBLANK(D45), NOT(AND(G45&gt;0, F45&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G45)) * F45)</f>
+      </c>
+      <c r="P45" s="50">
+        <f>IF(OR(ISBLANK(D45), NOT(AND(G45&gt;0, F45&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G45)) * F45)</f>
+      </c>
+      <c r="Q45" s="51">
+        <f>IF(ISBLANK(D45), "", IF(M45&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M45&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="46" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A46" s="39"/>
+      <c r="B46" s="40"/>
+      <c r="C46" s="41"/>
+      <c r="D46" s="42"/>
+      <c r="E46" s="43"/>
+      <c r="F46" s="43"/>
+      <c r="G46" s="44"/>
+      <c r="H46" s="45"/>
+      <c r="I46" s="46"/>
+      <c r="J46" s="39"/>
+      <c r="K46" s="39"/>
+      <c r="L46" s="47">
+        <f>IF(ISBLANK(D46), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M46" s="48">
+        <f>IF(ISBLANK(D46), "", IF(ISBLANK(I46), '⚙️ 全局核算参数 (Config)'!$B$13, I46))</f>
+      </c>
+      <c r="N46" s="49">
+        <f>IF(ISBLANK(D46), "", ROUND(((D46 * (1 + M46) + L46) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O46" s="50">
+        <f>IF(OR(ISBLANK(D46), NOT(AND(G46&gt;0, F46&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G46)) * F46)</f>
+      </c>
+      <c r="P46" s="50">
+        <f>IF(OR(ISBLANK(D46), NOT(AND(G46&gt;0, F46&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G46)) * F46)</f>
+      </c>
+      <c r="Q46" s="51">
+        <f>IF(ISBLANK(D46), "", IF(M46&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M46&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="47" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A47" s="52"/>
+      <c r="B47" s="53"/>
+      <c r="C47" s="54"/>
+      <c r="D47" s="55"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="56"/>
+      <c r="G47" s="57"/>
+      <c r="H47" s="58"/>
+      <c r="I47" s="59"/>
+      <c r="J47" s="52"/>
+      <c r="K47" s="52"/>
+      <c r="L47" s="47">
+        <f>IF(ISBLANK(D47), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M47" s="48">
+        <f>IF(ISBLANK(D47), "", IF(ISBLANK(I47), '⚙️ 全局核算参数 (Config)'!$B$13, I47))</f>
+      </c>
+      <c r="N47" s="49">
+        <f>IF(ISBLANK(D47), "", ROUND(((D47 * (1 + M47) + L47) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O47" s="50">
+        <f>IF(OR(ISBLANK(D47), NOT(AND(G47&gt;0, F47&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G47)) * F47)</f>
+      </c>
+      <c r="P47" s="50">
+        <f>IF(OR(ISBLANK(D47), NOT(AND(G47&gt;0, F47&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G47)) * F47)</f>
+      </c>
+      <c r="Q47" s="51">
+        <f>IF(ISBLANK(D47), "", IF(M47&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M47&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A48" s="39"/>
+      <c r="B48" s="40"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="42"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="44"/>
+      <c r="H48" s="45"/>
+      <c r="I48" s="46"/>
+      <c r="J48" s="39"/>
+      <c r="K48" s="39"/>
+      <c r="L48" s="47">
+        <f>IF(ISBLANK(D48), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M48" s="48">
+        <f>IF(ISBLANK(D48), "", IF(ISBLANK(I48), '⚙️ 全局核算参数 (Config)'!$B$13, I48))</f>
+      </c>
+      <c r="N48" s="49">
+        <f>IF(ISBLANK(D48), "", ROUND(((D48 * (1 + M48) + L48) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O48" s="50">
+        <f>IF(OR(ISBLANK(D48), NOT(AND(G48&gt;0, F48&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G48)) * F48)</f>
+      </c>
+      <c r="P48" s="50">
+        <f>IF(OR(ISBLANK(D48), NOT(AND(G48&gt;0, F48&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G48)) * F48)</f>
+      </c>
+      <c r="Q48" s="51">
+        <f>IF(ISBLANK(D48), "", IF(M48&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M48&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="49" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A49" s="52"/>
+      <c r="B49" s="53"/>
+      <c r="C49" s="54"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="57"/>
+      <c r="H49" s="58"/>
+      <c r="I49" s="59"/>
+      <c r="J49" s="52"/>
+      <c r="K49" s="52"/>
+      <c r="L49" s="47">
+        <f>IF(ISBLANK(D49), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M49" s="48">
+        <f>IF(ISBLANK(D49), "", IF(ISBLANK(I49), '⚙️ 全局核算参数 (Config)'!$B$13, I49))</f>
+      </c>
+      <c r="N49" s="49">
+        <f>IF(ISBLANK(D49), "", ROUND(((D49 * (1 + M49) + L49) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O49" s="50">
+        <f>IF(OR(ISBLANK(D49), NOT(AND(G49&gt;0, F49&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G49)) * F49)</f>
+      </c>
+      <c r="P49" s="50">
+        <f>IF(OR(ISBLANK(D49), NOT(AND(G49&gt;0, F49&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G49)) * F49)</f>
+      </c>
+      <c r="Q49" s="51">
+        <f>IF(ISBLANK(D49), "", IF(M49&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M49&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="50" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A50" s="39"/>
+      <c r="B50" s="40"/>
+      <c r="C50" s="41"/>
+      <c r="D50" s="42"/>
+      <c r="E50" s="43"/>
+      <c r="F50" s="43"/>
+      <c r="G50" s="44"/>
+      <c r="H50" s="45"/>
+      <c r="I50" s="46"/>
+      <c r="J50" s="39"/>
+      <c r="K50" s="39"/>
+      <c r="L50" s="47">
+        <f>IF(ISBLANK(D50), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M50" s="48">
+        <f>IF(ISBLANK(D50), "", IF(ISBLANK(I50), '⚙️ 全局核算参数 (Config)'!$B$13, I50))</f>
+      </c>
+      <c r="N50" s="49">
+        <f>IF(ISBLANK(D50), "", ROUND(((D50 * (1 + M50) + L50) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O50" s="50">
+        <f>IF(OR(ISBLANK(D50), NOT(AND(G50&gt;0, F50&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G50)) * F50)</f>
+      </c>
+      <c r="P50" s="50">
+        <f>IF(OR(ISBLANK(D50), NOT(AND(G50&gt;0, F50&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G50)) * F50)</f>
+      </c>
+      <c r="Q50" s="51">
+        <f>IF(ISBLANK(D50), "", IF(M50&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M50&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="51" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A51" s="52"/>
+      <c r="B51" s="53"/>
+      <c r="C51" s="54"/>
+      <c r="D51" s="55"/>
+      <c r="E51" s="56"/>
+      <c r="F51" s="56"/>
+      <c r="G51" s="57"/>
+      <c r="H51" s="58"/>
+      <c r="I51" s="59"/>
+      <c r="J51" s="52"/>
+      <c r="K51" s="52"/>
+      <c r="L51" s="47">
+        <f>IF(ISBLANK(D51), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M51" s="48">
+        <f>IF(ISBLANK(D51), "", IF(ISBLANK(I51), '⚙️ 全局核算参数 (Config)'!$B$13, I51))</f>
+      </c>
+      <c r="N51" s="49">
+        <f>IF(ISBLANK(D51), "", ROUND(((D51 * (1 + M51) + L51) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O51" s="50">
+        <f>IF(OR(ISBLANK(D51), NOT(AND(G51&gt;0, F51&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G51)) * F51)</f>
+      </c>
+      <c r="P51" s="50">
+        <f>IF(OR(ISBLANK(D51), NOT(AND(G51&gt;0, F51&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G51)) * F51)</f>
+      </c>
+      <c r="Q51" s="51">
+        <f>IF(ISBLANK(D51), "", IF(M51&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M51&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="52" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A52" s="39"/>
+      <c r="B52" s="40"/>
+      <c r="C52" s="41"/>
+      <c r="D52" s="42"/>
+      <c r="E52" s="43"/>
+      <c r="F52" s="43"/>
+      <c r="G52" s="44"/>
+      <c r="H52" s="45"/>
+      <c r="I52" s="46"/>
+      <c r="J52" s="39"/>
+      <c r="K52" s="39"/>
+      <c r="L52" s="47">
+        <f>IF(ISBLANK(D52), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M52" s="48">
+        <f>IF(ISBLANK(D52), "", IF(ISBLANK(I52), '⚙️ 全局核算参数 (Config)'!$B$13, I52))</f>
+      </c>
+      <c r="N52" s="49">
+        <f>IF(ISBLANK(D52), "", ROUND(((D52 * (1 + M52) + L52) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O52" s="50">
+        <f>IF(OR(ISBLANK(D52), NOT(AND(G52&gt;0, F52&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G52)) * F52)</f>
+      </c>
+      <c r="P52" s="50">
+        <f>IF(OR(ISBLANK(D52), NOT(AND(G52&gt;0, F52&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G52)) * F52)</f>
+      </c>
+      <c r="Q52" s="51">
+        <f>IF(ISBLANK(D52), "", IF(M52&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M52&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A53" s="52"/>
+      <c r="B53" s="53"/>
+      <c r="C53" s="54"/>
+      <c r="D53" s="55"/>
+      <c r="E53" s="56"/>
+      <c r="F53" s="56"/>
+      <c r="G53" s="57"/>
+      <c r="H53" s="58"/>
+      <c r="I53" s="59"/>
+      <c r="J53" s="52"/>
+      <c r="K53" s="52"/>
+      <c r="L53" s="47">
+        <f>IF(ISBLANK(D53), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M53" s="48">
+        <f>IF(ISBLANK(D53), "", IF(ISBLANK(I53), '⚙️ 全局核算参数 (Config)'!$B$13, I53))</f>
+      </c>
+      <c r="N53" s="49">
+        <f>IF(ISBLANK(D53), "", ROUND(((D53 * (1 + M53) + L53) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O53" s="50">
+        <f>IF(OR(ISBLANK(D53), NOT(AND(G53&gt;0, F53&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G53)) * F53)</f>
+      </c>
+      <c r="P53" s="50">
+        <f>IF(OR(ISBLANK(D53), NOT(AND(G53&gt;0, F53&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G53)) * F53)</f>
+      </c>
+      <c r="Q53" s="51">
+        <f>IF(ISBLANK(D53), "", IF(M53&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M53&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="54" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A54" s="39"/>
+      <c r="B54" s="40"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="42"/>
+      <c r="E54" s="43"/>
+      <c r="F54" s="43"/>
+      <c r="G54" s="44"/>
+      <c r="H54" s="45"/>
+      <c r="I54" s="46"/>
+      <c r="J54" s="39"/>
+      <c r="K54" s="39"/>
+      <c r="L54" s="47">
+        <f>IF(ISBLANK(D54), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M54" s="48">
+        <f>IF(ISBLANK(D54), "", IF(ISBLANK(I54), '⚙️ 全局核算参数 (Config)'!$B$13, I54))</f>
+      </c>
+      <c r="N54" s="49">
+        <f>IF(ISBLANK(D54), "", ROUND(((D54 * (1 + M54) + L54) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O54" s="50">
+        <f>IF(OR(ISBLANK(D54), NOT(AND(G54&gt;0, F54&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G54)) * F54)</f>
+      </c>
+      <c r="P54" s="50">
+        <f>IF(OR(ISBLANK(D54), NOT(AND(G54&gt;0, F54&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G54)) * F54)</f>
+      </c>
+      <c r="Q54" s="51">
+        <f>IF(ISBLANK(D54), "", IF(M54&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M54&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="55" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A55" s="52"/>
+      <c r="B55" s="53"/>
+      <c r="C55" s="54"/>
+      <c r="D55" s="55"/>
+      <c r="E55" s="56"/>
+      <c r="F55" s="56"/>
+      <c r="G55" s="57"/>
+      <c r="H55" s="58"/>
+      <c r="I55" s="59"/>
+      <c r="J55" s="52"/>
+      <c r="K55" s="52"/>
+      <c r="L55" s="47">
+        <f>IF(ISBLANK(D55), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M55" s="48">
+        <f>IF(ISBLANK(D55), "", IF(ISBLANK(I55), '⚙️ 全局核算参数 (Config)'!$B$13, I55))</f>
+      </c>
+      <c r="N55" s="49">
+        <f>IF(ISBLANK(D55), "", ROUND(((D55 * (1 + M55) + L55) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O55" s="50">
+        <f>IF(OR(ISBLANK(D55), NOT(AND(G55&gt;0, F55&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G55)) * F55)</f>
+      </c>
+      <c r="P55" s="50">
+        <f>IF(OR(ISBLANK(D55), NOT(AND(G55&gt;0, F55&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G55)) * F55)</f>
+      </c>
+      <c r="Q55" s="51">
+        <f>IF(ISBLANK(D55), "", IF(M55&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M55&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="56" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A56" s="39"/>
+      <c r="B56" s="40"/>
+      <c r="C56" s="41"/>
+      <c r="D56" s="42"/>
+      <c r="E56" s="43"/>
+      <c r="F56" s="43"/>
+      <c r="G56" s="44"/>
+      <c r="H56" s="45"/>
+      <c r="I56" s="46"/>
+      <c r="J56" s="39"/>
+      <c r="K56" s="39"/>
+      <c r="L56" s="47">
+        <f>IF(ISBLANK(D56), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M56" s="48">
+        <f>IF(ISBLANK(D56), "", IF(ISBLANK(I56), '⚙️ 全局核算参数 (Config)'!$B$13, I56))</f>
+      </c>
+      <c r="N56" s="49">
+        <f>IF(ISBLANK(D56), "", ROUND(((D56 * (1 + M56) + L56) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O56" s="50">
+        <f>IF(OR(ISBLANK(D56), NOT(AND(G56&gt;0, F56&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G56)) * F56)</f>
+      </c>
+      <c r="P56" s="50">
+        <f>IF(OR(ISBLANK(D56), NOT(AND(G56&gt;0, F56&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G56)) * F56)</f>
+      </c>
+      <c r="Q56" s="51">
+        <f>IF(ISBLANK(D56), "", IF(M56&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M56&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="57" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A57" s="52"/>
+      <c r="B57" s="53"/>
+      <c r="C57" s="54"/>
+      <c r="D57" s="55"/>
+      <c r="E57" s="56"/>
+      <c r="F57" s="56"/>
+      <c r="G57" s="57"/>
+      <c r="H57" s="58"/>
+      <c r="I57" s="59"/>
+      <c r="J57" s="52"/>
+      <c r="K57" s="52"/>
+      <c r="L57" s="47">
+        <f>IF(ISBLANK(D57), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M57" s="48">
+        <f>IF(ISBLANK(D57), "", IF(ISBLANK(I57), '⚙️ 全局核算参数 (Config)'!$B$13, I57))</f>
+      </c>
+      <c r="N57" s="49">
+        <f>IF(ISBLANK(D57), "", ROUND(((D57 * (1 + M57) + L57) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O57" s="50">
+        <f>IF(OR(ISBLANK(D57), NOT(AND(G57&gt;0, F57&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G57)) * F57)</f>
+      </c>
+      <c r="P57" s="50">
+        <f>IF(OR(ISBLANK(D57), NOT(AND(G57&gt;0, F57&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G57)) * F57)</f>
+      </c>
+      <c r="Q57" s="51">
+        <f>IF(ISBLANK(D57), "", IF(M57&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M57&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="58" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A58" s="39"/>
+      <c r="B58" s="40"/>
+      <c r="C58" s="41"/>
+      <c r="D58" s="42"/>
+      <c r="E58" s="43"/>
+      <c r="F58" s="43"/>
+      <c r="G58" s="44"/>
+      <c r="H58" s="45"/>
+      <c r="I58" s="46"/>
+      <c r="J58" s="39"/>
+      <c r="K58" s="39"/>
+      <c r="L58" s="47">
+        <f>IF(ISBLANK(D58), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M58" s="48">
+        <f>IF(ISBLANK(D58), "", IF(ISBLANK(I58), '⚙️ 全局核算参数 (Config)'!$B$13, I58))</f>
+      </c>
+      <c r="N58" s="49">
+        <f>IF(ISBLANK(D58), "", ROUND(((D58 * (1 + M58) + L58) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O58" s="50">
+        <f>IF(OR(ISBLANK(D58), NOT(AND(G58&gt;0, F58&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G58)) * F58)</f>
+      </c>
+      <c r="P58" s="50">
+        <f>IF(OR(ISBLANK(D58), NOT(AND(G58&gt;0, F58&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G58)) * F58)</f>
+      </c>
+      <c r="Q58" s="51">
+        <f>IF(ISBLANK(D58), "", IF(M58&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M58&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="59" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A59" s="52"/>
+      <c r="B59" s="53"/>
+      <c r="C59" s="54"/>
+      <c r="D59" s="55"/>
+      <c r="E59" s="56"/>
+      <c r="F59" s="56"/>
+      <c r="G59" s="57"/>
+      <c r="H59" s="58"/>
+      <c r="I59" s="59"/>
+      <c r="J59" s="52"/>
+      <c r="K59" s="52"/>
+      <c r="L59" s="47">
+        <f>IF(ISBLANK(D59), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M59" s="48">
+        <f>IF(ISBLANK(D59), "", IF(ISBLANK(I59), '⚙️ 全局核算参数 (Config)'!$B$13, I59))</f>
+      </c>
+      <c r="N59" s="49">
+        <f>IF(ISBLANK(D59), "", ROUND(((D59 * (1 + M59) + L59) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O59" s="50">
+        <f>IF(OR(ISBLANK(D59), NOT(AND(G59&gt;0, F59&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G59)) * F59)</f>
+      </c>
+      <c r="P59" s="50">
+        <f>IF(OR(ISBLANK(D59), NOT(AND(G59&gt;0, F59&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G59)) * F59)</f>
+      </c>
+      <c r="Q59" s="51">
+        <f>IF(ISBLANK(D59), "", IF(M59&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M59&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="60" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A60" s="39"/>
+      <c r="B60" s="40"/>
+      <c r="C60" s="41"/>
+      <c r="D60" s="42"/>
+      <c r="E60" s="43"/>
+      <c r="F60" s="43"/>
+      <c r="G60" s="44"/>
+      <c r="H60" s="45"/>
+      <c r="I60" s="46"/>
+      <c r="J60" s="39"/>
+      <c r="K60" s="39"/>
+      <c r="L60" s="47">
+        <f>IF(ISBLANK(D60), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M60" s="48">
+        <f>IF(ISBLANK(D60), "", IF(ISBLANK(I60), '⚙️ 全局核算参数 (Config)'!$B$13, I60))</f>
+      </c>
+      <c r="N60" s="49">
+        <f>IF(ISBLANK(D60), "", ROUND(((D60 * (1 + M60) + L60) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O60" s="50">
+        <f>IF(OR(ISBLANK(D60), NOT(AND(G60&gt;0, F60&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G60)) * F60)</f>
+      </c>
+      <c r="P60" s="50">
+        <f>IF(OR(ISBLANK(D60), NOT(AND(G60&gt;0, F60&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G60)) * F60)</f>
+      </c>
+      <c r="Q60" s="51">
+        <f>IF(ISBLANK(D60), "", IF(M60&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M60&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="61" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A61" s="52"/>
+      <c r="B61" s="53"/>
+      <c r="C61" s="54"/>
+      <c r="D61" s="55"/>
+      <c r="E61" s="56"/>
+      <c r="F61" s="56"/>
+      <c r="G61" s="57"/>
+      <c r="H61" s="58"/>
+      <c r="I61" s="59"/>
+      <c r="J61" s="52"/>
+      <c r="K61" s="52"/>
+      <c r="L61" s="47">
+        <f>IF(ISBLANK(D61), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M61" s="48">
+        <f>IF(ISBLANK(D61), "", IF(ISBLANK(I61), '⚙️ 全局核算参数 (Config)'!$B$13, I61))</f>
+      </c>
+      <c r="N61" s="49">
+        <f>IF(ISBLANK(D61), "", ROUND(((D61 * (1 + M61) + L61) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O61" s="50">
+        <f>IF(OR(ISBLANK(D61), NOT(AND(G61&gt;0, F61&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G61)) * F61)</f>
+      </c>
+      <c r="P61" s="50">
+        <f>IF(OR(ISBLANK(D61), NOT(AND(G61&gt;0, F61&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G61)) * F61)</f>
+      </c>
+      <c r="Q61" s="51">
+        <f>IF(ISBLANK(D61), "", IF(M61&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M61&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="62" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A62" s="39"/>
+      <c r="B62" s="40"/>
+      <c r="C62" s="41"/>
+      <c r="D62" s="42"/>
+      <c r="E62" s="43"/>
+      <c r="F62" s="43"/>
+      <c r="G62" s="44"/>
+      <c r="H62" s="45"/>
+      <c r="I62" s="46"/>
+      <c r="J62" s="39"/>
+      <c r="K62" s="39"/>
+      <c r="L62" s="47">
+        <f>IF(ISBLANK(D62), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M62" s="48">
+        <f>IF(ISBLANK(D62), "", IF(ISBLANK(I62), '⚙️ 全局核算参数 (Config)'!$B$13, I62))</f>
+      </c>
+      <c r="N62" s="49">
+        <f>IF(ISBLANK(D62), "", ROUND(((D62 * (1 + M62) + L62) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O62" s="50">
+        <f>IF(OR(ISBLANK(D62), NOT(AND(G62&gt;0, F62&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G62)) * F62)</f>
+      </c>
+      <c r="P62" s="50">
+        <f>IF(OR(ISBLANK(D62), NOT(AND(G62&gt;0, F62&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G62)) * F62)</f>
+      </c>
+      <c r="Q62" s="51">
+        <f>IF(ISBLANK(D62), "", IF(M62&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M62&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="63" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A63" s="52"/>
+      <c r="B63" s="53"/>
+      <c r="C63" s="54"/>
+      <c r="D63" s="55"/>
+      <c r="E63" s="56"/>
+      <c r="F63" s="56"/>
+      <c r="G63" s="57"/>
+      <c r="H63" s="58"/>
+      <c r="I63" s="59"/>
+      <c r="J63" s="52"/>
+      <c r="K63" s="52"/>
+      <c r="L63" s="47">
+        <f>IF(ISBLANK(D63), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M63" s="48">
+        <f>IF(ISBLANK(D63), "", IF(ISBLANK(I63), '⚙️ 全局核算参数 (Config)'!$B$13, I63))</f>
+      </c>
+      <c r="N63" s="49">
+        <f>IF(ISBLANK(D63), "", ROUND(((D63 * (1 + M63) + L63) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O63" s="50">
+        <f>IF(OR(ISBLANK(D63), NOT(AND(G63&gt;0, F63&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G63)) * F63)</f>
+      </c>
+      <c r="P63" s="50">
+        <f>IF(OR(ISBLANK(D63), NOT(AND(G63&gt;0, F63&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G63)) * F63)</f>
+      </c>
+      <c r="Q63" s="51">
+        <f>IF(ISBLANK(D63), "", IF(M63&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M63&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="64" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A64" s="39"/>
+      <c r="B64" s="40"/>
+      <c r="C64" s="41"/>
+      <c r="D64" s="42"/>
+      <c r="E64" s="43"/>
+      <c r="F64" s="43"/>
+      <c r="G64" s="44"/>
+      <c r="H64" s="45"/>
+      <c r="I64" s="46"/>
+      <c r="J64" s="39"/>
+      <c r="K64" s="39"/>
+      <c r="L64" s="47">
+        <f>IF(ISBLANK(D64), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M64" s="48">
+        <f>IF(ISBLANK(D64), "", IF(ISBLANK(I64), '⚙️ 全局核算参数 (Config)'!$B$13, I64))</f>
+      </c>
+      <c r="N64" s="49">
+        <f>IF(ISBLANK(D64), "", ROUND(((D64 * (1 + M64) + L64) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O64" s="50">
+        <f>IF(OR(ISBLANK(D64), NOT(AND(G64&gt;0, F64&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G64)) * F64)</f>
+      </c>
+      <c r="P64" s="50">
+        <f>IF(OR(ISBLANK(D64), NOT(AND(G64&gt;0, F64&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G64)) * F64)</f>
+      </c>
+      <c r="Q64" s="51">
+        <f>IF(ISBLANK(D64), "", IF(M64&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M64&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="65" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A65" s="52"/>
+      <c r="B65" s="53"/>
+      <c r="C65" s="54"/>
+      <c r="D65" s="55"/>
+      <c r="E65" s="56"/>
+      <c r="F65" s="56"/>
+      <c r="G65" s="57"/>
+      <c r="H65" s="58"/>
+      <c r="I65" s="59"/>
+      <c r="J65" s="52"/>
+      <c r="K65" s="52"/>
+      <c r="L65" s="47">
+        <f>IF(ISBLANK(D65), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M65" s="48">
+        <f>IF(ISBLANK(D65), "", IF(ISBLANK(I65), '⚙️ 全局核算参数 (Config)'!$B$13, I65))</f>
+      </c>
+      <c r="N65" s="49">
+        <f>IF(ISBLANK(D65), "", ROUND(((D65 * (1 + M65) + L65) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O65" s="50">
+        <f>IF(OR(ISBLANK(D65), NOT(AND(G65&gt;0, F65&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G65)) * F65)</f>
+      </c>
+      <c r="P65" s="50">
+        <f>IF(OR(ISBLANK(D65), NOT(AND(G65&gt;0, F65&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G65)) * F65)</f>
+      </c>
+      <c r="Q65" s="51">
+        <f>IF(ISBLANK(D65), "", IF(M65&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M65&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="66" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A66" s="39"/>
+      <c r="B66" s="40"/>
+      <c r="C66" s="41"/>
+      <c r="D66" s="42"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="44"/>
+      <c r="H66" s="45"/>
+      <c r="I66" s="46"/>
+      <c r="J66" s="39"/>
+      <c r="K66" s="39"/>
+      <c r="L66" s="47">
+        <f>IF(ISBLANK(D66), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M66" s="48">
+        <f>IF(ISBLANK(D66), "", IF(ISBLANK(I66), '⚙️ 全局核算参数 (Config)'!$B$13, I66))</f>
+      </c>
+      <c r="N66" s="49">
+        <f>IF(ISBLANK(D66), "", ROUND(((D66 * (1 + M66) + L66) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O66" s="50">
+        <f>IF(OR(ISBLANK(D66), NOT(AND(G66&gt;0, F66&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G66)) * F66)</f>
+      </c>
+      <c r="P66" s="50">
+        <f>IF(OR(ISBLANK(D66), NOT(AND(G66&gt;0, F66&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G66)) * F66)</f>
+      </c>
+      <c r="Q66" s="51">
+        <f>IF(ISBLANK(D66), "", IF(M66&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M66&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="67" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A67" s="52"/>
+      <c r="B67" s="53"/>
+      <c r="C67" s="54"/>
+      <c r="D67" s="55"/>
+      <c r="E67" s="56"/>
+      <c r="F67" s="56"/>
+      <c r="G67" s="57"/>
+      <c r="H67" s="58"/>
+      <c r="I67" s="59"/>
+      <c r="J67" s="52"/>
+      <c r="K67" s="52"/>
+      <c r="L67" s="47">
+        <f>IF(ISBLANK(D67), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M67" s="48">
+        <f>IF(ISBLANK(D67), "", IF(ISBLANK(I67), '⚙️ 全局核算参数 (Config)'!$B$13, I67))</f>
+      </c>
+      <c r="N67" s="49">
+        <f>IF(ISBLANK(D67), "", ROUND(((D67 * (1 + M67) + L67) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O67" s="50">
+        <f>IF(OR(ISBLANK(D67), NOT(AND(G67&gt;0, F67&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G67)) * F67)</f>
+      </c>
+      <c r="P67" s="50">
+        <f>IF(OR(ISBLANK(D67), NOT(AND(G67&gt;0, F67&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G67)) * F67)</f>
+      </c>
+      <c r="Q67" s="51">
+        <f>IF(ISBLANK(D67), "", IF(M67&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M67&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="68" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A68" s="39"/>
+      <c r="B68" s="40"/>
+      <c r="C68" s="41"/>
+      <c r="D68" s="42"/>
+      <c r="E68" s="43"/>
+      <c r="F68" s="43"/>
+      <c r="G68" s="44"/>
+      <c r="H68" s="45"/>
+      <c r="I68" s="46"/>
+      <c r="J68" s="39"/>
+      <c r="K68" s="39"/>
+      <c r="L68" s="47">
+        <f>IF(ISBLANK(D68), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M68" s="48">
+        <f>IF(ISBLANK(D68), "", IF(ISBLANK(I68), '⚙️ 全局核算参数 (Config)'!$B$13, I68))</f>
+      </c>
+      <c r="N68" s="49">
+        <f>IF(ISBLANK(D68), "", ROUND(((D68 * (1 + M68) + L68) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O68" s="50">
+        <f>IF(OR(ISBLANK(D68), NOT(AND(G68&gt;0, F68&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G68)) * F68)</f>
+      </c>
+      <c r="P68" s="50">
+        <f>IF(OR(ISBLANK(D68), NOT(AND(G68&gt;0, F68&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G68)) * F68)</f>
+      </c>
+      <c r="Q68" s="51">
+        <f>IF(ISBLANK(D68), "", IF(M68&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M68&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="69" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A69" s="52"/>
+      <c r="B69" s="53"/>
+      <c r="C69" s="54"/>
+      <c r="D69" s="55"/>
+      <c r="E69" s="56"/>
+      <c r="F69" s="56"/>
+      <c r="G69" s="57"/>
+      <c r="H69" s="58"/>
+      <c r="I69" s="59"/>
+      <c r="J69" s="52"/>
+      <c r="K69" s="52"/>
+      <c r="L69" s="47">
+        <f>IF(ISBLANK(D69), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M69" s="48">
+        <f>IF(ISBLANK(D69), "", IF(ISBLANK(I69), '⚙️ 全局核算参数 (Config)'!$B$13, I69))</f>
+      </c>
+      <c r="N69" s="49">
+        <f>IF(ISBLANK(D69), "", ROUND(((D69 * (1 + M69) + L69) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O69" s="50">
+        <f>IF(OR(ISBLANK(D69), NOT(AND(G69&gt;0, F69&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G69)) * F69)</f>
+      </c>
+      <c r="P69" s="50">
+        <f>IF(OR(ISBLANK(D69), NOT(AND(G69&gt;0, F69&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G69)) * F69)</f>
+      </c>
+      <c r="Q69" s="51">
+        <f>IF(ISBLANK(D69), "", IF(M69&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M69&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="70" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A70" s="39"/>
+      <c r="B70" s="40"/>
+      <c r="C70" s="41"/>
+      <c r="D70" s="42"/>
+      <c r="E70" s="43"/>
+      <c r="F70" s="43"/>
+      <c r="G70" s="44"/>
+      <c r="H70" s="45"/>
+      <c r="I70" s="46"/>
+      <c r="J70" s="39"/>
+      <c r="K70" s="39"/>
+      <c r="L70" s="47">
+        <f>IF(ISBLANK(D70), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M70" s="48">
+        <f>IF(ISBLANK(D70), "", IF(ISBLANK(I70), '⚙️ 全局核算参数 (Config)'!$B$13, I70))</f>
+      </c>
+      <c r="N70" s="49">
+        <f>IF(ISBLANK(D70), "", ROUND(((D70 * (1 + M70) + L70) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O70" s="50">
+        <f>IF(OR(ISBLANK(D70), NOT(AND(G70&gt;0, F70&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G70)) * F70)</f>
+      </c>
+      <c r="P70" s="50">
+        <f>IF(OR(ISBLANK(D70), NOT(AND(G70&gt;0, F70&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G70)) * F70)</f>
+      </c>
+      <c r="Q70" s="51">
+        <f>IF(ISBLANK(D70), "", IF(M70&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M70&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="71" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A71" s="52"/>
+      <c r="B71" s="53"/>
+      <c r="C71" s="54"/>
+      <c r="D71" s="55"/>
+      <c r="E71" s="56"/>
+      <c r="F71" s="56"/>
+      <c r="G71" s="57"/>
+      <c r="H71" s="58"/>
+      <c r="I71" s="59"/>
+      <c r="J71" s="52"/>
+      <c r="K71" s="52"/>
+      <c r="L71" s="47">
+        <f>IF(ISBLANK(D71), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M71" s="48">
+        <f>IF(ISBLANK(D71), "", IF(ISBLANK(I71), '⚙️ 全局核算参数 (Config)'!$B$13, I71))</f>
+      </c>
+      <c r="N71" s="49">
+        <f>IF(ISBLANK(D71), "", ROUND(((D71 * (1 + M71) + L71) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O71" s="50">
+        <f>IF(OR(ISBLANK(D71), NOT(AND(G71&gt;0, F71&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G71)) * F71)</f>
+      </c>
+      <c r="P71" s="50">
+        <f>IF(OR(ISBLANK(D71), NOT(AND(G71&gt;0, F71&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G71)) * F71)</f>
+      </c>
+      <c r="Q71" s="51">
+        <f>IF(ISBLANK(D71), "", IF(M71&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M71&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="72" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A72" s="39"/>
+      <c r="B72" s="40"/>
+      <c r="C72" s="41"/>
+      <c r="D72" s="42"/>
+      <c r="E72" s="43"/>
+      <c r="F72" s="43"/>
+      <c r="G72" s="44"/>
+      <c r="H72" s="45"/>
+      <c r="I72" s="46"/>
+      <c r="J72" s="39"/>
+      <c r="K72" s="39"/>
+      <c r="L72" s="47">
+        <f>IF(ISBLANK(D72), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M72" s="48">
+        <f>IF(ISBLANK(D72), "", IF(ISBLANK(I72), '⚙️ 全局核算参数 (Config)'!$B$13, I72))</f>
+      </c>
+      <c r="N72" s="49">
+        <f>IF(ISBLANK(D72), "", ROUND(((D72 * (1 + M72) + L72) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O72" s="50">
+        <f>IF(OR(ISBLANK(D72), NOT(AND(G72&gt;0, F72&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G72)) * F72)</f>
+      </c>
+      <c r="P72" s="50">
+        <f>IF(OR(ISBLANK(D72), NOT(AND(G72&gt;0, F72&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G72)) * F72)</f>
+      </c>
+      <c r="Q72" s="51">
+        <f>IF(ISBLANK(D72), "", IF(M72&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M72&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="73" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A73" s="52"/>
+      <c r="B73" s="53"/>
+      <c r="C73" s="54"/>
+      <c r="D73" s="55"/>
+      <c r="E73" s="56"/>
+      <c r="F73" s="56"/>
+      <c r="G73" s="57"/>
+      <c r="H73" s="58"/>
+      <c r="I73" s="59"/>
+      <c r="J73" s="52"/>
+      <c r="K73" s="52"/>
+      <c r="L73" s="47">
+        <f>IF(ISBLANK(D73), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M73" s="48">
+        <f>IF(ISBLANK(D73), "", IF(ISBLANK(I73), '⚙️ 全局核算参数 (Config)'!$B$13, I73))</f>
+      </c>
+      <c r="N73" s="49">
+        <f>IF(ISBLANK(D73), "", ROUND(((D73 * (1 + M73) + L73) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O73" s="50">
+        <f>IF(OR(ISBLANK(D73), NOT(AND(G73&gt;0, F73&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G73)) * F73)</f>
+      </c>
+      <c r="P73" s="50">
+        <f>IF(OR(ISBLANK(D73), NOT(AND(G73&gt;0, F73&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G73)) * F73)</f>
+      </c>
+      <c r="Q73" s="51">
+        <f>IF(ISBLANK(D73), "", IF(M73&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M73&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="74" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A74" s="39"/>
+      <c r="B74" s="40"/>
+      <c r="C74" s="41"/>
+      <c r="D74" s="42"/>
+      <c r="E74" s="43"/>
+      <c r="F74" s="43"/>
+      <c r="G74" s="44"/>
+      <c r="H74" s="45"/>
+      <c r="I74" s="46"/>
+      <c r="J74" s="39"/>
+      <c r="K74" s="39"/>
+      <c r="L74" s="47">
+        <f>IF(ISBLANK(D74), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M74" s="48">
+        <f>IF(ISBLANK(D74), "", IF(ISBLANK(I74), '⚙️ 全局核算参数 (Config)'!$B$13, I74))</f>
+      </c>
+      <c r="N74" s="49">
+        <f>IF(ISBLANK(D74), "", ROUND(((D74 * (1 + M74) + L74) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O74" s="50">
+        <f>IF(OR(ISBLANK(D74), NOT(AND(G74&gt;0, F74&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G74)) * F74)</f>
+      </c>
+      <c r="P74" s="50">
+        <f>IF(OR(ISBLANK(D74), NOT(AND(G74&gt;0, F74&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G74)) * F74)</f>
+      </c>
+      <c r="Q74" s="51">
+        <f>IF(ISBLANK(D74), "", IF(M74&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M74&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="75" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A75" s="52"/>
+      <c r="B75" s="53"/>
+      <c r="C75" s="54"/>
+      <c r="D75" s="55"/>
+      <c r="E75" s="56"/>
+      <c r="F75" s="56"/>
+      <c r="G75" s="57"/>
+      <c r="H75" s="58"/>
+      <c r="I75" s="59"/>
+      <c r="J75" s="52"/>
+      <c r="K75" s="52"/>
+      <c r="L75" s="47">
+        <f>IF(ISBLANK(D75), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M75" s="48">
+        <f>IF(ISBLANK(D75), "", IF(ISBLANK(I75), '⚙️ 全局核算参数 (Config)'!$B$13, I75))</f>
+      </c>
+      <c r="N75" s="49">
+        <f>IF(ISBLANK(D75), "", ROUND(((D75 * (1 + M75) + L75) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O75" s="50">
+        <f>IF(OR(ISBLANK(D75), NOT(AND(G75&gt;0, F75&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G75)) * F75)</f>
+      </c>
+      <c r="P75" s="50">
+        <f>IF(OR(ISBLANK(D75), NOT(AND(G75&gt;0, F75&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G75)) * F75)</f>
+      </c>
+      <c r="Q75" s="51">
+        <f>IF(ISBLANK(D75), "", IF(M75&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M75&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="76" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A76" s="39"/>
+      <c r="B76" s="40"/>
+      <c r="C76" s="41"/>
+      <c r="D76" s="42"/>
+      <c r="E76" s="43"/>
+      <c r="F76" s="43"/>
+      <c r="G76" s="44"/>
+      <c r="H76" s="45"/>
+      <c r="I76" s="46"/>
+      <c r="J76" s="39"/>
+      <c r="K76" s="39"/>
+      <c r="L76" s="47">
+        <f>IF(ISBLANK(D76), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M76" s="48">
+        <f>IF(ISBLANK(D76), "", IF(ISBLANK(I76), '⚙️ 全局核算参数 (Config)'!$B$13, I76))</f>
+      </c>
+      <c r="N76" s="49">
+        <f>IF(ISBLANK(D76), "", ROUND(((D76 * (1 + M76) + L76) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O76" s="50">
+        <f>IF(OR(ISBLANK(D76), NOT(AND(G76&gt;0, F76&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G76)) * F76)</f>
+      </c>
+      <c r="P76" s="50">
+        <f>IF(OR(ISBLANK(D76), NOT(AND(G76&gt;0, F76&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G76)) * F76)</f>
+      </c>
+      <c r="Q76" s="51">
+        <f>IF(ISBLANK(D76), "", IF(M76&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M76&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="77" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A77" s="52"/>
+      <c r="B77" s="53"/>
+      <c r="C77" s="54"/>
+      <c r="D77" s="55"/>
+      <c r="E77" s="56"/>
+      <c r="F77" s="56"/>
+      <c r="G77" s="57"/>
+      <c r="H77" s="58"/>
+      <c r="I77" s="59"/>
+      <c r="J77" s="52"/>
+      <c r="K77" s="52"/>
+      <c r="L77" s="47">
+        <f>IF(ISBLANK(D77), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M77" s="48">
+        <f>IF(ISBLANK(D77), "", IF(ISBLANK(I77), '⚙️ 全局核算参数 (Config)'!$B$13, I77))</f>
+      </c>
+      <c r="N77" s="49">
+        <f>IF(ISBLANK(D77), "", ROUND(((D77 * (1 + M77) + L77) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O77" s="50">
+        <f>IF(OR(ISBLANK(D77), NOT(AND(G77&gt;0, F77&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G77)) * F77)</f>
+      </c>
+      <c r="P77" s="50">
+        <f>IF(OR(ISBLANK(D77), NOT(AND(G77&gt;0, F77&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G77)) * F77)</f>
+      </c>
+      <c r="Q77" s="51">
+        <f>IF(ISBLANK(D77), "", IF(M77&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M77&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="78" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A78" s="39"/>
+      <c r="B78" s="40"/>
+      <c r="C78" s="41"/>
+      <c r="D78" s="42"/>
+      <c r="E78" s="43"/>
+      <c r="F78" s="43"/>
+      <c r="G78" s="44"/>
+      <c r="H78" s="45"/>
+      <c r="I78" s="46"/>
+      <c r="J78" s="39"/>
+      <c r="K78" s="39"/>
+      <c r="L78" s="47">
+        <f>IF(ISBLANK(D78), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M78" s="48">
+        <f>IF(ISBLANK(D78), "", IF(ISBLANK(I78), '⚙️ 全局核算参数 (Config)'!$B$13, I78))</f>
+      </c>
+      <c r="N78" s="49">
+        <f>IF(ISBLANK(D78), "", ROUND(((D78 * (1 + M78) + L78) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O78" s="50">
+        <f>IF(OR(ISBLANK(D78), NOT(AND(G78&gt;0, F78&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G78)) * F78)</f>
+      </c>
+      <c r="P78" s="50">
+        <f>IF(OR(ISBLANK(D78), NOT(AND(G78&gt;0, F78&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G78)) * F78)</f>
+      </c>
+      <c r="Q78" s="51">
+        <f>IF(ISBLANK(D78), "", IF(M78&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M78&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="79" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A79" s="52"/>
+      <c r="B79" s="53"/>
+      <c r="C79" s="54"/>
+      <c r="D79" s="55"/>
+      <c r="E79" s="56"/>
+      <c r="F79" s="56"/>
+      <c r="G79" s="57"/>
+      <c r="H79" s="58"/>
+      <c r="I79" s="59"/>
+      <c r="J79" s="52"/>
+      <c r="K79" s="52"/>
+      <c r="L79" s="47">
+        <f>IF(ISBLANK(D79), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M79" s="48">
+        <f>IF(ISBLANK(D79), "", IF(ISBLANK(I79), '⚙️ 全局核算参数 (Config)'!$B$13, I79))</f>
+      </c>
+      <c r="N79" s="49">
+        <f>IF(ISBLANK(D79), "", ROUND(((D79 * (1 + M79) + L79) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O79" s="50">
+        <f>IF(OR(ISBLANK(D79), NOT(AND(G79&gt;0, F79&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G79)) * F79)</f>
+      </c>
+      <c r="P79" s="50">
+        <f>IF(OR(ISBLANK(D79), NOT(AND(G79&gt;0, F79&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G79)) * F79)</f>
+      </c>
+      <c r="Q79" s="51">
+        <f>IF(ISBLANK(D79), "", IF(M79&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M79&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="80" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A80" s="39"/>
+      <c r="B80" s="40"/>
+      <c r="C80" s="41"/>
+      <c r="D80" s="42"/>
+      <c r="E80" s="43"/>
+      <c r="F80" s="43"/>
+      <c r="G80" s="44"/>
+      <c r="H80" s="45"/>
+      <c r="I80" s="46"/>
+      <c r="J80" s="39"/>
+      <c r="K80" s="39"/>
+      <c r="L80" s="47">
+        <f>IF(ISBLANK(D80), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M80" s="48">
+        <f>IF(ISBLANK(D80), "", IF(ISBLANK(I80), '⚙️ 全局核算参数 (Config)'!$B$13, I80))</f>
+      </c>
+      <c r="N80" s="49">
+        <f>IF(ISBLANK(D80), "", ROUND(((D80 * (1 + M80) + L80) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O80" s="50">
+        <f>IF(OR(ISBLANK(D80), NOT(AND(G80&gt;0, F80&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G80)) * F80)</f>
+      </c>
+      <c r="P80" s="50">
+        <f>IF(OR(ISBLANK(D80), NOT(AND(G80&gt;0, F80&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G80)) * F80)</f>
+      </c>
+      <c r="Q80" s="51">
+        <f>IF(ISBLANK(D80), "", IF(M80&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M80&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="81" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A81" s="52"/>
+      <c r="B81" s="53"/>
+      <c r="C81" s="54"/>
+      <c r="D81" s="55"/>
+      <c r="E81" s="56"/>
+      <c r="F81" s="56"/>
+      <c r="G81" s="57"/>
+      <c r="H81" s="58"/>
+      <c r="I81" s="59"/>
+      <c r="J81" s="52"/>
+      <c r="K81" s="52"/>
+      <c r="L81" s="47">
+        <f>IF(ISBLANK(D81), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M81" s="48">
+        <f>IF(ISBLANK(D81), "", IF(ISBLANK(I81), '⚙️ 全局核算参数 (Config)'!$B$13, I81))</f>
+      </c>
+      <c r="N81" s="49">
+        <f>IF(ISBLANK(D81), "", ROUND(((D81 * (1 + M81) + L81) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O81" s="50">
+        <f>IF(OR(ISBLANK(D81), NOT(AND(G81&gt;0, F81&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G81)) * F81)</f>
+      </c>
+      <c r="P81" s="50">
+        <f>IF(OR(ISBLANK(D81), NOT(AND(G81&gt;0, F81&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G81)) * F81)</f>
+      </c>
+      <c r="Q81" s="51">
+        <f>IF(ISBLANK(D81), "", IF(M81&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M81&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="82" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A82" s="39"/>
+      <c r="B82" s="40"/>
+      <c r="C82" s="41"/>
+      <c r="D82" s="42"/>
+      <c r="E82" s="43"/>
+      <c r="F82" s="43"/>
+      <c r="G82" s="44"/>
+      <c r="H82" s="45"/>
+      <c r="I82" s="46"/>
+      <c r="J82" s="39"/>
+      <c r="K82" s="39"/>
+      <c r="L82" s="47">
+        <f>IF(ISBLANK(D82), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M82" s="48">
+        <f>IF(ISBLANK(D82), "", IF(ISBLANK(I82), '⚙️ 全局核算参数 (Config)'!$B$13, I82))</f>
+      </c>
+      <c r="N82" s="49">
+        <f>IF(ISBLANK(D82), "", ROUND(((D82 * (1 + M82) + L82) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O82" s="50">
+        <f>IF(OR(ISBLANK(D82), NOT(AND(G82&gt;0, F82&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G82)) * F82)</f>
+      </c>
+      <c r="P82" s="50">
+        <f>IF(OR(ISBLANK(D82), NOT(AND(G82&gt;0, F82&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G82)) * F82)</f>
+      </c>
+      <c r="Q82" s="51">
+        <f>IF(ISBLANK(D82), "", IF(M82&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M82&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="83" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A83" s="52"/>
+      <c r="B83" s="53"/>
+      <c r="C83" s="54"/>
+      <c r="D83" s="55"/>
+      <c r="E83" s="56"/>
+      <c r="F83" s="56"/>
+      <c r="G83" s="57"/>
+      <c r="H83" s="58"/>
+      <c r="I83" s="59"/>
+      <c r="J83" s="52"/>
+      <c r="K83" s="52"/>
+      <c r="L83" s="47">
+        <f>IF(ISBLANK(D83), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M83" s="48">
+        <f>IF(ISBLANK(D83), "", IF(ISBLANK(I83), '⚙️ 全局核算参数 (Config)'!$B$13, I83))</f>
+      </c>
+      <c r="N83" s="49">
+        <f>IF(ISBLANK(D83), "", ROUND(((D83 * (1 + M83) + L83) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O83" s="50">
+        <f>IF(OR(ISBLANK(D83), NOT(AND(G83&gt;0, F83&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G83)) * F83)</f>
+      </c>
+      <c r="P83" s="50">
+        <f>IF(OR(ISBLANK(D83), NOT(AND(G83&gt;0, F83&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G83)) * F83)</f>
+      </c>
+      <c r="Q83" s="51">
+        <f>IF(ISBLANK(D83), "", IF(M83&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M83&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="84" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A84" s="39"/>
+      <c r="B84" s="40"/>
+      <c r="C84" s="41"/>
+      <c r="D84" s="42"/>
+      <c r="E84" s="43"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="44"/>
+      <c r="H84" s="45"/>
+      <c r="I84" s="46"/>
+      <c r="J84" s="39"/>
+      <c r="K84" s="39"/>
+      <c r="L84" s="47">
+        <f>IF(ISBLANK(D84), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M84" s="48">
+        <f>IF(ISBLANK(D84), "", IF(ISBLANK(I84), '⚙️ 全局核算参数 (Config)'!$B$13, I84))</f>
+      </c>
+      <c r="N84" s="49">
+        <f>IF(ISBLANK(D84), "", ROUND(((D84 * (1 + M84) + L84) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O84" s="50">
+        <f>IF(OR(ISBLANK(D84), NOT(AND(G84&gt;0, F84&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G84)) * F84)</f>
+      </c>
+      <c r="P84" s="50">
+        <f>IF(OR(ISBLANK(D84), NOT(AND(G84&gt;0, F84&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G84)) * F84)</f>
+      </c>
+      <c r="Q84" s="51">
+        <f>IF(ISBLANK(D84), "", IF(M84&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M84&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="85" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A85" s="52"/>
+      <c r="B85" s="53"/>
+      <c r="C85" s="54"/>
+      <c r="D85" s="55"/>
+      <c r="E85" s="56"/>
+      <c r="F85" s="56"/>
+      <c r="G85" s="57"/>
+      <c r="H85" s="58"/>
+      <c r="I85" s="59"/>
+      <c r="J85" s="52"/>
+      <c r="K85" s="52"/>
+      <c r="L85" s="47">
+        <f>IF(ISBLANK(D85), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M85" s="48">
+        <f>IF(ISBLANK(D85), "", IF(ISBLANK(I85), '⚙️ 全局核算参数 (Config)'!$B$13, I85))</f>
+      </c>
+      <c r="N85" s="49">
+        <f>IF(ISBLANK(D85), "", ROUND(((D85 * (1 + M85) + L85) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O85" s="50">
+        <f>IF(OR(ISBLANK(D85), NOT(AND(G85&gt;0, F85&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G85)) * F85)</f>
+      </c>
+      <c r="P85" s="50">
+        <f>IF(OR(ISBLANK(D85), NOT(AND(G85&gt;0, F85&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G85)) * F85)</f>
+      </c>
+      <c r="Q85" s="51">
+        <f>IF(ISBLANK(D85), "", IF(M85&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M85&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="86" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A86" s="39"/>
+      <c r="B86" s="40"/>
+      <c r="C86" s="41"/>
+      <c r="D86" s="42"/>
+      <c r="E86" s="43"/>
+      <c r="F86" s="43"/>
+      <c r="G86" s="44"/>
+      <c r="H86" s="45"/>
+      <c r="I86" s="46"/>
+      <c r="J86" s="39"/>
+      <c r="K86" s="39"/>
+      <c r="L86" s="47">
+        <f>IF(ISBLANK(D86), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M86" s="48">
+        <f>IF(ISBLANK(D86), "", IF(ISBLANK(I86), '⚙️ 全局核算参数 (Config)'!$B$13, I86))</f>
+      </c>
+      <c r="N86" s="49">
+        <f>IF(ISBLANK(D86), "", ROUND(((D86 * (1 + M86) + L86) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O86" s="50">
+        <f>IF(OR(ISBLANK(D86), NOT(AND(G86&gt;0, F86&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G86)) * F86)</f>
+      </c>
+      <c r="P86" s="50">
+        <f>IF(OR(ISBLANK(D86), NOT(AND(G86&gt;0, F86&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G86)) * F86)</f>
+      </c>
+      <c r="Q86" s="51">
+        <f>IF(ISBLANK(D86), "", IF(M86&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M86&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="87" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A87" s="52"/>
+      <c r="B87" s="53"/>
+      <c r="C87" s="54"/>
+      <c r="D87" s="55"/>
+      <c r="E87" s="56"/>
+      <c r="F87" s="56"/>
+      <c r="G87" s="57"/>
+      <c r="H87" s="58"/>
+      <c r="I87" s="59"/>
+      <c r="J87" s="52"/>
+      <c r="K87" s="52"/>
+      <c r="L87" s="47">
+        <f>IF(ISBLANK(D87), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M87" s="48">
+        <f>IF(ISBLANK(D87), "", IF(ISBLANK(I87), '⚙️ 全局核算参数 (Config)'!$B$13, I87))</f>
+      </c>
+      <c r="N87" s="49">
+        <f>IF(ISBLANK(D87), "", ROUND(((D87 * (1 + M87) + L87) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O87" s="50">
+        <f>IF(OR(ISBLANK(D87), NOT(AND(G87&gt;0, F87&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G87)) * F87)</f>
+      </c>
+      <c r="P87" s="50">
+        <f>IF(OR(ISBLANK(D87), NOT(AND(G87&gt;0, F87&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G87)) * F87)</f>
+      </c>
+      <c r="Q87" s="51">
+        <f>IF(ISBLANK(D87), "", IF(M87&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M87&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="88" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A88" s="39"/>
+      <c r="B88" s="40"/>
+      <c r="C88" s="41"/>
+      <c r="D88" s="42"/>
+      <c r="E88" s="43"/>
+      <c r="F88" s="43"/>
+      <c r="G88" s="44"/>
+      <c r="H88" s="45"/>
+      <c r="I88" s="46"/>
+      <c r="J88" s="39"/>
+      <c r="K88" s="39"/>
+      <c r="L88" s="47">
+        <f>IF(ISBLANK(D88), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M88" s="48">
+        <f>IF(ISBLANK(D88), "", IF(ISBLANK(I88), '⚙️ 全局核算参数 (Config)'!$B$13, I88))</f>
+      </c>
+      <c r="N88" s="49">
+        <f>IF(ISBLANK(D88), "", ROUND(((D88 * (1 + M88) + L88) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O88" s="50">
+        <f>IF(OR(ISBLANK(D88), NOT(AND(G88&gt;0, F88&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G88)) * F88)</f>
+      </c>
+      <c r="P88" s="50">
+        <f>IF(OR(ISBLANK(D88), NOT(AND(G88&gt;0, F88&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G88)) * F88)</f>
+      </c>
+      <c r="Q88" s="51">
+        <f>IF(ISBLANK(D88), "", IF(M88&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M88&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="89" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A89" s="52"/>
+      <c r="B89" s="53"/>
+      <c r="C89" s="54"/>
+      <c r="D89" s="55"/>
+      <c r="E89" s="56"/>
+      <c r="F89" s="56"/>
+      <c r="G89" s="57"/>
+      <c r="H89" s="58"/>
+      <c r="I89" s="59"/>
+      <c r="J89" s="52"/>
+      <c r="K89" s="52"/>
+      <c r="L89" s="47">
+        <f>IF(ISBLANK(D89), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M89" s="48">
+        <f>IF(ISBLANK(D89), "", IF(ISBLANK(I89), '⚙️ 全局核算参数 (Config)'!$B$13, I89))</f>
+      </c>
+      <c r="N89" s="49">
+        <f>IF(ISBLANK(D89), "", ROUND(((D89 * (1 + M89) + L89) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O89" s="50">
+        <f>IF(OR(ISBLANK(D89), NOT(AND(G89&gt;0, F89&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G89)) * F89)</f>
+      </c>
+      <c r="P89" s="50">
+        <f>IF(OR(ISBLANK(D89), NOT(AND(G89&gt;0, F89&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G89)) * F89)</f>
+      </c>
+      <c r="Q89" s="51">
+        <f>IF(ISBLANK(D89), "", IF(M89&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M89&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="90" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A90" s="39"/>
+      <c r="B90" s="40"/>
+      <c r="C90" s="41"/>
+      <c r="D90" s="42"/>
+      <c r="E90" s="43"/>
+      <c r="F90" s="43"/>
+      <c r="G90" s="44"/>
+      <c r="H90" s="45"/>
+      <c r="I90" s="46"/>
+      <c r="J90" s="39"/>
+      <c r="K90" s="39"/>
+      <c r="L90" s="47">
+        <f>IF(ISBLANK(D90), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M90" s="48">
+        <f>IF(ISBLANK(D90), "", IF(ISBLANK(I90), '⚙️ 全局核算参数 (Config)'!$B$13, I90))</f>
+      </c>
+      <c r="N90" s="49">
+        <f>IF(ISBLANK(D90), "", ROUND(((D90 * (1 + M90) + L90) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O90" s="50">
+        <f>IF(OR(ISBLANK(D90), NOT(AND(G90&gt;0, F90&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G90)) * F90)</f>
+      </c>
+      <c r="P90" s="50">
+        <f>IF(OR(ISBLANK(D90), NOT(AND(G90&gt;0, F90&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G90)) * F90)</f>
+      </c>
+      <c r="Q90" s="51">
+        <f>IF(ISBLANK(D90), "", IF(M90&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M90&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="91" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A91" s="52"/>
+      <c r="B91" s="53"/>
+      <c r="C91" s="54"/>
+      <c r="D91" s="55"/>
+      <c r="E91" s="56"/>
+      <c r="F91" s="56"/>
+      <c r="G91" s="57"/>
+      <c r="H91" s="58"/>
+      <c r="I91" s="59"/>
+      <c r="J91" s="52"/>
+      <c r="K91" s="52"/>
+      <c r="L91" s="47">
+        <f>IF(ISBLANK(D91), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M91" s="48">
+        <f>IF(ISBLANK(D91), "", IF(ISBLANK(I91), '⚙️ 全局核算参数 (Config)'!$B$13, I91))</f>
+      </c>
+      <c r="N91" s="49">
+        <f>IF(ISBLANK(D91), "", ROUND(((D91 * (1 + M91) + L91) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O91" s="50">
+        <f>IF(OR(ISBLANK(D91), NOT(AND(G91&gt;0, F91&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G91)) * F91)</f>
+      </c>
+      <c r="P91" s="50">
+        <f>IF(OR(ISBLANK(D91), NOT(AND(G91&gt;0, F91&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G91)) * F91)</f>
+      </c>
+      <c r="Q91" s="51">
+        <f>IF(ISBLANK(D91), "", IF(M91&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M91&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="92" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A92" s="39"/>
+      <c r="B92" s="40"/>
+      <c r="C92" s="41"/>
+      <c r="D92" s="42"/>
+      <c r="E92" s="43"/>
+      <c r="F92" s="43"/>
+      <c r="G92" s="44"/>
+      <c r="H92" s="45"/>
+      <c r="I92" s="46"/>
+      <c r="J92" s="39"/>
+      <c r="K92" s="39"/>
+      <c r="L92" s="47">
+        <f>IF(ISBLANK(D92), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M92" s="48">
+        <f>IF(ISBLANK(D92), "", IF(ISBLANK(I92), '⚙️ 全局核算参数 (Config)'!$B$13, I92))</f>
+      </c>
+      <c r="N92" s="49">
+        <f>IF(ISBLANK(D92), "", ROUND(((D92 * (1 + M92) + L92) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O92" s="50">
+        <f>IF(OR(ISBLANK(D92), NOT(AND(G92&gt;0, F92&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G92)) * F92)</f>
+      </c>
+      <c r="P92" s="50">
+        <f>IF(OR(ISBLANK(D92), NOT(AND(G92&gt;0, F92&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G92)) * F92)</f>
+      </c>
+      <c r="Q92" s="51">
+        <f>IF(ISBLANK(D92), "", IF(M92&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M92&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="93" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A93" s="52"/>
+      <c r="B93" s="53"/>
+      <c r="C93" s="54"/>
+      <c r="D93" s="55"/>
+      <c r="E93" s="56"/>
+      <c r="F93" s="56"/>
+      <c r="G93" s="57"/>
+      <c r="H93" s="58"/>
+      <c r="I93" s="59"/>
+      <c r="J93" s="52"/>
+      <c r="K93" s="52"/>
+      <c r="L93" s="47">
+        <f>IF(ISBLANK(D93), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M93" s="48">
+        <f>IF(ISBLANK(D93), "", IF(ISBLANK(I93), '⚙️ 全局核算参数 (Config)'!$B$13, I93))</f>
+      </c>
+      <c r="N93" s="49">
+        <f>IF(ISBLANK(D93), "", ROUND(((D93 * (1 + M93) + L93) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O93" s="50">
+        <f>IF(OR(ISBLANK(D93), NOT(AND(G93&gt;0, F93&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G93)) * F93)</f>
+      </c>
+      <c r="P93" s="50">
+        <f>IF(OR(ISBLANK(D93), NOT(AND(G93&gt;0, F93&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G93)) * F93)</f>
+      </c>
+      <c r="Q93" s="51">
+        <f>IF(ISBLANK(D93), "", IF(M93&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M93&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="94" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A94" s="39"/>
+      <c r="B94" s="40"/>
+      <c r="C94" s="41"/>
+      <c r="D94" s="42"/>
+      <c r="E94" s="43"/>
+      <c r="F94" s="43"/>
+      <c r="G94" s="44"/>
+      <c r="H94" s="45"/>
+      <c r="I94" s="46"/>
+      <c r="J94" s="39"/>
+      <c r="K94" s="39"/>
+      <c r="L94" s="47">
+        <f>IF(ISBLANK(D94), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M94" s="48">
+        <f>IF(ISBLANK(D94), "", IF(ISBLANK(I94), '⚙️ 全局核算参数 (Config)'!$B$13, I94))</f>
+      </c>
+      <c r="N94" s="49">
+        <f>IF(ISBLANK(D94), "", ROUND(((D94 * (1 + M94) + L94) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O94" s="50">
+        <f>IF(OR(ISBLANK(D94), NOT(AND(G94&gt;0, F94&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G94)) * F94)</f>
+      </c>
+      <c r="P94" s="50">
+        <f>IF(OR(ISBLANK(D94), NOT(AND(G94&gt;0, F94&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G94)) * F94)</f>
+      </c>
+      <c r="Q94" s="51">
+        <f>IF(ISBLANK(D94), "", IF(M94&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M94&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="95" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A95" s="52"/>
+      <c r="B95" s="53"/>
+      <c r="C95" s="54"/>
+      <c r="D95" s="55"/>
+      <c r="E95" s="56"/>
+      <c r="F95" s="56"/>
+      <c r="G95" s="57"/>
+      <c r="H95" s="58"/>
+      <c r="I95" s="59"/>
+      <c r="J95" s="52"/>
+      <c r="K95" s="52"/>
+      <c r="L95" s="47">
+        <f>IF(ISBLANK(D95), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M95" s="48">
+        <f>IF(ISBLANK(D95), "", IF(ISBLANK(I95), '⚙️ 全局核算参数 (Config)'!$B$13, I95))</f>
+      </c>
+      <c r="N95" s="49">
+        <f>IF(ISBLANK(D95), "", ROUND(((D95 * (1 + M95) + L95) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O95" s="50">
+        <f>IF(OR(ISBLANK(D95), NOT(AND(G95&gt;0, F95&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G95)) * F95)</f>
+      </c>
+      <c r="P95" s="50">
+        <f>IF(OR(ISBLANK(D95), NOT(AND(G95&gt;0, F95&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G95)) * F95)</f>
+      </c>
+      <c r="Q95" s="51">
+        <f>IF(ISBLANK(D95), "", IF(M95&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M95&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="96" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A96" s="39"/>
+      <c r="B96" s="40"/>
+      <c r="C96" s="41"/>
+      <c r="D96" s="42"/>
+      <c r="E96" s="43"/>
+      <c r="F96" s="43"/>
+      <c r="G96" s="44"/>
+      <c r="H96" s="45"/>
+      <c r="I96" s="46"/>
+      <c r="J96" s="39"/>
+      <c r="K96" s="39"/>
+      <c r="L96" s="47">
+        <f>IF(ISBLANK(D96), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M96" s="48">
+        <f>IF(ISBLANK(D96), "", IF(ISBLANK(I96), '⚙️ 全局核算参数 (Config)'!$B$13, I96))</f>
+      </c>
+      <c r="N96" s="49">
+        <f>IF(ISBLANK(D96), "", ROUND(((D96 * (1 + M96) + L96) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O96" s="50">
+        <f>IF(OR(ISBLANK(D96), NOT(AND(G96&gt;0, F96&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G96)) * F96)</f>
+      </c>
+      <c r="P96" s="50">
+        <f>IF(OR(ISBLANK(D96), NOT(AND(G96&gt;0, F96&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G96)) * F96)</f>
+      </c>
+      <c r="Q96" s="51">
+        <f>IF(ISBLANK(D96), "", IF(M96&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M96&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="97" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A97" s="52"/>
+      <c r="B97" s="53"/>
+      <c r="C97" s="54"/>
+      <c r="D97" s="55"/>
+      <c r="E97" s="56"/>
+      <c r="F97" s="56"/>
+      <c r="G97" s="57"/>
+      <c r="H97" s="58"/>
+      <c r="I97" s="59"/>
+      <c r="J97" s="52"/>
+      <c r="K97" s="52"/>
+      <c r="L97" s="47">
+        <f>IF(ISBLANK(D97), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M97" s="48">
+        <f>IF(ISBLANK(D97), "", IF(ISBLANK(I97), '⚙️ 全局核算参数 (Config)'!$B$13, I97))</f>
+      </c>
+      <c r="N97" s="49">
+        <f>IF(ISBLANK(D97), "", ROUND(((D97 * (1 + M97) + L97) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O97" s="50">
+        <f>IF(OR(ISBLANK(D97), NOT(AND(G97&gt;0, F97&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G97)) * F97)</f>
+      </c>
+      <c r="P97" s="50">
+        <f>IF(OR(ISBLANK(D97), NOT(AND(G97&gt;0, F97&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G97)) * F97)</f>
+      </c>
+      <c r="Q97" s="51">
+        <f>IF(ISBLANK(D97), "", IF(M97&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M97&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="98" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A98" s="39"/>
+      <c r="B98" s="40"/>
+      <c r="C98" s="41"/>
+      <c r="D98" s="42"/>
+      <c r="E98" s="43"/>
+      <c r="F98" s="43"/>
+      <c r="G98" s="44"/>
+      <c r="H98" s="45"/>
+      <c r="I98" s="46"/>
+      <c r="J98" s="39"/>
+      <c r="K98" s="39"/>
+      <c r="L98" s="47">
+        <f>IF(ISBLANK(D98), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M98" s="48">
+        <f>IF(ISBLANK(D98), "", IF(ISBLANK(I98), '⚙️ 全局核算参数 (Config)'!$B$13, I98))</f>
+      </c>
+      <c r="N98" s="49">
+        <f>IF(ISBLANK(D98), "", ROUND(((D98 * (1 + M98) + L98) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O98" s="50">
+        <f>IF(OR(ISBLANK(D98), NOT(AND(G98&gt;0, F98&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G98)) * F98)</f>
+      </c>
+      <c r="P98" s="50">
+        <f>IF(OR(ISBLANK(D98), NOT(AND(G98&gt;0, F98&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G98)) * F98)</f>
+      </c>
+      <c r="Q98" s="51">
+        <f>IF(ISBLANK(D98), "", IF(M98&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M98&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="99" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A99" s="52"/>
+      <c r="B99" s="53"/>
+      <c r="C99" s="54"/>
+      <c r="D99" s="55"/>
+      <c r="E99" s="56"/>
+      <c r="F99" s="56"/>
+      <c r="G99" s="57"/>
+      <c r="H99" s="58"/>
+      <c r="I99" s="59"/>
+      <c r="J99" s="52"/>
+      <c r="K99" s="52"/>
+      <c r="L99" s="47">
+        <f>IF(ISBLANK(D99), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M99" s="48">
+        <f>IF(ISBLANK(D99), "", IF(ISBLANK(I99), '⚙️ 全局核算参数 (Config)'!$B$13, I99))</f>
+      </c>
+      <c r="N99" s="49">
+        <f>IF(ISBLANK(D99), "", ROUND(((D99 * (1 + M99) + L99) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O99" s="50">
+        <f>IF(OR(ISBLANK(D99), NOT(AND(G99&gt;0, F99&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G99)) * F99)</f>
+      </c>
+      <c r="P99" s="50">
+        <f>IF(OR(ISBLANK(D99), NOT(AND(G99&gt;0, F99&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G99)) * F99)</f>
+      </c>
+      <c r="Q99" s="51">
+        <f>IF(ISBLANK(D99), "", IF(M99&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M99&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="100" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A100" s="39"/>
+      <c r="B100" s="40"/>
+      <c r="C100" s="41"/>
+      <c r="D100" s="42"/>
+      <c r="E100" s="43"/>
+      <c r="F100" s="43"/>
+      <c r="G100" s="44"/>
+      <c r="H100" s="45"/>
+      <c r="I100" s="46"/>
+      <c r="J100" s="39"/>
+      <c r="K100" s="39"/>
+      <c r="L100" s="47">
+        <f>IF(ISBLANK(D100), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M100" s="48">
+        <f>IF(ISBLANK(D100), "", IF(ISBLANK(I100), '⚙️ 全局核算参数 (Config)'!$B$13, I100))</f>
+      </c>
+      <c r="N100" s="49">
+        <f>IF(ISBLANK(D100), "", ROUND(((D100 * (1 + M100) + L100) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O100" s="50">
+        <f>IF(OR(ISBLANK(D100), NOT(AND(G100&gt;0, F100&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G100)) * F100)</f>
+      </c>
+      <c r="P100" s="50">
+        <f>IF(OR(ISBLANK(D100), NOT(AND(G100&gt;0, F100&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G100)) * F100)</f>
+      </c>
+      <c r="Q100" s="51">
+        <f>IF(ISBLANK(D100), "", IF(M100&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M100&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="101" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A101" s="52"/>
+      <c r="B101" s="53"/>
+      <c r="C101" s="54"/>
+      <c r="D101" s="55"/>
+      <c r="E101" s="56"/>
+      <c r="F101" s="56"/>
+      <c r="G101" s="57"/>
+      <c r="H101" s="58"/>
+      <c r="I101" s="59"/>
+      <c r="J101" s="52"/>
+      <c r="K101" s="52"/>
+      <c r="L101" s="47">
+        <f>IF(ISBLANK(D101), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M101" s="48">
+        <f>IF(ISBLANK(D101), "", IF(ISBLANK(I101), '⚙️ 全局核算参数 (Config)'!$B$13, I101))</f>
+      </c>
+      <c r="N101" s="49">
+        <f>IF(ISBLANK(D101), "", ROUND(((D101 * (1 + M101) + L101) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O101" s="50">
+        <f>IF(OR(ISBLANK(D101), NOT(AND(G101&gt;0, F101&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G101)) * F101)</f>
+      </c>
+      <c r="P101" s="50">
+        <f>IF(OR(ISBLANK(D101), NOT(AND(G101&gt;0, F101&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G101)) * F101)</f>
+      </c>
+      <c r="Q101" s="51">
+        <f>IF(ISBLANK(D101), "", IF(M101&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M101&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2998,7 +5168,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -3943,6 +6113,2036 @@
         <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A31), "", '📦 商品出厂底价库 (Products)'!J31)</f>
       </c>
     </row>
+    <row r="34" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A32), "", 31)</f>
+      </c>
+      <c r="B34" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A32), "", '📦 商品出厂底价库 (Products)'!A32)</f>
+      </c>
+      <c r="C34" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A32), "", '📦 商品出厂底价库 (Products)'!C32)</f>
+      </c>
+      <c r="D34" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A32), "", '📦 商品出厂底价库 (Products)'!E32)</f>
+      </c>
+      <c r="E34" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A32), "", '📦 商品出厂底价库 (Products)'!N32)</f>
+      </c>
+      <c r="F34" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A32), "", '📦 商品出厂底价库 (Products)'!F32)</f>
+      </c>
+      <c r="G34" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A32), "", '📦 商品出厂底价库 (Products)'!O32)</f>
+      </c>
+      <c r="H34" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A32), "", '📦 商品出厂底价库 (Products)'!P32)</f>
+      </c>
+      <c r="I34" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A32), "", '📦 商品出厂底价库 (Products)'!J32)</f>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A33), "", 32)</f>
+      </c>
+      <c r="B35" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A33), "", '📦 商品出厂底价库 (Products)'!A33)</f>
+      </c>
+      <c r="C35" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A33), "", '📦 商品出厂底价库 (Products)'!C33)</f>
+      </c>
+      <c r="D35" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A33), "", '📦 商品出厂底价库 (Products)'!E33)</f>
+      </c>
+      <c r="E35" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A33), "", '📦 商品出厂底价库 (Products)'!N33)</f>
+      </c>
+      <c r="F35" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A33), "", '📦 商品出厂底价库 (Products)'!F33)</f>
+      </c>
+      <c r="G35" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A33), "", '📦 商品出厂底价库 (Products)'!O33)</f>
+      </c>
+      <c r="H35" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A33), "", '📦 商品出厂底价库 (Products)'!P33)</f>
+      </c>
+      <c r="I35" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A33), "", '📦 商品出厂底价库 (Products)'!J33)</f>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A34), "", 33)</f>
+      </c>
+      <c r="B36" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A34), "", '📦 商品出厂底价库 (Products)'!A34)</f>
+      </c>
+      <c r="C36" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A34), "", '📦 商品出厂底价库 (Products)'!C34)</f>
+      </c>
+      <c r="D36" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A34), "", '📦 商品出厂底价库 (Products)'!E34)</f>
+      </c>
+      <c r="E36" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A34), "", '📦 商品出厂底价库 (Products)'!N34)</f>
+      </c>
+      <c r="F36" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A34), "", '📦 商品出厂底价库 (Products)'!F34)</f>
+      </c>
+      <c r="G36" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A34), "", '📦 商品出厂底价库 (Products)'!O34)</f>
+      </c>
+      <c r="H36" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A34), "", '📦 商品出厂底价库 (Products)'!P34)</f>
+      </c>
+      <c r="I36" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A34), "", '📦 商品出厂底价库 (Products)'!J34)</f>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A35), "", 34)</f>
+      </c>
+      <c r="B37" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A35), "", '📦 商品出厂底价库 (Products)'!A35)</f>
+      </c>
+      <c r="C37" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A35), "", '📦 商品出厂底价库 (Products)'!C35)</f>
+      </c>
+      <c r="D37" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A35), "", '📦 商品出厂底价库 (Products)'!E35)</f>
+      </c>
+      <c r="E37" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A35), "", '📦 商品出厂底价库 (Products)'!N35)</f>
+      </c>
+      <c r="F37" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A35), "", '📦 商品出厂底价库 (Products)'!F35)</f>
+      </c>
+      <c r="G37" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A35), "", '📦 商品出厂底价库 (Products)'!O35)</f>
+      </c>
+      <c r="H37" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A35), "", '📦 商品出厂底价库 (Products)'!P35)</f>
+      </c>
+      <c r="I37" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A35), "", '📦 商品出厂底价库 (Products)'!J35)</f>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A36), "", 35)</f>
+      </c>
+      <c r="B38" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A36), "", '📦 商品出厂底价库 (Products)'!A36)</f>
+      </c>
+      <c r="C38" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A36), "", '📦 商品出厂底价库 (Products)'!C36)</f>
+      </c>
+      <c r="D38" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A36), "", '📦 商品出厂底价库 (Products)'!E36)</f>
+      </c>
+      <c r="E38" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A36), "", '📦 商品出厂底价库 (Products)'!N36)</f>
+      </c>
+      <c r="F38" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A36), "", '📦 商品出厂底价库 (Products)'!F36)</f>
+      </c>
+      <c r="G38" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A36), "", '📦 商品出厂底价库 (Products)'!O36)</f>
+      </c>
+      <c r="H38" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A36), "", '📦 商品出厂底价库 (Products)'!P36)</f>
+      </c>
+      <c r="I38" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A36), "", '📦 商品出厂底价库 (Products)'!J36)</f>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A37), "", 36)</f>
+      </c>
+      <c r="B39" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A37), "", '📦 商品出厂底价库 (Products)'!A37)</f>
+      </c>
+      <c r="C39" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A37), "", '📦 商品出厂底价库 (Products)'!C37)</f>
+      </c>
+      <c r="D39" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A37), "", '📦 商品出厂底价库 (Products)'!E37)</f>
+      </c>
+      <c r="E39" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A37), "", '📦 商品出厂底价库 (Products)'!N37)</f>
+      </c>
+      <c r="F39" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A37), "", '📦 商品出厂底价库 (Products)'!F37)</f>
+      </c>
+      <c r="G39" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A37), "", '📦 商品出厂底价库 (Products)'!O37)</f>
+      </c>
+      <c r="H39" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A37), "", '📦 商品出厂底价库 (Products)'!P37)</f>
+      </c>
+      <c r="I39" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A37), "", '📦 商品出厂底价库 (Products)'!J37)</f>
+      </c>
+    </row>
+    <row r="40" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A38), "", 37)</f>
+      </c>
+      <c r="B40" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A38), "", '📦 商品出厂底价库 (Products)'!A38)</f>
+      </c>
+      <c r="C40" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A38), "", '📦 商品出厂底价库 (Products)'!C38)</f>
+      </c>
+      <c r="D40" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A38), "", '📦 商品出厂底价库 (Products)'!E38)</f>
+      </c>
+      <c r="E40" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A38), "", '📦 商品出厂底价库 (Products)'!N38)</f>
+      </c>
+      <c r="F40" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A38), "", '📦 商品出厂底价库 (Products)'!F38)</f>
+      </c>
+      <c r="G40" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A38), "", '📦 商品出厂底价库 (Products)'!O38)</f>
+      </c>
+      <c r="H40" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A38), "", '📦 商品出厂底价库 (Products)'!P38)</f>
+      </c>
+      <c r="I40" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A38), "", '📦 商品出厂底价库 (Products)'!J38)</f>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A39), "", 38)</f>
+      </c>
+      <c r="B41" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A39), "", '📦 商品出厂底价库 (Products)'!A39)</f>
+      </c>
+      <c r="C41" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A39), "", '📦 商品出厂底价库 (Products)'!C39)</f>
+      </c>
+      <c r="D41" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A39), "", '📦 商品出厂底价库 (Products)'!E39)</f>
+      </c>
+      <c r="E41" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A39), "", '📦 商品出厂底价库 (Products)'!N39)</f>
+      </c>
+      <c r="F41" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A39), "", '📦 商品出厂底价库 (Products)'!F39)</f>
+      </c>
+      <c r="G41" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A39), "", '📦 商品出厂底价库 (Products)'!O39)</f>
+      </c>
+      <c r="H41" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A39), "", '📦 商品出厂底价库 (Products)'!P39)</f>
+      </c>
+      <c r="I41" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A39), "", '📦 商品出厂底价库 (Products)'!J39)</f>
+      </c>
+    </row>
+    <row r="42" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A40), "", 39)</f>
+      </c>
+      <c r="B42" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A40), "", '📦 商品出厂底价库 (Products)'!A40)</f>
+      </c>
+      <c r="C42" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A40), "", '📦 商品出厂底价库 (Products)'!C40)</f>
+      </c>
+      <c r="D42" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A40), "", '📦 商品出厂底价库 (Products)'!E40)</f>
+      </c>
+      <c r="E42" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A40), "", '📦 商品出厂底价库 (Products)'!N40)</f>
+      </c>
+      <c r="F42" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A40), "", '📦 商品出厂底价库 (Products)'!F40)</f>
+      </c>
+      <c r="G42" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A40), "", '📦 商品出厂底价库 (Products)'!O40)</f>
+      </c>
+      <c r="H42" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A40), "", '📦 商品出厂底价库 (Products)'!P40)</f>
+      </c>
+      <c r="I42" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A40), "", '📦 商品出厂底价库 (Products)'!J40)</f>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A41), "", 40)</f>
+      </c>
+      <c r="B43" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A41), "", '📦 商品出厂底价库 (Products)'!A41)</f>
+      </c>
+      <c r="C43" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A41), "", '📦 商品出厂底价库 (Products)'!C41)</f>
+      </c>
+      <c r="D43" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A41), "", '📦 商品出厂底价库 (Products)'!E41)</f>
+      </c>
+      <c r="E43" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A41), "", '📦 商品出厂底价库 (Products)'!N41)</f>
+      </c>
+      <c r="F43" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A41), "", '📦 商品出厂底价库 (Products)'!F41)</f>
+      </c>
+      <c r="G43" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A41), "", '📦 商品出厂底价库 (Products)'!O41)</f>
+      </c>
+      <c r="H43" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A41), "", '📦 商品出厂底价库 (Products)'!P41)</f>
+      </c>
+      <c r="I43" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A41), "", '📦 商品出厂底价库 (Products)'!J41)</f>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A42), "", 41)</f>
+      </c>
+      <c r="B44" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A42), "", '📦 商品出厂底价库 (Products)'!A42)</f>
+      </c>
+      <c r="C44" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A42), "", '📦 商品出厂底价库 (Products)'!C42)</f>
+      </c>
+      <c r="D44" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A42), "", '📦 商品出厂底价库 (Products)'!E42)</f>
+      </c>
+      <c r="E44" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A42), "", '📦 商品出厂底价库 (Products)'!N42)</f>
+      </c>
+      <c r="F44" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A42), "", '📦 商品出厂底价库 (Products)'!F42)</f>
+      </c>
+      <c r="G44" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A42), "", '📦 商品出厂底价库 (Products)'!O42)</f>
+      </c>
+      <c r="H44" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A42), "", '📦 商品出厂底价库 (Products)'!P42)</f>
+      </c>
+      <c r="I44" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A42), "", '📦 商品出厂底价库 (Products)'!J42)</f>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A43), "", 42)</f>
+      </c>
+      <c r="B45" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A43), "", '📦 商品出厂底价库 (Products)'!A43)</f>
+      </c>
+      <c r="C45" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A43), "", '📦 商品出厂底价库 (Products)'!C43)</f>
+      </c>
+      <c r="D45" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A43), "", '📦 商品出厂底价库 (Products)'!E43)</f>
+      </c>
+      <c r="E45" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A43), "", '📦 商品出厂底价库 (Products)'!N43)</f>
+      </c>
+      <c r="F45" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A43), "", '📦 商品出厂底价库 (Products)'!F43)</f>
+      </c>
+      <c r="G45" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A43), "", '📦 商品出厂底价库 (Products)'!O43)</f>
+      </c>
+      <c r="H45" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A43), "", '📦 商品出厂底价库 (Products)'!P43)</f>
+      </c>
+      <c r="I45" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A43), "", '📦 商品出厂底价库 (Products)'!J43)</f>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A44), "", 43)</f>
+      </c>
+      <c r="B46" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A44), "", '📦 商品出厂底价库 (Products)'!A44)</f>
+      </c>
+      <c r="C46" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A44), "", '📦 商品出厂底价库 (Products)'!C44)</f>
+      </c>
+      <c r="D46" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A44), "", '📦 商品出厂底价库 (Products)'!E44)</f>
+      </c>
+      <c r="E46" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A44), "", '📦 商品出厂底价库 (Products)'!N44)</f>
+      </c>
+      <c r="F46" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A44), "", '📦 商品出厂底价库 (Products)'!F44)</f>
+      </c>
+      <c r="G46" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A44), "", '📦 商品出厂底价库 (Products)'!O44)</f>
+      </c>
+      <c r="H46" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A44), "", '📦 商品出厂底价库 (Products)'!P44)</f>
+      </c>
+      <c r="I46" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A44), "", '📦 商品出厂底价库 (Products)'!J44)</f>
+      </c>
+    </row>
+    <row r="47" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A45), "", 44)</f>
+      </c>
+      <c r="B47" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A45), "", '📦 商品出厂底价库 (Products)'!A45)</f>
+      </c>
+      <c r="C47" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A45), "", '📦 商品出厂底价库 (Products)'!C45)</f>
+      </c>
+      <c r="D47" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A45), "", '📦 商品出厂底价库 (Products)'!E45)</f>
+      </c>
+      <c r="E47" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A45), "", '📦 商品出厂底价库 (Products)'!N45)</f>
+      </c>
+      <c r="F47" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A45), "", '📦 商品出厂底价库 (Products)'!F45)</f>
+      </c>
+      <c r="G47" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A45), "", '📦 商品出厂底价库 (Products)'!O45)</f>
+      </c>
+      <c r="H47" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A45), "", '📦 商品出厂底价库 (Products)'!P45)</f>
+      </c>
+      <c r="I47" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A45), "", '📦 商品出厂底价库 (Products)'!J45)</f>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A46), "", 45)</f>
+      </c>
+      <c r="B48" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A46), "", '📦 商品出厂底价库 (Products)'!A46)</f>
+      </c>
+      <c r="C48" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A46), "", '📦 商品出厂底价库 (Products)'!C46)</f>
+      </c>
+      <c r="D48" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A46), "", '📦 商品出厂底价库 (Products)'!E46)</f>
+      </c>
+      <c r="E48" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A46), "", '📦 商品出厂底价库 (Products)'!N46)</f>
+      </c>
+      <c r="F48" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A46), "", '📦 商品出厂底价库 (Products)'!F46)</f>
+      </c>
+      <c r="G48" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A46), "", '📦 商品出厂底价库 (Products)'!O46)</f>
+      </c>
+      <c r="H48" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A46), "", '📦 商品出厂底价库 (Products)'!P46)</f>
+      </c>
+      <c r="I48" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A46), "", '📦 商品出厂底价库 (Products)'!J46)</f>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A47), "", 46)</f>
+      </c>
+      <c r="B49" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A47), "", '📦 商品出厂底价库 (Products)'!A47)</f>
+      </c>
+      <c r="C49" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A47), "", '📦 商品出厂底价库 (Products)'!C47)</f>
+      </c>
+      <c r="D49" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A47), "", '📦 商品出厂底价库 (Products)'!E47)</f>
+      </c>
+      <c r="E49" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A47), "", '📦 商品出厂底价库 (Products)'!N47)</f>
+      </c>
+      <c r="F49" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A47), "", '📦 商品出厂底价库 (Products)'!F47)</f>
+      </c>
+      <c r="G49" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A47), "", '📦 商品出厂底价库 (Products)'!O47)</f>
+      </c>
+      <c r="H49" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A47), "", '📦 商品出厂底价库 (Products)'!P47)</f>
+      </c>
+      <c r="I49" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A47), "", '📦 商品出厂底价库 (Products)'!J47)</f>
+      </c>
+    </row>
+    <row r="50" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A48), "", 47)</f>
+      </c>
+      <c r="B50" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A48), "", '📦 商品出厂底价库 (Products)'!A48)</f>
+      </c>
+      <c r="C50" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A48), "", '📦 商品出厂底价库 (Products)'!C48)</f>
+      </c>
+      <c r="D50" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A48), "", '📦 商品出厂底价库 (Products)'!E48)</f>
+      </c>
+      <c r="E50" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A48), "", '📦 商品出厂底价库 (Products)'!N48)</f>
+      </c>
+      <c r="F50" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A48), "", '📦 商品出厂底价库 (Products)'!F48)</f>
+      </c>
+      <c r="G50" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A48), "", '📦 商品出厂底价库 (Products)'!O48)</f>
+      </c>
+      <c r="H50" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A48), "", '📦 商品出厂底价库 (Products)'!P48)</f>
+      </c>
+      <c r="I50" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A48), "", '📦 商品出厂底价库 (Products)'!J48)</f>
+      </c>
+    </row>
+    <row r="51" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A49), "", 48)</f>
+      </c>
+      <c r="B51" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A49), "", '📦 商品出厂底价库 (Products)'!A49)</f>
+      </c>
+      <c r="C51" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A49), "", '📦 商品出厂底价库 (Products)'!C49)</f>
+      </c>
+      <c r="D51" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A49), "", '📦 商品出厂底价库 (Products)'!E49)</f>
+      </c>
+      <c r="E51" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A49), "", '📦 商品出厂底价库 (Products)'!N49)</f>
+      </c>
+      <c r="F51" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A49), "", '📦 商品出厂底价库 (Products)'!F49)</f>
+      </c>
+      <c r="G51" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A49), "", '📦 商品出厂底价库 (Products)'!O49)</f>
+      </c>
+      <c r="H51" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A49), "", '📦 商品出厂底价库 (Products)'!P49)</f>
+      </c>
+      <c r="I51" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A49), "", '📦 商品出厂底价库 (Products)'!J49)</f>
+      </c>
+    </row>
+    <row r="52" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A50), "", 49)</f>
+      </c>
+      <c r="B52" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A50), "", '📦 商品出厂底价库 (Products)'!A50)</f>
+      </c>
+      <c r="C52" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A50), "", '📦 商品出厂底价库 (Products)'!C50)</f>
+      </c>
+      <c r="D52" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A50), "", '📦 商品出厂底价库 (Products)'!E50)</f>
+      </c>
+      <c r="E52" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A50), "", '📦 商品出厂底价库 (Products)'!N50)</f>
+      </c>
+      <c r="F52" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A50), "", '📦 商品出厂底价库 (Products)'!F50)</f>
+      </c>
+      <c r="G52" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A50), "", '📦 商品出厂底价库 (Products)'!O50)</f>
+      </c>
+      <c r="H52" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A50), "", '📦 商品出厂底价库 (Products)'!P50)</f>
+      </c>
+      <c r="I52" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A50), "", '📦 商品出厂底价库 (Products)'!J50)</f>
+      </c>
+    </row>
+    <row r="53" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A51), "", 50)</f>
+      </c>
+      <c r="B53" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A51), "", '📦 商品出厂底价库 (Products)'!A51)</f>
+      </c>
+      <c r="C53" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A51), "", '📦 商品出厂底价库 (Products)'!C51)</f>
+      </c>
+      <c r="D53" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A51), "", '📦 商品出厂底价库 (Products)'!E51)</f>
+      </c>
+      <c r="E53" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A51), "", '📦 商品出厂底价库 (Products)'!N51)</f>
+      </c>
+      <c r="F53" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A51), "", '📦 商品出厂底价库 (Products)'!F51)</f>
+      </c>
+      <c r="G53" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A51), "", '📦 商品出厂底价库 (Products)'!O51)</f>
+      </c>
+      <c r="H53" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A51), "", '📦 商品出厂底价库 (Products)'!P51)</f>
+      </c>
+      <c r="I53" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A51), "", '📦 商品出厂底价库 (Products)'!J51)</f>
+      </c>
+    </row>
+    <row r="54" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A52), "", 51)</f>
+      </c>
+      <c r="B54" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A52), "", '📦 商品出厂底价库 (Products)'!A52)</f>
+      </c>
+      <c r="C54" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A52), "", '📦 商品出厂底价库 (Products)'!C52)</f>
+      </c>
+      <c r="D54" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A52), "", '📦 商品出厂底价库 (Products)'!E52)</f>
+      </c>
+      <c r="E54" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A52), "", '📦 商品出厂底价库 (Products)'!N52)</f>
+      </c>
+      <c r="F54" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A52), "", '📦 商品出厂底价库 (Products)'!F52)</f>
+      </c>
+      <c r="G54" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A52), "", '📦 商品出厂底价库 (Products)'!O52)</f>
+      </c>
+      <c r="H54" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A52), "", '📦 商品出厂底价库 (Products)'!P52)</f>
+      </c>
+      <c r="I54" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A52), "", '📦 商品出厂底价库 (Products)'!J52)</f>
+      </c>
+    </row>
+    <row r="55" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A53), "", 52)</f>
+      </c>
+      <c r="B55" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A53), "", '📦 商品出厂底价库 (Products)'!A53)</f>
+      </c>
+      <c r="C55" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A53), "", '📦 商品出厂底价库 (Products)'!C53)</f>
+      </c>
+      <c r="D55" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A53), "", '📦 商品出厂底价库 (Products)'!E53)</f>
+      </c>
+      <c r="E55" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A53), "", '📦 商品出厂底价库 (Products)'!N53)</f>
+      </c>
+      <c r="F55" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A53), "", '📦 商品出厂底价库 (Products)'!F53)</f>
+      </c>
+      <c r="G55" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A53), "", '📦 商品出厂底价库 (Products)'!O53)</f>
+      </c>
+      <c r="H55" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A53), "", '📦 商品出厂底价库 (Products)'!P53)</f>
+      </c>
+      <c r="I55" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A53), "", '📦 商品出厂底价库 (Products)'!J53)</f>
+      </c>
+    </row>
+    <row r="56" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A54), "", 53)</f>
+      </c>
+      <c r="B56" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A54), "", '📦 商品出厂底价库 (Products)'!A54)</f>
+      </c>
+      <c r="C56" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A54), "", '📦 商品出厂底价库 (Products)'!C54)</f>
+      </c>
+      <c r="D56" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A54), "", '📦 商品出厂底价库 (Products)'!E54)</f>
+      </c>
+      <c r="E56" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A54), "", '📦 商品出厂底价库 (Products)'!N54)</f>
+      </c>
+      <c r="F56" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A54), "", '📦 商品出厂底价库 (Products)'!F54)</f>
+      </c>
+      <c r="G56" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A54), "", '📦 商品出厂底价库 (Products)'!O54)</f>
+      </c>
+      <c r="H56" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A54), "", '📦 商品出厂底价库 (Products)'!P54)</f>
+      </c>
+      <c r="I56" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A54), "", '📦 商品出厂底价库 (Products)'!J54)</f>
+      </c>
+    </row>
+    <row r="57" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A55), "", 54)</f>
+      </c>
+      <c r="B57" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A55), "", '📦 商品出厂底价库 (Products)'!A55)</f>
+      </c>
+      <c r="C57" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A55), "", '📦 商品出厂底价库 (Products)'!C55)</f>
+      </c>
+      <c r="D57" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A55), "", '📦 商品出厂底价库 (Products)'!E55)</f>
+      </c>
+      <c r="E57" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A55), "", '📦 商品出厂底价库 (Products)'!N55)</f>
+      </c>
+      <c r="F57" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A55), "", '📦 商品出厂底价库 (Products)'!F55)</f>
+      </c>
+      <c r="G57" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A55), "", '📦 商品出厂底价库 (Products)'!O55)</f>
+      </c>
+      <c r="H57" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A55), "", '📦 商品出厂底价库 (Products)'!P55)</f>
+      </c>
+      <c r="I57" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A55), "", '📦 商品出厂底价库 (Products)'!J55)</f>
+      </c>
+    </row>
+    <row r="58" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A56), "", 55)</f>
+      </c>
+      <c r="B58" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A56), "", '📦 商品出厂底价库 (Products)'!A56)</f>
+      </c>
+      <c r="C58" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A56), "", '📦 商品出厂底价库 (Products)'!C56)</f>
+      </c>
+      <c r="D58" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A56), "", '📦 商品出厂底价库 (Products)'!E56)</f>
+      </c>
+      <c r="E58" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A56), "", '📦 商品出厂底价库 (Products)'!N56)</f>
+      </c>
+      <c r="F58" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A56), "", '📦 商品出厂底价库 (Products)'!F56)</f>
+      </c>
+      <c r="G58" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A56), "", '📦 商品出厂底价库 (Products)'!O56)</f>
+      </c>
+      <c r="H58" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A56), "", '📦 商品出厂底价库 (Products)'!P56)</f>
+      </c>
+      <c r="I58" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A56), "", '📦 商品出厂底价库 (Products)'!J56)</f>
+      </c>
+    </row>
+    <row r="59" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A57), "", 56)</f>
+      </c>
+      <c r="B59" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A57), "", '📦 商品出厂底价库 (Products)'!A57)</f>
+      </c>
+      <c r="C59" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A57), "", '📦 商品出厂底价库 (Products)'!C57)</f>
+      </c>
+      <c r="D59" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A57), "", '📦 商品出厂底价库 (Products)'!E57)</f>
+      </c>
+      <c r="E59" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A57), "", '📦 商品出厂底价库 (Products)'!N57)</f>
+      </c>
+      <c r="F59" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A57), "", '📦 商品出厂底价库 (Products)'!F57)</f>
+      </c>
+      <c r="G59" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A57), "", '📦 商品出厂底价库 (Products)'!O57)</f>
+      </c>
+      <c r="H59" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A57), "", '📦 商品出厂底价库 (Products)'!P57)</f>
+      </c>
+      <c r="I59" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A57), "", '📦 商品出厂底价库 (Products)'!J57)</f>
+      </c>
+    </row>
+    <row r="60" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A58), "", 57)</f>
+      </c>
+      <c r="B60" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A58), "", '📦 商品出厂底价库 (Products)'!A58)</f>
+      </c>
+      <c r="C60" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A58), "", '📦 商品出厂底价库 (Products)'!C58)</f>
+      </c>
+      <c r="D60" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A58), "", '📦 商品出厂底价库 (Products)'!E58)</f>
+      </c>
+      <c r="E60" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A58), "", '📦 商品出厂底价库 (Products)'!N58)</f>
+      </c>
+      <c r="F60" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A58), "", '📦 商品出厂底价库 (Products)'!F58)</f>
+      </c>
+      <c r="G60" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A58), "", '📦 商品出厂底价库 (Products)'!O58)</f>
+      </c>
+      <c r="H60" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A58), "", '📦 商品出厂底价库 (Products)'!P58)</f>
+      </c>
+      <c r="I60" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A58), "", '📦 商品出厂底价库 (Products)'!J58)</f>
+      </c>
+    </row>
+    <row r="61" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A59), "", 58)</f>
+      </c>
+      <c r="B61" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A59), "", '📦 商品出厂底价库 (Products)'!A59)</f>
+      </c>
+      <c r="C61" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A59), "", '📦 商品出厂底价库 (Products)'!C59)</f>
+      </c>
+      <c r="D61" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A59), "", '📦 商品出厂底价库 (Products)'!E59)</f>
+      </c>
+      <c r="E61" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A59), "", '📦 商品出厂底价库 (Products)'!N59)</f>
+      </c>
+      <c r="F61" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A59), "", '📦 商品出厂底价库 (Products)'!F59)</f>
+      </c>
+      <c r="G61" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A59), "", '📦 商品出厂底价库 (Products)'!O59)</f>
+      </c>
+      <c r="H61" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A59), "", '📦 商品出厂底价库 (Products)'!P59)</f>
+      </c>
+      <c r="I61" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A59), "", '📦 商品出厂底价库 (Products)'!J59)</f>
+      </c>
+    </row>
+    <row r="62" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A60), "", 59)</f>
+      </c>
+      <c r="B62" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A60), "", '📦 商品出厂底价库 (Products)'!A60)</f>
+      </c>
+      <c r="C62" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A60), "", '📦 商品出厂底价库 (Products)'!C60)</f>
+      </c>
+      <c r="D62" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A60), "", '📦 商品出厂底价库 (Products)'!E60)</f>
+      </c>
+      <c r="E62" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A60), "", '📦 商品出厂底价库 (Products)'!N60)</f>
+      </c>
+      <c r="F62" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A60), "", '📦 商品出厂底价库 (Products)'!F60)</f>
+      </c>
+      <c r="G62" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A60), "", '📦 商品出厂底价库 (Products)'!O60)</f>
+      </c>
+      <c r="H62" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A60), "", '📦 商品出厂底价库 (Products)'!P60)</f>
+      </c>
+      <c r="I62" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A60), "", '📦 商品出厂底价库 (Products)'!J60)</f>
+      </c>
+    </row>
+    <row r="63" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A61), "", 60)</f>
+      </c>
+      <c r="B63" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A61), "", '📦 商品出厂底价库 (Products)'!A61)</f>
+      </c>
+      <c r="C63" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A61), "", '📦 商品出厂底价库 (Products)'!C61)</f>
+      </c>
+      <c r="D63" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A61), "", '📦 商品出厂底价库 (Products)'!E61)</f>
+      </c>
+      <c r="E63" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A61), "", '📦 商品出厂底价库 (Products)'!N61)</f>
+      </c>
+      <c r="F63" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A61), "", '📦 商品出厂底价库 (Products)'!F61)</f>
+      </c>
+      <c r="G63" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A61), "", '📦 商品出厂底价库 (Products)'!O61)</f>
+      </c>
+      <c r="H63" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A61), "", '📦 商品出厂底价库 (Products)'!P61)</f>
+      </c>
+      <c r="I63" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A61), "", '📦 商品出厂底价库 (Products)'!J61)</f>
+      </c>
+    </row>
+    <row r="64" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A62), "", 61)</f>
+      </c>
+      <c r="B64" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A62), "", '📦 商品出厂底价库 (Products)'!A62)</f>
+      </c>
+      <c r="C64" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A62), "", '📦 商品出厂底价库 (Products)'!C62)</f>
+      </c>
+      <c r="D64" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A62), "", '📦 商品出厂底价库 (Products)'!E62)</f>
+      </c>
+      <c r="E64" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A62), "", '📦 商品出厂底价库 (Products)'!N62)</f>
+      </c>
+      <c r="F64" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A62), "", '📦 商品出厂底价库 (Products)'!F62)</f>
+      </c>
+      <c r="G64" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A62), "", '📦 商品出厂底价库 (Products)'!O62)</f>
+      </c>
+      <c r="H64" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A62), "", '📦 商品出厂底价库 (Products)'!P62)</f>
+      </c>
+      <c r="I64" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A62), "", '📦 商品出厂底价库 (Products)'!J62)</f>
+      </c>
+    </row>
+    <row r="65" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A63), "", 62)</f>
+      </c>
+      <c r="B65" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A63), "", '📦 商品出厂底价库 (Products)'!A63)</f>
+      </c>
+      <c r="C65" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A63), "", '📦 商品出厂底价库 (Products)'!C63)</f>
+      </c>
+      <c r="D65" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A63), "", '📦 商品出厂底价库 (Products)'!E63)</f>
+      </c>
+      <c r="E65" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A63), "", '📦 商品出厂底价库 (Products)'!N63)</f>
+      </c>
+      <c r="F65" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A63), "", '📦 商品出厂底价库 (Products)'!F63)</f>
+      </c>
+      <c r="G65" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A63), "", '📦 商品出厂底价库 (Products)'!O63)</f>
+      </c>
+      <c r="H65" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A63), "", '📦 商品出厂底价库 (Products)'!P63)</f>
+      </c>
+      <c r="I65" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A63), "", '📦 商品出厂底价库 (Products)'!J63)</f>
+      </c>
+    </row>
+    <row r="66" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A64), "", 63)</f>
+      </c>
+      <c r="B66" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A64), "", '📦 商品出厂底价库 (Products)'!A64)</f>
+      </c>
+      <c r="C66" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A64), "", '📦 商品出厂底价库 (Products)'!C64)</f>
+      </c>
+      <c r="D66" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A64), "", '📦 商品出厂底价库 (Products)'!E64)</f>
+      </c>
+      <c r="E66" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A64), "", '📦 商品出厂底价库 (Products)'!N64)</f>
+      </c>
+      <c r="F66" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A64), "", '📦 商品出厂底价库 (Products)'!F64)</f>
+      </c>
+      <c r="G66" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A64), "", '📦 商品出厂底价库 (Products)'!O64)</f>
+      </c>
+      <c r="H66" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A64), "", '📦 商品出厂底价库 (Products)'!P64)</f>
+      </c>
+      <c r="I66" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A64), "", '📦 商品出厂底价库 (Products)'!J64)</f>
+      </c>
+    </row>
+    <row r="67" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A67" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A65), "", 64)</f>
+      </c>
+      <c r="B67" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A65), "", '📦 商品出厂底价库 (Products)'!A65)</f>
+      </c>
+      <c r="C67" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A65), "", '📦 商品出厂底价库 (Products)'!C65)</f>
+      </c>
+      <c r="D67" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A65), "", '📦 商品出厂底价库 (Products)'!E65)</f>
+      </c>
+      <c r="E67" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A65), "", '📦 商品出厂底价库 (Products)'!N65)</f>
+      </c>
+      <c r="F67" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A65), "", '📦 商品出厂底价库 (Products)'!F65)</f>
+      </c>
+      <c r="G67" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A65), "", '📦 商品出厂底价库 (Products)'!O65)</f>
+      </c>
+      <c r="H67" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A65), "", '📦 商品出厂底价库 (Products)'!P65)</f>
+      </c>
+      <c r="I67" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A65), "", '📦 商品出厂底价库 (Products)'!J65)</f>
+      </c>
+    </row>
+    <row r="68" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A66), "", 65)</f>
+      </c>
+      <c r="B68" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A66), "", '📦 商品出厂底价库 (Products)'!A66)</f>
+      </c>
+      <c r="C68" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A66), "", '📦 商品出厂底价库 (Products)'!C66)</f>
+      </c>
+      <c r="D68" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A66), "", '📦 商品出厂底价库 (Products)'!E66)</f>
+      </c>
+      <c r="E68" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A66), "", '📦 商品出厂底价库 (Products)'!N66)</f>
+      </c>
+      <c r="F68" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A66), "", '📦 商品出厂底价库 (Products)'!F66)</f>
+      </c>
+      <c r="G68" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A66), "", '📦 商品出厂底价库 (Products)'!O66)</f>
+      </c>
+      <c r="H68" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A66), "", '📦 商品出厂底价库 (Products)'!P66)</f>
+      </c>
+      <c r="I68" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A66), "", '📦 商品出厂底价库 (Products)'!J66)</f>
+      </c>
+    </row>
+    <row r="69" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A67), "", 66)</f>
+      </c>
+      <c r="B69" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A67), "", '📦 商品出厂底价库 (Products)'!A67)</f>
+      </c>
+      <c r="C69" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A67), "", '📦 商品出厂底价库 (Products)'!C67)</f>
+      </c>
+      <c r="D69" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A67), "", '📦 商品出厂底价库 (Products)'!E67)</f>
+      </c>
+      <c r="E69" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A67), "", '📦 商品出厂底价库 (Products)'!N67)</f>
+      </c>
+      <c r="F69" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A67), "", '📦 商品出厂底价库 (Products)'!F67)</f>
+      </c>
+      <c r="G69" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A67), "", '📦 商品出厂底价库 (Products)'!O67)</f>
+      </c>
+      <c r="H69" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A67), "", '📦 商品出厂底价库 (Products)'!P67)</f>
+      </c>
+      <c r="I69" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A67), "", '📦 商品出厂底价库 (Products)'!J67)</f>
+      </c>
+    </row>
+    <row r="70" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A68), "", 67)</f>
+      </c>
+      <c r="B70" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A68), "", '📦 商品出厂底价库 (Products)'!A68)</f>
+      </c>
+      <c r="C70" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A68), "", '📦 商品出厂底价库 (Products)'!C68)</f>
+      </c>
+      <c r="D70" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A68), "", '📦 商品出厂底价库 (Products)'!E68)</f>
+      </c>
+      <c r="E70" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A68), "", '📦 商品出厂底价库 (Products)'!N68)</f>
+      </c>
+      <c r="F70" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A68), "", '📦 商品出厂底价库 (Products)'!F68)</f>
+      </c>
+      <c r="G70" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A68), "", '📦 商品出厂底价库 (Products)'!O68)</f>
+      </c>
+      <c r="H70" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A68), "", '📦 商品出厂底价库 (Products)'!P68)</f>
+      </c>
+      <c r="I70" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A68), "", '📦 商品出厂底价库 (Products)'!J68)</f>
+      </c>
+    </row>
+    <row r="71" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A71" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A69), "", 68)</f>
+      </c>
+      <c r="B71" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A69), "", '📦 商品出厂底价库 (Products)'!A69)</f>
+      </c>
+      <c r="C71" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A69), "", '📦 商品出厂底价库 (Products)'!C69)</f>
+      </c>
+      <c r="D71" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A69), "", '📦 商品出厂底价库 (Products)'!E69)</f>
+      </c>
+      <c r="E71" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A69), "", '📦 商品出厂底价库 (Products)'!N69)</f>
+      </c>
+      <c r="F71" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A69), "", '📦 商品出厂底价库 (Products)'!F69)</f>
+      </c>
+      <c r="G71" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A69), "", '📦 商品出厂底价库 (Products)'!O69)</f>
+      </c>
+      <c r="H71" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A69), "", '📦 商品出厂底价库 (Products)'!P69)</f>
+      </c>
+      <c r="I71" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A69), "", '📦 商品出厂底价库 (Products)'!J69)</f>
+      </c>
+    </row>
+    <row r="72" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A70), "", 69)</f>
+      </c>
+      <c r="B72" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A70), "", '📦 商品出厂底价库 (Products)'!A70)</f>
+      </c>
+      <c r="C72" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A70), "", '📦 商品出厂底价库 (Products)'!C70)</f>
+      </c>
+      <c r="D72" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A70), "", '📦 商品出厂底价库 (Products)'!E70)</f>
+      </c>
+      <c r="E72" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A70), "", '📦 商品出厂底价库 (Products)'!N70)</f>
+      </c>
+      <c r="F72" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A70), "", '📦 商品出厂底价库 (Products)'!F70)</f>
+      </c>
+      <c r="G72" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A70), "", '📦 商品出厂底价库 (Products)'!O70)</f>
+      </c>
+      <c r="H72" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A70), "", '📦 商品出厂底价库 (Products)'!P70)</f>
+      </c>
+      <c r="I72" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A70), "", '📦 商品出厂底价库 (Products)'!J70)</f>
+      </c>
+    </row>
+    <row r="73" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A73" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A71), "", 70)</f>
+      </c>
+      <c r="B73" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A71), "", '📦 商品出厂底价库 (Products)'!A71)</f>
+      </c>
+      <c r="C73" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A71), "", '📦 商品出厂底价库 (Products)'!C71)</f>
+      </c>
+      <c r="D73" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A71), "", '📦 商品出厂底价库 (Products)'!E71)</f>
+      </c>
+      <c r="E73" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A71), "", '📦 商品出厂底价库 (Products)'!N71)</f>
+      </c>
+      <c r="F73" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A71), "", '📦 商品出厂底价库 (Products)'!F71)</f>
+      </c>
+      <c r="G73" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A71), "", '📦 商品出厂底价库 (Products)'!O71)</f>
+      </c>
+      <c r="H73" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A71), "", '📦 商品出厂底价库 (Products)'!P71)</f>
+      </c>
+      <c r="I73" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A71), "", '📦 商品出厂底价库 (Products)'!J71)</f>
+      </c>
+    </row>
+    <row r="74" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A74" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A72), "", 71)</f>
+      </c>
+      <c r="B74" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A72), "", '📦 商品出厂底价库 (Products)'!A72)</f>
+      </c>
+      <c r="C74" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A72), "", '📦 商品出厂底价库 (Products)'!C72)</f>
+      </c>
+      <c r="D74" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A72), "", '📦 商品出厂底价库 (Products)'!E72)</f>
+      </c>
+      <c r="E74" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A72), "", '📦 商品出厂底价库 (Products)'!N72)</f>
+      </c>
+      <c r="F74" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A72), "", '📦 商品出厂底价库 (Products)'!F72)</f>
+      </c>
+      <c r="G74" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A72), "", '📦 商品出厂底价库 (Products)'!O72)</f>
+      </c>
+      <c r="H74" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A72), "", '📦 商品出厂底价库 (Products)'!P72)</f>
+      </c>
+      <c r="I74" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A72), "", '📦 商品出厂底价库 (Products)'!J72)</f>
+      </c>
+    </row>
+    <row r="75" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A75" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A73), "", 72)</f>
+      </c>
+      <c r="B75" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A73), "", '📦 商品出厂底价库 (Products)'!A73)</f>
+      </c>
+      <c r="C75" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A73), "", '📦 商品出厂底价库 (Products)'!C73)</f>
+      </c>
+      <c r="D75" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A73), "", '📦 商品出厂底价库 (Products)'!E73)</f>
+      </c>
+      <c r="E75" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A73), "", '📦 商品出厂底价库 (Products)'!N73)</f>
+      </c>
+      <c r="F75" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A73), "", '📦 商品出厂底价库 (Products)'!F73)</f>
+      </c>
+      <c r="G75" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A73), "", '📦 商品出厂底价库 (Products)'!O73)</f>
+      </c>
+      <c r="H75" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A73), "", '📦 商品出厂底价库 (Products)'!P73)</f>
+      </c>
+      <c r="I75" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A73), "", '📦 商品出厂底价库 (Products)'!J73)</f>
+      </c>
+    </row>
+    <row r="76" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A76" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A74), "", 73)</f>
+      </c>
+      <c r="B76" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A74), "", '📦 商品出厂底价库 (Products)'!A74)</f>
+      </c>
+      <c r="C76" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A74), "", '📦 商品出厂底价库 (Products)'!C74)</f>
+      </c>
+      <c r="D76" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A74), "", '📦 商品出厂底价库 (Products)'!E74)</f>
+      </c>
+      <c r="E76" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A74), "", '📦 商品出厂底价库 (Products)'!N74)</f>
+      </c>
+      <c r="F76" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A74), "", '📦 商品出厂底价库 (Products)'!F74)</f>
+      </c>
+      <c r="G76" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A74), "", '📦 商品出厂底价库 (Products)'!O74)</f>
+      </c>
+      <c r="H76" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A74), "", '📦 商品出厂底价库 (Products)'!P74)</f>
+      </c>
+      <c r="I76" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A74), "", '📦 商品出厂底价库 (Products)'!J74)</f>
+      </c>
+    </row>
+    <row r="77" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A77" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A75), "", 74)</f>
+      </c>
+      <c r="B77" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A75), "", '📦 商品出厂底价库 (Products)'!A75)</f>
+      </c>
+      <c r="C77" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A75), "", '📦 商品出厂底价库 (Products)'!C75)</f>
+      </c>
+      <c r="D77" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A75), "", '📦 商品出厂底价库 (Products)'!E75)</f>
+      </c>
+      <c r="E77" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A75), "", '📦 商品出厂底价库 (Products)'!N75)</f>
+      </c>
+      <c r="F77" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A75), "", '📦 商品出厂底价库 (Products)'!F75)</f>
+      </c>
+      <c r="G77" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A75), "", '📦 商品出厂底价库 (Products)'!O75)</f>
+      </c>
+      <c r="H77" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A75), "", '📦 商品出厂底价库 (Products)'!P75)</f>
+      </c>
+      <c r="I77" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A75), "", '📦 商品出厂底价库 (Products)'!J75)</f>
+      </c>
+    </row>
+    <row r="78" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A78" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A76), "", 75)</f>
+      </c>
+      <c r="B78" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A76), "", '📦 商品出厂底价库 (Products)'!A76)</f>
+      </c>
+      <c r="C78" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A76), "", '📦 商品出厂底价库 (Products)'!C76)</f>
+      </c>
+      <c r="D78" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A76), "", '📦 商品出厂底价库 (Products)'!E76)</f>
+      </c>
+      <c r="E78" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A76), "", '📦 商品出厂底价库 (Products)'!N76)</f>
+      </c>
+      <c r="F78" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A76), "", '📦 商品出厂底价库 (Products)'!F76)</f>
+      </c>
+      <c r="G78" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A76), "", '📦 商品出厂底价库 (Products)'!O76)</f>
+      </c>
+      <c r="H78" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A76), "", '📦 商品出厂底价库 (Products)'!P76)</f>
+      </c>
+      <c r="I78" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A76), "", '📦 商品出厂底价库 (Products)'!J76)</f>
+      </c>
+    </row>
+    <row r="79" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A79" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A77), "", 76)</f>
+      </c>
+      <c r="B79" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A77), "", '📦 商品出厂底价库 (Products)'!A77)</f>
+      </c>
+      <c r="C79" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A77), "", '📦 商品出厂底价库 (Products)'!C77)</f>
+      </c>
+      <c r="D79" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A77), "", '📦 商品出厂底价库 (Products)'!E77)</f>
+      </c>
+      <c r="E79" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A77), "", '📦 商品出厂底价库 (Products)'!N77)</f>
+      </c>
+      <c r="F79" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A77), "", '📦 商品出厂底价库 (Products)'!F77)</f>
+      </c>
+      <c r="G79" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A77), "", '📦 商品出厂底价库 (Products)'!O77)</f>
+      </c>
+      <c r="H79" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A77), "", '📦 商品出厂底价库 (Products)'!P77)</f>
+      </c>
+      <c r="I79" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A77), "", '📦 商品出厂底价库 (Products)'!J77)</f>
+      </c>
+    </row>
+    <row r="80" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A80" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A78), "", 77)</f>
+      </c>
+      <c r="B80" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A78), "", '📦 商品出厂底价库 (Products)'!A78)</f>
+      </c>
+      <c r="C80" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A78), "", '📦 商品出厂底价库 (Products)'!C78)</f>
+      </c>
+      <c r="D80" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A78), "", '📦 商品出厂底价库 (Products)'!E78)</f>
+      </c>
+      <c r="E80" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A78), "", '📦 商品出厂底价库 (Products)'!N78)</f>
+      </c>
+      <c r="F80" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A78), "", '📦 商品出厂底价库 (Products)'!F78)</f>
+      </c>
+      <c r="G80" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A78), "", '📦 商品出厂底价库 (Products)'!O78)</f>
+      </c>
+      <c r="H80" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A78), "", '📦 商品出厂底价库 (Products)'!P78)</f>
+      </c>
+      <c r="I80" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A78), "", '📦 商品出厂底价库 (Products)'!J78)</f>
+      </c>
+    </row>
+    <row r="81" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A81" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A79), "", 78)</f>
+      </c>
+      <c r="B81" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A79), "", '📦 商品出厂底价库 (Products)'!A79)</f>
+      </c>
+      <c r="C81" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A79), "", '📦 商品出厂底价库 (Products)'!C79)</f>
+      </c>
+      <c r="D81" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A79), "", '📦 商品出厂底价库 (Products)'!E79)</f>
+      </c>
+      <c r="E81" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A79), "", '📦 商品出厂底价库 (Products)'!N79)</f>
+      </c>
+      <c r="F81" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A79), "", '📦 商品出厂底价库 (Products)'!F79)</f>
+      </c>
+      <c r="G81" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A79), "", '📦 商品出厂底价库 (Products)'!O79)</f>
+      </c>
+      <c r="H81" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A79), "", '📦 商品出厂底价库 (Products)'!P79)</f>
+      </c>
+      <c r="I81" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A79), "", '📦 商品出厂底价库 (Products)'!J79)</f>
+      </c>
+    </row>
+    <row r="82" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A82" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A80), "", 79)</f>
+      </c>
+      <c r="B82" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A80), "", '📦 商品出厂底价库 (Products)'!A80)</f>
+      </c>
+      <c r="C82" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A80), "", '📦 商品出厂底价库 (Products)'!C80)</f>
+      </c>
+      <c r="D82" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A80), "", '📦 商品出厂底价库 (Products)'!E80)</f>
+      </c>
+      <c r="E82" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A80), "", '📦 商品出厂底价库 (Products)'!N80)</f>
+      </c>
+      <c r="F82" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A80), "", '📦 商品出厂底价库 (Products)'!F80)</f>
+      </c>
+      <c r="G82" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A80), "", '📦 商品出厂底价库 (Products)'!O80)</f>
+      </c>
+      <c r="H82" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A80), "", '📦 商品出厂底价库 (Products)'!P80)</f>
+      </c>
+      <c r="I82" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A80), "", '📦 商品出厂底价库 (Products)'!J80)</f>
+      </c>
+    </row>
+    <row r="83" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A83" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A81), "", 80)</f>
+      </c>
+      <c r="B83" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A81), "", '📦 商品出厂底价库 (Products)'!A81)</f>
+      </c>
+      <c r="C83" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A81), "", '📦 商品出厂底价库 (Products)'!C81)</f>
+      </c>
+      <c r="D83" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A81), "", '📦 商品出厂底价库 (Products)'!E81)</f>
+      </c>
+      <c r="E83" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A81), "", '📦 商品出厂底价库 (Products)'!N81)</f>
+      </c>
+      <c r="F83" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A81), "", '📦 商品出厂底价库 (Products)'!F81)</f>
+      </c>
+      <c r="G83" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A81), "", '📦 商品出厂底价库 (Products)'!O81)</f>
+      </c>
+      <c r="H83" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A81), "", '📦 商品出厂底价库 (Products)'!P81)</f>
+      </c>
+      <c r="I83" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A81), "", '📦 商品出厂底价库 (Products)'!J81)</f>
+      </c>
+    </row>
+    <row r="84" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A84" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A82), "", 81)</f>
+      </c>
+      <c r="B84" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A82), "", '📦 商品出厂底价库 (Products)'!A82)</f>
+      </c>
+      <c r="C84" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A82), "", '📦 商品出厂底价库 (Products)'!C82)</f>
+      </c>
+      <c r="D84" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A82), "", '📦 商品出厂底价库 (Products)'!E82)</f>
+      </c>
+      <c r="E84" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A82), "", '📦 商品出厂底价库 (Products)'!N82)</f>
+      </c>
+      <c r="F84" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A82), "", '📦 商品出厂底价库 (Products)'!F82)</f>
+      </c>
+      <c r="G84" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A82), "", '📦 商品出厂底价库 (Products)'!O82)</f>
+      </c>
+      <c r="H84" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A82), "", '📦 商品出厂底价库 (Products)'!P82)</f>
+      </c>
+      <c r="I84" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A82), "", '📦 商品出厂底价库 (Products)'!J82)</f>
+      </c>
+    </row>
+    <row r="85" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A85" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A83), "", 82)</f>
+      </c>
+      <c r="B85" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A83), "", '📦 商品出厂底价库 (Products)'!A83)</f>
+      </c>
+      <c r="C85" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A83), "", '📦 商品出厂底价库 (Products)'!C83)</f>
+      </c>
+      <c r="D85" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A83), "", '📦 商品出厂底价库 (Products)'!E83)</f>
+      </c>
+      <c r="E85" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A83), "", '📦 商品出厂底价库 (Products)'!N83)</f>
+      </c>
+      <c r="F85" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A83), "", '📦 商品出厂底价库 (Products)'!F83)</f>
+      </c>
+      <c r="G85" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A83), "", '📦 商品出厂底价库 (Products)'!O83)</f>
+      </c>
+      <c r="H85" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A83), "", '📦 商品出厂底价库 (Products)'!P83)</f>
+      </c>
+      <c r="I85" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A83), "", '📦 商品出厂底价库 (Products)'!J83)</f>
+      </c>
+    </row>
+    <row r="86" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A84), "", 83)</f>
+      </c>
+      <c r="B86" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A84), "", '📦 商品出厂底价库 (Products)'!A84)</f>
+      </c>
+      <c r="C86" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A84), "", '📦 商品出厂底价库 (Products)'!C84)</f>
+      </c>
+      <c r="D86" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A84), "", '📦 商品出厂底价库 (Products)'!E84)</f>
+      </c>
+      <c r="E86" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A84), "", '📦 商品出厂底价库 (Products)'!N84)</f>
+      </c>
+      <c r="F86" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A84), "", '📦 商品出厂底价库 (Products)'!F84)</f>
+      </c>
+      <c r="G86" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A84), "", '📦 商品出厂底价库 (Products)'!O84)</f>
+      </c>
+      <c r="H86" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A84), "", '📦 商品出厂底价库 (Products)'!P84)</f>
+      </c>
+      <c r="I86" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A84), "", '📦 商品出厂底价库 (Products)'!J84)</f>
+      </c>
+    </row>
+    <row r="87" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A85), "", 84)</f>
+      </c>
+      <c r="B87" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A85), "", '📦 商品出厂底价库 (Products)'!A85)</f>
+      </c>
+      <c r="C87" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A85), "", '📦 商品出厂底价库 (Products)'!C85)</f>
+      </c>
+      <c r="D87" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A85), "", '📦 商品出厂底价库 (Products)'!E85)</f>
+      </c>
+      <c r="E87" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A85), "", '📦 商品出厂底价库 (Products)'!N85)</f>
+      </c>
+      <c r="F87" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A85), "", '📦 商品出厂底价库 (Products)'!F85)</f>
+      </c>
+      <c r="G87" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A85), "", '📦 商品出厂底价库 (Products)'!O85)</f>
+      </c>
+      <c r="H87" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A85), "", '📦 商品出厂底价库 (Products)'!P85)</f>
+      </c>
+      <c r="I87" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A85), "", '📦 商品出厂底价库 (Products)'!J85)</f>
+      </c>
+    </row>
+    <row r="88" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A86), "", 85)</f>
+      </c>
+      <c r="B88" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A86), "", '📦 商品出厂底价库 (Products)'!A86)</f>
+      </c>
+      <c r="C88" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A86), "", '📦 商品出厂底价库 (Products)'!C86)</f>
+      </c>
+      <c r="D88" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A86), "", '📦 商品出厂底价库 (Products)'!E86)</f>
+      </c>
+      <c r="E88" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A86), "", '📦 商品出厂底价库 (Products)'!N86)</f>
+      </c>
+      <c r="F88" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A86), "", '📦 商品出厂底价库 (Products)'!F86)</f>
+      </c>
+      <c r="G88" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A86), "", '📦 商品出厂底价库 (Products)'!O86)</f>
+      </c>
+      <c r="H88" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A86), "", '📦 商品出厂底价库 (Products)'!P86)</f>
+      </c>
+      <c r="I88" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A86), "", '📦 商品出厂底价库 (Products)'!J86)</f>
+      </c>
+    </row>
+    <row r="89" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A87), "", 86)</f>
+      </c>
+      <c r="B89" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A87), "", '📦 商品出厂底价库 (Products)'!A87)</f>
+      </c>
+      <c r="C89" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A87), "", '📦 商品出厂底价库 (Products)'!C87)</f>
+      </c>
+      <c r="D89" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A87), "", '📦 商品出厂底价库 (Products)'!E87)</f>
+      </c>
+      <c r="E89" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A87), "", '📦 商品出厂底价库 (Products)'!N87)</f>
+      </c>
+      <c r="F89" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A87), "", '📦 商品出厂底价库 (Products)'!F87)</f>
+      </c>
+      <c r="G89" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A87), "", '📦 商品出厂底价库 (Products)'!O87)</f>
+      </c>
+      <c r="H89" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A87), "", '📦 商品出厂底价库 (Products)'!P87)</f>
+      </c>
+      <c r="I89" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A87), "", '📦 商品出厂底价库 (Products)'!J87)</f>
+      </c>
+    </row>
+    <row r="90" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A88), "", 87)</f>
+      </c>
+      <c r="B90" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A88), "", '📦 商品出厂底价库 (Products)'!A88)</f>
+      </c>
+      <c r="C90" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A88), "", '📦 商品出厂底价库 (Products)'!C88)</f>
+      </c>
+      <c r="D90" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A88), "", '📦 商品出厂底价库 (Products)'!E88)</f>
+      </c>
+      <c r="E90" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A88), "", '📦 商品出厂底价库 (Products)'!N88)</f>
+      </c>
+      <c r="F90" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A88), "", '📦 商品出厂底价库 (Products)'!F88)</f>
+      </c>
+      <c r="G90" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A88), "", '📦 商品出厂底价库 (Products)'!O88)</f>
+      </c>
+      <c r="H90" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A88), "", '📦 商品出厂底价库 (Products)'!P88)</f>
+      </c>
+      <c r="I90" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A88), "", '📦 商品出厂底价库 (Products)'!J88)</f>
+      </c>
+    </row>
+    <row r="91" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A91" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A89), "", 88)</f>
+      </c>
+      <c r="B91" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A89), "", '📦 商品出厂底价库 (Products)'!A89)</f>
+      </c>
+      <c r="C91" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A89), "", '📦 商品出厂底价库 (Products)'!C89)</f>
+      </c>
+      <c r="D91" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A89), "", '📦 商品出厂底价库 (Products)'!E89)</f>
+      </c>
+      <c r="E91" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A89), "", '📦 商品出厂底价库 (Products)'!N89)</f>
+      </c>
+      <c r="F91" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A89), "", '📦 商品出厂底价库 (Products)'!F89)</f>
+      </c>
+      <c r="G91" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A89), "", '📦 商品出厂底价库 (Products)'!O89)</f>
+      </c>
+      <c r="H91" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A89), "", '📦 商品出厂底价库 (Products)'!P89)</f>
+      </c>
+      <c r="I91" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A89), "", '📦 商品出厂底价库 (Products)'!J89)</f>
+      </c>
+    </row>
+    <row r="92" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A92" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A90), "", 89)</f>
+      </c>
+      <c r="B92" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A90), "", '📦 商品出厂底价库 (Products)'!A90)</f>
+      </c>
+      <c r="C92" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A90), "", '📦 商品出厂底价库 (Products)'!C90)</f>
+      </c>
+      <c r="D92" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A90), "", '📦 商品出厂底价库 (Products)'!E90)</f>
+      </c>
+      <c r="E92" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A90), "", '📦 商品出厂底价库 (Products)'!N90)</f>
+      </c>
+      <c r="F92" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A90), "", '📦 商品出厂底价库 (Products)'!F90)</f>
+      </c>
+      <c r="G92" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A90), "", '📦 商品出厂底价库 (Products)'!O90)</f>
+      </c>
+      <c r="H92" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A90), "", '📦 商品出厂底价库 (Products)'!P90)</f>
+      </c>
+      <c r="I92" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A90), "", '📦 商品出厂底价库 (Products)'!J90)</f>
+      </c>
+    </row>
+    <row r="93" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A91), "", 90)</f>
+      </c>
+      <c r="B93" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A91), "", '📦 商品出厂底价库 (Products)'!A91)</f>
+      </c>
+      <c r="C93" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A91), "", '📦 商品出厂底价库 (Products)'!C91)</f>
+      </c>
+      <c r="D93" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A91), "", '📦 商品出厂底价库 (Products)'!E91)</f>
+      </c>
+      <c r="E93" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A91), "", '📦 商品出厂底价库 (Products)'!N91)</f>
+      </c>
+      <c r="F93" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A91), "", '📦 商品出厂底价库 (Products)'!F91)</f>
+      </c>
+      <c r="G93" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A91), "", '📦 商品出厂底价库 (Products)'!O91)</f>
+      </c>
+      <c r="H93" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A91), "", '📦 商品出厂底价库 (Products)'!P91)</f>
+      </c>
+      <c r="I93" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A91), "", '📦 商品出厂底价库 (Products)'!J91)</f>
+      </c>
+    </row>
+    <row r="94" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A92), "", 91)</f>
+      </c>
+      <c r="B94" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A92), "", '📦 商品出厂底价库 (Products)'!A92)</f>
+      </c>
+      <c r="C94" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A92), "", '📦 商品出厂底价库 (Products)'!C92)</f>
+      </c>
+      <c r="D94" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A92), "", '📦 商品出厂底价库 (Products)'!E92)</f>
+      </c>
+      <c r="E94" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A92), "", '📦 商品出厂底价库 (Products)'!N92)</f>
+      </c>
+      <c r="F94" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A92), "", '📦 商品出厂底价库 (Products)'!F92)</f>
+      </c>
+      <c r="G94" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A92), "", '📦 商品出厂底价库 (Products)'!O92)</f>
+      </c>
+      <c r="H94" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A92), "", '📦 商品出厂底价库 (Products)'!P92)</f>
+      </c>
+      <c r="I94" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A92), "", '📦 商品出厂底价库 (Products)'!J92)</f>
+      </c>
+    </row>
+    <row r="95" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A93), "", 92)</f>
+      </c>
+      <c r="B95" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A93), "", '📦 商品出厂底价库 (Products)'!A93)</f>
+      </c>
+      <c r="C95" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A93), "", '📦 商品出厂底价库 (Products)'!C93)</f>
+      </c>
+      <c r="D95" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A93), "", '📦 商品出厂底价库 (Products)'!E93)</f>
+      </c>
+      <c r="E95" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A93), "", '📦 商品出厂底价库 (Products)'!N93)</f>
+      </c>
+      <c r="F95" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A93), "", '📦 商品出厂底价库 (Products)'!F93)</f>
+      </c>
+      <c r="G95" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A93), "", '📦 商品出厂底价库 (Products)'!O93)</f>
+      </c>
+      <c r="H95" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A93), "", '📦 商品出厂底价库 (Products)'!P93)</f>
+      </c>
+      <c r="I95" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A93), "", '📦 商品出厂底价库 (Products)'!J93)</f>
+      </c>
+    </row>
+    <row r="96" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A94), "", 93)</f>
+      </c>
+      <c r="B96" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A94), "", '📦 商品出厂底价库 (Products)'!A94)</f>
+      </c>
+      <c r="C96" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A94), "", '📦 商品出厂底价库 (Products)'!C94)</f>
+      </c>
+      <c r="D96" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A94), "", '📦 商品出厂底价库 (Products)'!E94)</f>
+      </c>
+      <c r="E96" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A94), "", '📦 商品出厂底价库 (Products)'!N94)</f>
+      </c>
+      <c r="F96" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A94), "", '📦 商品出厂底价库 (Products)'!F94)</f>
+      </c>
+      <c r="G96" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A94), "", '📦 商品出厂底价库 (Products)'!O94)</f>
+      </c>
+      <c r="H96" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A94), "", '📦 商品出厂底价库 (Products)'!P94)</f>
+      </c>
+      <c r="I96" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A94), "", '📦 商品出厂底价库 (Products)'!J94)</f>
+      </c>
+    </row>
+    <row r="97" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A95), "", 94)</f>
+      </c>
+      <c r="B97" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A95), "", '📦 商品出厂底价库 (Products)'!A95)</f>
+      </c>
+      <c r="C97" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A95), "", '📦 商品出厂底价库 (Products)'!C95)</f>
+      </c>
+      <c r="D97" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A95), "", '📦 商品出厂底价库 (Products)'!E95)</f>
+      </c>
+      <c r="E97" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A95), "", '📦 商品出厂底价库 (Products)'!N95)</f>
+      </c>
+      <c r="F97" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A95), "", '📦 商品出厂底价库 (Products)'!F95)</f>
+      </c>
+      <c r="G97" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A95), "", '📦 商品出厂底价库 (Products)'!O95)</f>
+      </c>
+      <c r="H97" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A95), "", '📦 商品出厂底价库 (Products)'!P95)</f>
+      </c>
+      <c r="I97" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A95), "", '📦 商品出厂底价库 (Products)'!J95)</f>
+      </c>
+    </row>
+    <row r="98" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A96), "", 95)</f>
+      </c>
+      <c r="B98" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A96), "", '📦 商品出厂底价库 (Products)'!A96)</f>
+      </c>
+      <c r="C98" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A96), "", '📦 商品出厂底价库 (Products)'!C96)</f>
+      </c>
+      <c r="D98" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A96), "", '📦 商品出厂底价库 (Products)'!E96)</f>
+      </c>
+      <c r="E98" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A96), "", '📦 商品出厂底价库 (Products)'!N96)</f>
+      </c>
+      <c r="F98" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A96), "", '📦 商品出厂底价库 (Products)'!F96)</f>
+      </c>
+      <c r="G98" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A96), "", '📦 商品出厂底价库 (Products)'!O96)</f>
+      </c>
+      <c r="H98" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A96), "", '📦 商品出厂底价库 (Products)'!P96)</f>
+      </c>
+      <c r="I98" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A96), "", '📦 商品出厂底价库 (Products)'!J96)</f>
+      </c>
+    </row>
+    <row r="99" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A97), "", 96)</f>
+      </c>
+      <c r="B99" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A97), "", '📦 商品出厂底价库 (Products)'!A97)</f>
+      </c>
+      <c r="C99" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A97), "", '📦 商品出厂底价库 (Products)'!C97)</f>
+      </c>
+      <c r="D99" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A97), "", '📦 商品出厂底价库 (Products)'!E97)</f>
+      </c>
+      <c r="E99" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A97), "", '📦 商品出厂底价库 (Products)'!N97)</f>
+      </c>
+      <c r="F99" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A97), "", '📦 商品出厂底价库 (Products)'!F97)</f>
+      </c>
+      <c r="G99" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A97), "", '📦 商品出厂底价库 (Products)'!O97)</f>
+      </c>
+      <c r="H99" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A97), "", '📦 商品出厂底价库 (Products)'!P97)</f>
+      </c>
+      <c r="I99" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A97), "", '📦 商品出厂底价库 (Products)'!J97)</f>
+      </c>
+    </row>
+    <row r="100" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A98), "", 97)</f>
+      </c>
+      <c r="B100" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A98), "", '📦 商品出厂底价库 (Products)'!A98)</f>
+      </c>
+      <c r="C100" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A98), "", '📦 商品出厂底价库 (Products)'!C98)</f>
+      </c>
+      <c r="D100" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A98), "", '📦 商品出厂底价库 (Products)'!E98)</f>
+      </c>
+      <c r="E100" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A98), "", '📦 商品出厂底价库 (Products)'!N98)</f>
+      </c>
+      <c r="F100" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A98), "", '📦 商品出厂底价库 (Products)'!F98)</f>
+      </c>
+      <c r="G100" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A98), "", '📦 商品出厂底价库 (Products)'!O98)</f>
+      </c>
+      <c r="H100" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A98), "", '📦 商品出厂底价库 (Products)'!P98)</f>
+      </c>
+      <c r="I100" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A98), "", '📦 商品出厂底价库 (Products)'!J98)</f>
+      </c>
+    </row>
+    <row r="101" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A101" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A99), "", 98)</f>
+      </c>
+      <c r="B101" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A99), "", '📦 商品出厂底价库 (Products)'!A99)</f>
+      </c>
+      <c r="C101" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A99), "", '📦 商品出厂底价库 (Products)'!C99)</f>
+      </c>
+      <c r="D101" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A99), "", '📦 商品出厂底价库 (Products)'!E99)</f>
+      </c>
+      <c r="E101" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A99), "", '📦 商品出厂底价库 (Products)'!N99)</f>
+      </c>
+      <c r="F101" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A99), "", '📦 商品出厂底价库 (Products)'!F99)</f>
+      </c>
+      <c r="G101" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A99), "", '📦 商品出厂底价库 (Products)'!O99)</f>
+      </c>
+      <c r="H101" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A99), "", '📦 商品出厂底价库 (Products)'!P99)</f>
+      </c>
+      <c r="I101" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A99), "", '📦 商品出厂底价库 (Products)'!J99)</f>
+      </c>
+    </row>
+    <row r="102" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A100), "", 99)</f>
+      </c>
+      <c r="B102" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A100), "", '📦 商品出厂底价库 (Products)'!A100)</f>
+      </c>
+      <c r="C102" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A100), "", '📦 商品出厂底价库 (Products)'!C100)</f>
+      </c>
+      <c r="D102" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A100), "", '📦 商品出厂底价库 (Products)'!E100)</f>
+      </c>
+      <c r="E102" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A100), "", '📦 商品出厂底价库 (Products)'!N100)</f>
+      </c>
+      <c r="F102" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A100), "", '📦 商品出厂底价库 (Products)'!F100)</f>
+      </c>
+      <c r="G102" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A100), "", '📦 商品出厂底价库 (Products)'!O100)</f>
+      </c>
+      <c r="H102" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A100), "", '📦 商品出厂底价库 (Products)'!P100)</f>
+      </c>
+      <c r="I102" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A100), "", '📦 商品出厂底价库 (Products)'!J100)</f>
+      </c>
+    </row>
+    <row r="103" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A103" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", 100)</f>
+      </c>
+      <c r="B103" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", '📦 商品出厂底价库 (Products)'!A101)</f>
+      </c>
+      <c r="C103" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", '📦 商品出厂底价库 (Products)'!C101)</f>
+      </c>
+      <c r="D103" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", '📦 商品出厂底价库 (Products)'!E101)</f>
+      </c>
+      <c r="E103" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", '📦 商品出厂底价库 (Products)'!N101)</f>
+      </c>
+      <c r="F103" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", '📦 商品出厂底价库 (Products)'!F101)</f>
+      </c>
+      <c r="G103" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", '📦 商品出厂底价库 (Products)'!O101)</f>
+      </c>
+      <c r="H103" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", '📦 商品出厂底价库 (Products)'!P101)</f>
+      </c>
+      <c r="I103" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", '📦 商品出厂底价库 (Products)'!J101)</f>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
feat(lead_magnets): expand smart formula capacity to 150 pre-populated rows
</commit_message>
<xml_diff>
--- a/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
+++ b/lead_magnets/2026外贸出厂底价表与智能核价模板.xlsx
@@ -1863,7 +1863,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q101"/>
+  <dimension ref="A1:Q151"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -5160,6 +5160,1556 @@
         <f>IF(ISBLANK(D101), "", IF(M101&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M101&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
       </c>
     </row>
+    <row r="102" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A102" s="39"/>
+      <c r="B102" s="40"/>
+      <c r="C102" s="41"/>
+      <c r="D102" s="42"/>
+      <c r="E102" s="43"/>
+      <c r="F102" s="43"/>
+      <c r="G102" s="44"/>
+      <c r="H102" s="45"/>
+      <c r="I102" s="46"/>
+      <c r="J102" s="39"/>
+      <c r="K102" s="39"/>
+      <c r="L102" s="47">
+        <f>IF(ISBLANK(D102), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M102" s="48">
+        <f>IF(ISBLANK(D102), "", IF(ISBLANK(I102), '⚙️ 全局核算参数 (Config)'!$B$13, I102))</f>
+      </c>
+      <c r="N102" s="49">
+        <f>IF(ISBLANK(D102), "", ROUND(((D102 * (1 + M102) + L102) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O102" s="50">
+        <f>IF(OR(ISBLANK(D102), NOT(AND(G102&gt;0, F102&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G102)) * F102)</f>
+      </c>
+      <c r="P102" s="50">
+        <f>IF(OR(ISBLANK(D102), NOT(AND(G102&gt;0, F102&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G102)) * F102)</f>
+      </c>
+      <c r="Q102" s="51">
+        <f>IF(ISBLANK(D102), "", IF(M102&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M102&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="103" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A103" s="52"/>
+      <c r="B103" s="53"/>
+      <c r="C103" s="54"/>
+      <c r="D103" s="55"/>
+      <c r="E103" s="56"/>
+      <c r="F103" s="56"/>
+      <c r="G103" s="57"/>
+      <c r="H103" s="58"/>
+      <c r="I103" s="59"/>
+      <c r="J103" s="52"/>
+      <c r="K103" s="52"/>
+      <c r="L103" s="47">
+        <f>IF(ISBLANK(D103), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M103" s="48">
+        <f>IF(ISBLANK(D103), "", IF(ISBLANK(I103), '⚙️ 全局核算参数 (Config)'!$B$13, I103))</f>
+      </c>
+      <c r="N103" s="49">
+        <f>IF(ISBLANK(D103), "", ROUND(((D103 * (1 + M103) + L103) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O103" s="50">
+        <f>IF(OR(ISBLANK(D103), NOT(AND(G103&gt;0, F103&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G103)) * F103)</f>
+      </c>
+      <c r="P103" s="50">
+        <f>IF(OR(ISBLANK(D103), NOT(AND(G103&gt;0, F103&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G103)) * F103)</f>
+      </c>
+      <c r="Q103" s="51">
+        <f>IF(ISBLANK(D103), "", IF(M103&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M103&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="104" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A104" s="39"/>
+      <c r="B104" s="40"/>
+      <c r="C104" s="41"/>
+      <c r="D104" s="42"/>
+      <c r="E104" s="43"/>
+      <c r="F104" s="43"/>
+      <c r="G104" s="44"/>
+      <c r="H104" s="45"/>
+      <c r="I104" s="46"/>
+      <c r="J104" s="39"/>
+      <c r="K104" s="39"/>
+      <c r="L104" s="47">
+        <f>IF(ISBLANK(D104), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M104" s="48">
+        <f>IF(ISBLANK(D104), "", IF(ISBLANK(I104), '⚙️ 全局核算参数 (Config)'!$B$13, I104))</f>
+      </c>
+      <c r="N104" s="49">
+        <f>IF(ISBLANK(D104), "", ROUND(((D104 * (1 + M104) + L104) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O104" s="50">
+        <f>IF(OR(ISBLANK(D104), NOT(AND(G104&gt;0, F104&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G104)) * F104)</f>
+      </c>
+      <c r="P104" s="50">
+        <f>IF(OR(ISBLANK(D104), NOT(AND(G104&gt;0, F104&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G104)) * F104)</f>
+      </c>
+      <c r="Q104" s="51">
+        <f>IF(ISBLANK(D104), "", IF(M104&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M104&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="105" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A105" s="52"/>
+      <c r="B105" s="53"/>
+      <c r="C105" s="54"/>
+      <c r="D105" s="55"/>
+      <c r="E105" s="56"/>
+      <c r="F105" s="56"/>
+      <c r="G105" s="57"/>
+      <c r="H105" s="58"/>
+      <c r="I105" s="59"/>
+      <c r="J105" s="52"/>
+      <c r="K105" s="52"/>
+      <c r="L105" s="47">
+        <f>IF(ISBLANK(D105), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M105" s="48">
+        <f>IF(ISBLANK(D105), "", IF(ISBLANK(I105), '⚙️ 全局核算参数 (Config)'!$B$13, I105))</f>
+      </c>
+      <c r="N105" s="49">
+        <f>IF(ISBLANK(D105), "", ROUND(((D105 * (1 + M105) + L105) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O105" s="50">
+        <f>IF(OR(ISBLANK(D105), NOT(AND(G105&gt;0, F105&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G105)) * F105)</f>
+      </c>
+      <c r="P105" s="50">
+        <f>IF(OR(ISBLANK(D105), NOT(AND(G105&gt;0, F105&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G105)) * F105)</f>
+      </c>
+      <c r="Q105" s="51">
+        <f>IF(ISBLANK(D105), "", IF(M105&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M105&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="106" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A106" s="39"/>
+      <c r="B106" s="40"/>
+      <c r="C106" s="41"/>
+      <c r="D106" s="42"/>
+      <c r="E106" s="43"/>
+      <c r="F106" s="43"/>
+      <c r="G106" s="44"/>
+      <c r="H106" s="45"/>
+      <c r="I106" s="46"/>
+      <c r="J106" s="39"/>
+      <c r="K106" s="39"/>
+      <c r="L106" s="47">
+        <f>IF(ISBLANK(D106), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M106" s="48">
+        <f>IF(ISBLANK(D106), "", IF(ISBLANK(I106), '⚙️ 全局核算参数 (Config)'!$B$13, I106))</f>
+      </c>
+      <c r="N106" s="49">
+        <f>IF(ISBLANK(D106), "", ROUND(((D106 * (1 + M106) + L106) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O106" s="50">
+        <f>IF(OR(ISBLANK(D106), NOT(AND(G106&gt;0, F106&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G106)) * F106)</f>
+      </c>
+      <c r="P106" s="50">
+        <f>IF(OR(ISBLANK(D106), NOT(AND(G106&gt;0, F106&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G106)) * F106)</f>
+      </c>
+      <c r="Q106" s="51">
+        <f>IF(ISBLANK(D106), "", IF(M106&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M106&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="107" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A107" s="52"/>
+      <c r="B107" s="53"/>
+      <c r="C107" s="54"/>
+      <c r="D107" s="55"/>
+      <c r="E107" s="56"/>
+      <c r="F107" s="56"/>
+      <c r="G107" s="57"/>
+      <c r="H107" s="58"/>
+      <c r="I107" s="59"/>
+      <c r="J107" s="52"/>
+      <c r="K107" s="52"/>
+      <c r="L107" s="47">
+        <f>IF(ISBLANK(D107), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M107" s="48">
+        <f>IF(ISBLANK(D107), "", IF(ISBLANK(I107), '⚙️ 全局核算参数 (Config)'!$B$13, I107))</f>
+      </c>
+      <c r="N107" s="49">
+        <f>IF(ISBLANK(D107), "", ROUND(((D107 * (1 + M107) + L107) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O107" s="50">
+        <f>IF(OR(ISBLANK(D107), NOT(AND(G107&gt;0, F107&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G107)) * F107)</f>
+      </c>
+      <c r="P107" s="50">
+        <f>IF(OR(ISBLANK(D107), NOT(AND(G107&gt;0, F107&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G107)) * F107)</f>
+      </c>
+      <c r="Q107" s="51">
+        <f>IF(ISBLANK(D107), "", IF(M107&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M107&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="108" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A108" s="39"/>
+      <c r="B108" s="40"/>
+      <c r="C108" s="41"/>
+      <c r="D108" s="42"/>
+      <c r="E108" s="43"/>
+      <c r="F108" s="43"/>
+      <c r="G108" s="44"/>
+      <c r="H108" s="45"/>
+      <c r="I108" s="46"/>
+      <c r="J108" s="39"/>
+      <c r="K108" s="39"/>
+      <c r="L108" s="47">
+        <f>IF(ISBLANK(D108), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M108" s="48">
+        <f>IF(ISBLANK(D108), "", IF(ISBLANK(I108), '⚙️ 全局核算参数 (Config)'!$B$13, I108))</f>
+      </c>
+      <c r="N108" s="49">
+        <f>IF(ISBLANK(D108), "", ROUND(((D108 * (1 + M108) + L108) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O108" s="50">
+        <f>IF(OR(ISBLANK(D108), NOT(AND(G108&gt;0, F108&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G108)) * F108)</f>
+      </c>
+      <c r="P108" s="50">
+        <f>IF(OR(ISBLANK(D108), NOT(AND(G108&gt;0, F108&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G108)) * F108)</f>
+      </c>
+      <c r="Q108" s="51">
+        <f>IF(ISBLANK(D108), "", IF(M108&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M108&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="109" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A109" s="52"/>
+      <c r="B109" s="53"/>
+      <c r="C109" s="54"/>
+      <c r="D109" s="55"/>
+      <c r="E109" s="56"/>
+      <c r="F109" s="56"/>
+      <c r="G109" s="57"/>
+      <c r="H109" s="58"/>
+      <c r="I109" s="59"/>
+      <c r="J109" s="52"/>
+      <c r="K109" s="52"/>
+      <c r="L109" s="47">
+        <f>IF(ISBLANK(D109), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M109" s="48">
+        <f>IF(ISBLANK(D109), "", IF(ISBLANK(I109), '⚙️ 全局核算参数 (Config)'!$B$13, I109))</f>
+      </c>
+      <c r="N109" s="49">
+        <f>IF(ISBLANK(D109), "", ROUND(((D109 * (1 + M109) + L109) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O109" s="50">
+        <f>IF(OR(ISBLANK(D109), NOT(AND(G109&gt;0, F109&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G109)) * F109)</f>
+      </c>
+      <c r="P109" s="50">
+        <f>IF(OR(ISBLANK(D109), NOT(AND(G109&gt;0, F109&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G109)) * F109)</f>
+      </c>
+      <c r="Q109" s="51">
+        <f>IF(ISBLANK(D109), "", IF(M109&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M109&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="110" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A110" s="39"/>
+      <c r="B110" s="40"/>
+      <c r="C110" s="41"/>
+      <c r="D110" s="42"/>
+      <c r="E110" s="43"/>
+      <c r="F110" s="43"/>
+      <c r="G110" s="44"/>
+      <c r="H110" s="45"/>
+      <c r="I110" s="46"/>
+      <c r="J110" s="39"/>
+      <c r="K110" s="39"/>
+      <c r="L110" s="47">
+        <f>IF(ISBLANK(D110), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M110" s="48">
+        <f>IF(ISBLANK(D110), "", IF(ISBLANK(I110), '⚙️ 全局核算参数 (Config)'!$B$13, I110))</f>
+      </c>
+      <c r="N110" s="49">
+        <f>IF(ISBLANK(D110), "", ROUND(((D110 * (1 + M110) + L110) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O110" s="50">
+        <f>IF(OR(ISBLANK(D110), NOT(AND(G110&gt;0, F110&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G110)) * F110)</f>
+      </c>
+      <c r="P110" s="50">
+        <f>IF(OR(ISBLANK(D110), NOT(AND(G110&gt;0, F110&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G110)) * F110)</f>
+      </c>
+      <c r="Q110" s="51">
+        <f>IF(ISBLANK(D110), "", IF(M110&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M110&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="111" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A111" s="52"/>
+      <c r="B111" s="53"/>
+      <c r="C111" s="54"/>
+      <c r="D111" s="55"/>
+      <c r="E111" s="56"/>
+      <c r="F111" s="56"/>
+      <c r="G111" s="57"/>
+      <c r="H111" s="58"/>
+      <c r="I111" s="59"/>
+      <c r="J111" s="52"/>
+      <c r="K111" s="52"/>
+      <c r="L111" s="47">
+        <f>IF(ISBLANK(D111), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M111" s="48">
+        <f>IF(ISBLANK(D111), "", IF(ISBLANK(I111), '⚙️ 全局核算参数 (Config)'!$B$13, I111))</f>
+      </c>
+      <c r="N111" s="49">
+        <f>IF(ISBLANK(D111), "", ROUND(((D111 * (1 + M111) + L111) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O111" s="50">
+        <f>IF(OR(ISBLANK(D111), NOT(AND(G111&gt;0, F111&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G111)) * F111)</f>
+      </c>
+      <c r="P111" s="50">
+        <f>IF(OR(ISBLANK(D111), NOT(AND(G111&gt;0, F111&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G111)) * F111)</f>
+      </c>
+      <c r="Q111" s="51">
+        <f>IF(ISBLANK(D111), "", IF(M111&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M111&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="112" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A112" s="39"/>
+      <c r="B112" s="40"/>
+      <c r="C112" s="41"/>
+      <c r="D112" s="42"/>
+      <c r="E112" s="43"/>
+      <c r="F112" s="43"/>
+      <c r="G112" s="44"/>
+      <c r="H112" s="45"/>
+      <c r="I112" s="46"/>
+      <c r="J112" s="39"/>
+      <c r="K112" s="39"/>
+      <c r="L112" s="47">
+        <f>IF(ISBLANK(D112), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M112" s="48">
+        <f>IF(ISBLANK(D112), "", IF(ISBLANK(I112), '⚙️ 全局核算参数 (Config)'!$B$13, I112))</f>
+      </c>
+      <c r="N112" s="49">
+        <f>IF(ISBLANK(D112), "", ROUND(((D112 * (1 + M112) + L112) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O112" s="50">
+        <f>IF(OR(ISBLANK(D112), NOT(AND(G112&gt;0, F112&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G112)) * F112)</f>
+      </c>
+      <c r="P112" s="50">
+        <f>IF(OR(ISBLANK(D112), NOT(AND(G112&gt;0, F112&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G112)) * F112)</f>
+      </c>
+      <c r="Q112" s="51">
+        <f>IF(ISBLANK(D112), "", IF(M112&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M112&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="113" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A113" s="52"/>
+      <c r="B113" s="53"/>
+      <c r="C113" s="54"/>
+      <c r="D113" s="55"/>
+      <c r="E113" s="56"/>
+      <c r="F113" s="56"/>
+      <c r="G113" s="57"/>
+      <c r="H113" s="58"/>
+      <c r="I113" s="59"/>
+      <c r="J113" s="52"/>
+      <c r="K113" s="52"/>
+      <c r="L113" s="47">
+        <f>IF(ISBLANK(D113), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M113" s="48">
+        <f>IF(ISBLANK(D113), "", IF(ISBLANK(I113), '⚙️ 全局核算参数 (Config)'!$B$13, I113))</f>
+      </c>
+      <c r="N113" s="49">
+        <f>IF(ISBLANK(D113), "", ROUND(((D113 * (1 + M113) + L113) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O113" s="50">
+        <f>IF(OR(ISBLANK(D113), NOT(AND(G113&gt;0, F113&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G113)) * F113)</f>
+      </c>
+      <c r="P113" s="50">
+        <f>IF(OR(ISBLANK(D113), NOT(AND(G113&gt;0, F113&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G113)) * F113)</f>
+      </c>
+      <c r="Q113" s="51">
+        <f>IF(ISBLANK(D113), "", IF(M113&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M113&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="114" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A114" s="39"/>
+      <c r="B114" s="40"/>
+      <c r="C114" s="41"/>
+      <c r="D114" s="42"/>
+      <c r="E114" s="43"/>
+      <c r="F114" s="43"/>
+      <c r="G114" s="44"/>
+      <c r="H114" s="45"/>
+      <c r="I114" s="46"/>
+      <c r="J114" s="39"/>
+      <c r="K114" s="39"/>
+      <c r="L114" s="47">
+        <f>IF(ISBLANK(D114), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M114" s="48">
+        <f>IF(ISBLANK(D114), "", IF(ISBLANK(I114), '⚙️ 全局核算参数 (Config)'!$B$13, I114))</f>
+      </c>
+      <c r="N114" s="49">
+        <f>IF(ISBLANK(D114), "", ROUND(((D114 * (1 + M114) + L114) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O114" s="50">
+        <f>IF(OR(ISBLANK(D114), NOT(AND(G114&gt;0, F114&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G114)) * F114)</f>
+      </c>
+      <c r="P114" s="50">
+        <f>IF(OR(ISBLANK(D114), NOT(AND(G114&gt;0, F114&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G114)) * F114)</f>
+      </c>
+      <c r="Q114" s="51">
+        <f>IF(ISBLANK(D114), "", IF(M114&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M114&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="115" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A115" s="52"/>
+      <c r="B115" s="53"/>
+      <c r="C115" s="54"/>
+      <c r="D115" s="55"/>
+      <c r="E115" s="56"/>
+      <c r="F115" s="56"/>
+      <c r="G115" s="57"/>
+      <c r="H115" s="58"/>
+      <c r="I115" s="59"/>
+      <c r="J115" s="52"/>
+      <c r="K115" s="52"/>
+      <c r="L115" s="47">
+        <f>IF(ISBLANK(D115), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M115" s="48">
+        <f>IF(ISBLANK(D115), "", IF(ISBLANK(I115), '⚙️ 全局核算参数 (Config)'!$B$13, I115))</f>
+      </c>
+      <c r="N115" s="49">
+        <f>IF(ISBLANK(D115), "", ROUND(((D115 * (1 + M115) + L115) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O115" s="50">
+        <f>IF(OR(ISBLANK(D115), NOT(AND(G115&gt;0, F115&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G115)) * F115)</f>
+      </c>
+      <c r="P115" s="50">
+        <f>IF(OR(ISBLANK(D115), NOT(AND(G115&gt;0, F115&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G115)) * F115)</f>
+      </c>
+      <c r="Q115" s="51">
+        <f>IF(ISBLANK(D115), "", IF(M115&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M115&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="116" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A116" s="39"/>
+      <c r="B116" s="40"/>
+      <c r="C116" s="41"/>
+      <c r="D116" s="42"/>
+      <c r="E116" s="43"/>
+      <c r="F116" s="43"/>
+      <c r="G116" s="44"/>
+      <c r="H116" s="45"/>
+      <c r="I116" s="46"/>
+      <c r="J116" s="39"/>
+      <c r="K116" s="39"/>
+      <c r="L116" s="47">
+        <f>IF(ISBLANK(D116), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M116" s="48">
+        <f>IF(ISBLANK(D116), "", IF(ISBLANK(I116), '⚙️ 全局核算参数 (Config)'!$B$13, I116))</f>
+      </c>
+      <c r="N116" s="49">
+        <f>IF(ISBLANK(D116), "", ROUND(((D116 * (1 + M116) + L116) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O116" s="50">
+        <f>IF(OR(ISBLANK(D116), NOT(AND(G116&gt;0, F116&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G116)) * F116)</f>
+      </c>
+      <c r="P116" s="50">
+        <f>IF(OR(ISBLANK(D116), NOT(AND(G116&gt;0, F116&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G116)) * F116)</f>
+      </c>
+      <c r="Q116" s="51">
+        <f>IF(ISBLANK(D116), "", IF(M116&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M116&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="117" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A117" s="52"/>
+      <c r="B117" s="53"/>
+      <c r="C117" s="54"/>
+      <c r="D117" s="55"/>
+      <c r="E117" s="56"/>
+      <c r="F117" s="56"/>
+      <c r="G117" s="57"/>
+      <c r="H117" s="58"/>
+      <c r="I117" s="59"/>
+      <c r="J117" s="52"/>
+      <c r="K117" s="52"/>
+      <c r="L117" s="47">
+        <f>IF(ISBLANK(D117), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M117" s="48">
+        <f>IF(ISBLANK(D117), "", IF(ISBLANK(I117), '⚙️ 全局核算参数 (Config)'!$B$13, I117))</f>
+      </c>
+      <c r="N117" s="49">
+        <f>IF(ISBLANK(D117), "", ROUND(((D117 * (1 + M117) + L117) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O117" s="50">
+        <f>IF(OR(ISBLANK(D117), NOT(AND(G117&gt;0, F117&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G117)) * F117)</f>
+      </c>
+      <c r="P117" s="50">
+        <f>IF(OR(ISBLANK(D117), NOT(AND(G117&gt;0, F117&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G117)) * F117)</f>
+      </c>
+      <c r="Q117" s="51">
+        <f>IF(ISBLANK(D117), "", IF(M117&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M117&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="118" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A118" s="39"/>
+      <c r="B118" s="40"/>
+      <c r="C118" s="41"/>
+      <c r="D118" s="42"/>
+      <c r="E118" s="43"/>
+      <c r="F118" s="43"/>
+      <c r="G118" s="44"/>
+      <c r="H118" s="45"/>
+      <c r="I118" s="46"/>
+      <c r="J118" s="39"/>
+      <c r="K118" s="39"/>
+      <c r="L118" s="47">
+        <f>IF(ISBLANK(D118), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M118" s="48">
+        <f>IF(ISBLANK(D118), "", IF(ISBLANK(I118), '⚙️ 全局核算参数 (Config)'!$B$13, I118))</f>
+      </c>
+      <c r="N118" s="49">
+        <f>IF(ISBLANK(D118), "", ROUND(((D118 * (1 + M118) + L118) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O118" s="50">
+        <f>IF(OR(ISBLANK(D118), NOT(AND(G118&gt;0, F118&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G118)) * F118)</f>
+      </c>
+      <c r="P118" s="50">
+        <f>IF(OR(ISBLANK(D118), NOT(AND(G118&gt;0, F118&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G118)) * F118)</f>
+      </c>
+      <c r="Q118" s="51">
+        <f>IF(ISBLANK(D118), "", IF(M118&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M118&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="119" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A119" s="52"/>
+      <c r="B119" s="53"/>
+      <c r="C119" s="54"/>
+      <c r="D119" s="55"/>
+      <c r="E119" s="56"/>
+      <c r="F119" s="56"/>
+      <c r="G119" s="57"/>
+      <c r="H119" s="58"/>
+      <c r="I119" s="59"/>
+      <c r="J119" s="52"/>
+      <c r="K119" s="52"/>
+      <c r="L119" s="47">
+        <f>IF(ISBLANK(D119), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M119" s="48">
+        <f>IF(ISBLANK(D119), "", IF(ISBLANK(I119), '⚙️ 全局核算参数 (Config)'!$B$13, I119))</f>
+      </c>
+      <c r="N119" s="49">
+        <f>IF(ISBLANK(D119), "", ROUND(((D119 * (1 + M119) + L119) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O119" s="50">
+        <f>IF(OR(ISBLANK(D119), NOT(AND(G119&gt;0, F119&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G119)) * F119)</f>
+      </c>
+      <c r="P119" s="50">
+        <f>IF(OR(ISBLANK(D119), NOT(AND(G119&gt;0, F119&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G119)) * F119)</f>
+      </c>
+      <c r="Q119" s="51">
+        <f>IF(ISBLANK(D119), "", IF(M119&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M119&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="120" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A120" s="39"/>
+      <c r="B120" s="40"/>
+      <c r="C120" s="41"/>
+      <c r="D120" s="42"/>
+      <c r="E120" s="43"/>
+      <c r="F120" s="43"/>
+      <c r="G120" s="44"/>
+      <c r="H120" s="45"/>
+      <c r="I120" s="46"/>
+      <c r="J120" s="39"/>
+      <c r="K120" s="39"/>
+      <c r="L120" s="47">
+        <f>IF(ISBLANK(D120), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M120" s="48">
+        <f>IF(ISBLANK(D120), "", IF(ISBLANK(I120), '⚙️ 全局核算参数 (Config)'!$B$13, I120))</f>
+      </c>
+      <c r="N120" s="49">
+        <f>IF(ISBLANK(D120), "", ROUND(((D120 * (1 + M120) + L120) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O120" s="50">
+        <f>IF(OR(ISBLANK(D120), NOT(AND(G120&gt;0, F120&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G120)) * F120)</f>
+      </c>
+      <c r="P120" s="50">
+        <f>IF(OR(ISBLANK(D120), NOT(AND(G120&gt;0, F120&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G120)) * F120)</f>
+      </c>
+      <c r="Q120" s="51">
+        <f>IF(ISBLANK(D120), "", IF(M120&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M120&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="121" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A121" s="52"/>
+      <c r="B121" s="53"/>
+      <c r="C121" s="54"/>
+      <c r="D121" s="55"/>
+      <c r="E121" s="56"/>
+      <c r="F121" s="56"/>
+      <c r="G121" s="57"/>
+      <c r="H121" s="58"/>
+      <c r="I121" s="59"/>
+      <c r="J121" s="52"/>
+      <c r="K121" s="52"/>
+      <c r="L121" s="47">
+        <f>IF(ISBLANK(D121), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M121" s="48">
+        <f>IF(ISBLANK(D121), "", IF(ISBLANK(I121), '⚙️ 全局核算参数 (Config)'!$B$13, I121))</f>
+      </c>
+      <c r="N121" s="49">
+        <f>IF(ISBLANK(D121), "", ROUND(((D121 * (1 + M121) + L121) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O121" s="50">
+        <f>IF(OR(ISBLANK(D121), NOT(AND(G121&gt;0, F121&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G121)) * F121)</f>
+      </c>
+      <c r="P121" s="50">
+        <f>IF(OR(ISBLANK(D121), NOT(AND(G121&gt;0, F121&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G121)) * F121)</f>
+      </c>
+      <c r="Q121" s="51">
+        <f>IF(ISBLANK(D121), "", IF(M121&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M121&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="122" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A122" s="39"/>
+      <c r="B122" s="40"/>
+      <c r="C122" s="41"/>
+      <c r="D122" s="42"/>
+      <c r="E122" s="43"/>
+      <c r="F122" s="43"/>
+      <c r="G122" s="44"/>
+      <c r="H122" s="45"/>
+      <c r="I122" s="46"/>
+      <c r="J122" s="39"/>
+      <c r="K122" s="39"/>
+      <c r="L122" s="47">
+        <f>IF(ISBLANK(D122), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M122" s="48">
+        <f>IF(ISBLANK(D122), "", IF(ISBLANK(I122), '⚙️ 全局核算参数 (Config)'!$B$13, I122))</f>
+      </c>
+      <c r="N122" s="49">
+        <f>IF(ISBLANK(D122), "", ROUND(((D122 * (1 + M122) + L122) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O122" s="50">
+        <f>IF(OR(ISBLANK(D122), NOT(AND(G122&gt;0, F122&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G122)) * F122)</f>
+      </c>
+      <c r="P122" s="50">
+        <f>IF(OR(ISBLANK(D122), NOT(AND(G122&gt;0, F122&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G122)) * F122)</f>
+      </c>
+      <c r="Q122" s="51">
+        <f>IF(ISBLANK(D122), "", IF(M122&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M122&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="123" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A123" s="52"/>
+      <c r="B123" s="53"/>
+      <c r="C123" s="54"/>
+      <c r="D123" s="55"/>
+      <c r="E123" s="56"/>
+      <c r="F123" s="56"/>
+      <c r="G123" s="57"/>
+      <c r="H123" s="58"/>
+      <c r="I123" s="59"/>
+      <c r="J123" s="52"/>
+      <c r="K123" s="52"/>
+      <c r="L123" s="47">
+        <f>IF(ISBLANK(D123), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M123" s="48">
+        <f>IF(ISBLANK(D123), "", IF(ISBLANK(I123), '⚙️ 全局核算参数 (Config)'!$B$13, I123))</f>
+      </c>
+      <c r="N123" s="49">
+        <f>IF(ISBLANK(D123), "", ROUND(((D123 * (1 + M123) + L123) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O123" s="50">
+        <f>IF(OR(ISBLANK(D123), NOT(AND(G123&gt;0, F123&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G123)) * F123)</f>
+      </c>
+      <c r="P123" s="50">
+        <f>IF(OR(ISBLANK(D123), NOT(AND(G123&gt;0, F123&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G123)) * F123)</f>
+      </c>
+      <c r="Q123" s="51">
+        <f>IF(ISBLANK(D123), "", IF(M123&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M123&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="124" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A124" s="39"/>
+      <c r="B124" s="40"/>
+      <c r="C124" s="41"/>
+      <c r="D124" s="42"/>
+      <c r="E124" s="43"/>
+      <c r="F124" s="43"/>
+      <c r="G124" s="44"/>
+      <c r="H124" s="45"/>
+      <c r="I124" s="46"/>
+      <c r="J124" s="39"/>
+      <c r="K124" s="39"/>
+      <c r="L124" s="47">
+        <f>IF(ISBLANK(D124), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M124" s="48">
+        <f>IF(ISBLANK(D124), "", IF(ISBLANK(I124), '⚙️ 全局核算参数 (Config)'!$B$13, I124))</f>
+      </c>
+      <c r="N124" s="49">
+        <f>IF(ISBLANK(D124), "", ROUND(((D124 * (1 + M124) + L124) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O124" s="50">
+        <f>IF(OR(ISBLANK(D124), NOT(AND(G124&gt;0, F124&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G124)) * F124)</f>
+      </c>
+      <c r="P124" s="50">
+        <f>IF(OR(ISBLANK(D124), NOT(AND(G124&gt;0, F124&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G124)) * F124)</f>
+      </c>
+      <c r="Q124" s="51">
+        <f>IF(ISBLANK(D124), "", IF(M124&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M124&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="125" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A125" s="52"/>
+      <c r="B125" s="53"/>
+      <c r="C125" s="54"/>
+      <c r="D125" s="55"/>
+      <c r="E125" s="56"/>
+      <c r="F125" s="56"/>
+      <c r="G125" s="57"/>
+      <c r="H125" s="58"/>
+      <c r="I125" s="59"/>
+      <c r="J125" s="52"/>
+      <c r="K125" s="52"/>
+      <c r="L125" s="47">
+        <f>IF(ISBLANK(D125), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M125" s="48">
+        <f>IF(ISBLANK(D125), "", IF(ISBLANK(I125), '⚙️ 全局核算参数 (Config)'!$B$13, I125))</f>
+      </c>
+      <c r="N125" s="49">
+        <f>IF(ISBLANK(D125), "", ROUND(((D125 * (1 + M125) + L125) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O125" s="50">
+        <f>IF(OR(ISBLANK(D125), NOT(AND(G125&gt;0, F125&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G125)) * F125)</f>
+      </c>
+      <c r="P125" s="50">
+        <f>IF(OR(ISBLANK(D125), NOT(AND(G125&gt;0, F125&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G125)) * F125)</f>
+      </c>
+      <c r="Q125" s="51">
+        <f>IF(ISBLANK(D125), "", IF(M125&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M125&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="126" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A126" s="39"/>
+      <c r="B126" s="40"/>
+      <c r="C126" s="41"/>
+      <c r="D126" s="42"/>
+      <c r="E126" s="43"/>
+      <c r="F126" s="43"/>
+      <c r="G126" s="44"/>
+      <c r="H126" s="45"/>
+      <c r="I126" s="46"/>
+      <c r="J126" s="39"/>
+      <c r="K126" s="39"/>
+      <c r="L126" s="47">
+        <f>IF(ISBLANK(D126), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M126" s="48">
+        <f>IF(ISBLANK(D126), "", IF(ISBLANK(I126), '⚙️ 全局核算参数 (Config)'!$B$13, I126))</f>
+      </c>
+      <c r="N126" s="49">
+        <f>IF(ISBLANK(D126), "", ROUND(((D126 * (1 + M126) + L126) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O126" s="50">
+        <f>IF(OR(ISBLANK(D126), NOT(AND(G126&gt;0, F126&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G126)) * F126)</f>
+      </c>
+      <c r="P126" s="50">
+        <f>IF(OR(ISBLANK(D126), NOT(AND(G126&gt;0, F126&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G126)) * F126)</f>
+      </c>
+      <c r="Q126" s="51">
+        <f>IF(ISBLANK(D126), "", IF(M126&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M126&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="127" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A127" s="52"/>
+      <c r="B127" s="53"/>
+      <c r="C127" s="54"/>
+      <c r="D127" s="55"/>
+      <c r="E127" s="56"/>
+      <c r="F127" s="56"/>
+      <c r="G127" s="57"/>
+      <c r="H127" s="58"/>
+      <c r="I127" s="59"/>
+      <c r="J127" s="52"/>
+      <c r="K127" s="52"/>
+      <c r="L127" s="47">
+        <f>IF(ISBLANK(D127), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M127" s="48">
+        <f>IF(ISBLANK(D127), "", IF(ISBLANK(I127), '⚙️ 全局核算参数 (Config)'!$B$13, I127))</f>
+      </c>
+      <c r="N127" s="49">
+        <f>IF(ISBLANK(D127), "", ROUND(((D127 * (1 + M127) + L127) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O127" s="50">
+        <f>IF(OR(ISBLANK(D127), NOT(AND(G127&gt;0, F127&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G127)) * F127)</f>
+      </c>
+      <c r="P127" s="50">
+        <f>IF(OR(ISBLANK(D127), NOT(AND(G127&gt;0, F127&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G127)) * F127)</f>
+      </c>
+      <c r="Q127" s="51">
+        <f>IF(ISBLANK(D127), "", IF(M127&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M127&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="128" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A128" s="39"/>
+      <c r="B128" s="40"/>
+      <c r="C128" s="41"/>
+      <c r="D128" s="42"/>
+      <c r="E128" s="43"/>
+      <c r="F128" s="43"/>
+      <c r="G128" s="44"/>
+      <c r="H128" s="45"/>
+      <c r="I128" s="46"/>
+      <c r="J128" s="39"/>
+      <c r="K128" s="39"/>
+      <c r="L128" s="47">
+        <f>IF(ISBLANK(D128), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M128" s="48">
+        <f>IF(ISBLANK(D128), "", IF(ISBLANK(I128), '⚙️ 全局核算参数 (Config)'!$B$13, I128))</f>
+      </c>
+      <c r="N128" s="49">
+        <f>IF(ISBLANK(D128), "", ROUND(((D128 * (1 + M128) + L128) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O128" s="50">
+        <f>IF(OR(ISBLANK(D128), NOT(AND(G128&gt;0, F128&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G128)) * F128)</f>
+      </c>
+      <c r="P128" s="50">
+        <f>IF(OR(ISBLANK(D128), NOT(AND(G128&gt;0, F128&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G128)) * F128)</f>
+      </c>
+      <c r="Q128" s="51">
+        <f>IF(ISBLANK(D128), "", IF(M128&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M128&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="129" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A129" s="52"/>
+      <c r="B129" s="53"/>
+      <c r="C129" s="54"/>
+      <c r="D129" s="55"/>
+      <c r="E129" s="56"/>
+      <c r="F129" s="56"/>
+      <c r="G129" s="57"/>
+      <c r="H129" s="58"/>
+      <c r="I129" s="59"/>
+      <c r="J129" s="52"/>
+      <c r="K129" s="52"/>
+      <c r="L129" s="47">
+        <f>IF(ISBLANK(D129), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M129" s="48">
+        <f>IF(ISBLANK(D129), "", IF(ISBLANK(I129), '⚙️ 全局核算参数 (Config)'!$B$13, I129))</f>
+      </c>
+      <c r="N129" s="49">
+        <f>IF(ISBLANK(D129), "", ROUND(((D129 * (1 + M129) + L129) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O129" s="50">
+        <f>IF(OR(ISBLANK(D129), NOT(AND(G129&gt;0, F129&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G129)) * F129)</f>
+      </c>
+      <c r="P129" s="50">
+        <f>IF(OR(ISBLANK(D129), NOT(AND(G129&gt;0, F129&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G129)) * F129)</f>
+      </c>
+      <c r="Q129" s="51">
+        <f>IF(ISBLANK(D129), "", IF(M129&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M129&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="130" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A130" s="39"/>
+      <c r="B130" s="40"/>
+      <c r="C130" s="41"/>
+      <c r="D130" s="42"/>
+      <c r="E130" s="43"/>
+      <c r="F130" s="43"/>
+      <c r="G130" s="44"/>
+      <c r="H130" s="45"/>
+      <c r="I130" s="46"/>
+      <c r="J130" s="39"/>
+      <c r="K130" s="39"/>
+      <c r="L130" s="47">
+        <f>IF(ISBLANK(D130), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M130" s="48">
+        <f>IF(ISBLANK(D130), "", IF(ISBLANK(I130), '⚙️ 全局核算参数 (Config)'!$B$13, I130))</f>
+      </c>
+      <c r="N130" s="49">
+        <f>IF(ISBLANK(D130), "", ROUND(((D130 * (1 + M130) + L130) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O130" s="50">
+        <f>IF(OR(ISBLANK(D130), NOT(AND(G130&gt;0, F130&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G130)) * F130)</f>
+      </c>
+      <c r="P130" s="50">
+        <f>IF(OR(ISBLANK(D130), NOT(AND(G130&gt;0, F130&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G130)) * F130)</f>
+      </c>
+      <c r="Q130" s="51">
+        <f>IF(ISBLANK(D130), "", IF(M130&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M130&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="131" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A131" s="52"/>
+      <c r="B131" s="53"/>
+      <c r="C131" s="54"/>
+      <c r="D131" s="55"/>
+      <c r="E131" s="56"/>
+      <c r="F131" s="56"/>
+      <c r="G131" s="57"/>
+      <c r="H131" s="58"/>
+      <c r="I131" s="59"/>
+      <c r="J131" s="52"/>
+      <c r="K131" s="52"/>
+      <c r="L131" s="47">
+        <f>IF(ISBLANK(D131), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M131" s="48">
+        <f>IF(ISBLANK(D131), "", IF(ISBLANK(I131), '⚙️ 全局核算参数 (Config)'!$B$13, I131))</f>
+      </c>
+      <c r="N131" s="49">
+        <f>IF(ISBLANK(D131), "", ROUND(((D131 * (1 + M131) + L131) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O131" s="50">
+        <f>IF(OR(ISBLANK(D131), NOT(AND(G131&gt;0, F131&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G131)) * F131)</f>
+      </c>
+      <c r="P131" s="50">
+        <f>IF(OR(ISBLANK(D131), NOT(AND(G131&gt;0, F131&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G131)) * F131)</f>
+      </c>
+      <c r="Q131" s="51">
+        <f>IF(ISBLANK(D131), "", IF(M131&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M131&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="132" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A132" s="39"/>
+      <c r="B132" s="40"/>
+      <c r="C132" s="41"/>
+      <c r="D132" s="42"/>
+      <c r="E132" s="43"/>
+      <c r="F132" s="43"/>
+      <c r="G132" s="44"/>
+      <c r="H132" s="45"/>
+      <c r="I132" s="46"/>
+      <c r="J132" s="39"/>
+      <c r="K132" s="39"/>
+      <c r="L132" s="47">
+        <f>IF(ISBLANK(D132), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M132" s="48">
+        <f>IF(ISBLANK(D132), "", IF(ISBLANK(I132), '⚙️ 全局核算参数 (Config)'!$B$13, I132))</f>
+      </c>
+      <c r="N132" s="49">
+        <f>IF(ISBLANK(D132), "", ROUND(((D132 * (1 + M132) + L132) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O132" s="50">
+        <f>IF(OR(ISBLANK(D132), NOT(AND(G132&gt;0, F132&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G132)) * F132)</f>
+      </c>
+      <c r="P132" s="50">
+        <f>IF(OR(ISBLANK(D132), NOT(AND(G132&gt;0, F132&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G132)) * F132)</f>
+      </c>
+      <c r="Q132" s="51">
+        <f>IF(ISBLANK(D132), "", IF(M132&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M132&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="133" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A133" s="52"/>
+      <c r="B133" s="53"/>
+      <c r="C133" s="54"/>
+      <c r="D133" s="55"/>
+      <c r="E133" s="56"/>
+      <c r="F133" s="56"/>
+      <c r="G133" s="57"/>
+      <c r="H133" s="58"/>
+      <c r="I133" s="59"/>
+      <c r="J133" s="52"/>
+      <c r="K133" s="52"/>
+      <c r="L133" s="47">
+        <f>IF(ISBLANK(D133), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M133" s="48">
+        <f>IF(ISBLANK(D133), "", IF(ISBLANK(I133), '⚙️ 全局核算参数 (Config)'!$B$13, I133))</f>
+      </c>
+      <c r="N133" s="49">
+        <f>IF(ISBLANK(D133), "", ROUND(((D133 * (1 + M133) + L133) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O133" s="50">
+        <f>IF(OR(ISBLANK(D133), NOT(AND(G133&gt;0, F133&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G133)) * F133)</f>
+      </c>
+      <c r="P133" s="50">
+        <f>IF(OR(ISBLANK(D133), NOT(AND(G133&gt;0, F133&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G133)) * F133)</f>
+      </c>
+      <c r="Q133" s="51">
+        <f>IF(ISBLANK(D133), "", IF(M133&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M133&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="134" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A134" s="39"/>
+      <c r="B134" s="40"/>
+      <c r="C134" s="41"/>
+      <c r="D134" s="42"/>
+      <c r="E134" s="43"/>
+      <c r="F134" s="43"/>
+      <c r="G134" s="44"/>
+      <c r="H134" s="45"/>
+      <c r="I134" s="46"/>
+      <c r="J134" s="39"/>
+      <c r="K134" s="39"/>
+      <c r="L134" s="47">
+        <f>IF(ISBLANK(D134), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M134" s="48">
+        <f>IF(ISBLANK(D134), "", IF(ISBLANK(I134), '⚙️ 全局核算参数 (Config)'!$B$13, I134))</f>
+      </c>
+      <c r="N134" s="49">
+        <f>IF(ISBLANK(D134), "", ROUND(((D134 * (1 + M134) + L134) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O134" s="50">
+        <f>IF(OR(ISBLANK(D134), NOT(AND(G134&gt;0, F134&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G134)) * F134)</f>
+      </c>
+      <c r="P134" s="50">
+        <f>IF(OR(ISBLANK(D134), NOT(AND(G134&gt;0, F134&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G134)) * F134)</f>
+      </c>
+      <c r="Q134" s="51">
+        <f>IF(ISBLANK(D134), "", IF(M134&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M134&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="135" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A135" s="52"/>
+      <c r="B135" s="53"/>
+      <c r="C135" s="54"/>
+      <c r="D135" s="55"/>
+      <c r="E135" s="56"/>
+      <c r="F135" s="56"/>
+      <c r="G135" s="57"/>
+      <c r="H135" s="58"/>
+      <c r="I135" s="59"/>
+      <c r="J135" s="52"/>
+      <c r="K135" s="52"/>
+      <c r="L135" s="47">
+        <f>IF(ISBLANK(D135), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M135" s="48">
+        <f>IF(ISBLANK(D135), "", IF(ISBLANK(I135), '⚙️ 全局核算参数 (Config)'!$B$13, I135))</f>
+      </c>
+      <c r="N135" s="49">
+        <f>IF(ISBLANK(D135), "", ROUND(((D135 * (1 + M135) + L135) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O135" s="50">
+        <f>IF(OR(ISBLANK(D135), NOT(AND(G135&gt;0, F135&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G135)) * F135)</f>
+      </c>
+      <c r="P135" s="50">
+        <f>IF(OR(ISBLANK(D135), NOT(AND(G135&gt;0, F135&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G135)) * F135)</f>
+      </c>
+      <c r="Q135" s="51">
+        <f>IF(ISBLANK(D135), "", IF(M135&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M135&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="136" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A136" s="39"/>
+      <c r="B136" s="40"/>
+      <c r="C136" s="41"/>
+      <c r="D136" s="42"/>
+      <c r="E136" s="43"/>
+      <c r="F136" s="43"/>
+      <c r="G136" s="44"/>
+      <c r="H136" s="45"/>
+      <c r="I136" s="46"/>
+      <c r="J136" s="39"/>
+      <c r="K136" s="39"/>
+      <c r="L136" s="47">
+        <f>IF(ISBLANK(D136), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M136" s="48">
+        <f>IF(ISBLANK(D136), "", IF(ISBLANK(I136), '⚙️ 全局核算参数 (Config)'!$B$13, I136))</f>
+      </c>
+      <c r="N136" s="49">
+        <f>IF(ISBLANK(D136), "", ROUND(((D136 * (1 + M136) + L136) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O136" s="50">
+        <f>IF(OR(ISBLANK(D136), NOT(AND(G136&gt;0, F136&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G136)) * F136)</f>
+      </c>
+      <c r="P136" s="50">
+        <f>IF(OR(ISBLANK(D136), NOT(AND(G136&gt;0, F136&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G136)) * F136)</f>
+      </c>
+      <c r="Q136" s="51">
+        <f>IF(ISBLANK(D136), "", IF(M136&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M136&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="137" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A137" s="52"/>
+      <c r="B137" s="53"/>
+      <c r="C137" s="54"/>
+      <c r="D137" s="55"/>
+      <c r="E137" s="56"/>
+      <c r="F137" s="56"/>
+      <c r="G137" s="57"/>
+      <c r="H137" s="58"/>
+      <c r="I137" s="59"/>
+      <c r="J137" s="52"/>
+      <c r="K137" s="52"/>
+      <c r="L137" s="47">
+        <f>IF(ISBLANK(D137), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M137" s="48">
+        <f>IF(ISBLANK(D137), "", IF(ISBLANK(I137), '⚙️ 全局核算参数 (Config)'!$B$13, I137))</f>
+      </c>
+      <c r="N137" s="49">
+        <f>IF(ISBLANK(D137), "", ROUND(((D137 * (1 + M137) + L137) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O137" s="50">
+        <f>IF(OR(ISBLANK(D137), NOT(AND(G137&gt;0, F137&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G137)) * F137)</f>
+      </c>
+      <c r="P137" s="50">
+        <f>IF(OR(ISBLANK(D137), NOT(AND(G137&gt;0, F137&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G137)) * F137)</f>
+      </c>
+      <c r="Q137" s="51">
+        <f>IF(ISBLANK(D137), "", IF(M137&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M137&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="138" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A138" s="39"/>
+      <c r="B138" s="40"/>
+      <c r="C138" s="41"/>
+      <c r="D138" s="42"/>
+      <c r="E138" s="43"/>
+      <c r="F138" s="43"/>
+      <c r="G138" s="44"/>
+      <c r="H138" s="45"/>
+      <c r="I138" s="46"/>
+      <c r="J138" s="39"/>
+      <c r="K138" s="39"/>
+      <c r="L138" s="47">
+        <f>IF(ISBLANK(D138), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M138" s="48">
+        <f>IF(ISBLANK(D138), "", IF(ISBLANK(I138), '⚙️ 全局核算参数 (Config)'!$B$13, I138))</f>
+      </c>
+      <c r="N138" s="49">
+        <f>IF(ISBLANK(D138), "", ROUND(((D138 * (1 + M138) + L138) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O138" s="50">
+        <f>IF(OR(ISBLANK(D138), NOT(AND(G138&gt;0, F138&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G138)) * F138)</f>
+      </c>
+      <c r="P138" s="50">
+        <f>IF(OR(ISBLANK(D138), NOT(AND(G138&gt;0, F138&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G138)) * F138)</f>
+      </c>
+      <c r="Q138" s="51">
+        <f>IF(ISBLANK(D138), "", IF(M138&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M138&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="139" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A139" s="52"/>
+      <c r="B139" s="53"/>
+      <c r="C139" s="54"/>
+      <c r="D139" s="55"/>
+      <c r="E139" s="56"/>
+      <c r="F139" s="56"/>
+      <c r="G139" s="57"/>
+      <c r="H139" s="58"/>
+      <c r="I139" s="59"/>
+      <c r="J139" s="52"/>
+      <c r="K139" s="52"/>
+      <c r="L139" s="47">
+        <f>IF(ISBLANK(D139), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M139" s="48">
+        <f>IF(ISBLANK(D139), "", IF(ISBLANK(I139), '⚙️ 全局核算参数 (Config)'!$B$13, I139))</f>
+      </c>
+      <c r="N139" s="49">
+        <f>IF(ISBLANK(D139), "", ROUND(((D139 * (1 + M139) + L139) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O139" s="50">
+        <f>IF(OR(ISBLANK(D139), NOT(AND(G139&gt;0, F139&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G139)) * F139)</f>
+      </c>
+      <c r="P139" s="50">
+        <f>IF(OR(ISBLANK(D139), NOT(AND(G139&gt;0, F139&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G139)) * F139)</f>
+      </c>
+      <c r="Q139" s="51">
+        <f>IF(ISBLANK(D139), "", IF(M139&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M139&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="140" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A140" s="39"/>
+      <c r="B140" s="40"/>
+      <c r="C140" s="41"/>
+      <c r="D140" s="42"/>
+      <c r="E140" s="43"/>
+      <c r="F140" s="43"/>
+      <c r="G140" s="44"/>
+      <c r="H140" s="45"/>
+      <c r="I140" s="46"/>
+      <c r="J140" s="39"/>
+      <c r="K140" s="39"/>
+      <c r="L140" s="47">
+        <f>IF(ISBLANK(D140), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M140" s="48">
+        <f>IF(ISBLANK(D140), "", IF(ISBLANK(I140), '⚙️ 全局核算参数 (Config)'!$B$13, I140))</f>
+      </c>
+      <c r="N140" s="49">
+        <f>IF(ISBLANK(D140), "", ROUND(((D140 * (1 + M140) + L140) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O140" s="50">
+        <f>IF(OR(ISBLANK(D140), NOT(AND(G140&gt;0, F140&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G140)) * F140)</f>
+      </c>
+      <c r="P140" s="50">
+        <f>IF(OR(ISBLANK(D140), NOT(AND(G140&gt;0, F140&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G140)) * F140)</f>
+      </c>
+      <c r="Q140" s="51">
+        <f>IF(ISBLANK(D140), "", IF(M140&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M140&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="141" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A141" s="52"/>
+      <c r="B141" s="53"/>
+      <c r="C141" s="54"/>
+      <c r="D141" s="55"/>
+      <c r="E141" s="56"/>
+      <c r="F141" s="56"/>
+      <c r="G141" s="57"/>
+      <c r="H141" s="58"/>
+      <c r="I141" s="59"/>
+      <c r="J141" s="52"/>
+      <c r="K141" s="52"/>
+      <c r="L141" s="47">
+        <f>IF(ISBLANK(D141), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M141" s="48">
+        <f>IF(ISBLANK(D141), "", IF(ISBLANK(I141), '⚙️ 全局核算参数 (Config)'!$B$13, I141))</f>
+      </c>
+      <c r="N141" s="49">
+        <f>IF(ISBLANK(D141), "", ROUND(((D141 * (1 + M141) + L141) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O141" s="50">
+        <f>IF(OR(ISBLANK(D141), NOT(AND(G141&gt;0, F141&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G141)) * F141)</f>
+      </c>
+      <c r="P141" s="50">
+        <f>IF(OR(ISBLANK(D141), NOT(AND(G141&gt;0, F141&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G141)) * F141)</f>
+      </c>
+      <c r="Q141" s="51">
+        <f>IF(ISBLANK(D141), "", IF(M141&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M141&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="142" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A142" s="39"/>
+      <c r="B142" s="40"/>
+      <c r="C142" s="41"/>
+      <c r="D142" s="42"/>
+      <c r="E142" s="43"/>
+      <c r="F142" s="43"/>
+      <c r="G142" s="44"/>
+      <c r="H142" s="45"/>
+      <c r="I142" s="46"/>
+      <c r="J142" s="39"/>
+      <c r="K142" s="39"/>
+      <c r="L142" s="47">
+        <f>IF(ISBLANK(D142), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M142" s="48">
+        <f>IF(ISBLANK(D142), "", IF(ISBLANK(I142), '⚙️ 全局核算参数 (Config)'!$B$13, I142))</f>
+      </c>
+      <c r="N142" s="49">
+        <f>IF(ISBLANK(D142), "", ROUND(((D142 * (1 + M142) + L142) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O142" s="50">
+        <f>IF(OR(ISBLANK(D142), NOT(AND(G142&gt;0, F142&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G142)) * F142)</f>
+      </c>
+      <c r="P142" s="50">
+        <f>IF(OR(ISBLANK(D142), NOT(AND(G142&gt;0, F142&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G142)) * F142)</f>
+      </c>
+      <c r="Q142" s="51">
+        <f>IF(ISBLANK(D142), "", IF(M142&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M142&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="143" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A143" s="52"/>
+      <c r="B143" s="53"/>
+      <c r="C143" s="54"/>
+      <c r="D143" s="55"/>
+      <c r="E143" s="56"/>
+      <c r="F143" s="56"/>
+      <c r="G143" s="57"/>
+      <c r="H143" s="58"/>
+      <c r="I143" s="59"/>
+      <c r="J143" s="52"/>
+      <c r="K143" s="52"/>
+      <c r="L143" s="47">
+        <f>IF(ISBLANK(D143), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M143" s="48">
+        <f>IF(ISBLANK(D143), "", IF(ISBLANK(I143), '⚙️ 全局核算参数 (Config)'!$B$13, I143))</f>
+      </c>
+      <c r="N143" s="49">
+        <f>IF(ISBLANK(D143), "", ROUND(((D143 * (1 + M143) + L143) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O143" s="50">
+        <f>IF(OR(ISBLANK(D143), NOT(AND(G143&gt;0, F143&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G143)) * F143)</f>
+      </c>
+      <c r="P143" s="50">
+        <f>IF(OR(ISBLANK(D143), NOT(AND(G143&gt;0, F143&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G143)) * F143)</f>
+      </c>
+      <c r="Q143" s="51">
+        <f>IF(ISBLANK(D143), "", IF(M143&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M143&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="144" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A144" s="39"/>
+      <c r="B144" s="40"/>
+      <c r="C144" s="41"/>
+      <c r="D144" s="42"/>
+      <c r="E144" s="43"/>
+      <c r="F144" s="43"/>
+      <c r="G144" s="44"/>
+      <c r="H144" s="45"/>
+      <c r="I144" s="46"/>
+      <c r="J144" s="39"/>
+      <c r="K144" s="39"/>
+      <c r="L144" s="47">
+        <f>IF(ISBLANK(D144), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M144" s="48">
+        <f>IF(ISBLANK(D144), "", IF(ISBLANK(I144), '⚙️ 全局核算参数 (Config)'!$B$13, I144))</f>
+      </c>
+      <c r="N144" s="49">
+        <f>IF(ISBLANK(D144), "", ROUND(((D144 * (1 + M144) + L144) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O144" s="50">
+        <f>IF(OR(ISBLANK(D144), NOT(AND(G144&gt;0, F144&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G144)) * F144)</f>
+      </c>
+      <c r="P144" s="50">
+        <f>IF(OR(ISBLANK(D144), NOT(AND(G144&gt;0, F144&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G144)) * F144)</f>
+      </c>
+      <c r="Q144" s="51">
+        <f>IF(ISBLANK(D144), "", IF(M144&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M144&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="145" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A145" s="52"/>
+      <c r="B145" s="53"/>
+      <c r="C145" s="54"/>
+      <c r="D145" s="55"/>
+      <c r="E145" s="56"/>
+      <c r="F145" s="56"/>
+      <c r="G145" s="57"/>
+      <c r="H145" s="58"/>
+      <c r="I145" s="59"/>
+      <c r="J145" s="52"/>
+      <c r="K145" s="52"/>
+      <c r="L145" s="47">
+        <f>IF(ISBLANK(D145), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M145" s="48">
+        <f>IF(ISBLANK(D145), "", IF(ISBLANK(I145), '⚙️ 全局核算参数 (Config)'!$B$13, I145))</f>
+      </c>
+      <c r="N145" s="49">
+        <f>IF(ISBLANK(D145), "", ROUND(((D145 * (1 + M145) + L145) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O145" s="50">
+        <f>IF(OR(ISBLANK(D145), NOT(AND(G145&gt;0, F145&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G145)) * F145)</f>
+      </c>
+      <c r="P145" s="50">
+        <f>IF(OR(ISBLANK(D145), NOT(AND(G145&gt;0, F145&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G145)) * F145)</f>
+      </c>
+      <c r="Q145" s="51">
+        <f>IF(ISBLANK(D145), "", IF(M145&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M145&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="146" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A146" s="39"/>
+      <c r="B146" s="40"/>
+      <c r="C146" s="41"/>
+      <c r="D146" s="42"/>
+      <c r="E146" s="43"/>
+      <c r="F146" s="43"/>
+      <c r="G146" s="44"/>
+      <c r="H146" s="45"/>
+      <c r="I146" s="46"/>
+      <c r="J146" s="39"/>
+      <c r="K146" s="39"/>
+      <c r="L146" s="47">
+        <f>IF(ISBLANK(D146), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M146" s="48">
+        <f>IF(ISBLANK(D146), "", IF(ISBLANK(I146), '⚙️ 全局核算参数 (Config)'!$B$13, I146))</f>
+      </c>
+      <c r="N146" s="49">
+        <f>IF(ISBLANK(D146), "", ROUND(((D146 * (1 + M146) + L146) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O146" s="50">
+        <f>IF(OR(ISBLANK(D146), NOT(AND(G146&gt;0, F146&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G146)) * F146)</f>
+      </c>
+      <c r="P146" s="50">
+        <f>IF(OR(ISBLANK(D146), NOT(AND(G146&gt;0, F146&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G146)) * F146)</f>
+      </c>
+      <c r="Q146" s="51">
+        <f>IF(ISBLANK(D146), "", IF(M146&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M146&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="147" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A147" s="52"/>
+      <c r="B147" s="53"/>
+      <c r="C147" s="54"/>
+      <c r="D147" s="55"/>
+      <c r="E147" s="56"/>
+      <c r="F147" s="56"/>
+      <c r="G147" s="57"/>
+      <c r="H147" s="58"/>
+      <c r="I147" s="59"/>
+      <c r="J147" s="52"/>
+      <c r="K147" s="52"/>
+      <c r="L147" s="47">
+        <f>IF(ISBLANK(D147), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M147" s="48">
+        <f>IF(ISBLANK(D147), "", IF(ISBLANK(I147), '⚙️ 全局核算参数 (Config)'!$B$13, I147))</f>
+      </c>
+      <c r="N147" s="49">
+        <f>IF(ISBLANK(D147), "", ROUND(((D147 * (1 + M147) + L147) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O147" s="50">
+        <f>IF(OR(ISBLANK(D147), NOT(AND(G147&gt;0, F147&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G147)) * F147)</f>
+      </c>
+      <c r="P147" s="50">
+        <f>IF(OR(ISBLANK(D147), NOT(AND(G147&gt;0, F147&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G147)) * F147)</f>
+      </c>
+      <c r="Q147" s="51">
+        <f>IF(ISBLANK(D147), "", IF(M147&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M147&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="148" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A148" s="39"/>
+      <c r="B148" s="40"/>
+      <c r="C148" s="41"/>
+      <c r="D148" s="42"/>
+      <c r="E148" s="43"/>
+      <c r="F148" s="43"/>
+      <c r="G148" s="44"/>
+      <c r="H148" s="45"/>
+      <c r="I148" s="46"/>
+      <c r="J148" s="39"/>
+      <c r="K148" s="39"/>
+      <c r="L148" s="47">
+        <f>IF(ISBLANK(D148), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M148" s="48">
+        <f>IF(ISBLANK(D148), "", IF(ISBLANK(I148), '⚙️ 全局核算参数 (Config)'!$B$13, I148))</f>
+      </c>
+      <c r="N148" s="49">
+        <f>IF(ISBLANK(D148), "", ROUND(((D148 * (1 + M148) + L148) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O148" s="50">
+        <f>IF(OR(ISBLANK(D148), NOT(AND(G148&gt;0, F148&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G148)) * F148)</f>
+      </c>
+      <c r="P148" s="50">
+        <f>IF(OR(ISBLANK(D148), NOT(AND(G148&gt;0, F148&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G148)) * F148)</f>
+      </c>
+      <c r="Q148" s="51">
+        <f>IF(ISBLANK(D148), "", IF(M148&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M148&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="149" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A149" s="52"/>
+      <c r="B149" s="53"/>
+      <c r="C149" s="54"/>
+      <c r="D149" s="55"/>
+      <c r="E149" s="56"/>
+      <c r="F149" s="56"/>
+      <c r="G149" s="57"/>
+      <c r="H149" s="58"/>
+      <c r="I149" s="59"/>
+      <c r="J149" s="52"/>
+      <c r="K149" s="52"/>
+      <c r="L149" s="47">
+        <f>IF(ISBLANK(D149), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M149" s="48">
+        <f>IF(ISBLANK(D149), "", IF(ISBLANK(I149), '⚙️ 全局核算参数 (Config)'!$B$13, I149))</f>
+      </c>
+      <c r="N149" s="49">
+        <f>IF(ISBLANK(D149), "", ROUND(((D149 * (1 + M149) + L149) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O149" s="50">
+        <f>IF(OR(ISBLANK(D149), NOT(AND(G149&gt;0, F149&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G149)) * F149)</f>
+      </c>
+      <c r="P149" s="50">
+        <f>IF(OR(ISBLANK(D149), NOT(AND(G149&gt;0, F149&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G149)) * F149)</f>
+      </c>
+      <c r="Q149" s="51">
+        <f>IF(ISBLANK(D149), "", IF(M149&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M149&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="150" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A150" s="39"/>
+      <c r="B150" s="40"/>
+      <c r="C150" s="41"/>
+      <c r="D150" s="42"/>
+      <c r="E150" s="43"/>
+      <c r="F150" s="43"/>
+      <c r="G150" s="44"/>
+      <c r="H150" s="45"/>
+      <c r="I150" s="46"/>
+      <c r="J150" s="39"/>
+      <c r="K150" s="39"/>
+      <c r="L150" s="47">
+        <f>IF(ISBLANK(D150), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M150" s="48">
+        <f>IF(ISBLANK(D150), "", IF(ISBLANK(I150), '⚙️ 全局核算参数 (Config)'!$B$13, I150))</f>
+      </c>
+      <c r="N150" s="49">
+        <f>IF(ISBLANK(D150), "", ROUND(((D150 * (1 + M150) + L150) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O150" s="50">
+        <f>IF(OR(ISBLANK(D150), NOT(AND(G150&gt;0, F150&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G150)) * F150)</f>
+      </c>
+      <c r="P150" s="50">
+        <f>IF(OR(ISBLANK(D150), NOT(AND(G150&gt;0, F150&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G150)) * F150)</f>
+      </c>
+      <c r="Q150" s="51">
+        <f>IF(ISBLANK(D150), "", IF(M150&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M150&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
+    <row r="151" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A151" s="52"/>
+      <c r="B151" s="53"/>
+      <c r="C151" s="54"/>
+      <c r="D151" s="55"/>
+      <c r="E151" s="56"/>
+      <c r="F151" s="56"/>
+      <c r="G151" s="57"/>
+      <c r="H151" s="58"/>
+      <c r="I151" s="59"/>
+      <c r="J151" s="52"/>
+      <c r="K151" s="52"/>
+      <c r="L151" s="47">
+        <f>IF(ISBLANK(D151), "", '⚙️ 全局核算参数 (Config)'!$C$21)</f>
+      </c>
+      <c r="M151" s="48">
+        <f>IF(ISBLANK(D151), "", IF(ISBLANK(I151), '⚙️ 全局核算参数 (Config)'!$B$13, I151))</f>
+      </c>
+      <c r="N151" s="49">
+        <f>IF(ISBLANK(D151), "", ROUND(((D151 * (1 + M151) + L151) / '⚙️ 全局核算参数 (Config)'!$C$4), 2))</f>
+      </c>
+      <c r="O151" s="50">
+        <f>IF(OR(ISBLANK(D151), NOT(AND(G151&gt;0, F151&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$32 / G151)) * F151)</f>
+      </c>
+      <c r="P151" s="50">
+        <f>IF(OR(ISBLANK(D151), NOT(AND(G151&gt;0, F151&gt;0))), "", INT(('⚙️ 全局核算参数 (Config)'!$B$34 / G151)) * F151)</f>
+      </c>
+      <c r="Q151" s="51">
+        <f>IF(ISBLANK(D151), "", IF(M151&lt;'⚙️ 全局核算参数 (Config)'!$B$14, "🚨 穿透红线", IF(M151&gt;=0.25, "💎 高毛利款", "✅ 利润健康")))</f>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -5168,7 +6718,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I153"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -8143,6 +9693,1456 @@
         <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A101), "", '📦 商品出厂底价库 (Products)'!J101)</f>
       </c>
     </row>
+    <row r="104" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A102), "", 101)</f>
+      </c>
+      <c r="B104" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A102), "", '📦 商品出厂底价库 (Products)'!A102)</f>
+      </c>
+      <c r="C104" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A102), "", '📦 商品出厂底价库 (Products)'!C102)</f>
+      </c>
+      <c r="D104" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A102), "", '📦 商品出厂底价库 (Products)'!E102)</f>
+      </c>
+      <c r="E104" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A102), "", '📦 商品出厂底价库 (Products)'!N102)</f>
+      </c>
+      <c r="F104" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A102), "", '📦 商品出厂底价库 (Products)'!F102)</f>
+      </c>
+      <c r="G104" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A102), "", '📦 商品出厂底价库 (Products)'!O102)</f>
+      </c>
+      <c r="H104" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A102), "", '📦 商品出厂底价库 (Products)'!P102)</f>
+      </c>
+      <c r="I104" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A102), "", '📦 商品出厂底价库 (Products)'!J102)</f>
+      </c>
+    </row>
+    <row r="105" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A103), "", 102)</f>
+      </c>
+      <c r="B105" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A103), "", '📦 商品出厂底价库 (Products)'!A103)</f>
+      </c>
+      <c r="C105" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A103), "", '📦 商品出厂底价库 (Products)'!C103)</f>
+      </c>
+      <c r="D105" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A103), "", '📦 商品出厂底价库 (Products)'!E103)</f>
+      </c>
+      <c r="E105" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A103), "", '📦 商品出厂底价库 (Products)'!N103)</f>
+      </c>
+      <c r="F105" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A103), "", '📦 商品出厂底价库 (Products)'!F103)</f>
+      </c>
+      <c r="G105" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A103), "", '📦 商品出厂底价库 (Products)'!O103)</f>
+      </c>
+      <c r="H105" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A103), "", '📦 商品出厂底价库 (Products)'!P103)</f>
+      </c>
+      <c r="I105" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A103), "", '📦 商品出厂底价库 (Products)'!J103)</f>
+      </c>
+    </row>
+    <row r="106" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A104), "", 103)</f>
+      </c>
+      <c r="B106" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A104), "", '📦 商品出厂底价库 (Products)'!A104)</f>
+      </c>
+      <c r="C106" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A104), "", '📦 商品出厂底价库 (Products)'!C104)</f>
+      </c>
+      <c r="D106" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A104), "", '📦 商品出厂底价库 (Products)'!E104)</f>
+      </c>
+      <c r="E106" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A104), "", '📦 商品出厂底价库 (Products)'!N104)</f>
+      </c>
+      <c r="F106" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A104), "", '📦 商品出厂底价库 (Products)'!F104)</f>
+      </c>
+      <c r="G106" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A104), "", '📦 商品出厂底价库 (Products)'!O104)</f>
+      </c>
+      <c r="H106" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A104), "", '📦 商品出厂底价库 (Products)'!P104)</f>
+      </c>
+      <c r="I106" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A104), "", '📦 商品出厂底价库 (Products)'!J104)</f>
+      </c>
+    </row>
+    <row r="107" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A105), "", 104)</f>
+      </c>
+      <c r="B107" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A105), "", '📦 商品出厂底价库 (Products)'!A105)</f>
+      </c>
+      <c r="C107" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A105), "", '📦 商品出厂底价库 (Products)'!C105)</f>
+      </c>
+      <c r="D107" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A105), "", '📦 商品出厂底价库 (Products)'!E105)</f>
+      </c>
+      <c r="E107" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A105), "", '📦 商品出厂底价库 (Products)'!N105)</f>
+      </c>
+      <c r="F107" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A105), "", '📦 商品出厂底价库 (Products)'!F105)</f>
+      </c>
+      <c r="G107" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A105), "", '📦 商品出厂底价库 (Products)'!O105)</f>
+      </c>
+      <c r="H107" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A105), "", '📦 商品出厂底价库 (Products)'!P105)</f>
+      </c>
+      <c r="I107" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A105), "", '📦 商品出厂底价库 (Products)'!J105)</f>
+      </c>
+    </row>
+    <row r="108" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A106), "", 105)</f>
+      </c>
+      <c r="B108" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A106), "", '📦 商品出厂底价库 (Products)'!A106)</f>
+      </c>
+      <c r="C108" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A106), "", '📦 商品出厂底价库 (Products)'!C106)</f>
+      </c>
+      <c r="D108" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A106), "", '📦 商品出厂底价库 (Products)'!E106)</f>
+      </c>
+      <c r="E108" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A106), "", '📦 商品出厂底价库 (Products)'!N106)</f>
+      </c>
+      <c r="F108" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A106), "", '📦 商品出厂底价库 (Products)'!F106)</f>
+      </c>
+      <c r="G108" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A106), "", '📦 商品出厂底价库 (Products)'!O106)</f>
+      </c>
+      <c r="H108" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A106), "", '📦 商品出厂底价库 (Products)'!P106)</f>
+      </c>
+      <c r="I108" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A106), "", '📦 商品出厂底价库 (Products)'!J106)</f>
+      </c>
+    </row>
+    <row r="109" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A107), "", 106)</f>
+      </c>
+      <c r="B109" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A107), "", '📦 商品出厂底价库 (Products)'!A107)</f>
+      </c>
+      <c r="C109" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A107), "", '📦 商品出厂底价库 (Products)'!C107)</f>
+      </c>
+      <c r="D109" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A107), "", '📦 商品出厂底价库 (Products)'!E107)</f>
+      </c>
+      <c r="E109" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A107), "", '📦 商品出厂底价库 (Products)'!N107)</f>
+      </c>
+      <c r="F109" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A107), "", '📦 商品出厂底价库 (Products)'!F107)</f>
+      </c>
+      <c r="G109" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A107), "", '📦 商品出厂底价库 (Products)'!O107)</f>
+      </c>
+      <c r="H109" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A107), "", '📦 商品出厂底价库 (Products)'!P107)</f>
+      </c>
+      <c r="I109" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A107), "", '📦 商品出厂底价库 (Products)'!J107)</f>
+      </c>
+    </row>
+    <row r="110" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A108), "", 107)</f>
+      </c>
+      <c r="B110" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A108), "", '📦 商品出厂底价库 (Products)'!A108)</f>
+      </c>
+      <c r="C110" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A108), "", '📦 商品出厂底价库 (Products)'!C108)</f>
+      </c>
+      <c r="D110" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A108), "", '📦 商品出厂底价库 (Products)'!E108)</f>
+      </c>
+      <c r="E110" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A108), "", '📦 商品出厂底价库 (Products)'!N108)</f>
+      </c>
+      <c r="F110" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A108), "", '📦 商品出厂底价库 (Products)'!F108)</f>
+      </c>
+      <c r="G110" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A108), "", '📦 商品出厂底价库 (Products)'!O108)</f>
+      </c>
+      <c r="H110" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A108), "", '📦 商品出厂底价库 (Products)'!P108)</f>
+      </c>
+      <c r="I110" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A108), "", '📦 商品出厂底价库 (Products)'!J108)</f>
+      </c>
+    </row>
+    <row r="111" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A109), "", 108)</f>
+      </c>
+      <c r="B111" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A109), "", '📦 商品出厂底价库 (Products)'!A109)</f>
+      </c>
+      <c r="C111" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A109), "", '📦 商品出厂底价库 (Products)'!C109)</f>
+      </c>
+      <c r="D111" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A109), "", '📦 商品出厂底价库 (Products)'!E109)</f>
+      </c>
+      <c r="E111" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A109), "", '📦 商品出厂底价库 (Products)'!N109)</f>
+      </c>
+      <c r="F111" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A109), "", '📦 商品出厂底价库 (Products)'!F109)</f>
+      </c>
+      <c r="G111" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A109), "", '📦 商品出厂底价库 (Products)'!O109)</f>
+      </c>
+      <c r="H111" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A109), "", '📦 商品出厂底价库 (Products)'!P109)</f>
+      </c>
+      <c r="I111" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A109), "", '📦 商品出厂底价库 (Products)'!J109)</f>
+      </c>
+    </row>
+    <row r="112" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A112" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A110), "", 109)</f>
+      </c>
+      <c r="B112" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A110), "", '📦 商品出厂底价库 (Products)'!A110)</f>
+      </c>
+      <c r="C112" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A110), "", '📦 商品出厂底价库 (Products)'!C110)</f>
+      </c>
+      <c r="D112" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A110), "", '📦 商品出厂底价库 (Products)'!E110)</f>
+      </c>
+      <c r="E112" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A110), "", '📦 商品出厂底价库 (Products)'!N110)</f>
+      </c>
+      <c r="F112" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A110), "", '📦 商品出厂底价库 (Products)'!F110)</f>
+      </c>
+      <c r="G112" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A110), "", '📦 商品出厂底价库 (Products)'!O110)</f>
+      </c>
+      <c r="H112" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A110), "", '📦 商品出厂底价库 (Products)'!P110)</f>
+      </c>
+      <c r="I112" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A110), "", '📦 商品出厂底价库 (Products)'!J110)</f>
+      </c>
+    </row>
+    <row r="113" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A111), "", 110)</f>
+      </c>
+      <c r="B113" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A111), "", '📦 商品出厂底价库 (Products)'!A111)</f>
+      </c>
+      <c r="C113" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A111), "", '📦 商品出厂底价库 (Products)'!C111)</f>
+      </c>
+      <c r="D113" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A111), "", '📦 商品出厂底价库 (Products)'!E111)</f>
+      </c>
+      <c r="E113" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A111), "", '📦 商品出厂底价库 (Products)'!N111)</f>
+      </c>
+      <c r="F113" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A111), "", '📦 商品出厂底价库 (Products)'!F111)</f>
+      </c>
+      <c r="G113" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A111), "", '📦 商品出厂底价库 (Products)'!O111)</f>
+      </c>
+      <c r="H113" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A111), "", '📦 商品出厂底价库 (Products)'!P111)</f>
+      </c>
+      <c r="I113" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A111), "", '📦 商品出厂底价库 (Products)'!J111)</f>
+      </c>
+    </row>
+    <row r="114" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A112), "", 111)</f>
+      </c>
+      <c r="B114" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A112), "", '📦 商品出厂底价库 (Products)'!A112)</f>
+      </c>
+      <c r="C114" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A112), "", '📦 商品出厂底价库 (Products)'!C112)</f>
+      </c>
+      <c r="D114" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A112), "", '📦 商品出厂底价库 (Products)'!E112)</f>
+      </c>
+      <c r="E114" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A112), "", '📦 商品出厂底价库 (Products)'!N112)</f>
+      </c>
+      <c r="F114" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A112), "", '📦 商品出厂底价库 (Products)'!F112)</f>
+      </c>
+      <c r="G114" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A112), "", '📦 商品出厂底价库 (Products)'!O112)</f>
+      </c>
+      <c r="H114" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A112), "", '📦 商品出厂底价库 (Products)'!P112)</f>
+      </c>
+      <c r="I114" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A112), "", '📦 商品出厂底价库 (Products)'!J112)</f>
+      </c>
+    </row>
+    <row r="115" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A115" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A113), "", 112)</f>
+      </c>
+      <c r="B115" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A113), "", '📦 商品出厂底价库 (Products)'!A113)</f>
+      </c>
+      <c r="C115" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A113), "", '📦 商品出厂底价库 (Products)'!C113)</f>
+      </c>
+      <c r="D115" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A113), "", '📦 商品出厂底价库 (Products)'!E113)</f>
+      </c>
+      <c r="E115" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A113), "", '📦 商品出厂底价库 (Products)'!N113)</f>
+      </c>
+      <c r="F115" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A113), "", '📦 商品出厂底价库 (Products)'!F113)</f>
+      </c>
+      <c r="G115" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A113), "", '📦 商品出厂底价库 (Products)'!O113)</f>
+      </c>
+      <c r="H115" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A113), "", '📦 商品出厂底价库 (Products)'!P113)</f>
+      </c>
+      <c r="I115" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A113), "", '📦 商品出厂底价库 (Products)'!J113)</f>
+      </c>
+    </row>
+    <row r="116" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A116" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A114), "", 113)</f>
+      </c>
+      <c r="B116" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A114), "", '📦 商品出厂底价库 (Products)'!A114)</f>
+      </c>
+      <c r="C116" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A114), "", '📦 商品出厂底价库 (Products)'!C114)</f>
+      </c>
+      <c r="D116" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A114), "", '📦 商品出厂底价库 (Products)'!E114)</f>
+      </c>
+      <c r="E116" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A114), "", '📦 商品出厂底价库 (Products)'!N114)</f>
+      </c>
+      <c r="F116" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A114), "", '📦 商品出厂底价库 (Products)'!F114)</f>
+      </c>
+      <c r="G116" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A114), "", '📦 商品出厂底价库 (Products)'!O114)</f>
+      </c>
+      <c r="H116" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A114), "", '📦 商品出厂底价库 (Products)'!P114)</f>
+      </c>
+      <c r="I116" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A114), "", '📦 商品出厂底价库 (Products)'!J114)</f>
+      </c>
+    </row>
+    <row r="117" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A117" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A115), "", 114)</f>
+      </c>
+      <c r="B117" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A115), "", '📦 商品出厂底价库 (Products)'!A115)</f>
+      </c>
+      <c r="C117" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A115), "", '📦 商品出厂底价库 (Products)'!C115)</f>
+      </c>
+      <c r="D117" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A115), "", '📦 商品出厂底价库 (Products)'!E115)</f>
+      </c>
+      <c r="E117" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A115), "", '📦 商品出厂底价库 (Products)'!N115)</f>
+      </c>
+      <c r="F117" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A115), "", '📦 商品出厂底价库 (Products)'!F115)</f>
+      </c>
+      <c r="G117" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A115), "", '📦 商品出厂底价库 (Products)'!O115)</f>
+      </c>
+      <c r="H117" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A115), "", '📦 商品出厂底价库 (Products)'!P115)</f>
+      </c>
+      <c r="I117" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A115), "", '📦 商品出厂底价库 (Products)'!J115)</f>
+      </c>
+    </row>
+    <row r="118" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A118" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A116), "", 115)</f>
+      </c>
+      <c r="B118" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A116), "", '📦 商品出厂底价库 (Products)'!A116)</f>
+      </c>
+      <c r="C118" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A116), "", '📦 商品出厂底价库 (Products)'!C116)</f>
+      </c>
+      <c r="D118" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A116), "", '📦 商品出厂底价库 (Products)'!E116)</f>
+      </c>
+      <c r="E118" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A116), "", '📦 商品出厂底价库 (Products)'!N116)</f>
+      </c>
+      <c r="F118" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A116), "", '📦 商品出厂底价库 (Products)'!F116)</f>
+      </c>
+      <c r="G118" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A116), "", '📦 商品出厂底价库 (Products)'!O116)</f>
+      </c>
+      <c r="H118" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A116), "", '📦 商品出厂底价库 (Products)'!P116)</f>
+      </c>
+      <c r="I118" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A116), "", '📦 商品出厂底价库 (Products)'!J116)</f>
+      </c>
+    </row>
+    <row r="119" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A119" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A117), "", 116)</f>
+      </c>
+      <c r="B119" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A117), "", '📦 商品出厂底价库 (Products)'!A117)</f>
+      </c>
+      <c r="C119" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A117), "", '📦 商品出厂底价库 (Products)'!C117)</f>
+      </c>
+      <c r="D119" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A117), "", '📦 商品出厂底价库 (Products)'!E117)</f>
+      </c>
+      <c r="E119" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A117), "", '📦 商品出厂底价库 (Products)'!N117)</f>
+      </c>
+      <c r="F119" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A117), "", '📦 商品出厂底价库 (Products)'!F117)</f>
+      </c>
+      <c r="G119" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A117), "", '📦 商品出厂底价库 (Products)'!O117)</f>
+      </c>
+      <c r="H119" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A117), "", '📦 商品出厂底价库 (Products)'!P117)</f>
+      </c>
+      <c r="I119" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A117), "", '📦 商品出厂底价库 (Products)'!J117)</f>
+      </c>
+    </row>
+    <row r="120" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A120" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A118), "", 117)</f>
+      </c>
+      <c r="B120" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A118), "", '📦 商品出厂底价库 (Products)'!A118)</f>
+      </c>
+      <c r="C120" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A118), "", '📦 商品出厂底价库 (Products)'!C118)</f>
+      </c>
+      <c r="D120" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A118), "", '📦 商品出厂底价库 (Products)'!E118)</f>
+      </c>
+      <c r="E120" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A118), "", '📦 商品出厂底价库 (Products)'!N118)</f>
+      </c>
+      <c r="F120" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A118), "", '📦 商品出厂底价库 (Products)'!F118)</f>
+      </c>
+      <c r="G120" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A118), "", '📦 商品出厂底价库 (Products)'!O118)</f>
+      </c>
+      <c r="H120" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A118), "", '📦 商品出厂底价库 (Products)'!P118)</f>
+      </c>
+      <c r="I120" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A118), "", '📦 商品出厂底价库 (Products)'!J118)</f>
+      </c>
+    </row>
+    <row r="121" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A121" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A119), "", 118)</f>
+      </c>
+      <c r="B121" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A119), "", '📦 商品出厂底价库 (Products)'!A119)</f>
+      </c>
+      <c r="C121" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A119), "", '📦 商品出厂底价库 (Products)'!C119)</f>
+      </c>
+      <c r="D121" s="71">
+        <f>IF(ISBLANK('�� 商品出厂底价库 (Products)'!A119), "", '📦 商品出厂底价库 (Products)'!E119)</f>
+      </c>
+      <c r="E121" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A119), "", '📦 商品出厂底价库 (Products)'!N119)</f>
+      </c>
+      <c r="F121" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A119), "", '📦 商品出厂底价库 (Products)'!F119)</f>
+      </c>
+      <c r="G121" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A119), "", '📦 商品出厂底价库 (Products)'!O119)</f>
+      </c>
+      <c r="H121" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A119), "", '📦 商品出厂底价库 (Products)'!P119)</f>
+      </c>
+      <c r="I121" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A119), "", '📦 商品出厂底价库 (Products)'!J119)</f>
+      </c>
+    </row>
+    <row r="122" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A122" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A120), "", 119)</f>
+      </c>
+      <c r="B122" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A120), "", '📦 商品出厂底价库 (Products)'!A120)</f>
+      </c>
+      <c r="C122" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A120), "", '📦 商品出厂底价库 (Products)'!C120)</f>
+      </c>
+      <c r="D122" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A120), "", '📦 商品出厂底价库 (Products)'!E120)</f>
+      </c>
+      <c r="E122" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A120), "", '📦 商品出厂底价库 (Products)'!N120)</f>
+      </c>
+      <c r="F122" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A120), "", '📦 商品出厂底价库 (Products)'!F120)</f>
+      </c>
+      <c r="G122" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A120), "", '📦 商品出厂底价库 (Products)'!O120)</f>
+      </c>
+      <c r="H122" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A120), "", '📦 商品出厂底价库 (Products)'!P120)</f>
+      </c>
+      <c r="I122" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A120), "", '📦 商品出厂底价库 (Products)'!J120)</f>
+      </c>
+    </row>
+    <row r="123" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A123" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A121), "", 120)</f>
+      </c>
+      <c r="B123" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A121), "", '📦 商品出厂底价库 (Products)'!A121)</f>
+      </c>
+      <c r="C123" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A121), "", '📦 商品出厂底价库 (Products)'!C121)</f>
+      </c>
+      <c r="D123" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A121), "", '📦 商品出厂底价库 (Products)'!E121)</f>
+      </c>
+      <c r="E123" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A121), "", '📦 商品出厂底价库 (Products)'!N121)</f>
+      </c>
+      <c r="F123" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A121), "", '📦 商品出厂底价库 (Products)'!F121)</f>
+      </c>
+      <c r="G123" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A121), "", '📦 商品出厂底价库 (Products)'!O121)</f>
+      </c>
+      <c r="H123" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A121), "", '📦 商品出厂底价库 (Products)'!P121)</f>
+      </c>
+      <c r="I123" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A121), "", '📦 商品出厂底价库 (Products)'!J121)</f>
+      </c>
+    </row>
+    <row r="124" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A124" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A122), "", 121)</f>
+      </c>
+      <c r="B124" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A122), "", '📦 商品出厂底价库 (Products)'!A122)</f>
+      </c>
+      <c r="C124" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A122), "", '📦 商品出厂底价库 (Products)'!C122)</f>
+      </c>
+      <c r="D124" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A122), "", '📦 商品出厂底价库 (Products)'!E122)</f>
+      </c>
+      <c r="E124" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A122), "", '📦 商品出厂底价库 (Products)'!N122)</f>
+      </c>
+      <c r="F124" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A122), "", '📦 商品出厂底价库 (Products)'!F122)</f>
+      </c>
+      <c r="G124" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A122), "", '📦 商品出厂底价库 (Products)'!O122)</f>
+      </c>
+      <c r="H124" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A122), "", '📦 商品出厂底价库 (Products)'!P122)</f>
+      </c>
+      <c r="I124" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A122), "", '📦 商品出厂底价库 (Products)'!J122)</f>
+      </c>
+    </row>
+    <row r="125" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A125" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A123), "", 122)</f>
+      </c>
+      <c r="B125" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A123), "", '📦 商品出厂底价库 (Products)'!A123)</f>
+      </c>
+      <c r="C125" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A123), "", '📦 商品出厂底价库 (Products)'!C123)</f>
+      </c>
+      <c r="D125" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A123), "", '📦 商品出厂底价库 (Products)'!E123)</f>
+      </c>
+      <c r="E125" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A123), "", '📦 商品出厂底价库 (Products)'!N123)</f>
+      </c>
+      <c r="F125" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A123), "", '📦 商品出厂底价库 (Products)'!F123)</f>
+      </c>
+      <c r="G125" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A123), "", '📦 商品出厂底价库 (Products)'!O123)</f>
+      </c>
+      <c r="H125" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A123), "", '📦 商品出厂底价库 (Products)'!P123)</f>
+      </c>
+      <c r="I125" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A123), "", '📦 商品出厂底价库 (Products)'!J123)</f>
+      </c>
+    </row>
+    <row r="126" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A126" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A124), "", 123)</f>
+      </c>
+      <c r="B126" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A124), "", '📦 商品出厂底价库 (Products)'!A124)</f>
+      </c>
+      <c r="C126" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A124), "", '📦 商品出厂底价库 (Products)'!C124)</f>
+      </c>
+      <c r="D126" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A124), "", '📦 商品出厂底价库 (Products)'!E124)</f>
+      </c>
+      <c r="E126" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A124), "", '📦 商品出厂底价库 (Products)'!N124)</f>
+      </c>
+      <c r="F126" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A124), "", '📦 商品出厂底价库 (Products)'!F124)</f>
+      </c>
+      <c r="G126" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A124), "", '📦 商品出厂底价库 (Products)'!O124)</f>
+      </c>
+      <c r="H126" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A124), "", '📦 商品出厂底价库 (Products)'!P124)</f>
+      </c>
+      <c r="I126" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A124), "", '📦 商品出厂底价库 (Products)'!J124)</f>
+      </c>
+    </row>
+    <row r="127" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A127" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A125), "", 124)</f>
+      </c>
+      <c r="B127" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A125), "", '📦 商品出厂底价库 (Products)'!A125)</f>
+      </c>
+      <c r="C127" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A125), "", '📦 商品出厂底价库 (Products)'!C125)</f>
+      </c>
+      <c r="D127" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A125), "", '📦 商品出厂底价库 (Products)'!E125)</f>
+      </c>
+      <c r="E127" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A125), "", '📦 商品出厂底价库 (Products)'!N125)</f>
+      </c>
+      <c r="F127" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A125), "", '📦 商品出厂底价库 (Products)'!F125)</f>
+      </c>
+      <c r="G127" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A125), "", '📦 商品出厂底价库 (Products)'!O125)</f>
+      </c>
+      <c r="H127" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A125), "", '📦 商品出厂底价库 (Products)'!P125)</f>
+      </c>
+      <c r="I127" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A125), "", '📦 商品出厂底价库 (Products)'!J125)</f>
+      </c>
+    </row>
+    <row r="128" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A128" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A126), "", 125)</f>
+      </c>
+      <c r="B128" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A126), "", '📦 商品出厂底价库 (Products)'!A126)</f>
+      </c>
+      <c r="C128" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A126), "", '📦 商品出厂底价库 (Products)'!C126)</f>
+      </c>
+      <c r="D128" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A126), "", '📦 商品出厂底价库 (Products)'!E126)</f>
+      </c>
+      <c r="E128" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A126), "", '📦 商品出厂底价库 (Products)'!N126)</f>
+      </c>
+      <c r="F128" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A126), "", '📦 商品出厂底价库 (Products)'!F126)</f>
+      </c>
+      <c r="G128" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A126), "", '📦 商品出厂底价库 (Products)'!O126)</f>
+      </c>
+      <c r="H128" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A126), "", '📦 商品出厂底价库 (Products)'!P126)</f>
+      </c>
+      <c r="I128" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A126), "", '📦 商品出厂底价库 (Products)'!J126)</f>
+      </c>
+    </row>
+    <row r="129" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A129" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A127), "", 126)</f>
+      </c>
+      <c r="B129" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A127), "", '📦 商品出厂底价库 (Products)'!A127)</f>
+      </c>
+      <c r="C129" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A127), "", '📦 商品出厂底价库 (Products)'!C127)</f>
+      </c>
+      <c r="D129" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A127), "", '📦 商品出厂底价库 (Products)'!E127)</f>
+      </c>
+      <c r="E129" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A127), "", '📦 商品出厂底价库 (Products)'!N127)</f>
+      </c>
+      <c r="F129" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A127), "", '📦 商品出厂底价库 (Products)'!F127)</f>
+      </c>
+      <c r="G129" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A127), "", '📦 商品出厂底价库 (Products)'!O127)</f>
+      </c>
+      <c r="H129" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A127), "", '📦 商品出厂底价库 (Products)'!P127)</f>
+      </c>
+      <c r="I129" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A127), "", '📦 商品出厂底价库 (Products)'!J127)</f>
+      </c>
+    </row>
+    <row r="130" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A130" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A128), "", 127)</f>
+      </c>
+      <c r="B130" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A128), "", '📦 商品出厂底价库 (Products)'!A128)</f>
+      </c>
+      <c r="C130" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A128), "", '📦 商品出厂底价库 (Products)'!C128)</f>
+      </c>
+      <c r="D130" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A128), "", '📦 商品出厂底价库 (Products)'!E128)</f>
+      </c>
+      <c r="E130" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A128), "", '📦 商品出厂底价库 (Products)'!N128)</f>
+      </c>
+      <c r="F130" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A128), "", '📦 商品出厂底价库 (Products)'!F128)</f>
+      </c>
+      <c r="G130" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A128), "", '📦 商品出厂底价库 (Products)'!O128)</f>
+      </c>
+      <c r="H130" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A128), "", '📦 商品出厂底价库 (Products)'!P128)</f>
+      </c>
+      <c r="I130" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A128), "", '📦 商品出厂底价库 (Products)'!J128)</f>
+      </c>
+    </row>
+    <row r="131" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A131" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A129), "", 128)</f>
+      </c>
+      <c r="B131" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A129), "", '📦 商品出厂底价库 (Products)'!A129)</f>
+      </c>
+      <c r="C131" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A129), "", '📦 商品出厂底价库 (Products)'!C129)</f>
+      </c>
+      <c r="D131" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A129), "", '📦 商品出厂底价库 (Products)'!E129)</f>
+      </c>
+      <c r="E131" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A129), "", '📦 商品出厂底价库 (Products)'!N129)</f>
+      </c>
+      <c r="F131" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A129), "", '📦 商品出厂底价库 (Products)'!F129)</f>
+      </c>
+      <c r="G131" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A129), "", '📦 商品出厂底价库 (Products)'!O129)</f>
+      </c>
+      <c r="H131" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A129), "", '📦 商品出厂底价库 (Products)'!P129)</f>
+      </c>
+      <c r="I131" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A129), "", '📦 商品出厂底价库 (Products)'!J129)</f>
+      </c>
+    </row>
+    <row r="132" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A132" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A130), "", 129)</f>
+      </c>
+      <c r="B132" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A130), "", '📦 商品出厂底价库 (Products)'!A130)</f>
+      </c>
+      <c r="C132" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A130), "", '📦 商品出厂底价库 (Products)'!C130)</f>
+      </c>
+      <c r="D132" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A130), "", '📦 商品出厂底价库 (Products)'!E130)</f>
+      </c>
+      <c r="E132" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A130), "", '📦 商品出厂底价库 (Products)'!N130)</f>
+      </c>
+      <c r="F132" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A130), "", '📦 商品出厂底价库 (Products)'!F130)</f>
+      </c>
+      <c r="G132" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A130), "", '📦 商品出厂底价库 (Products)'!O130)</f>
+      </c>
+      <c r="H132" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A130), "", '📦 商品出厂底价库 (Products)'!P130)</f>
+      </c>
+      <c r="I132" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A130), "", '📦 商品出厂底价库 (Products)'!J130)</f>
+      </c>
+    </row>
+    <row r="133" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A133" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A131), "", 130)</f>
+      </c>
+      <c r="B133" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A131), "", '📦 商品出厂底价库 (Products)'!A131)</f>
+      </c>
+      <c r="C133" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A131), "", '📦 商品出厂底价库 (Products)'!C131)</f>
+      </c>
+      <c r="D133" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A131), "", '📦 商品出厂底价库 (Products)'!E131)</f>
+      </c>
+      <c r="E133" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A131), "", '📦 商品出厂底价库 (Products)'!N131)</f>
+      </c>
+      <c r="F133" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A131), "", '📦 商品出厂底价库 (Products)'!F131)</f>
+      </c>
+      <c r="G133" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A131), "", '📦 商品出厂底价库 (Products)'!O131)</f>
+      </c>
+      <c r="H133" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A131), "", '📦 商品出厂底价库 (Products)'!P131)</f>
+      </c>
+      <c r="I133" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A131), "", '📦 商品出厂底价库 (Products)'!J131)</f>
+      </c>
+    </row>
+    <row r="134" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A134" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A132), "", 131)</f>
+      </c>
+      <c r="B134" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A132), "", '📦 商品出厂底价库 (Products)'!A132)</f>
+      </c>
+      <c r="C134" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A132), "", '📦 商品出厂底价库 (Products)'!C132)</f>
+      </c>
+      <c r="D134" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A132), "", '📦 商品出厂底价库 (Products)'!E132)</f>
+      </c>
+      <c r="E134" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A132), "", '📦 商品出厂底价库 (Products)'!N132)</f>
+      </c>
+      <c r="F134" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A132), "", '📦 商品出厂底价库 (Products)'!F132)</f>
+      </c>
+      <c r="G134" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A132), "", '📦 商品出厂底价库 (Products)'!O132)</f>
+      </c>
+      <c r="H134" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A132), "", '📦 商品出厂底价库 (Products)'!P132)</f>
+      </c>
+      <c r="I134" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A132), "", '📦 商品出厂底价库 (Products)'!J132)</f>
+      </c>
+    </row>
+    <row r="135" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A135" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A133), "", 132)</f>
+      </c>
+      <c r="B135" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A133), "", '📦 商品出厂底价库 (Products)'!A133)</f>
+      </c>
+      <c r="C135" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A133), "", '📦 商品出厂底价库 (Products)'!C133)</f>
+      </c>
+      <c r="D135" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A133), "", '📦 商品出厂底价库 (Products)'!E133)</f>
+      </c>
+      <c r="E135" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A133), "", '📦 商品出厂底价库 (Products)'!N133)</f>
+      </c>
+      <c r="F135" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A133), "", '📦 商品出厂底价库 (Products)'!F133)</f>
+      </c>
+      <c r="G135" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A133), "", '📦 商品出厂底价库 (Products)'!O133)</f>
+      </c>
+      <c r="H135" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A133), "", '📦 商品出厂底价库 (Products)'!P133)</f>
+      </c>
+      <c r="I135" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A133), "", '📦 商品出厂底价库 (Products)'!J133)</f>
+      </c>
+    </row>
+    <row r="136" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A136" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A134), "", 133)</f>
+      </c>
+      <c r="B136" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A134), "", '📦 商品出厂底价库 (Products)'!A134)</f>
+      </c>
+      <c r="C136" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A134), "", '📦 商品出厂底价库 (Products)'!C134)</f>
+      </c>
+      <c r="D136" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A134), "", '📦 商品出厂底价库 (Products)'!E134)</f>
+      </c>
+      <c r="E136" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A134), "", '📦 商品出厂底价库 (Products)'!N134)</f>
+      </c>
+      <c r="F136" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A134), "", '📦 商品出厂底价库 (Products)'!F134)</f>
+      </c>
+      <c r="G136" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A134), "", '📦 商品出厂底价库 (Products)'!O134)</f>
+      </c>
+      <c r="H136" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A134), "", '📦 商品出厂底价库 (Products)'!P134)</f>
+      </c>
+      <c r="I136" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A134), "", '📦 商品出厂底价库 (Products)'!J134)</f>
+      </c>
+    </row>
+    <row r="137" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A137" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A135), "", 134)</f>
+      </c>
+      <c r="B137" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A135), "", '📦 商品出厂底价库 (Products)'!A135)</f>
+      </c>
+      <c r="C137" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A135), "", '📦 商品出厂底价库 (Products)'!C135)</f>
+      </c>
+      <c r="D137" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A135), "", '📦 商品出厂底价库 (Products)'!E135)</f>
+      </c>
+      <c r="E137" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A135), "", '📦 商品出厂底价库 (Products)'!N135)</f>
+      </c>
+      <c r="F137" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A135), "", '📦 商品出厂底价库 (Products)'!F135)</f>
+      </c>
+      <c r="G137" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A135), "", '📦 商品出厂底价库 (Products)'!O135)</f>
+      </c>
+      <c r="H137" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A135), "", '📦 商品出厂底价库 (Products)'!P135)</f>
+      </c>
+      <c r="I137" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A135), "", '📦 商品出厂底价库 (Products)'!J135)</f>
+      </c>
+    </row>
+    <row r="138" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A138" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A136), "", 135)</f>
+      </c>
+      <c r="B138" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A136), "", '📦 商品出厂底价库 (Products)'!A136)</f>
+      </c>
+      <c r="C138" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A136), "", '📦 商品出厂底价库 (Products)'!C136)</f>
+      </c>
+      <c r="D138" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A136), "", '📦 商品出厂底价库 (Products)'!E136)</f>
+      </c>
+      <c r="E138" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A136), "", '📦 商品出厂底价库 (Products)'!N136)</f>
+      </c>
+      <c r="F138" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A136), "", '📦 商品出厂底价库 (Products)'!F136)</f>
+      </c>
+      <c r="G138" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A136), "", '📦 商品出厂底价库 (Products)'!O136)</f>
+      </c>
+      <c r="H138" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A136), "", '📦 商品出厂底价库 (Products)'!P136)</f>
+      </c>
+      <c r="I138" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A136), "", '📦 商品出厂底价库 (Products)'!J136)</f>
+      </c>
+    </row>
+    <row r="139" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A139" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A137), "", 136)</f>
+      </c>
+      <c r="B139" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A137), "", '📦 商品出厂底价库 (Products)'!A137)</f>
+      </c>
+      <c r="C139" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A137), "", '📦 商品出厂底价库 (Products)'!C137)</f>
+      </c>
+      <c r="D139" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A137), "", '📦 商品出厂底价库 (Products)'!E137)</f>
+      </c>
+      <c r="E139" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A137), "", '📦 商品出厂底价库 (Products)'!N137)</f>
+      </c>
+      <c r="F139" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A137), "", '📦 商品出厂底价库 (Products)'!F137)</f>
+      </c>
+      <c r="G139" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A137), "", '📦 商品出厂底价库 (Products)'!O137)</f>
+      </c>
+      <c r="H139" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A137), "", '📦 商品出厂底价库 (Products)'!P137)</f>
+      </c>
+      <c r="I139" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A137), "", '📦 商品出厂底价库 (Products)'!J137)</f>
+      </c>
+    </row>
+    <row r="140" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A140" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A138), "", 137)</f>
+      </c>
+      <c r="B140" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A138), "", '📦 商品出厂底价库 (Products)'!A138)</f>
+      </c>
+      <c r="C140" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A138), "", '📦 商品出厂底价库 (Products)'!C138)</f>
+      </c>
+      <c r="D140" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A138), "", '📦 商品出厂底价库 (Products)'!E138)</f>
+      </c>
+      <c r="E140" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A138), "", '📦 商品出厂底价库 (Products)'!N138)</f>
+      </c>
+      <c r="F140" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A138), "", '📦 商品出厂底价库 (Products)'!F138)</f>
+      </c>
+      <c r="G140" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A138), "", '📦 商品出厂底价库 (Products)'!O138)</f>
+      </c>
+      <c r="H140" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A138), "", '📦 商品出厂底价库 (Products)'!P138)</f>
+      </c>
+      <c r="I140" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A138), "", '📦 商品出厂底价库 (Products)'!J138)</f>
+      </c>
+    </row>
+    <row r="141" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A141" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A139), "", 138)</f>
+      </c>
+      <c r="B141" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A139), "", '📦 商品出厂底价库 (Products)'!A139)</f>
+      </c>
+      <c r="C141" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A139), "", '📦 商品出厂底价库 (Products)'!C139)</f>
+      </c>
+      <c r="D141" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A139), "", '📦 商品出厂底价库 (Products)'!E139)</f>
+      </c>
+      <c r="E141" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A139), "", '📦 商品出厂底价库 (Products)'!N139)</f>
+      </c>
+      <c r="F141" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A139), "", '📦 商品出厂底价库 (Products)'!F139)</f>
+      </c>
+      <c r="G141" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A139), "", '📦 商品出厂底价库 (Products)'!O139)</f>
+      </c>
+      <c r="H141" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A139), "", '📦 商品出厂底价库 (Products)'!P139)</f>
+      </c>
+      <c r="I141" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A139), "", '📦 商品出厂底价库 (Products)'!J139)</f>
+      </c>
+    </row>
+    <row r="142" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A142" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A140), "", 139)</f>
+      </c>
+      <c r="B142" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A140), "", '📦 商品出厂底价库 (Products)'!A140)</f>
+      </c>
+      <c r="C142" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A140), "", '📦 商品出厂底价库 (Products)'!C140)</f>
+      </c>
+      <c r="D142" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A140), "", '📦 商品出厂底价库 (Products)'!E140)</f>
+      </c>
+      <c r="E142" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A140), "", '📦 商品出厂底价库 (Products)'!N140)</f>
+      </c>
+      <c r="F142" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A140), "", '📦 商品出厂底价库 (Products)'!F140)</f>
+      </c>
+      <c r="G142" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A140), "", '📦 商品出厂底价库 (Products)'!O140)</f>
+      </c>
+      <c r="H142" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A140), "", '📦 商品出厂底价库 (Products)'!P140)</f>
+      </c>
+      <c r="I142" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A140), "", '📦 商品出厂底价库 (Products)'!J140)</f>
+      </c>
+    </row>
+    <row r="143" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A143" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A141), "", 140)</f>
+      </c>
+      <c r="B143" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A141), "", '📦 商品出厂底价库 (Products)'!A141)</f>
+      </c>
+      <c r="C143" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A141), "", '📦 商品出厂底价库 (Products)'!C141)</f>
+      </c>
+      <c r="D143" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A141), "", '📦 商品出厂底价库 (Products)'!E141)</f>
+      </c>
+      <c r="E143" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A141), "", '📦 商品出厂底价库 (Products)'!N141)</f>
+      </c>
+      <c r="F143" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A141), "", '📦 商品出厂底价库 (Products)'!F141)</f>
+      </c>
+      <c r="G143" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A141), "", '📦 商品出厂底价库 (Products)'!O141)</f>
+      </c>
+      <c r="H143" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A141), "", '📦 商品出厂底价库 (Products)'!P141)</f>
+      </c>
+      <c r="I143" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A141), "", '📦 商品出厂底价库 (Products)'!J141)</f>
+      </c>
+    </row>
+    <row r="144" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A144" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A142), "", 141)</f>
+      </c>
+      <c r="B144" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A142), "", '📦 商品出厂底价库 (Products)'!A142)</f>
+      </c>
+      <c r="C144" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A142), "", '📦 商品出厂底价库 (Products)'!C142)</f>
+      </c>
+      <c r="D144" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A142), "", '📦 商品出厂底价库 (Products)'!E142)</f>
+      </c>
+      <c r="E144" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A142), "", '📦 商品出厂底价库 (Products)'!N142)</f>
+      </c>
+      <c r="F144" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A142), "", '📦 商品出厂底价库 (Products)'!F142)</f>
+      </c>
+      <c r="G144" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A142), "", '📦 商品出厂底价库 (Products)'!O142)</f>
+      </c>
+      <c r="H144" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A142), "", '📦 商品出厂底价库 (Products)'!P142)</f>
+      </c>
+      <c r="I144" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A142), "", '📦 商品出厂底价库 (Products)'!J142)</f>
+      </c>
+    </row>
+    <row r="145" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A145" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A143), "", 142)</f>
+      </c>
+      <c r="B145" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A143), "", '📦 商品出厂底价库 (Products)'!A143)</f>
+      </c>
+      <c r="C145" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A143), "", '📦 商品出厂底价库 (Products)'!C143)</f>
+      </c>
+      <c r="D145" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A143), "", '📦 商品出厂底价库 (Products)'!E143)</f>
+      </c>
+      <c r="E145" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A143), "", '📦 商品出厂底价库 (Products)'!N143)</f>
+      </c>
+      <c r="F145" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A143), "", '📦 商品出厂底价库 (Products)'!F143)</f>
+      </c>
+      <c r="G145" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A143), "", '📦 商品出厂底价库 (Products)'!O143)</f>
+      </c>
+      <c r="H145" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A143), "", '📦 商品出厂底价库 (Products)'!P143)</f>
+      </c>
+      <c r="I145" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A143), "", '📦 商品出厂底价库 (Products)'!J143)</f>
+      </c>
+    </row>
+    <row r="146" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A146" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A144), "", 143)</f>
+      </c>
+      <c r="B146" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A144), "", '📦 商品出厂底价库 (Products)'!A144)</f>
+      </c>
+      <c r="C146" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A144), "", '📦 商品出厂底价库 (Products)'!C144)</f>
+      </c>
+      <c r="D146" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A144), "", '📦 商品出厂底价库 (Products)'!E144)</f>
+      </c>
+      <c r="E146" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A144), "", '📦 商品出厂底价库 (Products)'!N144)</f>
+      </c>
+      <c r="F146" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A144), "", '📦 商品出厂底价库 (Products)'!F144)</f>
+      </c>
+      <c r="G146" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A144), "", '📦 商品出厂底价库 (Products)'!O144)</f>
+      </c>
+      <c r="H146" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A144), "", '📦 商品出厂底价库 (Products)'!P144)</f>
+      </c>
+      <c r="I146" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A144), "", '📦 商品出厂底价库 (Products)'!J144)</f>
+      </c>
+    </row>
+    <row r="147" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A147" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A145), "", 144)</f>
+      </c>
+      <c r="B147" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A145), "", '📦 商品出厂底价库 (Products)'!A145)</f>
+      </c>
+      <c r="C147" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A145), "", '📦 商品出厂底价库 (Products)'!C145)</f>
+      </c>
+      <c r="D147" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A145), "", '📦 商品出厂底价库 (Products)'!E145)</f>
+      </c>
+      <c r="E147" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A145), "", '📦 商品出厂底价库 (Products)'!N145)</f>
+      </c>
+      <c r="F147" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A145), "", '📦 商品出厂底价库 (Products)'!F145)</f>
+      </c>
+      <c r="G147" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A145), "", '📦 商品出厂底价库 (Products)'!O145)</f>
+      </c>
+      <c r="H147" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A145), "", '📦 商品出厂底价库 (Products)'!P145)</f>
+      </c>
+      <c r="I147" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A145), "", '📦 商品出厂底价库 (Products)'!J145)</f>
+      </c>
+    </row>
+    <row r="148" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A148" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A146), "", 145)</f>
+      </c>
+      <c r="B148" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A146), "", '📦 商品出厂底价库 (Products)'!A146)</f>
+      </c>
+      <c r="C148" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A146), "", '📦 商品出厂底价库 (Products)'!C146)</f>
+      </c>
+      <c r="D148" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A146), "", '📦 商品出厂底价库 (Products)'!E146)</f>
+      </c>
+      <c r="E148" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A146), "", '📦 商品出厂底价库 (Products)'!N146)</f>
+      </c>
+      <c r="F148" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A146), "", '📦 商品出厂底价库 (Products)'!F146)</f>
+      </c>
+      <c r="G148" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A146), "", '📦 商品出厂底价库 (Products)'!O146)</f>
+      </c>
+      <c r="H148" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A146), "", '📦 商品出厂底价库 (Products)'!P146)</f>
+      </c>
+      <c r="I148" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A146), "", '📦 商品出厂底价库 (Products)'!J146)</f>
+      </c>
+    </row>
+    <row r="149" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A149" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A147), "", 146)</f>
+      </c>
+      <c r="B149" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A147), "", '📦 商品出厂底价库 (Products)'!A147)</f>
+      </c>
+      <c r="C149" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A147), "", '📦 商品出厂底价库 (Products)'!C147)</f>
+      </c>
+      <c r="D149" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A147), "", '📦 商品出厂底价库 (Products)'!E147)</f>
+      </c>
+      <c r="E149" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A147), "", '📦 商品出厂底价库 (Products)'!N147)</f>
+      </c>
+      <c r="F149" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A147), "", '📦 商品出厂底价库 (Products)'!F147)</f>
+      </c>
+      <c r="G149" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A147), "", '📦 商品出厂底价库 (Products)'!O147)</f>
+      </c>
+      <c r="H149" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A147), "", '📦 商品出厂底价库 (Products)'!P147)</f>
+      </c>
+      <c r="I149" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A147), "", '📦 商品出厂底价库 (Products)'!J147)</f>
+      </c>
+    </row>
+    <row r="150" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A150" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A148), "", 147)</f>
+      </c>
+      <c r="B150" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A148), "", '📦 商品出厂底价库 (Products)'!A148)</f>
+      </c>
+      <c r="C150" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A148), "", '📦 商品出厂底价库 (Products)'!C148)</f>
+      </c>
+      <c r="D150" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A148), "", '📦 商品出厂底价库 (Products)'!E148)</f>
+      </c>
+      <c r="E150" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A148), "", '📦 商品出厂底价库 (Products)'!N148)</f>
+      </c>
+      <c r="F150" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A148), "", '📦 商品出厂底价库 (Products)'!F148)</f>
+      </c>
+      <c r="G150" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A148), "", '📦 商品出厂底价库 (Products)'!O148)</f>
+      </c>
+      <c r="H150" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A148), "", '📦 商品出厂底价库 (Products)'!P148)</f>
+      </c>
+      <c r="I150" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A148), "", '📦 商品出厂底价库 (Products)'!J148)</f>
+      </c>
+    </row>
+    <row r="151" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A151" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A149), "", 148)</f>
+      </c>
+      <c r="B151" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A149), "", '📦 商品出厂底价库 (Products)'!A149)</f>
+      </c>
+      <c r="C151" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A149), "", '📦 商品出厂底价库 (Products)'!C149)</f>
+      </c>
+      <c r="D151" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A149), "", '📦 商品出厂底价库 (Products)'!E149)</f>
+      </c>
+      <c r="E151" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A149), "", '📦 商品出厂底价库 (Products)'!N149)</f>
+      </c>
+      <c r="F151" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A149), "", '📦 商品出厂底价库 (Products)'!F149)</f>
+      </c>
+      <c r="G151" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A149), "", '📦 商品出厂底价库 (Products)'!O149)</f>
+      </c>
+      <c r="H151" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A149), "", '📦 商品出厂底价库 (Products)'!P149)</f>
+      </c>
+      <c r="I151" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A149), "", '📦 商品出厂底价库 (Products)'!J149)</f>
+      </c>
+    </row>
+    <row r="152" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A152" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A150), "", 149)</f>
+      </c>
+      <c r="B152" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A150), "", '📦 商品出厂底价库 (Products)'!A150)</f>
+      </c>
+      <c r="C152" s="66">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A150), "", '📦 商品出厂底价库 (Products)'!C150)</f>
+      </c>
+      <c r="D152" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A150), "", '📦 商品出厂底价库 (Products)'!E150)</f>
+      </c>
+      <c r="E152" s="68">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A150), "", '📦 商品出厂底价库 (Products)'!N150)</f>
+      </c>
+      <c r="F152" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A150), "", '📦 商品出厂底价库 (Products)'!F150)</f>
+      </c>
+      <c r="G152" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A150), "", '📦 商品出厂底价库 (Products)'!O150)</f>
+      </c>
+      <c r="H152" s="67">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A150), "", '📦 商品出厂底价库 (Products)'!P150)</f>
+      </c>
+      <c r="I152" s="65">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A150), "", '📦 商品出厂底价库 (Products)'!J150)</f>
+      </c>
+    </row>
+    <row r="153" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A153" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A151), "", 150)</f>
+      </c>
+      <c r="B153" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A151), "", '📦 商品出厂底价库 (Products)'!A151)</f>
+      </c>
+      <c r="C153" s="70">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A151), "", '📦 商品出厂底价库 (Products)'!C151)</f>
+      </c>
+      <c r="D153" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A151), "", '📦 商品出厂底价库 (Products)'!E151)</f>
+      </c>
+      <c r="E153" s="72">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A151), "", '📦 商品出厂底价库 (Products)'!N151)</f>
+      </c>
+      <c r="F153" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A151), "", '📦 商品出厂底价库 (Products)'!F151)</f>
+      </c>
+      <c r="G153" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A151), "", '📦 商品出厂底价库 (Products)'!O151)</f>
+      </c>
+      <c r="H153" s="71">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A151), "", '📦 商品出厂底价库 (Products)'!P151)</f>
+      </c>
+      <c r="I153" s="69">
+        <f>IF(ISBLANK('📦 商品出厂底价库 (Products)'!A151), "", '📦 商品出厂底价库 (Products)'!J151)</f>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:B1"/>

</xml_diff>